<commit_message>
fix(tds): expand Simple template's worked example to 3 linked entries
The worked example previously showed one Challan row + a single Entry
row, which doesn't actually demonstrate the pattern this template
exists for: one challan covering several deductees. Expanded to one
Challan row + three linked Entry rows (rows 4-7), all sharing the
example Challan ID, so a client sees the multi-entry grouping at a
glance rather than just the field formats.

Data rows now start at row 8 (was row 6); formulas, validations, and
conditional formatting ranges shifted accordingly. Re-verified
end-to-end: the real 5-entry/2-challan fixture still resolves BSR
Code/Challan No correctly with the expanded example left in place, and
the blank template still yields zero rows.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/TDS_Data_Entry_Simple_Template.xlsx
+++ b/public/templates/TDS_Data_Entry_Simple_Template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="76">
   <si>
     <t>TDS DATA ENTRY TEMPLATE (SIMPLE, CHALLAN-WISE)</t>
   </si>
@@ -41,7 +41,7 @@
     <t>One challan can have MANY entries. Just keep adding Entry rows with that Challan ID before moving to the next challan.</t>
   </si>
   <si>
-    <t>Rows 4–5 are a WORKED EXAMPLE (one Challan row + one Entry row), shown in gray. You may delete them, overwrite them, or leave them — the software recognises the example Challan ID (EXAMPLE-DO-NOT-IMPORT) and always excludes both rows from import.</t>
+    <t>Rows 4–7 are a WORKED EXAMPLE (one Challan row + THREE linked Entry rows — showing one challan covering several deductees), shown in gray. You may delete them, overwrite them, or leave them — the software recognises the example Challan ID (EXAMPLE-DO-NOT-IMPORT) and always excludes all four rows from import.</t>
   </si>
   <si>
     <t>Columns D–H (blue) are Challan-only fields — leave them blank on Entry rows. Columns I–P (yellow) are Entry-only fields — leave them blank on Challan rows.</t>
@@ -83,7 +83,7 @@
     <t>Total Challan Amount (₹)*</t>
   </si>
   <si>
-    <t>The total amount (TDS + interest, if any) actually deposited via this challan.  Example: 5,558</t>
+    <t>The total amount (TDS + interest, if any) actually deposited via this challan.  Example: 6,558</t>
   </si>
   <si>
     <t>Bank Name</t>
@@ -170,7 +170,7 @@
     <t>TDS DATA  —  each Challan row's full details, followed by its Entry rows</t>
   </si>
   <si>
-    <t>Rows 4–5 (gray) are a worked example — the example Challan ID is auto-excluded on import, so delete them, overwrite them, or leave them as-is.</t>
+    <t>Rows 4–7 (gray) are a worked example — one Challan with THREE linked entries — the example Challan ID is auto-excluded on import, so delete them, overwrite them, or leave them as-is.</t>
   </si>
   <si>
     <t>Sr. No.</t>
@@ -219,6 +219,27 @@
   </si>
   <si>
     <t>194C</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>A-ONE CHEM TRADE PVT. LTD.</t>
+  </si>
+  <si>
+    <t>AAGCA2480D</t>
+  </si>
+  <si>
+    <t>KHYATI CHEMICALS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>AAACK6277E</t>
+  </si>
+  <si>
+    <t>194J</t>
+  </si>
+  <si>
+    <t>NIL rate, LDC on file</t>
   </si>
 </sst>
 </file>
@@ -1080,7 +1101,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S205"/>
+  <dimension ref="A1:S207"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -1208,7 +1229,7 @@
         <v>46177</v>
       </c>
       <c r="G4" s="13">
-        <v>5558</v>
+        <v>6558</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>62</v>
@@ -1270,67 +1291,105 @@
       <c r="P5" s="13">
         <v>0</v>
       </c>
-      <c r="Q5" s="10"/>
+      <c r="Q5" s="10" t="s">
+        <v>69</v>
+      </c>
       <c r="R5" s="10"/>
       <c r="S5" s="10"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
-        <f>IF($B6="Entry",COUNTIF($B$6:$B6,"Entry"),"")</f>
-      </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="24"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="24"/>
-      <c r="P6" s="24"/>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="27">
-        <f>IF($B6&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C6,$O$6:$O$205)+SUMIF($C$6:$C$205,$C6,$P$6:$P$205))</f>
-      </c>
-      <c r="S6" s="27">
-        <f>IF(OR($B6&lt;&gt;"Challan",$C6="",G6=0),"",IF(ROUND(G6-R6,2)=0,"Matches","Check Entries"))</f>
-      </c>
+      <c r="A6" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="L6" s="12">
+        <v>46173</v>
+      </c>
+      <c r="M6" s="13">
+        <v>500000</v>
+      </c>
+      <c r="N6" s="14">
+        <v>0.2</v>
+      </c>
+      <c r="O6" s="13">
+        <v>1000</v>
+      </c>
+      <c r="P6" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="R6" s="10"/>
+      <c r="S6" s="10"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
-        <f>IF($B7="Entry",COUNTIF($B$6:$B7,"Entry"),"")</f>
-      </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="24"/>
-      <c r="P7" s="24"/>
-      <c r="Q7" s="26"/>
-      <c r="R7" s="27">
-        <f>IF($B7&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C7,$O$6:$O$205)+SUMIF($C$6:$C$205,$C7,$P$6:$P$205))</f>
-      </c>
-      <c r="S7" s="27">
-        <f>IF(OR($B7&lt;&gt;"Challan",$C7="",G7=0),"",IF(ROUND(G7-R7,2)=0,"Matches","Check Entries"))</f>
-      </c>
+      <c r="A7" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="L7" s="12">
+        <v>46173</v>
+      </c>
+      <c r="M7" s="13">
+        <v>100000</v>
+      </c>
+      <c r="N7" s="14">
+        <v>0</v>
+      </c>
+      <c r="O7" s="13">
+        <v>0</v>
+      </c>
+      <c r="P7" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
-        <f>IF($B8="Entry",COUNTIF($B$6:$B8,"Entry"),"")</f>
+        <f>IF($B8="Entry",COUNTIF($B$8:$B8,"Entry"),"")</f>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="17"/>
@@ -1349,7 +1408,7 @@
       <c r="P8" s="24"/>
       <c r="Q8" s="26"/>
       <c r="R8" s="27">
-        <f>IF($B8&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C8,$O$6:$O$205)+SUMIF($C$6:$C$205,$C8,$P$6:$P$205))</f>
+        <f>IF($B8&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C8,$O$8:$O$207)+SUMIF($C$8:$C$207,$C8,$P$8:$P$207))</f>
       </c>
       <c r="S8" s="27">
         <f>IF(OR($B8&lt;&gt;"Challan",$C8="",G8=0),"",IF(ROUND(G8-R8,2)=0,"Matches","Check Entries"))</f>
@@ -1357,7 +1416,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
-        <f>IF($B9="Entry",COUNTIF($B$6:$B9,"Entry"),"")</f>
+        <f>IF($B9="Entry",COUNTIF($B$8:$B9,"Entry"),"")</f>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="17"/>
@@ -1376,7 +1435,7 @@
       <c r="P9" s="24"/>
       <c r="Q9" s="26"/>
       <c r="R9" s="27">
-        <f>IF($B9&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C9,$O$6:$O$205)+SUMIF($C$6:$C$205,$C9,$P$6:$P$205))</f>
+        <f>IF($B9&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C9,$O$8:$O$207)+SUMIF($C$8:$C$207,$C9,$P$8:$P$207))</f>
       </c>
       <c r="S9" s="27">
         <f>IF(OR($B9&lt;&gt;"Challan",$C9="",G9=0),"",IF(ROUND(G9-R9,2)=0,"Matches","Check Entries"))</f>
@@ -1384,7 +1443,7 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
-        <f>IF($B10="Entry",COUNTIF($B$6:$B10,"Entry"),"")</f>
+        <f>IF($B10="Entry",COUNTIF($B$8:$B10,"Entry"),"")</f>
       </c>
       <c r="B10" s="16"/>
       <c r="C10" s="17"/>
@@ -1403,7 +1462,7 @@
       <c r="P10" s="24"/>
       <c r="Q10" s="26"/>
       <c r="R10" s="27">
-        <f>IF($B10&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C10,$O$6:$O$205)+SUMIF($C$6:$C$205,$C10,$P$6:$P$205))</f>
+        <f>IF($B10&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C10,$O$8:$O$207)+SUMIF($C$8:$C$207,$C10,$P$8:$P$207))</f>
       </c>
       <c r="S10" s="27">
         <f>IF(OR($B10&lt;&gt;"Challan",$C10="",G10=0),"",IF(ROUND(G10-R10,2)=0,"Matches","Check Entries"))</f>
@@ -1411,7 +1470,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
-        <f>IF($B11="Entry",COUNTIF($B$6:$B11,"Entry"),"")</f>
+        <f>IF($B11="Entry",COUNTIF($B$8:$B11,"Entry"),"")</f>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="17"/>
@@ -1430,7 +1489,7 @@
       <c r="P11" s="24"/>
       <c r="Q11" s="26"/>
       <c r="R11" s="27">
-        <f>IF($B11&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C11,$O$6:$O$205)+SUMIF($C$6:$C$205,$C11,$P$6:$P$205))</f>
+        <f>IF($B11&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C11,$O$8:$O$207)+SUMIF($C$8:$C$207,$C11,$P$8:$P$207))</f>
       </c>
       <c r="S11" s="27">
         <f>IF(OR($B11&lt;&gt;"Challan",$C11="",G11=0),"",IF(ROUND(G11-R11,2)=0,"Matches","Check Entries"))</f>
@@ -1438,7 +1497,7 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
-        <f>IF($B12="Entry",COUNTIF($B$6:$B12,"Entry"),"")</f>
+        <f>IF($B12="Entry",COUNTIF($B$8:$B12,"Entry"),"")</f>
       </c>
       <c r="B12" s="16"/>
       <c r="C12" s="17"/>
@@ -1457,7 +1516,7 @@
       <c r="P12" s="24"/>
       <c r="Q12" s="26"/>
       <c r="R12" s="27">
-        <f>IF($B12&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C12,$O$6:$O$205)+SUMIF($C$6:$C$205,$C12,$P$6:$P$205))</f>
+        <f>IF($B12&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C12,$O$8:$O$207)+SUMIF($C$8:$C$207,$C12,$P$8:$P$207))</f>
       </c>
       <c r="S12" s="27">
         <f>IF(OR($B12&lt;&gt;"Challan",$C12="",G12=0),"",IF(ROUND(G12-R12,2)=0,"Matches","Check Entries"))</f>
@@ -1465,7 +1524,7 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
-        <f>IF($B13="Entry",COUNTIF($B$6:$B13,"Entry"),"")</f>
+        <f>IF($B13="Entry",COUNTIF($B$8:$B13,"Entry"),"")</f>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="17"/>
@@ -1484,7 +1543,7 @@
       <c r="P13" s="24"/>
       <c r="Q13" s="26"/>
       <c r="R13" s="27">
-        <f>IF($B13&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C13,$O$6:$O$205)+SUMIF($C$6:$C$205,$C13,$P$6:$P$205))</f>
+        <f>IF($B13&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C13,$O$8:$O$207)+SUMIF($C$8:$C$207,$C13,$P$8:$P$207))</f>
       </c>
       <c r="S13" s="27">
         <f>IF(OR($B13&lt;&gt;"Challan",$C13="",G13=0),"",IF(ROUND(G13-R13,2)=0,"Matches","Check Entries"))</f>
@@ -1492,7 +1551,7 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
-        <f>IF($B14="Entry",COUNTIF($B$6:$B14,"Entry"),"")</f>
+        <f>IF($B14="Entry",COUNTIF($B$8:$B14,"Entry"),"")</f>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="17"/>
@@ -1511,7 +1570,7 @@
       <c r="P14" s="24"/>
       <c r="Q14" s="26"/>
       <c r="R14" s="27">
-        <f>IF($B14&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C14,$O$6:$O$205)+SUMIF($C$6:$C$205,$C14,$P$6:$P$205))</f>
+        <f>IF($B14&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C14,$O$8:$O$207)+SUMIF($C$8:$C$207,$C14,$P$8:$P$207))</f>
       </c>
       <c r="S14" s="27">
         <f>IF(OR($B14&lt;&gt;"Challan",$C14="",G14=0),"",IF(ROUND(G14-R14,2)=0,"Matches","Check Entries"))</f>
@@ -1519,7 +1578,7 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
-        <f>IF($B15="Entry",COUNTIF($B$6:$B15,"Entry"),"")</f>
+        <f>IF($B15="Entry",COUNTIF($B$8:$B15,"Entry"),"")</f>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="17"/>
@@ -1538,7 +1597,7 @@
       <c r="P15" s="24"/>
       <c r="Q15" s="26"/>
       <c r="R15" s="27">
-        <f>IF($B15&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C15,$O$6:$O$205)+SUMIF($C$6:$C$205,$C15,$P$6:$P$205))</f>
+        <f>IF($B15&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C15,$O$8:$O$207)+SUMIF($C$8:$C$207,$C15,$P$8:$P$207))</f>
       </c>
       <c r="S15" s="27">
         <f>IF(OR($B15&lt;&gt;"Challan",$C15="",G15=0),"",IF(ROUND(G15-R15,2)=0,"Matches","Check Entries"))</f>
@@ -1546,7 +1605,7 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
-        <f>IF($B16="Entry",COUNTIF($B$6:$B16,"Entry"),"")</f>
+        <f>IF($B16="Entry",COUNTIF($B$8:$B16,"Entry"),"")</f>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="17"/>
@@ -1565,7 +1624,7 @@
       <c r="P16" s="24"/>
       <c r="Q16" s="26"/>
       <c r="R16" s="27">
-        <f>IF($B16&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C16,$O$6:$O$205)+SUMIF($C$6:$C$205,$C16,$P$6:$P$205))</f>
+        <f>IF($B16&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C16,$O$8:$O$207)+SUMIF($C$8:$C$207,$C16,$P$8:$P$207))</f>
       </c>
       <c r="S16" s="27">
         <f>IF(OR($B16&lt;&gt;"Challan",$C16="",G16=0),"",IF(ROUND(G16-R16,2)=0,"Matches","Check Entries"))</f>
@@ -1573,7 +1632,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
-        <f>IF($B17="Entry",COUNTIF($B$6:$B17,"Entry"),"")</f>
+        <f>IF($B17="Entry",COUNTIF($B$8:$B17,"Entry"),"")</f>
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="17"/>
@@ -1592,7 +1651,7 @@
       <c r="P17" s="24"/>
       <c r="Q17" s="26"/>
       <c r="R17" s="27">
-        <f>IF($B17&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C17,$O$6:$O$205)+SUMIF($C$6:$C$205,$C17,$P$6:$P$205))</f>
+        <f>IF($B17&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C17,$O$8:$O$207)+SUMIF($C$8:$C$207,$C17,$P$8:$P$207))</f>
       </c>
       <c r="S17" s="27">
         <f>IF(OR($B17&lt;&gt;"Challan",$C17="",G17=0),"",IF(ROUND(G17-R17,2)=0,"Matches","Check Entries"))</f>
@@ -1600,7 +1659,7 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
-        <f>IF($B18="Entry",COUNTIF($B$6:$B18,"Entry"),"")</f>
+        <f>IF($B18="Entry",COUNTIF($B$8:$B18,"Entry"),"")</f>
       </c>
       <c r="B18" s="16"/>
       <c r="C18" s="17"/>
@@ -1619,7 +1678,7 @@
       <c r="P18" s="24"/>
       <c r="Q18" s="26"/>
       <c r="R18" s="27">
-        <f>IF($B18&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C18,$O$6:$O$205)+SUMIF($C$6:$C$205,$C18,$P$6:$P$205))</f>
+        <f>IF($B18&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C18,$O$8:$O$207)+SUMIF($C$8:$C$207,$C18,$P$8:$P$207))</f>
       </c>
       <c r="S18" s="27">
         <f>IF(OR($B18&lt;&gt;"Challan",$C18="",G18=0),"",IF(ROUND(G18-R18,2)=0,"Matches","Check Entries"))</f>
@@ -1627,7 +1686,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
-        <f>IF($B19="Entry",COUNTIF($B$6:$B19,"Entry"),"")</f>
+        <f>IF($B19="Entry",COUNTIF($B$8:$B19,"Entry"),"")</f>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="17"/>
@@ -1646,7 +1705,7 @@
       <c r="P19" s="24"/>
       <c r="Q19" s="26"/>
       <c r="R19" s="27">
-        <f>IF($B19&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C19,$O$6:$O$205)+SUMIF($C$6:$C$205,$C19,$P$6:$P$205))</f>
+        <f>IF($B19&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C19,$O$8:$O$207)+SUMIF($C$8:$C$207,$C19,$P$8:$P$207))</f>
       </c>
       <c r="S19" s="27">
         <f>IF(OR($B19&lt;&gt;"Challan",$C19="",G19=0),"",IF(ROUND(G19-R19,2)=0,"Matches","Check Entries"))</f>
@@ -1654,7 +1713,7 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
-        <f>IF($B20="Entry",COUNTIF($B$6:$B20,"Entry"),"")</f>
+        <f>IF($B20="Entry",COUNTIF($B$8:$B20,"Entry"),"")</f>
       </c>
       <c r="B20" s="16"/>
       <c r="C20" s="17"/>
@@ -1673,7 +1732,7 @@
       <c r="P20" s="24"/>
       <c r="Q20" s="26"/>
       <c r="R20" s="27">
-        <f>IF($B20&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C20,$O$6:$O$205)+SUMIF($C$6:$C$205,$C20,$P$6:$P$205))</f>
+        <f>IF($B20&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C20,$O$8:$O$207)+SUMIF($C$8:$C$207,$C20,$P$8:$P$207))</f>
       </c>
       <c r="S20" s="27">
         <f>IF(OR($B20&lt;&gt;"Challan",$C20="",G20=0),"",IF(ROUND(G20-R20,2)=0,"Matches","Check Entries"))</f>
@@ -1681,7 +1740,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
-        <f>IF($B21="Entry",COUNTIF($B$6:$B21,"Entry"),"")</f>
+        <f>IF($B21="Entry",COUNTIF($B$8:$B21,"Entry"),"")</f>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="17"/>
@@ -1700,7 +1759,7 @@
       <c r="P21" s="24"/>
       <c r="Q21" s="26"/>
       <c r="R21" s="27">
-        <f>IF($B21&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C21,$O$6:$O$205)+SUMIF($C$6:$C$205,$C21,$P$6:$P$205))</f>
+        <f>IF($B21&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C21,$O$8:$O$207)+SUMIF($C$8:$C$207,$C21,$P$8:$P$207))</f>
       </c>
       <c r="S21" s="27">
         <f>IF(OR($B21&lt;&gt;"Challan",$C21="",G21=0),"",IF(ROUND(G21-R21,2)=0,"Matches","Check Entries"))</f>
@@ -1708,7 +1767,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
-        <f>IF($B22="Entry",COUNTIF($B$6:$B22,"Entry"),"")</f>
+        <f>IF($B22="Entry",COUNTIF($B$8:$B22,"Entry"),"")</f>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="17"/>
@@ -1727,7 +1786,7 @@
       <c r="P22" s="24"/>
       <c r="Q22" s="26"/>
       <c r="R22" s="27">
-        <f>IF($B22&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C22,$O$6:$O$205)+SUMIF($C$6:$C$205,$C22,$P$6:$P$205))</f>
+        <f>IF($B22&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C22,$O$8:$O$207)+SUMIF($C$8:$C$207,$C22,$P$8:$P$207))</f>
       </c>
       <c r="S22" s="27">
         <f>IF(OR($B22&lt;&gt;"Challan",$C22="",G22=0),"",IF(ROUND(G22-R22,2)=0,"Matches","Check Entries"))</f>
@@ -1735,7 +1794,7 @@
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
-        <f>IF($B23="Entry",COUNTIF($B$6:$B23,"Entry"),"")</f>
+        <f>IF($B23="Entry",COUNTIF($B$8:$B23,"Entry"),"")</f>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="17"/>
@@ -1754,7 +1813,7 @@
       <c r="P23" s="24"/>
       <c r="Q23" s="26"/>
       <c r="R23" s="27">
-        <f>IF($B23&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C23,$O$6:$O$205)+SUMIF($C$6:$C$205,$C23,$P$6:$P$205))</f>
+        <f>IF($B23&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C23,$O$8:$O$207)+SUMIF($C$8:$C$207,$C23,$P$8:$P$207))</f>
       </c>
       <c r="S23" s="27">
         <f>IF(OR($B23&lt;&gt;"Challan",$C23="",G23=0),"",IF(ROUND(G23-R23,2)=0,"Matches","Check Entries"))</f>
@@ -1762,7 +1821,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
-        <f>IF($B24="Entry",COUNTIF($B$6:$B24,"Entry"),"")</f>
+        <f>IF($B24="Entry",COUNTIF($B$8:$B24,"Entry"),"")</f>
       </c>
       <c r="B24" s="16"/>
       <c r="C24" s="17"/>
@@ -1781,7 +1840,7 @@
       <c r="P24" s="24"/>
       <c r="Q24" s="26"/>
       <c r="R24" s="27">
-        <f>IF($B24&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C24,$O$6:$O$205)+SUMIF($C$6:$C$205,$C24,$P$6:$P$205))</f>
+        <f>IF($B24&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C24,$O$8:$O$207)+SUMIF($C$8:$C$207,$C24,$P$8:$P$207))</f>
       </c>
       <c r="S24" s="27">
         <f>IF(OR($B24&lt;&gt;"Challan",$C24="",G24=0),"",IF(ROUND(G24-R24,2)=0,"Matches","Check Entries"))</f>
@@ -1789,7 +1848,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
-        <f>IF($B25="Entry",COUNTIF($B$6:$B25,"Entry"),"")</f>
+        <f>IF($B25="Entry",COUNTIF($B$8:$B25,"Entry"),"")</f>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="17"/>
@@ -1808,7 +1867,7 @@
       <c r="P25" s="24"/>
       <c r="Q25" s="26"/>
       <c r="R25" s="27">
-        <f>IF($B25&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C25,$O$6:$O$205)+SUMIF($C$6:$C$205,$C25,$P$6:$P$205))</f>
+        <f>IF($B25&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C25,$O$8:$O$207)+SUMIF($C$8:$C$207,$C25,$P$8:$P$207))</f>
       </c>
       <c r="S25" s="27">
         <f>IF(OR($B25&lt;&gt;"Challan",$C25="",G25=0),"",IF(ROUND(G25-R25,2)=0,"Matches","Check Entries"))</f>
@@ -1816,7 +1875,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
-        <f>IF($B26="Entry",COUNTIF($B$6:$B26,"Entry"),"")</f>
+        <f>IF($B26="Entry",COUNTIF($B$8:$B26,"Entry"),"")</f>
       </c>
       <c r="B26" s="16"/>
       <c r="C26" s="17"/>
@@ -1835,7 +1894,7 @@
       <c r="P26" s="24"/>
       <c r="Q26" s="26"/>
       <c r="R26" s="27">
-        <f>IF($B26&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C26,$O$6:$O$205)+SUMIF($C$6:$C$205,$C26,$P$6:$P$205))</f>
+        <f>IF($B26&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C26,$O$8:$O$207)+SUMIF($C$8:$C$207,$C26,$P$8:$P$207))</f>
       </c>
       <c r="S26" s="27">
         <f>IF(OR($B26&lt;&gt;"Challan",$C26="",G26=0),"",IF(ROUND(G26-R26,2)=0,"Matches","Check Entries"))</f>
@@ -1843,7 +1902,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
-        <f>IF($B27="Entry",COUNTIF($B$6:$B27,"Entry"),"")</f>
+        <f>IF($B27="Entry",COUNTIF($B$8:$B27,"Entry"),"")</f>
       </c>
       <c r="B27" s="16"/>
       <c r="C27" s="17"/>
@@ -1862,7 +1921,7 @@
       <c r="P27" s="24"/>
       <c r="Q27" s="26"/>
       <c r="R27" s="27">
-        <f>IF($B27&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C27,$O$6:$O$205)+SUMIF($C$6:$C$205,$C27,$P$6:$P$205))</f>
+        <f>IF($B27&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C27,$O$8:$O$207)+SUMIF($C$8:$C$207,$C27,$P$8:$P$207))</f>
       </c>
       <c r="S27" s="27">
         <f>IF(OR($B27&lt;&gt;"Challan",$C27="",G27=0),"",IF(ROUND(G27-R27,2)=0,"Matches","Check Entries"))</f>
@@ -1870,7 +1929,7 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
-        <f>IF($B28="Entry",COUNTIF($B$6:$B28,"Entry"),"")</f>
+        <f>IF($B28="Entry",COUNTIF($B$8:$B28,"Entry"),"")</f>
       </c>
       <c r="B28" s="16"/>
       <c r="C28" s="17"/>
@@ -1889,7 +1948,7 @@
       <c r="P28" s="24"/>
       <c r="Q28" s="26"/>
       <c r="R28" s="27">
-        <f>IF($B28&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C28,$O$6:$O$205)+SUMIF($C$6:$C$205,$C28,$P$6:$P$205))</f>
+        <f>IF($B28&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C28,$O$8:$O$207)+SUMIF($C$8:$C$207,$C28,$P$8:$P$207))</f>
       </c>
       <c r="S28" s="27">
         <f>IF(OR($B28&lt;&gt;"Challan",$C28="",G28=0),"",IF(ROUND(G28-R28,2)=0,"Matches","Check Entries"))</f>
@@ -1897,7 +1956,7 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
-        <f>IF($B29="Entry",COUNTIF($B$6:$B29,"Entry"),"")</f>
+        <f>IF($B29="Entry",COUNTIF($B$8:$B29,"Entry"),"")</f>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="17"/>
@@ -1916,7 +1975,7 @@
       <c r="P29" s="24"/>
       <c r="Q29" s="26"/>
       <c r="R29" s="27">
-        <f>IF($B29&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C29,$O$6:$O$205)+SUMIF($C$6:$C$205,$C29,$P$6:$P$205))</f>
+        <f>IF($B29&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C29,$O$8:$O$207)+SUMIF($C$8:$C$207,$C29,$P$8:$P$207))</f>
       </c>
       <c r="S29" s="27">
         <f>IF(OR($B29&lt;&gt;"Challan",$C29="",G29=0),"",IF(ROUND(G29-R29,2)=0,"Matches","Check Entries"))</f>
@@ -1924,7 +1983,7 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
-        <f>IF($B30="Entry",COUNTIF($B$6:$B30,"Entry"),"")</f>
+        <f>IF($B30="Entry",COUNTIF($B$8:$B30,"Entry"),"")</f>
       </c>
       <c r="B30" s="16"/>
       <c r="C30" s="17"/>
@@ -1943,7 +2002,7 @@
       <c r="P30" s="24"/>
       <c r="Q30" s="26"/>
       <c r="R30" s="27">
-        <f>IF($B30&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C30,$O$6:$O$205)+SUMIF($C$6:$C$205,$C30,$P$6:$P$205))</f>
+        <f>IF($B30&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C30,$O$8:$O$207)+SUMIF($C$8:$C$207,$C30,$P$8:$P$207))</f>
       </c>
       <c r="S30" s="27">
         <f>IF(OR($B30&lt;&gt;"Challan",$C30="",G30=0),"",IF(ROUND(G30-R30,2)=0,"Matches","Check Entries"))</f>
@@ -1951,7 +2010,7 @@
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="15">
-        <f>IF($B31="Entry",COUNTIF($B$6:$B31,"Entry"),"")</f>
+        <f>IF($B31="Entry",COUNTIF($B$8:$B31,"Entry"),"")</f>
       </c>
       <c r="B31" s="16"/>
       <c r="C31" s="17"/>
@@ -1970,7 +2029,7 @@
       <c r="P31" s="24"/>
       <c r="Q31" s="26"/>
       <c r="R31" s="27">
-        <f>IF($B31&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C31,$O$6:$O$205)+SUMIF($C$6:$C$205,$C31,$P$6:$P$205))</f>
+        <f>IF($B31&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C31,$O$8:$O$207)+SUMIF($C$8:$C$207,$C31,$P$8:$P$207))</f>
       </c>
       <c r="S31" s="27">
         <f>IF(OR($B31&lt;&gt;"Challan",$C31="",G31=0),"",IF(ROUND(G31-R31,2)=0,"Matches","Check Entries"))</f>
@@ -1978,7 +2037,7 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="15">
-        <f>IF($B32="Entry",COUNTIF($B$6:$B32,"Entry"),"")</f>
+        <f>IF($B32="Entry",COUNTIF($B$8:$B32,"Entry"),"")</f>
       </c>
       <c r="B32" s="16"/>
       <c r="C32" s="17"/>
@@ -1997,7 +2056,7 @@
       <c r="P32" s="24"/>
       <c r="Q32" s="26"/>
       <c r="R32" s="27">
-        <f>IF($B32&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C32,$O$6:$O$205)+SUMIF($C$6:$C$205,$C32,$P$6:$P$205))</f>
+        <f>IF($B32&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C32,$O$8:$O$207)+SUMIF($C$8:$C$207,$C32,$P$8:$P$207))</f>
       </c>
       <c r="S32" s="27">
         <f>IF(OR($B32&lt;&gt;"Challan",$C32="",G32=0),"",IF(ROUND(G32-R32,2)=0,"Matches","Check Entries"))</f>
@@ -2005,7 +2064,7 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="15">
-        <f>IF($B33="Entry",COUNTIF($B$6:$B33,"Entry"),"")</f>
+        <f>IF($B33="Entry",COUNTIF($B$8:$B33,"Entry"),"")</f>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="17"/>
@@ -2024,7 +2083,7 @@
       <c r="P33" s="24"/>
       <c r="Q33" s="26"/>
       <c r="R33" s="27">
-        <f>IF($B33&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C33,$O$6:$O$205)+SUMIF($C$6:$C$205,$C33,$P$6:$P$205))</f>
+        <f>IF($B33&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C33,$O$8:$O$207)+SUMIF($C$8:$C$207,$C33,$P$8:$P$207))</f>
       </c>
       <c r="S33" s="27">
         <f>IF(OR($B33&lt;&gt;"Challan",$C33="",G33=0),"",IF(ROUND(G33-R33,2)=0,"Matches","Check Entries"))</f>
@@ -2032,7 +2091,7 @@
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="15">
-        <f>IF($B34="Entry",COUNTIF($B$6:$B34,"Entry"),"")</f>
+        <f>IF($B34="Entry",COUNTIF($B$8:$B34,"Entry"),"")</f>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="17"/>
@@ -2051,7 +2110,7 @@
       <c r="P34" s="24"/>
       <c r="Q34" s="26"/>
       <c r="R34" s="27">
-        <f>IF($B34&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C34,$O$6:$O$205)+SUMIF($C$6:$C$205,$C34,$P$6:$P$205))</f>
+        <f>IF($B34&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C34,$O$8:$O$207)+SUMIF($C$8:$C$207,$C34,$P$8:$P$207))</f>
       </c>
       <c r="S34" s="27">
         <f>IF(OR($B34&lt;&gt;"Challan",$C34="",G34=0),"",IF(ROUND(G34-R34,2)=0,"Matches","Check Entries"))</f>
@@ -2059,7 +2118,7 @@
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="15">
-        <f>IF($B35="Entry",COUNTIF($B$6:$B35,"Entry"),"")</f>
+        <f>IF($B35="Entry",COUNTIF($B$8:$B35,"Entry"),"")</f>
       </c>
       <c r="B35" s="16"/>
       <c r="C35" s="17"/>
@@ -2078,7 +2137,7 @@
       <c r="P35" s="24"/>
       <c r="Q35" s="26"/>
       <c r="R35" s="27">
-        <f>IF($B35&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C35,$O$6:$O$205)+SUMIF($C$6:$C$205,$C35,$P$6:$P$205))</f>
+        <f>IF($B35&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C35,$O$8:$O$207)+SUMIF($C$8:$C$207,$C35,$P$8:$P$207))</f>
       </c>
       <c r="S35" s="27">
         <f>IF(OR($B35&lt;&gt;"Challan",$C35="",G35=0),"",IF(ROUND(G35-R35,2)=0,"Matches","Check Entries"))</f>
@@ -2086,7 +2145,7 @@
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
-        <f>IF($B36="Entry",COUNTIF($B$6:$B36,"Entry"),"")</f>
+        <f>IF($B36="Entry",COUNTIF($B$8:$B36,"Entry"),"")</f>
       </c>
       <c r="B36" s="16"/>
       <c r="C36" s="17"/>
@@ -2105,7 +2164,7 @@
       <c r="P36" s="24"/>
       <c r="Q36" s="26"/>
       <c r="R36" s="27">
-        <f>IF($B36&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C36,$O$6:$O$205)+SUMIF($C$6:$C$205,$C36,$P$6:$P$205))</f>
+        <f>IF($B36&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C36,$O$8:$O$207)+SUMIF($C$8:$C$207,$C36,$P$8:$P$207))</f>
       </c>
       <c r="S36" s="27">
         <f>IF(OR($B36&lt;&gt;"Challan",$C36="",G36=0),"",IF(ROUND(G36-R36,2)=0,"Matches","Check Entries"))</f>
@@ -2113,7 +2172,7 @@
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
-        <f>IF($B37="Entry",COUNTIF($B$6:$B37,"Entry"),"")</f>
+        <f>IF($B37="Entry",COUNTIF($B$8:$B37,"Entry"),"")</f>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="17"/>
@@ -2132,7 +2191,7 @@
       <c r="P37" s="24"/>
       <c r="Q37" s="26"/>
       <c r="R37" s="27">
-        <f>IF($B37&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C37,$O$6:$O$205)+SUMIF($C$6:$C$205,$C37,$P$6:$P$205))</f>
+        <f>IF($B37&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C37,$O$8:$O$207)+SUMIF($C$8:$C$207,$C37,$P$8:$P$207))</f>
       </c>
       <c r="S37" s="27">
         <f>IF(OR($B37&lt;&gt;"Challan",$C37="",G37=0),"",IF(ROUND(G37-R37,2)=0,"Matches","Check Entries"))</f>
@@ -2140,7 +2199,7 @@
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="15">
-        <f>IF($B38="Entry",COUNTIF($B$6:$B38,"Entry"),"")</f>
+        <f>IF($B38="Entry",COUNTIF($B$8:$B38,"Entry"),"")</f>
       </c>
       <c r="B38" s="16"/>
       <c r="C38" s="17"/>
@@ -2159,7 +2218,7 @@
       <c r="P38" s="24"/>
       <c r="Q38" s="26"/>
       <c r="R38" s="27">
-        <f>IF($B38&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C38,$O$6:$O$205)+SUMIF($C$6:$C$205,$C38,$P$6:$P$205))</f>
+        <f>IF($B38&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C38,$O$8:$O$207)+SUMIF($C$8:$C$207,$C38,$P$8:$P$207))</f>
       </c>
       <c r="S38" s="27">
         <f>IF(OR($B38&lt;&gt;"Challan",$C38="",G38=0),"",IF(ROUND(G38-R38,2)=0,"Matches","Check Entries"))</f>
@@ -2167,7 +2226,7 @@
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="15">
-        <f>IF($B39="Entry",COUNTIF($B$6:$B39,"Entry"),"")</f>
+        <f>IF($B39="Entry",COUNTIF($B$8:$B39,"Entry"),"")</f>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="17"/>
@@ -2186,7 +2245,7 @@
       <c r="P39" s="24"/>
       <c r="Q39" s="26"/>
       <c r="R39" s="27">
-        <f>IF($B39&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C39,$O$6:$O$205)+SUMIF($C$6:$C$205,$C39,$P$6:$P$205))</f>
+        <f>IF($B39&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C39,$O$8:$O$207)+SUMIF($C$8:$C$207,$C39,$P$8:$P$207))</f>
       </c>
       <c r="S39" s="27">
         <f>IF(OR($B39&lt;&gt;"Challan",$C39="",G39=0),"",IF(ROUND(G39-R39,2)=0,"Matches","Check Entries"))</f>
@@ -2194,7 +2253,7 @@
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
-        <f>IF($B40="Entry",COUNTIF($B$6:$B40,"Entry"),"")</f>
+        <f>IF($B40="Entry",COUNTIF($B$8:$B40,"Entry"),"")</f>
       </c>
       <c r="B40" s="16"/>
       <c r="C40" s="17"/>
@@ -2213,7 +2272,7 @@
       <c r="P40" s="24"/>
       <c r="Q40" s="26"/>
       <c r="R40" s="27">
-        <f>IF($B40&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C40,$O$6:$O$205)+SUMIF($C$6:$C$205,$C40,$P$6:$P$205))</f>
+        <f>IF($B40&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C40,$O$8:$O$207)+SUMIF($C$8:$C$207,$C40,$P$8:$P$207))</f>
       </c>
       <c r="S40" s="27">
         <f>IF(OR($B40&lt;&gt;"Challan",$C40="",G40=0),"",IF(ROUND(G40-R40,2)=0,"Matches","Check Entries"))</f>
@@ -2221,7 +2280,7 @@
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
-        <f>IF($B41="Entry",COUNTIF($B$6:$B41,"Entry"),"")</f>
+        <f>IF($B41="Entry",COUNTIF($B$8:$B41,"Entry"),"")</f>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="17"/>
@@ -2240,7 +2299,7 @@
       <c r="P41" s="24"/>
       <c r="Q41" s="26"/>
       <c r="R41" s="27">
-        <f>IF($B41&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C41,$O$6:$O$205)+SUMIF($C$6:$C$205,$C41,$P$6:$P$205))</f>
+        <f>IF($B41&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C41,$O$8:$O$207)+SUMIF($C$8:$C$207,$C41,$P$8:$P$207))</f>
       </c>
       <c r="S41" s="27">
         <f>IF(OR($B41&lt;&gt;"Challan",$C41="",G41=0),"",IF(ROUND(G41-R41,2)=0,"Matches","Check Entries"))</f>
@@ -2248,7 +2307,7 @@
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="15">
-        <f>IF($B42="Entry",COUNTIF($B$6:$B42,"Entry"),"")</f>
+        <f>IF($B42="Entry",COUNTIF($B$8:$B42,"Entry"),"")</f>
       </c>
       <c r="B42" s="16"/>
       <c r="C42" s="17"/>
@@ -2267,7 +2326,7 @@
       <c r="P42" s="24"/>
       <c r="Q42" s="26"/>
       <c r="R42" s="27">
-        <f>IF($B42&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C42,$O$6:$O$205)+SUMIF($C$6:$C$205,$C42,$P$6:$P$205))</f>
+        <f>IF($B42&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C42,$O$8:$O$207)+SUMIF($C$8:$C$207,$C42,$P$8:$P$207))</f>
       </c>
       <c r="S42" s="27">
         <f>IF(OR($B42&lt;&gt;"Challan",$C42="",G42=0),"",IF(ROUND(G42-R42,2)=0,"Matches","Check Entries"))</f>
@@ -2275,7 +2334,7 @@
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="15">
-        <f>IF($B43="Entry",COUNTIF($B$6:$B43,"Entry"),"")</f>
+        <f>IF($B43="Entry",COUNTIF($B$8:$B43,"Entry"),"")</f>
       </c>
       <c r="B43" s="16"/>
       <c r="C43" s="17"/>
@@ -2294,7 +2353,7 @@
       <c r="P43" s="24"/>
       <c r="Q43" s="26"/>
       <c r="R43" s="27">
-        <f>IF($B43&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C43,$O$6:$O$205)+SUMIF($C$6:$C$205,$C43,$P$6:$P$205))</f>
+        <f>IF($B43&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C43,$O$8:$O$207)+SUMIF($C$8:$C$207,$C43,$P$8:$P$207))</f>
       </c>
       <c r="S43" s="27">
         <f>IF(OR($B43&lt;&gt;"Challan",$C43="",G43=0),"",IF(ROUND(G43-R43,2)=0,"Matches","Check Entries"))</f>
@@ -2302,7 +2361,7 @@
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
-        <f>IF($B44="Entry",COUNTIF($B$6:$B44,"Entry"),"")</f>
+        <f>IF($B44="Entry",COUNTIF($B$8:$B44,"Entry"),"")</f>
       </c>
       <c r="B44" s="16"/>
       <c r="C44" s="17"/>
@@ -2321,7 +2380,7 @@
       <c r="P44" s="24"/>
       <c r="Q44" s="26"/>
       <c r="R44" s="27">
-        <f>IF($B44&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C44,$O$6:$O$205)+SUMIF($C$6:$C$205,$C44,$P$6:$P$205))</f>
+        <f>IF($B44&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C44,$O$8:$O$207)+SUMIF($C$8:$C$207,$C44,$P$8:$P$207))</f>
       </c>
       <c r="S44" s="27">
         <f>IF(OR($B44&lt;&gt;"Challan",$C44="",G44=0),"",IF(ROUND(G44-R44,2)=0,"Matches","Check Entries"))</f>
@@ -2329,7 +2388,7 @@
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
-        <f>IF($B45="Entry",COUNTIF($B$6:$B45,"Entry"),"")</f>
+        <f>IF($B45="Entry",COUNTIF($B$8:$B45,"Entry"),"")</f>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="17"/>
@@ -2348,7 +2407,7 @@
       <c r="P45" s="24"/>
       <c r="Q45" s="26"/>
       <c r="R45" s="27">
-        <f>IF($B45&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C45,$O$6:$O$205)+SUMIF($C$6:$C$205,$C45,$P$6:$P$205))</f>
+        <f>IF($B45&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C45,$O$8:$O$207)+SUMIF($C$8:$C$207,$C45,$P$8:$P$207))</f>
       </c>
       <c r="S45" s="27">
         <f>IF(OR($B45&lt;&gt;"Challan",$C45="",G45=0),"",IF(ROUND(G45-R45,2)=0,"Matches","Check Entries"))</f>
@@ -2356,7 +2415,7 @@
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="15">
-        <f>IF($B46="Entry",COUNTIF($B$6:$B46,"Entry"),"")</f>
+        <f>IF($B46="Entry",COUNTIF($B$8:$B46,"Entry"),"")</f>
       </c>
       <c r="B46" s="16"/>
       <c r="C46" s="17"/>
@@ -2375,7 +2434,7 @@
       <c r="P46" s="24"/>
       <c r="Q46" s="26"/>
       <c r="R46" s="27">
-        <f>IF($B46&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C46,$O$6:$O$205)+SUMIF($C$6:$C$205,$C46,$P$6:$P$205))</f>
+        <f>IF($B46&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C46,$O$8:$O$207)+SUMIF($C$8:$C$207,$C46,$P$8:$P$207))</f>
       </c>
       <c r="S46" s="27">
         <f>IF(OR($B46&lt;&gt;"Challan",$C46="",G46=0),"",IF(ROUND(G46-R46,2)=0,"Matches","Check Entries"))</f>
@@ -2383,7 +2442,7 @@
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="15">
-        <f>IF($B47="Entry",COUNTIF($B$6:$B47,"Entry"),"")</f>
+        <f>IF($B47="Entry",COUNTIF($B$8:$B47,"Entry"),"")</f>
       </c>
       <c r="B47" s="16"/>
       <c r="C47" s="17"/>
@@ -2402,7 +2461,7 @@
       <c r="P47" s="24"/>
       <c r="Q47" s="26"/>
       <c r="R47" s="27">
-        <f>IF($B47&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C47,$O$6:$O$205)+SUMIF($C$6:$C$205,$C47,$P$6:$P$205))</f>
+        <f>IF($B47&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C47,$O$8:$O$207)+SUMIF($C$8:$C$207,$C47,$P$8:$P$207))</f>
       </c>
       <c r="S47" s="27">
         <f>IF(OR($B47&lt;&gt;"Challan",$C47="",G47=0),"",IF(ROUND(G47-R47,2)=0,"Matches","Check Entries"))</f>
@@ -2410,7 +2469,7 @@
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
-        <f>IF($B48="Entry",COUNTIF($B$6:$B48,"Entry"),"")</f>
+        <f>IF($B48="Entry",COUNTIF($B$8:$B48,"Entry"),"")</f>
       </c>
       <c r="B48" s="16"/>
       <c r="C48" s="17"/>
@@ -2429,7 +2488,7 @@
       <c r="P48" s="24"/>
       <c r="Q48" s="26"/>
       <c r="R48" s="27">
-        <f>IF($B48&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C48,$O$6:$O$205)+SUMIF($C$6:$C$205,$C48,$P$6:$P$205))</f>
+        <f>IF($B48&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C48,$O$8:$O$207)+SUMIF($C$8:$C$207,$C48,$P$8:$P$207))</f>
       </c>
       <c r="S48" s="27">
         <f>IF(OR($B48&lt;&gt;"Challan",$C48="",G48=0),"",IF(ROUND(G48-R48,2)=0,"Matches","Check Entries"))</f>
@@ -2437,7 +2496,7 @@
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
-        <f>IF($B49="Entry",COUNTIF($B$6:$B49,"Entry"),"")</f>
+        <f>IF($B49="Entry",COUNTIF($B$8:$B49,"Entry"),"")</f>
       </c>
       <c r="B49" s="16"/>
       <c r="C49" s="17"/>
@@ -2456,7 +2515,7 @@
       <c r="P49" s="24"/>
       <c r="Q49" s="26"/>
       <c r="R49" s="27">
-        <f>IF($B49&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C49,$O$6:$O$205)+SUMIF($C$6:$C$205,$C49,$P$6:$P$205))</f>
+        <f>IF($B49&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C49,$O$8:$O$207)+SUMIF($C$8:$C$207,$C49,$P$8:$P$207))</f>
       </c>
       <c r="S49" s="27">
         <f>IF(OR($B49&lt;&gt;"Challan",$C49="",G49=0),"",IF(ROUND(G49-R49,2)=0,"Matches","Check Entries"))</f>
@@ -2464,7 +2523,7 @@
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
-        <f>IF($B50="Entry",COUNTIF($B$6:$B50,"Entry"),"")</f>
+        <f>IF($B50="Entry",COUNTIF($B$8:$B50,"Entry"),"")</f>
       </c>
       <c r="B50" s="16"/>
       <c r="C50" s="17"/>
@@ -2483,7 +2542,7 @@
       <c r="P50" s="24"/>
       <c r="Q50" s="26"/>
       <c r="R50" s="27">
-        <f>IF($B50&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C50,$O$6:$O$205)+SUMIF($C$6:$C$205,$C50,$P$6:$P$205))</f>
+        <f>IF($B50&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C50,$O$8:$O$207)+SUMIF($C$8:$C$207,$C50,$P$8:$P$207))</f>
       </c>
       <c r="S50" s="27">
         <f>IF(OR($B50&lt;&gt;"Challan",$C50="",G50=0),"",IF(ROUND(G50-R50,2)=0,"Matches","Check Entries"))</f>
@@ -2491,7 +2550,7 @@
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
-        <f>IF($B51="Entry",COUNTIF($B$6:$B51,"Entry"),"")</f>
+        <f>IF($B51="Entry",COUNTIF($B$8:$B51,"Entry"),"")</f>
       </c>
       <c r="B51" s="16"/>
       <c r="C51" s="17"/>
@@ -2510,7 +2569,7 @@
       <c r="P51" s="24"/>
       <c r="Q51" s="26"/>
       <c r="R51" s="27">
-        <f>IF($B51&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C51,$O$6:$O$205)+SUMIF($C$6:$C$205,$C51,$P$6:$P$205))</f>
+        <f>IF($B51&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C51,$O$8:$O$207)+SUMIF($C$8:$C$207,$C51,$P$8:$P$207))</f>
       </c>
       <c r="S51" s="27">
         <f>IF(OR($B51&lt;&gt;"Challan",$C51="",G51=0),"",IF(ROUND(G51-R51,2)=0,"Matches","Check Entries"))</f>
@@ -2518,7 +2577,7 @@
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
-        <f>IF($B52="Entry",COUNTIF($B$6:$B52,"Entry"),"")</f>
+        <f>IF($B52="Entry",COUNTIF($B$8:$B52,"Entry"),"")</f>
       </c>
       <c r="B52" s="16"/>
       <c r="C52" s="17"/>
@@ -2537,7 +2596,7 @@
       <c r="P52" s="24"/>
       <c r="Q52" s="26"/>
       <c r="R52" s="27">
-        <f>IF($B52&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C52,$O$6:$O$205)+SUMIF($C$6:$C$205,$C52,$P$6:$P$205))</f>
+        <f>IF($B52&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C52,$O$8:$O$207)+SUMIF($C$8:$C$207,$C52,$P$8:$P$207))</f>
       </c>
       <c r="S52" s="27">
         <f>IF(OR($B52&lt;&gt;"Challan",$C52="",G52=0),"",IF(ROUND(G52-R52,2)=0,"Matches","Check Entries"))</f>
@@ -2545,7 +2604,7 @@
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
-        <f>IF($B53="Entry",COUNTIF($B$6:$B53,"Entry"),"")</f>
+        <f>IF($B53="Entry",COUNTIF($B$8:$B53,"Entry"),"")</f>
       </c>
       <c r="B53" s="16"/>
       <c r="C53" s="17"/>
@@ -2564,7 +2623,7 @@
       <c r="P53" s="24"/>
       <c r="Q53" s="26"/>
       <c r="R53" s="27">
-        <f>IF($B53&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C53,$O$6:$O$205)+SUMIF($C$6:$C$205,$C53,$P$6:$P$205))</f>
+        <f>IF($B53&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C53,$O$8:$O$207)+SUMIF($C$8:$C$207,$C53,$P$8:$P$207))</f>
       </c>
       <c r="S53" s="27">
         <f>IF(OR($B53&lt;&gt;"Challan",$C53="",G53=0),"",IF(ROUND(G53-R53,2)=0,"Matches","Check Entries"))</f>
@@ -2572,7 +2631,7 @@
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="15">
-        <f>IF($B54="Entry",COUNTIF($B$6:$B54,"Entry"),"")</f>
+        <f>IF($B54="Entry",COUNTIF($B$8:$B54,"Entry"),"")</f>
       </c>
       <c r="B54" s="16"/>
       <c r="C54" s="17"/>
@@ -2591,7 +2650,7 @@
       <c r="P54" s="24"/>
       <c r="Q54" s="26"/>
       <c r="R54" s="27">
-        <f>IF($B54&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C54,$O$6:$O$205)+SUMIF($C$6:$C$205,$C54,$P$6:$P$205))</f>
+        <f>IF($B54&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C54,$O$8:$O$207)+SUMIF($C$8:$C$207,$C54,$P$8:$P$207))</f>
       </c>
       <c r="S54" s="27">
         <f>IF(OR($B54&lt;&gt;"Challan",$C54="",G54=0),"",IF(ROUND(G54-R54,2)=0,"Matches","Check Entries"))</f>
@@ -2599,7 +2658,7 @@
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" s="15">
-        <f>IF($B55="Entry",COUNTIF($B$6:$B55,"Entry"),"")</f>
+        <f>IF($B55="Entry",COUNTIF($B$8:$B55,"Entry"),"")</f>
       </c>
       <c r="B55" s="16"/>
       <c r="C55" s="17"/>
@@ -2618,7 +2677,7 @@
       <c r="P55" s="24"/>
       <c r="Q55" s="26"/>
       <c r="R55" s="27">
-        <f>IF($B55&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C55,$O$6:$O$205)+SUMIF($C$6:$C$205,$C55,$P$6:$P$205))</f>
+        <f>IF($B55&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C55,$O$8:$O$207)+SUMIF($C$8:$C$207,$C55,$P$8:$P$207))</f>
       </c>
       <c r="S55" s="27">
         <f>IF(OR($B55&lt;&gt;"Challan",$C55="",G55=0),"",IF(ROUND(G55-R55,2)=0,"Matches","Check Entries"))</f>
@@ -2626,7 +2685,7 @@
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
-        <f>IF($B56="Entry",COUNTIF($B$6:$B56,"Entry"),"")</f>
+        <f>IF($B56="Entry",COUNTIF($B$8:$B56,"Entry"),"")</f>
       </c>
       <c r="B56" s="16"/>
       <c r="C56" s="17"/>
@@ -2645,7 +2704,7 @@
       <c r="P56" s="24"/>
       <c r="Q56" s="26"/>
       <c r="R56" s="27">
-        <f>IF($B56&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C56,$O$6:$O$205)+SUMIF($C$6:$C$205,$C56,$P$6:$P$205))</f>
+        <f>IF($B56&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C56,$O$8:$O$207)+SUMIF($C$8:$C$207,$C56,$P$8:$P$207))</f>
       </c>
       <c r="S56" s="27">
         <f>IF(OR($B56&lt;&gt;"Challan",$C56="",G56=0),"",IF(ROUND(G56-R56,2)=0,"Matches","Check Entries"))</f>
@@ -2653,7 +2712,7 @@
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
-        <f>IF($B57="Entry",COUNTIF($B$6:$B57,"Entry"),"")</f>
+        <f>IF($B57="Entry",COUNTIF($B$8:$B57,"Entry"),"")</f>
       </c>
       <c r="B57" s="16"/>
       <c r="C57" s="17"/>
@@ -2672,7 +2731,7 @@
       <c r="P57" s="24"/>
       <c r="Q57" s="26"/>
       <c r="R57" s="27">
-        <f>IF($B57&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C57,$O$6:$O$205)+SUMIF($C$6:$C$205,$C57,$P$6:$P$205))</f>
+        <f>IF($B57&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C57,$O$8:$O$207)+SUMIF($C$8:$C$207,$C57,$P$8:$P$207))</f>
       </c>
       <c r="S57" s="27">
         <f>IF(OR($B57&lt;&gt;"Challan",$C57="",G57=0),"",IF(ROUND(G57-R57,2)=0,"Matches","Check Entries"))</f>
@@ -2680,7 +2739,7 @@
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="15">
-        <f>IF($B58="Entry",COUNTIF($B$6:$B58,"Entry"),"")</f>
+        <f>IF($B58="Entry",COUNTIF($B$8:$B58,"Entry"),"")</f>
       </c>
       <c r="B58" s="16"/>
       <c r="C58" s="17"/>
@@ -2699,7 +2758,7 @@
       <c r="P58" s="24"/>
       <c r="Q58" s="26"/>
       <c r="R58" s="27">
-        <f>IF($B58&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C58,$O$6:$O$205)+SUMIF($C$6:$C$205,$C58,$P$6:$P$205))</f>
+        <f>IF($B58&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C58,$O$8:$O$207)+SUMIF($C$8:$C$207,$C58,$P$8:$P$207))</f>
       </c>
       <c r="S58" s="27">
         <f>IF(OR($B58&lt;&gt;"Challan",$C58="",G58=0),"",IF(ROUND(G58-R58,2)=0,"Matches","Check Entries"))</f>
@@ -2707,7 +2766,7 @@
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="15">
-        <f>IF($B59="Entry",COUNTIF($B$6:$B59,"Entry"),"")</f>
+        <f>IF($B59="Entry",COUNTIF($B$8:$B59,"Entry"),"")</f>
       </c>
       <c r="B59" s="16"/>
       <c r="C59" s="17"/>
@@ -2726,7 +2785,7 @@
       <c r="P59" s="24"/>
       <c r="Q59" s="26"/>
       <c r="R59" s="27">
-        <f>IF($B59&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C59,$O$6:$O$205)+SUMIF($C$6:$C$205,$C59,$P$6:$P$205))</f>
+        <f>IF($B59&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C59,$O$8:$O$207)+SUMIF($C$8:$C$207,$C59,$P$8:$P$207))</f>
       </c>
       <c r="S59" s="27">
         <f>IF(OR($B59&lt;&gt;"Challan",$C59="",G59=0),"",IF(ROUND(G59-R59,2)=0,"Matches","Check Entries"))</f>
@@ -2734,7 +2793,7 @@
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
-        <f>IF($B60="Entry",COUNTIF($B$6:$B60,"Entry"),"")</f>
+        <f>IF($B60="Entry",COUNTIF($B$8:$B60,"Entry"),"")</f>
       </c>
       <c r="B60" s="16"/>
       <c r="C60" s="17"/>
@@ -2753,7 +2812,7 @@
       <c r="P60" s="24"/>
       <c r="Q60" s="26"/>
       <c r="R60" s="27">
-        <f>IF($B60&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C60,$O$6:$O$205)+SUMIF($C$6:$C$205,$C60,$P$6:$P$205))</f>
+        <f>IF($B60&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C60,$O$8:$O$207)+SUMIF($C$8:$C$207,$C60,$P$8:$P$207))</f>
       </c>
       <c r="S60" s="27">
         <f>IF(OR($B60&lt;&gt;"Challan",$C60="",G60=0),"",IF(ROUND(G60-R60,2)=0,"Matches","Check Entries"))</f>
@@ -2761,7 +2820,7 @@
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
-        <f>IF($B61="Entry",COUNTIF($B$6:$B61,"Entry"),"")</f>
+        <f>IF($B61="Entry",COUNTIF($B$8:$B61,"Entry"),"")</f>
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="17"/>
@@ -2780,7 +2839,7 @@
       <c r="P61" s="24"/>
       <c r="Q61" s="26"/>
       <c r="R61" s="27">
-        <f>IF($B61&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C61,$O$6:$O$205)+SUMIF($C$6:$C$205,$C61,$P$6:$P$205))</f>
+        <f>IF($B61&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C61,$O$8:$O$207)+SUMIF($C$8:$C$207,$C61,$P$8:$P$207))</f>
       </c>
       <c r="S61" s="27">
         <f>IF(OR($B61&lt;&gt;"Challan",$C61="",G61=0),"",IF(ROUND(G61-R61,2)=0,"Matches","Check Entries"))</f>
@@ -2788,7 +2847,7 @@
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A62" s="15">
-        <f>IF($B62="Entry",COUNTIF($B$6:$B62,"Entry"),"")</f>
+        <f>IF($B62="Entry",COUNTIF($B$8:$B62,"Entry"),"")</f>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="17"/>
@@ -2807,7 +2866,7 @@
       <c r="P62" s="24"/>
       <c r="Q62" s="26"/>
       <c r="R62" s="27">
-        <f>IF($B62&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C62,$O$6:$O$205)+SUMIF($C$6:$C$205,$C62,$P$6:$P$205))</f>
+        <f>IF($B62&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C62,$O$8:$O$207)+SUMIF($C$8:$C$207,$C62,$P$8:$P$207))</f>
       </c>
       <c r="S62" s="27">
         <f>IF(OR($B62&lt;&gt;"Challan",$C62="",G62=0),"",IF(ROUND(G62-R62,2)=0,"Matches","Check Entries"))</f>
@@ -2815,7 +2874,7 @@
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A63" s="15">
-        <f>IF($B63="Entry",COUNTIF($B$6:$B63,"Entry"),"")</f>
+        <f>IF($B63="Entry",COUNTIF($B$8:$B63,"Entry"),"")</f>
       </c>
       <c r="B63" s="16"/>
       <c r="C63" s="17"/>
@@ -2834,7 +2893,7 @@
       <c r="P63" s="24"/>
       <c r="Q63" s="26"/>
       <c r="R63" s="27">
-        <f>IF($B63&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C63,$O$6:$O$205)+SUMIF($C$6:$C$205,$C63,$P$6:$P$205))</f>
+        <f>IF($B63&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C63,$O$8:$O$207)+SUMIF($C$8:$C$207,$C63,$P$8:$P$207))</f>
       </c>
       <c r="S63" s="27">
         <f>IF(OR($B63&lt;&gt;"Challan",$C63="",G63=0),"",IF(ROUND(G63-R63,2)=0,"Matches","Check Entries"))</f>
@@ -2842,7 +2901,7 @@
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A64" s="15">
-        <f>IF($B64="Entry",COUNTIF($B$6:$B64,"Entry"),"")</f>
+        <f>IF($B64="Entry",COUNTIF($B$8:$B64,"Entry"),"")</f>
       </c>
       <c r="B64" s="16"/>
       <c r="C64" s="17"/>
@@ -2861,7 +2920,7 @@
       <c r="P64" s="24"/>
       <c r="Q64" s="26"/>
       <c r="R64" s="27">
-        <f>IF($B64&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C64,$O$6:$O$205)+SUMIF($C$6:$C$205,$C64,$P$6:$P$205))</f>
+        <f>IF($B64&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C64,$O$8:$O$207)+SUMIF($C$8:$C$207,$C64,$P$8:$P$207))</f>
       </c>
       <c r="S64" s="27">
         <f>IF(OR($B64&lt;&gt;"Challan",$C64="",G64=0),"",IF(ROUND(G64-R64,2)=0,"Matches","Check Entries"))</f>
@@ -2869,7 +2928,7 @@
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A65" s="15">
-        <f>IF($B65="Entry",COUNTIF($B$6:$B65,"Entry"),"")</f>
+        <f>IF($B65="Entry",COUNTIF($B$8:$B65,"Entry"),"")</f>
       </c>
       <c r="B65" s="16"/>
       <c r="C65" s="17"/>
@@ -2888,7 +2947,7 @@
       <c r="P65" s="24"/>
       <c r="Q65" s="26"/>
       <c r="R65" s="27">
-        <f>IF($B65&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C65,$O$6:$O$205)+SUMIF($C$6:$C$205,$C65,$P$6:$P$205))</f>
+        <f>IF($B65&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C65,$O$8:$O$207)+SUMIF($C$8:$C$207,$C65,$P$8:$P$207))</f>
       </c>
       <c r="S65" s="27">
         <f>IF(OR($B65&lt;&gt;"Challan",$C65="",G65=0),"",IF(ROUND(G65-R65,2)=0,"Matches","Check Entries"))</f>
@@ -2896,7 +2955,7 @@
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A66" s="15">
-        <f>IF($B66="Entry",COUNTIF($B$6:$B66,"Entry"),"")</f>
+        <f>IF($B66="Entry",COUNTIF($B$8:$B66,"Entry"),"")</f>
       </c>
       <c r="B66" s="16"/>
       <c r="C66" s="17"/>
@@ -2915,7 +2974,7 @@
       <c r="P66" s="24"/>
       <c r="Q66" s="26"/>
       <c r="R66" s="27">
-        <f>IF($B66&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C66,$O$6:$O$205)+SUMIF($C$6:$C$205,$C66,$P$6:$P$205))</f>
+        <f>IF($B66&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C66,$O$8:$O$207)+SUMIF($C$8:$C$207,$C66,$P$8:$P$207))</f>
       </c>
       <c r="S66" s="27">
         <f>IF(OR($B66&lt;&gt;"Challan",$C66="",G66=0),"",IF(ROUND(G66-R66,2)=0,"Matches","Check Entries"))</f>
@@ -2923,7 +2982,7 @@
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A67" s="15">
-        <f>IF($B67="Entry",COUNTIF($B$6:$B67,"Entry"),"")</f>
+        <f>IF($B67="Entry",COUNTIF($B$8:$B67,"Entry"),"")</f>
       </c>
       <c r="B67" s="16"/>
       <c r="C67" s="17"/>
@@ -2942,7 +3001,7 @@
       <c r="P67" s="24"/>
       <c r="Q67" s="26"/>
       <c r="R67" s="27">
-        <f>IF($B67&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C67,$O$6:$O$205)+SUMIF($C$6:$C$205,$C67,$P$6:$P$205))</f>
+        <f>IF($B67&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C67,$O$8:$O$207)+SUMIF($C$8:$C$207,$C67,$P$8:$P$207))</f>
       </c>
       <c r="S67" s="27">
         <f>IF(OR($B67&lt;&gt;"Challan",$C67="",G67=0),"",IF(ROUND(G67-R67,2)=0,"Matches","Check Entries"))</f>
@@ -2950,7 +3009,7 @@
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A68" s="15">
-        <f>IF($B68="Entry",COUNTIF($B$6:$B68,"Entry"),"")</f>
+        <f>IF($B68="Entry",COUNTIF($B$8:$B68,"Entry"),"")</f>
       </c>
       <c r="B68" s="16"/>
       <c r="C68" s="17"/>
@@ -2969,7 +3028,7 @@
       <c r="P68" s="24"/>
       <c r="Q68" s="26"/>
       <c r="R68" s="27">
-        <f>IF($B68&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C68,$O$6:$O$205)+SUMIF($C$6:$C$205,$C68,$P$6:$P$205))</f>
+        <f>IF($B68&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C68,$O$8:$O$207)+SUMIF($C$8:$C$207,$C68,$P$8:$P$207))</f>
       </c>
       <c r="S68" s="27">
         <f>IF(OR($B68&lt;&gt;"Challan",$C68="",G68=0),"",IF(ROUND(G68-R68,2)=0,"Matches","Check Entries"))</f>
@@ -2977,7 +3036,7 @@
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A69" s="15">
-        <f>IF($B69="Entry",COUNTIF($B$6:$B69,"Entry"),"")</f>
+        <f>IF($B69="Entry",COUNTIF($B$8:$B69,"Entry"),"")</f>
       </c>
       <c r="B69" s="16"/>
       <c r="C69" s="17"/>
@@ -2996,7 +3055,7 @@
       <c r="P69" s="24"/>
       <c r="Q69" s="26"/>
       <c r="R69" s="27">
-        <f>IF($B69&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C69,$O$6:$O$205)+SUMIF($C$6:$C$205,$C69,$P$6:$P$205))</f>
+        <f>IF($B69&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C69,$O$8:$O$207)+SUMIF($C$8:$C$207,$C69,$P$8:$P$207))</f>
       </c>
       <c r="S69" s="27">
         <f>IF(OR($B69&lt;&gt;"Challan",$C69="",G69=0),"",IF(ROUND(G69-R69,2)=0,"Matches","Check Entries"))</f>
@@ -3004,7 +3063,7 @@
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70" s="15">
-        <f>IF($B70="Entry",COUNTIF($B$6:$B70,"Entry"),"")</f>
+        <f>IF($B70="Entry",COUNTIF($B$8:$B70,"Entry"),"")</f>
       </c>
       <c r="B70" s="16"/>
       <c r="C70" s="17"/>
@@ -3023,7 +3082,7 @@
       <c r="P70" s="24"/>
       <c r="Q70" s="26"/>
       <c r="R70" s="27">
-        <f>IF($B70&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C70,$O$6:$O$205)+SUMIF($C$6:$C$205,$C70,$P$6:$P$205))</f>
+        <f>IF($B70&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C70,$O$8:$O$207)+SUMIF($C$8:$C$207,$C70,$P$8:$P$207))</f>
       </c>
       <c r="S70" s="27">
         <f>IF(OR($B70&lt;&gt;"Challan",$C70="",G70=0),"",IF(ROUND(G70-R70,2)=0,"Matches","Check Entries"))</f>
@@ -3031,7 +3090,7 @@
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A71" s="15">
-        <f>IF($B71="Entry",COUNTIF($B$6:$B71,"Entry"),"")</f>
+        <f>IF($B71="Entry",COUNTIF($B$8:$B71,"Entry"),"")</f>
       </c>
       <c r="B71" s="16"/>
       <c r="C71" s="17"/>
@@ -3050,7 +3109,7 @@
       <c r="P71" s="24"/>
       <c r="Q71" s="26"/>
       <c r="R71" s="27">
-        <f>IF($B71&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C71,$O$6:$O$205)+SUMIF($C$6:$C$205,$C71,$P$6:$P$205))</f>
+        <f>IF($B71&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C71,$O$8:$O$207)+SUMIF($C$8:$C$207,$C71,$P$8:$P$207))</f>
       </c>
       <c r="S71" s="27">
         <f>IF(OR($B71&lt;&gt;"Challan",$C71="",G71=0),"",IF(ROUND(G71-R71,2)=0,"Matches","Check Entries"))</f>
@@ -3058,7 +3117,7 @@
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A72" s="15">
-        <f>IF($B72="Entry",COUNTIF($B$6:$B72,"Entry"),"")</f>
+        <f>IF($B72="Entry",COUNTIF($B$8:$B72,"Entry"),"")</f>
       </c>
       <c r="B72" s="16"/>
       <c r="C72" s="17"/>
@@ -3077,7 +3136,7 @@
       <c r="P72" s="24"/>
       <c r="Q72" s="26"/>
       <c r="R72" s="27">
-        <f>IF($B72&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C72,$O$6:$O$205)+SUMIF($C$6:$C$205,$C72,$P$6:$P$205))</f>
+        <f>IF($B72&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C72,$O$8:$O$207)+SUMIF($C$8:$C$207,$C72,$P$8:$P$207))</f>
       </c>
       <c r="S72" s="27">
         <f>IF(OR($B72&lt;&gt;"Challan",$C72="",G72=0),"",IF(ROUND(G72-R72,2)=0,"Matches","Check Entries"))</f>
@@ -3085,7 +3144,7 @@
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A73" s="15">
-        <f>IF($B73="Entry",COUNTIF($B$6:$B73,"Entry"),"")</f>
+        <f>IF($B73="Entry",COUNTIF($B$8:$B73,"Entry"),"")</f>
       </c>
       <c r="B73" s="16"/>
       <c r="C73" s="17"/>
@@ -3104,7 +3163,7 @@
       <c r="P73" s="24"/>
       <c r="Q73" s="26"/>
       <c r="R73" s="27">
-        <f>IF($B73&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C73,$O$6:$O$205)+SUMIF($C$6:$C$205,$C73,$P$6:$P$205))</f>
+        <f>IF($B73&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C73,$O$8:$O$207)+SUMIF($C$8:$C$207,$C73,$P$8:$P$207))</f>
       </c>
       <c r="S73" s="27">
         <f>IF(OR($B73&lt;&gt;"Challan",$C73="",G73=0),"",IF(ROUND(G73-R73,2)=0,"Matches","Check Entries"))</f>
@@ -3112,7 +3171,7 @@
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A74" s="15">
-        <f>IF($B74="Entry",COUNTIF($B$6:$B74,"Entry"),"")</f>
+        <f>IF($B74="Entry",COUNTIF($B$8:$B74,"Entry"),"")</f>
       </c>
       <c r="B74" s="16"/>
       <c r="C74" s="17"/>
@@ -3131,7 +3190,7 @@
       <c r="P74" s="24"/>
       <c r="Q74" s="26"/>
       <c r="R74" s="27">
-        <f>IF($B74&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C74,$O$6:$O$205)+SUMIF($C$6:$C$205,$C74,$P$6:$P$205))</f>
+        <f>IF($B74&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C74,$O$8:$O$207)+SUMIF($C$8:$C$207,$C74,$P$8:$P$207))</f>
       </c>
       <c r="S74" s="27">
         <f>IF(OR($B74&lt;&gt;"Challan",$C74="",G74=0),"",IF(ROUND(G74-R74,2)=0,"Matches","Check Entries"))</f>
@@ -3139,7 +3198,7 @@
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A75" s="15">
-        <f>IF($B75="Entry",COUNTIF($B$6:$B75,"Entry"),"")</f>
+        <f>IF($B75="Entry",COUNTIF($B$8:$B75,"Entry"),"")</f>
       </c>
       <c r="B75" s="16"/>
       <c r="C75" s="17"/>
@@ -3158,7 +3217,7 @@
       <c r="P75" s="24"/>
       <c r="Q75" s="26"/>
       <c r="R75" s="27">
-        <f>IF($B75&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C75,$O$6:$O$205)+SUMIF($C$6:$C$205,$C75,$P$6:$P$205))</f>
+        <f>IF($B75&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C75,$O$8:$O$207)+SUMIF($C$8:$C$207,$C75,$P$8:$P$207))</f>
       </c>
       <c r="S75" s="27">
         <f>IF(OR($B75&lt;&gt;"Challan",$C75="",G75=0),"",IF(ROUND(G75-R75,2)=0,"Matches","Check Entries"))</f>
@@ -3166,7 +3225,7 @@
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A76" s="15">
-        <f>IF($B76="Entry",COUNTIF($B$6:$B76,"Entry"),"")</f>
+        <f>IF($B76="Entry",COUNTIF($B$8:$B76,"Entry"),"")</f>
       </c>
       <c r="B76" s="16"/>
       <c r="C76" s="17"/>
@@ -3185,7 +3244,7 @@
       <c r="P76" s="24"/>
       <c r="Q76" s="26"/>
       <c r="R76" s="27">
-        <f>IF($B76&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C76,$O$6:$O$205)+SUMIF($C$6:$C$205,$C76,$P$6:$P$205))</f>
+        <f>IF($B76&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C76,$O$8:$O$207)+SUMIF($C$8:$C$207,$C76,$P$8:$P$207))</f>
       </c>
       <c r="S76" s="27">
         <f>IF(OR($B76&lt;&gt;"Challan",$C76="",G76=0),"",IF(ROUND(G76-R76,2)=0,"Matches","Check Entries"))</f>
@@ -3193,7 +3252,7 @@
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77" s="15">
-        <f>IF($B77="Entry",COUNTIF($B$6:$B77,"Entry"),"")</f>
+        <f>IF($B77="Entry",COUNTIF($B$8:$B77,"Entry"),"")</f>
       </c>
       <c r="B77" s="16"/>
       <c r="C77" s="17"/>
@@ -3212,7 +3271,7 @@
       <c r="P77" s="24"/>
       <c r="Q77" s="26"/>
       <c r="R77" s="27">
-        <f>IF($B77&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C77,$O$6:$O$205)+SUMIF($C$6:$C$205,$C77,$P$6:$P$205))</f>
+        <f>IF($B77&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C77,$O$8:$O$207)+SUMIF($C$8:$C$207,$C77,$P$8:$P$207))</f>
       </c>
       <c r="S77" s="27">
         <f>IF(OR($B77&lt;&gt;"Challan",$C77="",G77=0),"",IF(ROUND(G77-R77,2)=0,"Matches","Check Entries"))</f>
@@ -3220,7 +3279,7 @@
     </row>
     <row r="78" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A78" s="15">
-        <f>IF($B78="Entry",COUNTIF($B$6:$B78,"Entry"),"")</f>
+        <f>IF($B78="Entry",COUNTIF($B$8:$B78,"Entry"),"")</f>
       </c>
       <c r="B78" s="16"/>
       <c r="C78" s="17"/>
@@ -3239,7 +3298,7 @@
       <c r="P78" s="24"/>
       <c r="Q78" s="26"/>
       <c r="R78" s="27">
-        <f>IF($B78&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C78,$O$6:$O$205)+SUMIF($C$6:$C$205,$C78,$P$6:$P$205))</f>
+        <f>IF($B78&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C78,$O$8:$O$207)+SUMIF($C$8:$C$207,$C78,$P$8:$P$207))</f>
       </c>
       <c r="S78" s="27">
         <f>IF(OR($B78&lt;&gt;"Challan",$C78="",G78=0),"",IF(ROUND(G78-R78,2)=0,"Matches","Check Entries"))</f>
@@ -3247,7 +3306,7 @@
     </row>
     <row r="79" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A79" s="15">
-        <f>IF($B79="Entry",COUNTIF($B$6:$B79,"Entry"),"")</f>
+        <f>IF($B79="Entry",COUNTIF($B$8:$B79,"Entry"),"")</f>
       </c>
       <c r="B79" s="16"/>
       <c r="C79" s="17"/>
@@ -3266,7 +3325,7 @@
       <c r="P79" s="24"/>
       <c r="Q79" s="26"/>
       <c r="R79" s="27">
-        <f>IF($B79&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C79,$O$6:$O$205)+SUMIF($C$6:$C$205,$C79,$P$6:$P$205))</f>
+        <f>IF($B79&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C79,$O$8:$O$207)+SUMIF($C$8:$C$207,$C79,$P$8:$P$207))</f>
       </c>
       <c r="S79" s="27">
         <f>IF(OR($B79&lt;&gt;"Challan",$C79="",G79=0),"",IF(ROUND(G79-R79,2)=0,"Matches","Check Entries"))</f>
@@ -3274,7 +3333,7 @@
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80" s="15">
-        <f>IF($B80="Entry",COUNTIF($B$6:$B80,"Entry"),"")</f>
+        <f>IF($B80="Entry",COUNTIF($B$8:$B80,"Entry"),"")</f>
       </c>
       <c r="B80" s="16"/>
       <c r="C80" s="17"/>
@@ -3293,7 +3352,7 @@
       <c r="P80" s="24"/>
       <c r="Q80" s="26"/>
       <c r="R80" s="27">
-        <f>IF($B80&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C80,$O$6:$O$205)+SUMIF($C$6:$C$205,$C80,$P$6:$P$205))</f>
+        <f>IF($B80&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C80,$O$8:$O$207)+SUMIF($C$8:$C$207,$C80,$P$8:$P$207))</f>
       </c>
       <c r="S80" s="27">
         <f>IF(OR($B80&lt;&gt;"Challan",$C80="",G80=0),"",IF(ROUND(G80-R80,2)=0,"Matches","Check Entries"))</f>
@@ -3301,7 +3360,7 @@
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" s="15">
-        <f>IF($B81="Entry",COUNTIF($B$6:$B81,"Entry"),"")</f>
+        <f>IF($B81="Entry",COUNTIF($B$8:$B81,"Entry"),"")</f>
       </c>
       <c r="B81" s="16"/>
       <c r="C81" s="17"/>
@@ -3320,7 +3379,7 @@
       <c r="P81" s="24"/>
       <c r="Q81" s="26"/>
       <c r="R81" s="27">
-        <f>IF($B81&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C81,$O$6:$O$205)+SUMIF($C$6:$C$205,$C81,$P$6:$P$205))</f>
+        <f>IF($B81&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C81,$O$8:$O$207)+SUMIF($C$8:$C$207,$C81,$P$8:$P$207))</f>
       </c>
       <c r="S81" s="27">
         <f>IF(OR($B81&lt;&gt;"Challan",$C81="",G81=0),"",IF(ROUND(G81-R81,2)=0,"Matches","Check Entries"))</f>
@@ -3328,7 +3387,7 @@
     </row>
     <row r="82" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A82" s="15">
-        <f>IF($B82="Entry",COUNTIF($B$6:$B82,"Entry"),"")</f>
+        <f>IF($B82="Entry",COUNTIF($B$8:$B82,"Entry"),"")</f>
       </c>
       <c r="B82" s="16"/>
       <c r="C82" s="17"/>
@@ -3347,7 +3406,7 @@
       <c r="P82" s="24"/>
       <c r="Q82" s="26"/>
       <c r="R82" s="27">
-        <f>IF($B82&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C82,$O$6:$O$205)+SUMIF($C$6:$C$205,$C82,$P$6:$P$205))</f>
+        <f>IF($B82&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C82,$O$8:$O$207)+SUMIF($C$8:$C$207,$C82,$P$8:$P$207))</f>
       </c>
       <c r="S82" s="27">
         <f>IF(OR($B82&lt;&gt;"Challan",$C82="",G82=0),"",IF(ROUND(G82-R82,2)=0,"Matches","Check Entries"))</f>
@@ -3355,7 +3414,7 @@
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83" s="15">
-        <f>IF($B83="Entry",COUNTIF($B$6:$B83,"Entry"),"")</f>
+        <f>IF($B83="Entry",COUNTIF($B$8:$B83,"Entry"),"")</f>
       </c>
       <c r="B83" s="16"/>
       <c r="C83" s="17"/>
@@ -3374,7 +3433,7 @@
       <c r="P83" s="24"/>
       <c r="Q83" s="26"/>
       <c r="R83" s="27">
-        <f>IF($B83&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C83,$O$6:$O$205)+SUMIF($C$6:$C$205,$C83,$P$6:$P$205))</f>
+        <f>IF($B83&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C83,$O$8:$O$207)+SUMIF($C$8:$C$207,$C83,$P$8:$P$207))</f>
       </c>
       <c r="S83" s="27">
         <f>IF(OR($B83&lt;&gt;"Challan",$C83="",G83=0),"",IF(ROUND(G83-R83,2)=0,"Matches","Check Entries"))</f>
@@ -3382,7 +3441,7 @@
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84" s="15">
-        <f>IF($B84="Entry",COUNTIF($B$6:$B84,"Entry"),"")</f>
+        <f>IF($B84="Entry",COUNTIF($B$8:$B84,"Entry"),"")</f>
       </c>
       <c r="B84" s="16"/>
       <c r="C84" s="17"/>
@@ -3401,7 +3460,7 @@
       <c r="P84" s="24"/>
       <c r="Q84" s="26"/>
       <c r="R84" s="27">
-        <f>IF($B84&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C84,$O$6:$O$205)+SUMIF($C$6:$C$205,$C84,$P$6:$P$205))</f>
+        <f>IF($B84&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C84,$O$8:$O$207)+SUMIF($C$8:$C$207,$C84,$P$8:$P$207))</f>
       </c>
       <c r="S84" s="27">
         <f>IF(OR($B84&lt;&gt;"Challan",$C84="",G84=0),"",IF(ROUND(G84-R84,2)=0,"Matches","Check Entries"))</f>
@@ -3409,7 +3468,7 @@
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85" s="15">
-        <f>IF($B85="Entry",COUNTIF($B$6:$B85,"Entry"),"")</f>
+        <f>IF($B85="Entry",COUNTIF($B$8:$B85,"Entry"),"")</f>
       </c>
       <c r="B85" s="16"/>
       <c r="C85" s="17"/>
@@ -3428,7 +3487,7 @@
       <c r="P85" s="24"/>
       <c r="Q85" s="26"/>
       <c r="R85" s="27">
-        <f>IF($B85&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C85,$O$6:$O$205)+SUMIF($C$6:$C$205,$C85,$P$6:$P$205))</f>
+        <f>IF($B85&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C85,$O$8:$O$207)+SUMIF($C$8:$C$207,$C85,$P$8:$P$207))</f>
       </c>
       <c r="S85" s="27">
         <f>IF(OR($B85&lt;&gt;"Challan",$C85="",G85=0),"",IF(ROUND(G85-R85,2)=0,"Matches","Check Entries"))</f>
@@ -3436,7 +3495,7 @@
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" s="15">
-        <f>IF($B86="Entry",COUNTIF($B$6:$B86,"Entry"),"")</f>
+        <f>IF($B86="Entry",COUNTIF($B$8:$B86,"Entry"),"")</f>
       </c>
       <c r="B86" s="16"/>
       <c r="C86" s="17"/>
@@ -3455,7 +3514,7 @@
       <c r="P86" s="24"/>
       <c r="Q86" s="26"/>
       <c r="R86" s="27">
-        <f>IF($B86&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C86,$O$6:$O$205)+SUMIF($C$6:$C$205,$C86,$P$6:$P$205))</f>
+        <f>IF($B86&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C86,$O$8:$O$207)+SUMIF($C$8:$C$207,$C86,$P$8:$P$207))</f>
       </c>
       <c r="S86" s="27">
         <f>IF(OR($B86&lt;&gt;"Challan",$C86="",G86=0),"",IF(ROUND(G86-R86,2)=0,"Matches","Check Entries"))</f>
@@ -3463,7 +3522,7 @@
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87" s="15">
-        <f>IF($B87="Entry",COUNTIF($B$6:$B87,"Entry"),"")</f>
+        <f>IF($B87="Entry",COUNTIF($B$8:$B87,"Entry"),"")</f>
       </c>
       <c r="B87" s="16"/>
       <c r="C87" s="17"/>
@@ -3482,7 +3541,7 @@
       <c r="P87" s="24"/>
       <c r="Q87" s="26"/>
       <c r="R87" s="27">
-        <f>IF($B87&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C87,$O$6:$O$205)+SUMIF($C$6:$C$205,$C87,$P$6:$P$205))</f>
+        <f>IF($B87&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C87,$O$8:$O$207)+SUMIF($C$8:$C$207,$C87,$P$8:$P$207))</f>
       </c>
       <c r="S87" s="27">
         <f>IF(OR($B87&lt;&gt;"Challan",$C87="",G87=0),"",IF(ROUND(G87-R87,2)=0,"Matches","Check Entries"))</f>
@@ -3490,7 +3549,7 @@
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88" s="15">
-        <f>IF($B88="Entry",COUNTIF($B$6:$B88,"Entry"),"")</f>
+        <f>IF($B88="Entry",COUNTIF($B$8:$B88,"Entry"),"")</f>
       </c>
       <c r="B88" s="16"/>
       <c r="C88" s="17"/>
@@ -3509,7 +3568,7 @@
       <c r="P88" s="24"/>
       <c r="Q88" s="26"/>
       <c r="R88" s="27">
-        <f>IF($B88&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C88,$O$6:$O$205)+SUMIF($C$6:$C$205,$C88,$P$6:$P$205))</f>
+        <f>IF($B88&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C88,$O$8:$O$207)+SUMIF($C$8:$C$207,$C88,$P$8:$P$207))</f>
       </c>
       <c r="S88" s="27">
         <f>IF(OR($B88&lt;&gt;"Challan",$C88="",G88=0),"",IF(ROUND(G88-R88,2)=0,"Matches","Check Entries"))</f>
@@ -3517,7 +3576,7 @@
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89" s="15">
-        <f>IF($B89="Entry",COUNTIF($B$6:$B89,"Entry"),"")</f>
+        <f>IF($B89="Entry",COUNTIF($B$8:$B89,"Entry"),"")</f>
       </c>
       <c r="B89" s="16"/>
       <c r="C89" s="17"/>
@@ -3536,7 +3595,7 @@
       <c r="P89" s="24"/>
       <c r="Q89" s="26"/>
       <c r="R89" s="27">
-        <f>IF($B89&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C89,$O$6:$O$205)+SUMIF($C$6:$C$205,$C89,$P$6:$P$205))</f>
+        <f>IF($B89&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C89,$O$8:$O$207)+SUMIF($C$8:$C$207,$C89,$P$8:$P$207))</f>
       </c>
       <c r="S89" s="27">
         <f>IF(OR($B89&lt;&gt;"Challan",$C89="",G89=0),"",IF(ROUND(G89-R89,2)=0,"Matches","Check Entries"))</f>
@@ -3544,7 +3603,7 @@
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90" s="15">
-        <f>IF($B90="Entry",COUNTIF($B$6:$B90,"Entry"),"")</f>
+        <f>IF($B90="Entry",COUNTIF($B$8:$B90,"Entry"),"")</f>
       </c>
       <c r="B90" s="16"/>
       <c r="C90" s="17"/>
@@ -3563,7 +3622,7 @@
       <c r="P90" s="24"/>
       <c r="Q90" s="26"/>
       <c r="R90" s="27">
-        <f>IF($B90&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C90,$O$6:$O$205)+SUMIF($C$6:$C$205,$C90,$P$6:$P$205))</f>
+        <f>IF($B90&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C90,$O$8:$O$207)+SUMIF($C$8:$C$207,$C90,$P$8:$P$207))</f>
       </c>
       <c r="S90" s="27">
         <f>IF(OR($B90&lt;&gt;"Challan",$C90="",G90=0),"",IF(ROUND(G90-R90,2)=0,"Matches","Check Entries"))</f>
@@ -3571,7 +3630,7 @@
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91" s="15">
-        <f>IF($B91="Entry",COUNTIF($B$6:$B91,"Entry"),"")</f>
+        <f>IF($B91="Entry",COUNTIF($B$8:$B91,"Entry"),"")</f>
       </c>
       <c r="B91" s="16"/>
       <c r="C91" s="17"/>
@@ -3590,7 +3649,7 @@
       <c r="P91" s="24"/>
       <c r="Q91" s="26"/>
       <c r="R91" s="27">
-        <f>IF($B91&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C91,$O$6:$O$205)+SUMIF($C$6:$C$205,$C91,$P$6:$P$205))</f>
+        <f>IF($B91&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C91,$O$8:$O$207)+SUMIF($C$8:$C$207,$C91,$P$8:$P$207))</f>
       </c>
       <c r="S91" s="27">
         <f>IF(OR($B91&lt;&gt;"Challan",$C91="",G91=0),"",IF(ROUND(G91-R91,2)=0,"Matches","Check Entries"))</f>
@@ -3598,7 +3657,7 @@
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92" s="15">
-        <f>IF($B92="Entry",COUNTIF($B$6:$B92,"Entry"),"")</f>
+        <f>IF($B92="Entry",COUNTIF($B$8:$B92,"Entry"),"")</f>
       </c>
       <c r="B92" s="16"/>
       <c r="C92" s="17"/>
@@ -3617,7 +3676,7 @@
       <c r="P92" s="24"/>
       <c r="Q92" s="26"/>
       <c r="R92" s="27">
-        <f>IF($B92&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C92,$O$6:$O$205)+SUMIF($C$6:$C$205,$C92,$P$6:$P$205))</f>
+        <f>IF($B92&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C92,$O$8:$O$207)+SUMIF($C$8:$C$207,$C92,$P$8:$P$207))</f>
       </c>
       <c r="S92" s="27">
         <f>IF(OR($B92&lt;&gt;"Challan",$C92="",G92=0),"",IF(ROUND(G92-R92,2)=0,"Matches","Check Entries"))</f>
@@ -3625,7 +3684,7 @@
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93" s="15">
-        <f>IF($B93="Entry",COUNTIF($B$6:$B93,"Entry"),"")</f>
+        <f>IF($B93="Entry",COUNTIF($B$8:$B93,"Entry"),"")</f>
       </c>
       <c r="B93" s="16"/>
       <c r="C93" s="17"/>
@@ -3644,7 +3703,7 @@
       <c r="P93" s="24"/>
       <c r="Q93" s="26"/>
       <c r="R93" s="27">
-        <f>IF($B93&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C93,$O$6:$O$205)+SUMIF($C$6:$C$205,$C93,$P$6:$P$205))</f>
+        <f>IF($B93&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C93,$O$8:$O$207)+SUMIF($C$8:$C$207,$C93,$P$8:$P$207))</f>
       </c>
       <c r="S93" s="27">
         <f>IF(OR($B93&lt;&gt;"Challan",$C93="",G93=0),"",IF(ROUND(G93-R93,2)=0,"Matches","Check Entries"))</f>
@@ -3652,7 +3711,7 @@
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94" s="15">
-        <f>IF($B94="Entry",COUNTIF($B$6:$B94,"Entry"),"")</f>
+        <f>IF($B94="Entry",COUNTIF($B$8:$B94,"Entry"),"")</f>
       </c>
       <c r="B94" s="16"/>
       <c r="C94" s="17"/>
@@ -3671,7 +3730,7 @@
       <c r="P94" s="24"/>
       <c r="Q94" s="26"/>
       <c r="R94" s="27">
-        <f>IF($B94&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C94,$O$6:$O$205)+SUMIF($C$6:$C$205,$C94,$P$6:$P$205))</f>
+        <f>IF($B94&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C94,$O$8:$O$207)+SUMIF($C$8:$C$207,$C94,$P$8:$P$207))</f>
       </c>
       <c r="S94" s="27">
         <f>IF(OR($B94&lt;&gt;"Challan",$C94="",G94=0),"",IF(ROUND(G94-R94,2)=0,"Matches","Check Entries"))</f>
@@ -3679,7 +3738,7 @@
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95" s="15">
-        <f>IF($B95="Entry",COUNTIF($B$6:$B95,"Entry"),"")</f>
+        <f>IF($B95="Entry",COUNTIF($B$8:$B95,"Entry"),"")</f>
       </c>
       <c r="B95" s="16"/>
       <c r="C95" s="17"/>
@@ -3698,7 +3757,7 @@
       <c r="P95" s="24"/>
       <c r="Q95" s="26"/>
       <c r="R95" s="27">
-        <f>IF($B95&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C95,$O$6:$O$205)+SUMIF($C$6:$C$205,$C95,$P$6:$P$205))</f>
+        <f>IF($B95&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C95,$O$8:$O$207)+SUMIF($C$8:$C$207,$C95,$P$8:$P$207))</f>
       </c>
       <c r="S95" s="27">
         <f>IF(OR($B95&lt;&gt;"Challan",$C95="",G95=0),"",IF(ROUND(G95-R95,2)=0,"Matches","Check Entries"))</f>
@@ -3706,7 +3765,7 @@
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A96" s="15">
-        <f>IF($B96="Entry",COUNTIF($B$6:$B96,"Entry"),"")</f>
+        <f>IF($B96="Entry",COUNTIF($B$8:$B96,"Entry"),"")</f>
       </c>
       <c r="B96" s="16"/>
       <c r="C96" s="17"/>
@@ -3725,7 +3784,7 @@
       <c r="P96" s="24"/>
       <c r="Q96" s="26"/>
       <c r="R96" s="27">
-        <f>IF($B96&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C96,$O$6:$O$205)+SUMIF($C$6:$C$205,$C96,$P$6:$P$205))</f>
+        <f>IF($B96&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C96,$O$8:$O$207)+SUMIF($C$8:$C$207,$C96,$P$8:$P$207))</f>
       </c>
       <c r="S96" s="27">
         <f>IF(OR($B96&lt;&gt;"Challan",$C96="",G96=0),"",IF(ROUND(G96-R96,2)=0,"Matches","Check Entries"))</f>
@@ -3733,7 +3792,7 @@
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A97" s="15">
-        <f>IF($B97="Entry",COUNTIF($B$6:$B97,"Entry"),"")</f>
+        <f>IF($B97="Entry",COUNTIF($B$8:$B97,"Entry"),"")</f>
       </c>
       <c r="B97" s="16"/>
       <c r="C97" s="17"/>
@@ -3752,7 +3811,7 @@
       <c r="P97" s="24"/>
       <c r="Q97" s="26"/>
       <c r="R97" s="27">
-        <f>IF($B97&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C97,$O$6:$O$205)+SUMIF($C$6:$C$205,$C97,$P$6:$P$205))</f>
+        <f>IF($B97&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C97,$O$8:$O$207)+SUMIF($C$8:$C$207,$C97,$P$8:$P$207))</f>
       </c>
       <c r="S97" s="27">
         <f>IF(OR($B97&lt;&gt;"Challan",$C97="",G97=0),"",IF(ROUND(G97-R97,2)=0,"Matches","Check Entries"))</f>
@@ -3760,7 +3819,7 @@
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A98" s="15">
-        <f>IF($B98="Entry",COUNTIF($B$6:$B98,"Entry"),"")</f>
+        <f>IF($B98="Entry",COUNTIF($B$8:$B98,"Entry"),"")</f>
       </c>
       <c r="B98" s="16"/>
       <c r="C98" s="17"/>
@@ -3779,7 +3838,7 @@
       <c r="P98" s="24"/>
       <c r="Q98" s="26"/>
       <c r="R98" s="27">
-        <f>IF($B98&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C98,$O$6:$O$205)+SUMIF($C$6:$C$205,$C98,$P$6:$P$205))</f>
+        <f>IF($B98&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C98,$O$8:$O$207)+SUMIF($C$8:$C$207,$C98,$P$8:$P$207))</f>
       </c>
       <c r="S98" s="27">
         <f>IF(OR($B98&lt;&gt;"Challan",$C98="",G98=0),"",IF(ROUND(G98-R98,2)=0,"Matches","Check Entries"))</f>
@@ -3787,7 +3846,7 @@
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A99" s="15">
-        <f>IF($B99="Entry",COUNTIF($B$6:$B99,"Entry"),"")</f>
+        <f>IF($B99="Entry",COUNTIF($B$8:$B99,"Entry"),"")</f>
       </c>
       <c r="B99" s="16"/>
       <c r="C99" s="17"/>
@@ -3806,7 +3865,7 @@
       <c r="P99" s="24"/>
       <c r="Q99" s="26"/>
       <c r="R99" s="27">
-        <f>IF($B99&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C99,$O$6:$O$205)+SUMIF($C$6:$C$205,$C99,$P$6:$P$205))</f>
+        <f>IF($B99&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C99,$O$8:$O$207)+SUMIF($C$8:$C$207,$C99,$P$8:$P$207))</f>
       </c>
       <c r="S99" s="27">
         <f>IF(OR($B99&lt;&gt;"Challan",$C99="",G99=0),"",IF(ROUND(G99-R99,2)=0,"Matches","Check Entries"))</f>
@@ -3814,7 +3873,7 @@
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A100" s="15">
-        <f>IF($B100="Entry",COUNTIF($B$6:$B100,"Entry"),"")</f>
+        <f>IF($B100="Entry",COUNTIF($B$8:$B100,"Entry"),"")</f>
       </c>
       <c r="B100" s="16"/>
       <c r="C100" s="17"/>
@@ -3833,7 +3892,7 @@
       <c r="P100" s="24"/>
       <c r="Q100" s="26"/>
       <c r="R100" s="27">
-        <f>IF($B100&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C100,$O$6:$O$205)+SUMIF($C$6:$C$205,$C100,$P$6:$P$205))</f>
+        <f>IF($B100&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C100,$O$8:$O$207)+SUMIF($C$8:$C$207,$C100,$P$8:$P$207))</f>
       </c>
       <c r="S100" s="27">
         <f>IF(OR($B100&lt;&gt;"Challan",$C100="",G100=0),"",IF(ROUND(G100-R100,2)=0,"Matches","Check Entries"))</f>
@@ -3841,7 +3900,7 @@
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A101" s="15">
-        <f>IF($B101="Entry",COUNTIF($B$6:$B101,"Entry"),"")</f>
+        <f>IF($B101="Entry",COUNTIF($B$8:$B101,"Entry"),"")</f>
       </c>
       <c r="B101" s="16"/>
       <c r="C101" s="17"/>
@@ -3860,7 +3919,7 @@
       <c r="P101" s="24"/>
       <c r="Q101" s="26"/>
       <c r="R101" s="27">
-        <f>IF($B101&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C101,$O$6:$O$205)+SUMIF($C$6:$C$205,$C101,$P$6:$P$205))</f>
+        <f>IF($B101&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C101,$O$8:$O$207)+SUMIF($C$8:$C$207,$C101,$P$8:$P$207))</f>
       </c>
       <c r="S101" s="27">
         <f>IF(OR($B101&lt;&gt;"Challan",$C101="",G101=0),"",IF(ROUND(G101-R101,2)=0,"Matches","Check Entries"))</f>
@@ -3868,7 +3927,7 @@
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A102" s="15">
-        <f>IF($B102="Entry",COUNTIF($B$6:$B102,"Entry"),"")</f>
+        <f>IF($B102="Entry",COUNTIF($B$8:$B102,"Entry"),"")</f>
       </c>
       <c r="B102" s="16"/>
       <c r="C102" s="17"/>
@@ -3887,7 +3946,7 @@
       <c r="P102" s="24"/>
       <c r="Q102" s="26"/>
       <c r="R102" s="27">
-        <f>IF($B102&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C102,$O$6:$O$205)+SUMIF($C$6:$C$205,$C102,$P$6:$P$205))</f>
+        <f>IF($B102&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C102,$O$8:$O$207)+SUMIF($C$8:$C$207,$C102,$P$8:$P$207))</f>
       </c>
       <c r="S102" s="27">
         <f>IF(OR($B102&lt;&gt;"Challan",$C102="",G102=0),"",IF(ROUND(G102-R102,2)=0,"Matches","Check Entries"))</f>
@@ -3895,7 +3954,7 @@
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A103" s="15">
-        <f>IF($B103="Entry",COUNTIF($B$6:$B103,"Entry"),"")</f>
+        <f>IF($B103="Entry",COUNTIF($B$8:$B103,"Entry"),"")</f>
       </c>
       <c r="B103" s="16"/>
       <c r="C103" s="17"/>
@@ -3914,7 +3973,7 @@
       <c r="P103" s="24"/>
       <c r="Q103" s="26"/>
       <c r="R103" s="27">
-        <f>IF($B103&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C103,$O$6:$O$205)+SUMIF($C$6:$C$205,$C103,$P$6:$P$205))</f>
+        <f>IF($B103&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C103,$O$8:$O$207)+SUMIF($C$8:$C$207,$C103,$P$8:$P$207))</f>
       </c>
       <c r="S103" s="27">
         <f>IF(OR($B103&lt;&gt;"Challan",$C103="",G103=0),"",IF(ROUND(G103-R103,2)=0,"Matches","Check Entries"))</f>
@@ -3922,7 +3981,7 @@
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A104" s="15">
-        <f>IF($B104="Entry",COUNTIF($B$6:$B104,"Entry"),"")</f>
+        <f>IF($B104="Entry",COUNTIF($B$8:$B104,"Entry"),"")</f>
       </c>
       <c r="B104" s="16"/>
       <c r="C104" s="17"/>
@@ -3941,7 +4000,7 @@
       <c r="P104" s="24"/>
       <c r="Q104" s="26"/>
       <c r="R104" s="27">
-        <f>IF($B104&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C104,$O$6:$O$205)+SUMIF($C$6:$C$205,$C104,$P$6:$P$205))</f>
+        <f>IF($B104&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C104,$O$8:$O$207)+SUMIF($C$8:$C$207,$C104,$P$8:$P$207))</f>
       </c>
       <c r="S104" s="27">
         <f>IF(OR($B104&lt;&gt;"Challan",$C104="",G104=0),"",IF(ROUND(G104-R104,2)=0,"Matches","Check Entries"))</f>
@@ -3949,7 +4008,7 @@
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A105" s="15">
-        <f>IF($B105="Entry",COUNTIF($B$6:$B105,"Entry"),"")</f>
+        <f>IF($B105="Entry",COUNTIF($B$8:$B105,"Entry"),"")</f>
       </c>
       <c r="B105" s="16"/>
       <c r="C105" s="17"/>
@@ -3968,7 +4027,7 @@
       <c r="P105" s="24"/>
       <c r="Q105" s="26"/>
       <c r="R105" s="27">
-        <f>IF($B105&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C105,$O$6:$O$205)+SUMIF($C$6:$C$205,$C105,$P$6:$P$205))</f>
+        <f>IF($B105&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C105,$O$8:$O$207)+SUMIF($C$8:$C$207,$C105,$P$8:$P$207))</f>
       </c>
       <c r="S105" s="27">
         <f>IF(OR($B105&lt;&gt;"Challan",$C105="",G105=0),"",IF(ROUND(G105-R105,2)=0,"Matches","Check Entries"))</f>
@@ -3976,7 +4035,7 @@
     </row>
     <row r="106" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A106" s="15">
-        <f>IF($B106="Entry",COUNTIF($B$6:$B106,"Entry"),"")</f>
+        <f>IF($B106="Entry",COUNTIF($B$8:$B106,"Entry"),"")</f>
       </c>
       <c r="B106" s="16"/>
       <c r="C106" s="17"/>
@@ -3995,7 +4054,7 @@
       <c r="P106" s="24"/>
       <c r="Q106" s="26"/>
       <c r="R106" s="27">
-        <f>IF($B106&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C106,$O$6:$O$205)+SUMIF($C$6:$C$205,$C106,$P$6:$P$205))</f>
+        <f>IF($B106&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C106,$O$8:$O$207)+SUMIF($C$8:$C$207,$C106,$P$8:$P$207))</f>
       </c>
       <c r="S106" s="27">
         <f>IF(OR($B106&lt;&gt;"Challan",$C106="",G106=0),"",IF(ROUND(G106-R106,2)=0,"Matches","Check Entries"))</f>
@@ -4003,7 +4062,7 @@
     </row>
     <row r="107" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A107" s="15">
-        <f>IF($B107="Entry",COUNTIF($B$6:$B107,"Entry"),"")</f>
+        <f>IF($B107="Entry",COUNTIF($B$8:$B107,"Entry"),"")</f>
       </c>
       <c r="B107" s="16"/>
       <c r="C107" s="17"/>
@@ -4022,7 +4081,7 @@
       <c r="P107" s="24"/>
       <c r="Q107" s="26"/>
       <c r="R107" s="27">
-        <f>IF($B107&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C107,$O$6:$O$205)+SUMIF($C$6:$C$205,$C107,$P$6:$P$205))</f>
+        <f>IF($B107&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C107,$O$8:$O$207)+SUMIF($C$8:$C$207,$C107,$P$8:$P$207))</f>
       </c>
       <c r="S107" s="27">
         <f>IF(OR($B107&lt;&gt;"Challan",$C107="",G107=0),"",IF(ROUND(G107-R107,2)=0,"Matches","Check Entries"))</f>
@@ -4030,7 +4089,7 @@
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A108" s="15">
-        <f>IF($B108="Entry",COUNTIF($B$6:$B108,"Entry"),"")</f>
+        <f>IF($B108="Entry",COUNTIF($B$8:$B108,"Entry"),"")</f>
       </c>
       <c r="B108" s="16"/>
       <c r="C108" s="17"/>
@@ -4049,7 +4108,7 @@
       <c r="P108" s="24"/>
       <c r="Q108" s="26"/>
       <c r="R108" s="27">
-        <f>IF($B108&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C108,$O$6:$O$205)+SUMIF($C$6:$C$205,$C108,$P$6:$P$205))</f>
+        <f>IF($B108&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C108,$O$8:$O$207)+SUMIF($C$8:$C$207,$C108,$P$8:$P$207))</f>
       </c>
       <c r="S108" s="27">
         <f>IF(OR($B108&lt;&gt;"Challan",$C108="",G108=0),"",IF(ROUND(G108-R108,2)=0,"Matches","Check Entries"))</f>
@@ -4057,7 +4116,7 @@
     </row>
     <row r="109" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A109" s="15">
-        <f>IF($B109="Entry",COUNTIF($B$6:$B109,"Entry"),"")</f>
+        <f>IF($B109="Entry",COUNTIF($B$8:$B109,"Entry"),"")</f>
       </c>
       <c r="B109" s="16"/>
       <c r="C109" s="17"/>
@@ -4076,7 +4135,7 @@
       <c r="P109" s="24"/>
       <c r="Q109" s="26"/>
       <c r="R109" s="27">
-        <f>IF($B109&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C109,$O$6:$O$205)+SUMIF($C$6:$C$205,$C109,$P$6:$P$205))</f>
+        <f>IF($B109&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C109,$O$8:$O$207)+SUMIF($C$8:$C$207,$C109,$P$8:$P$207))</f>
       </c>
       <c r="S109" s="27">
         <f>IF(OR($B109&lt;&gt;"Challan",$C109="",G109=0),"",IF(ROUND(G109-R109,2)=0,"Matches","Check Entries"))</f>
@@ -4084,7 +4143,7 @@
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A110" s="15">
-        <f>IF($B110="Entry",COUNTIF($B$6:$B110,"Entry"),"")</f>
+        <f>IF($B110="Entry",COUNTIF($B$8:$B110,"Entry"),"")</f>
       </c>
       <c r="B110" s="16"/>
       <c r="C110" s="17"/>
@@ -4103,7 +4162,7 @@
       <c r="P110" s="24"/>
       <c r="Q110" s="26"/>
       <c r="R110" s="27">
-        <f>IF($B110&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C110,$O$6:$O$205)+SUMIF($C$6:$C$205,$C110,$P$6:$P$205))</f>
+        <f>IF($B110&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C110,$O$8:$O$207)+SUMIF($C$8:$C$207,$C110,$P$8:$P$207))</f>
       </c>
       <c r="S110" s="27">
         <f>IF(OR($B110&lt;&gt;"Challan",$C110="",G110=0),"",IF(ROUND(G110-R110,2)=0,"Matches","Check Entries"))</f>
@@ -4111,7 +4170,7 @@
     </row>
     <row r="111" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A111" s="15">
-        <f>IF($B111="Entry",COUNTIF($B$6:$B111,"Entry"),"")</f>
+        <f>IF($B111="Entry",COUNTIF($B$8:$B111,"Entry"),"")</f>
       </c>
       <c r="B111" s="16"/>
       <c r="C111" s="17"/>
@@ -4130,7 +4189,7 @@
       <c r="P111" s="24"/>
       <c r="Q111" s="26"/>
       <c r="R111" s="27">
-        <f>IF($B111&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C111,$O$6:$O$205)+SUMIF($C$6:$C$205,$C111,$P$6:$P$205))</f>
+        <f>IF($B111&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C111,$O$8:$O$207)+SUMIF($C$8:$C$207,$C111,$P$8:$P$207))</f>
       </c>
       <c r="S111" s="27">
         <f>IF(OR($B111&lt;&gt;"Challan",$C111="",G111=0),"",IF(ROUND(G111-R111,2)=0,"Matches","Check Entries"))</f>
@@ -4138,7 +4197,7 @@
     </row>
     <row r="112" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A112" s="15">
-        <f>IF($B112="Entry",COUNTIF($B$6:$B112,"Entry"),"")</f>
+        <f>IF($B112="Entry",COUNTIF($B$8:$B112,"Entry"),"")</f>
       </c>
       <c r="B112" s="16"/>
       <c r="C112" s="17"/>
@@ -4157,7 +4216,7 @@
       <c r="P112" s="24"/>
       <c r="Q112" s="26"/>
       <c r="R112" s="27">
-        <f>IF($B112&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C112,$O$6:$O$205)+SUMIF($C$6:$C$205,$C112,$P$6:$P$205))</f>
+        <f>IF($B112&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C112,$O$8:$O$207)+SUMIF($C$8:$C$207,$C112,$P$8:$P$207))</f>
       </c>
       <c r="S112" s="27">
         <f>IF(OR($B112&lt;&gt;"Challan",$C112="",G112=0),"",IF(ROUND(G112-R112,2)=0,"Matches","Check Entries"))</f>
@@ -4165,7 +4224,7 @@
     </row>
     <row r="113" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A113" s="15">
-        <f>IF($B113="Entry",COUNTIF($B$6:$B113,"Entry"),"")</f>
+        <f>IF($B113="Entry",COUNTIF($B$8:$B113,"Entry"),"")</f>
       </c>
       <c r="B113" s="16"/>
       <c r="C113" s="17"/>
@@ -4184,7 +4243,7 @@
       <c r="P113" s="24"/>
       <c r="Q113" s="26"/>
       <c r="R113" s="27">
-        <f>IF($B113&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C113,$O$6:$O$205)+SUMIF($C$6:$C$205,$C113,$P$6:$P$205))</f>
+        <f>IF($B113&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C113,$O$8:$O$207)+SUMIF($C$8:$C$207,$C113,$P$8:$P$207))</f>
       </c>
       <c r="S113" s="27">
         <f>IF(OR($B113&lt;&gt;"Challan",$C113="",G113=0),"",IF(ROUND(G113-R113,2)=0,"Matches","Check Entries"))</f>
@@ -4192,7 +4251,7 @@
     </row>
     <row r="114" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A114" s="15">
-        <f>IF($B114="Entry",COUNTIF($B$6:$B114,"Entry"),"")</f>
+        <f>IF($B114="Entry",COUNTIF($B$8:$B114,"Entry"),"")</f>
       </c>
       <c r="B114" s="16"/>
       <c r="C114" s="17"/>
@@ -4211,7 +4270,7 @@
       <c r="P114" s="24"/>
       <c r="Q114" s="26"/>
       <c r="R114" s="27">
-        <f>IF($B114&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C114,$O$6:$O$205)+SUMIF($C$6:$C$205,$C114,$P$6:$P$205))</f>
+        <f>IF($B114&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C114,$O$8:$O$207)+SUMIF($C$8:$C$207,$C114,$P$8:$P$207))</f>
       </c>
       <c r="S114" s="27">
         <f>IF(OR($B114&lt;&gt;"Challan",$C114="",G114=0),"",IF(ROUND(G114-R114,2)=0,"Matches","Check Entries"))</f>
@@ -4219,7 +4278,7 @@
     </row>
     <row r="115" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A115" s="15">
-        <f>IF($B115="Entry",COUNTIF($B$6:$B115,"Entry"),"")</f>
+        <f>IF($B115="Entry",COUNTIF($B$8:$B115,"Entry"),"")</f>
       </c>
       <c r="B115" s="16"/>
       <c r="C115" s="17"/>
@@ -4238,7 +4297,7 @@
       <c r="P115" s="24"/>
       <c r="Q115" s="26"/>
       <c r="R115" s="27">
-        <f>IF($B115&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C115,$O$6:$O$205)+SUMIF($C$6:$C$205,$C115,$P$6:$P$205))</f>
+        <f>IF($B115&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C115,$O$8:$O$207)+SUMIF($C$8:$C$207,$C115,$P$8:$P$207))</f>
       </c>
       <c r="S115" s="27">
         <f>IF(OR($B115&lt;&gt;"Challan",$C115="",G115=0),"",IF(ROUND(G115-R115,2)=0,"Matches","Check Entries"))</f>
@@ -4246,7 +4305,7 @@
     </row>
     <row r="116" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A116" s="15">
-        <f>IF($B116="Entry",COUNTIF($B$6:$B116,"Entry"),"")</f>
+        <f>IF($B116="Entry",COUNTIF($B$8:$B116,"Entry"),"")</f>
       </c>
       <c r="B116" s="16"/>
       <c r="C116" s="17"/>
@@ -4265,7 +4324,7 @@
       <c r="P116" s="24"/>
       <c r="Q116" s="26"/>
       <c r="R116" s="27">
-        <f>IF($B116&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C116,$O$6:$O$205)+SUMIF($C$6:$C$205,$C116,$P$6:$P$205))</f>
+        <f>IF($B116&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C116,$O$8:$O$207)+SUMIF($C$8:$C$207,$C116,$P$8:$P$207))</f>
       </c>
       <c r="S116" s="27">
         <f>IF(OR($B116&lt;&gt;"Challan",$C116="",G116=0),"",IF(ROUND(G116-R116,2)=0,"Matches","Check Entries"))</f>
@@ -4273,7 +4332,7 @@
     </row>
     <row r="117" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A117" s="15">
-        <f>IF($B117="Entry",COUNTIF($B$6:$B117,"Entry"),"")</f>
+        <f>IF($B117="Entry",COUNTIF($B$8:$B117,"Entry"),"")</f>
       </c>
       <c r="B117" s="16"/>
       <c r="C117" s="17"/>
@@ -4292,7 +4351,7 @@
       <c r="P117" s="24"/>
       <c r="Q117" s="26"/>
       <c r="R117" s="27">
-        <f>IF($B117&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C117,$O$6:$O$205)+SUMIF($C$6:$C$205,$C117,$P$6:$P$205))</f>
+        <f>IF($B117&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C117,$O$8:$O$207)+SUMIF($C$8:$C$207,$C117,$P$8:$P$207))</f>
       </c>
       <c r="S117" s="27">
         <f>IF(OR($B117&lt;&gt;"Challan",$C117="",G117=0),"",IF(ROUND(G117-R117,2)=0,"Matches","Check Entries"))</f>
@@ -4300,7 +4359,7 @@
     </row>
     <row r="118" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A118" s="15">
-        <f>IF($B118="Entry",COUNTIF($B$6:$B118,"Entry"),"")</f>
+        <f>IF($B118="Entry",COUNTIF($B$8:$B118,"Entry"),"")</f>
       </c>
       <c r="B118" s="16"/>
       <c r="C118" s="17"/>
@@ -4319,7 +4378,7 @@
       <c r="P118" s="24"/>
       <c r="Q118" s="26"/>
       <c r="R118" s="27">
-        <f>IF($B118&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C118,$O$6:$O$205)+SUMIF($C$6:$C$205,$C118,$P$6:$P$205))</f>
+        <f>IF($B118&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C118,$O$8:$O$207)+SUMIF($C$8:$C$207,$C118,$P$8:$P$207))</f>
       </c>
       <c r="S118" s="27">
         <f>IF(OR($B118&lt;&gt;"Challan",$C118="",G118=0),"",IF(ROUND(G118-R118,2)=0,"Matches","Check Entries"))</f>
@@ -4327,7 +4386,7 @@
     </row>
     <row r="119" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A119" s="15">
-        <f>IF($B119="Entry",COUNTIF($B$6:$B119,"Entry"),"")</f>
+        <f>IF($B119="Entry",COUNTIF($B$8:$B119,"Entry"),"")</f>
       </c>
       <c r="B119" s="16"/>
       <c r="C119" s="17"/>
@@ -4346,7 +4405,7 @@
       <c r="P119" s="24"/>
       <c r="Q119" s="26"/>
       <c r="R119" s="27">
-        <f>IF($B119&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C119,$O$6:$O$205)+SUMIF($C$6:$C$205,$C119,$P$6:$P$205))</f>
+        <f>IF($B119&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C119,$O$8:$O$207)+SUMIF($C$8:$C$207,$C119,$P$8:$P$207))</f>
       </c>
       <c r="S119" s="27">
         <f>IF(OR($B119&lt;&gt;"Challan",$C119="",G119=0),"",IF(ROUND(G119-R119,2)=0,"Matches","Check Entries"))</f>
@@ -4354,7 +4413,7 @@
     </row>
     <row r="120" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A120" s="15">
-        <f>IF($B120="Entry",COUNTIF($B$6:$B120,"Entry"),"")</f>
+        <f>IF($B120="Entry",COUNTIF($B$8:$B120,"Entry"),"")</f>
       </c>
       <c r="B120" s="16"/>
       <c r="C120" s="17"/>
@@ -4373,7 +4432,7 @@
       <c r="P120" s="24"/>
       <c r="Q120" s="26"/>
       <c r="R120" s="27">
-        <f>IF($B120&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C120,$O$6:$O$205)+SUMIF($C$6:$C$205,$C120,$P$6:$P$205))</f>
+        <f>IF($B120&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C120,$O$8:$O$207)+SUMIF($C$8:$C$207,$C120,$P$8:$P$207))</f>
       </c>
       <c r="S120" s="27">
         <f>IF(OR($B120&lt;&gt;"Challan",$C120="",G120=0),"",IF(ROUND(G120-R120,2)=0,"Matches","Check Entries"))</f>
@@ -4381,7 +4440,7 @@
     </row>
     <row r="121" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A121" s="15">
-        <f>IF($B121="Entry",COUNTIF($B$6:$B121,"Entry"),"")</f>
+        <f>IF($B121="Entry",COUNTIF($B$8:$B121,"Entry"),"")</f>
       </c>
       <c r="B121" s="16"/>
       <c r="C121" s="17"/>
@@ -4400,7 +4459,7 @@
       <c r="P121" s="24"/>
       <c r="Q121" s="26"/>
       <c r="R121" s="27">
-        <f>IF($B121&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C121,$O$6:$O$205)+SUMIF($C$6:$C$205,$C121,$P$6:$P$205))</f>
+        <f>IF($B121&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C121,$O$8:$O$207)+SUMIF($C$8:$C$207,$C121,$P$8:$P$207))</f>
       </c>
       <c r="S121" s="27">
         <f>IF(OR($B121&lt;&gt;"Challan",$C121="",G121=0),"",IF(ROUND(G121-R121,2)=0,"Matches","Check Entries"))</f>
@@ -4408,7 +4467,7 @@
     </row>
     <row r="122" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="15">
-        <f>IF($B122="Entry",COUNTIF($B$6:$B122,"Entry"),"")</f>
+        <f>IF($B122="Entry",COUNTIF($B$8:$B122,"Entry"),"")</f>
       </c>
       <c r="B122" s="16"/>
       <c r="C122" s="17"/>
@@ -4427,7 +4486,7 @@
       <c r="P122" s="24"/>
       <c r="Q122" s="26"/>
       <c r="R122" s="27">
-        <f>IF($B122&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C122,$O$6:$O$205)+SUMIF($C$6:$C$205,$C122,$P$6:$P$205))</f>
+        <f>IF($B122&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C122,$O$8:$O$207)+SUMIF($C$8:$C$207,$C122,$P$8:$P$207))</f>
       </c>
       <c r="S122" s="27">
         <f>IF(OR($B122&lt;&gt;"Challan",$C122="",G122=0),"",IF(ROUND(G122-R122,2)=0,"Matches","Check Entries"))</f>
@@ -4435,7 +4494,7 @@
     </row>
     <row r="123" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A123" s="15">
-        <f>IF($B123="Entry",COUNTIF($B$6:$B123,"Entry"),"")</f>
+        <f>IF($B123="Entry",COUNTIF($B$8:$B123,"Entry"),"")</f>
       </c>
       <c r="B123" s="16"/>
       <c r="C123" s="17"/>
@@ -4454,7 +4513,7 @@
       <c r="P123" s="24"/>
       <c r="Q123" s="26"/>
       <c r="R123" s="27">
-        <f>IF($B123&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C123,$O$6:$O$205)+SUMIF($C$6:$C$205,$C123,$P$6:$P$205))</f>
+        <f>IF($B123&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C123,$O$8:$O$207)+SUMIF($C$8:$C$207,$C123,$P$8:$P$207))</f>
       </c>
       <c r="S123" s="27">
         <f>IF(OR($B123&lt;&gt;"Challan",$C123="",G123=0),"",IF(ROUND(G123-R123,2)=0,"Matches","Check Entries"))</f>
@@ -4462,7 +4521,7 @@
     </row>
     <row r="124" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A124" s="15">
-        <f>IF($B124="Entry",COUNTIF($B$6:$B124,"Entry"),"")</f>
+        <f>IF($B124="Entry",COUNTIF($B$8:$B124,"Entry"),"")</f>
       </c>
       <c r="B124" s="16"/>
       <c r="C124" s="17"/>
@@ -4481,7 +4540,7 @@
       <c r="P124" s="24"/>
       <c r="Q124" s="26"/>
       <c r="R124" s="27">
-        <f>IF($B124&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C124,$O$6:$O$205)+SUMIF($C$6:$C$205,$C124,$P$6:$P$205))</f>
+        <f>IF($B124&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C124,$O$8:$O$207)+SUMIF($C$8:$C$207,$C124,$P$8:$P$207))</f>
       </c>
       <c r="S124" s="27">
         <f>IF(OR($B124&lt;&gt;"Challan",$C124="",G124=0),"",IF(ROUND(G124-R124,2)=0,"Matches","Check Entries"))</f>
@@ -4489,7 +4548,7 @@
     </row>
     <row r="125" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A125" s="15">
-        <f>IF($B125="Entry",COUNTIF($B$6:$B125,"Entry"),"")</f>
+        <f>IF($B125="Entry",COUNTIF($B$8:$B125,"Entry"),"")</f>
       </c>
       <c r="B125" s="16"/>
       <c r="C125" s="17"/>
@@ -4508,7 +4567,7 @@
       <c r="P125" s="24"/>
       <c r="Q125" s="26"/>
       <c r="R125" s="27">
-        <f>IF($B125&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C125,$O$6:$O$205)+SUMIF($C$6:$C$205,$C125,$P$6:$P$205))</f>
+        <f>IF($B125&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C125,$O$8:$O$207)+SUMIF($C$8:$C$207,$C125,$P$8:$P$207))</f>
       </c>
       <c r="S125" s="27">
         <f>IF(OR($B125&lt;&gt;"Challan",$C125="",G125=0),"",IF(ROUND(G125-R125,2)=0,"Matches","Check Entries"))</f>
@@ -4516,7 +4575,7 @@
     </row>
     <row r="126" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A126" s="15">
-        <f>IF($B126="Entry",COUNTIF($B$6:$B126,"Entry"),"")</f>
+        <f>IF($B126="Entry",COUNTIF($B$8:$B126,"Entry"),"")</f>
       </c>
       <c r="B126" s="16"/>
       <c r="C126" s="17"/>
@@ -4535,7 +4594,7 @@
       <c r="P126" s="24"/>
       <c r="Q126" s="26"/>
       <c r="R126" s="27">
-        <f>IF($B126&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C126,$O$6:$O$205)+SUMIF($C$6:$C$205,$C126,$P$6:$P$205))</f>
+        <f>IF($B126&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C126,$O$8:$O$207)+SUMIF($C$8:$C$207,$C126,$P$8:$P$207))</f>
       </c>
       <c r="S126" s="27">
         <f>IF(OR($B126&lt;&gt;"Challan",$C126="",G126=0),"",IF(ROUND(G126-R126,2)=0,"Matches","Check Entries"))</f>
@@ -4543,7 +4602,7 @@
     </row>
     <row r="127" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A127" s="15">
-        <f>IF($B127="Entry",COUNTIF($B$6:$B127,"Entry"),"")</f>
+        <f>IF($B127="Entry",COUNTIF($B$8:$B127,"Entry"),"")</f>
       </c>
       <c r="B127" s="16"/>
       <c r="C127" s="17"/>
@@ -4562,7 +4621,7 @@
       <c r="P127" s="24"/>
       <c r="Q127" s="26"/>
       <c r="R127" s="27">
-        <f>IF($B127&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C127,$O$6:$O$205)+SUMIF($C$6:$C$205,$C127,$P$6:$P$205))</f>
+        <f>IF($B127&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C127,$O$8:$O$207)+SUMIF($C$8:$C$207,$C127,$P$8:$P$207))</f>
       </c>
       <c r="S127" s="27">
         <f>IF(OR($B127&lt;&gt;"Challan",$C127="",G127=0),"",IF(ROUND(G127-R127,2)=0,"Matches","Check Entries"))</f>
@@ -4570,7 +4629,7 @@
     </row>
     <row r="128" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A128" s="15">
-        <f>IF($B128="Entry",COUNTIF($B$6:$B128,"Entry"),"")</f>
+        <f>IF($B128="Entry",COUNTIF($B$8:$B128,"Entry"),"")</f>
       </c>
       <c r="B128" s="16"/>
       <c r="C128" s="17"/>
@@ -4589,7 +4648,7 @@
       <c r="P128" s="24"/>
       <c r="Q128" s="26"/>
       <c r="R128" s="27">
-        <f>IF($B128&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C128,$O$6:$O$205)+SUMIF($C$6:$C$205,$C128,$P$6:$P$205))</f>
+        <f>IF($B128&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C128,$O$8:$O$207)+SUMIF($C$8:$C$207,$C128,$P$8:$P$207))</f>
       </c>
       <c r="S128" s="27">
         <f>IF(OR($B128&lt;&gt;"Challan",$C128="",G128=0),"",IF(ROUND(G128-R128,2)=0,"Matches","Check Entries"))</f>
@@ -4597,7 +4656,7 @@
     </row>
     <row r="129" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A129" s="15">
-        <f>IF($B129="Entry",COUNTIF($B$6:$B129,"Entry"),"")</f>
+        <f>IF($B129="Entry",COUNTIF($B$8:$B129,"Entry"),"")</f>
       </c>
       <c r="B129" s="16"/>
       <c r="C129" s="17"/>
@@ -4616,7 +4675,7 @@
       <c r="P129" s="24"/>
       <c r="Q129" s="26"/>
       <c r="R129" s="27">
-        <f>IF($B129&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C129,$O$6:$O$205)+SUMIF($C$6:$C$205,$C129,$P$6:$P$205))</f>
+        <f>IF($B129&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C129,$O$8:$O$207)+SUMIF($C$8:$C$207,$C129,$P$8:$P$207))</f>
       </c>
       <c r="S129" s="27">
         <f>IF(OR($B129&lt;&gt;"Challan",$C129="",G129=0),"",IF(ROUND(G129-R129,2)=0,"Matches","Check Entries"))</f>
@@ -4624,7 +4683,7 @@
     </row>
     <row r="130" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A130" s="15">
-        <f>IF($B130="Entry",COUNTIF($B$6:$B130,"Entry"),"")</f>
+        <f>IF($B130="Entry",COUNTIF($B$8:$B130,"Entry"),"")</f>
       </c>
       <c r="B130" s="16"/>
       <c r="C130" s="17"/>
@@ -4643,7 +4702,7 @@
       <c r="P130" s="24"/>
       <c r="Q130" s="26"/>
       <c r="R130" s="27">
-        <f>IF($B130&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C130,$O$6:$O$205)+SUMIF($C$6:$C$205,$C130,$P$6:$P$205))</f>
+        <f>IF($B130&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C130,$O$8:$O$207)+SUMIF($C$8:$C$207,$C130,$P$8:$P$207))</f>
       </c>
       <c r="S130" s="27">
         <f>IF(OR($B130&lt;&gt;"Challan",$C130="",G130=0),"",IF(ROUND(G130-R130,2)=0,"Matches","Check Entries"))</f>
@@ -4651,7 +4710,7 @@
     </row>
     <row r="131" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A131" s="15">
-        <f>IF($B131="Entry",COUNTIF($B$6:$B131,"Entry"),"")</f>
+        <f>IF($B131="Entry",COUNTIF($B$8:$B131,"Entry"),"")</f>
       </c>
       <c r="B131" s="16"/>
       <c r="C131" s="17"/>
@@ -4670,7 +4729,7 @@
       <c r="P131" s="24"/>
       <c r="Q131" s="26"/>
       <c r="R131" s="27">
-        <f>IF($B131&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C131,$O$6:$O$205)+SUMIF($C$6:$C$205,$C131,$P$6:$P$205))</f>
+        <f>IF($B131&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C131,$O$8:$O$207)+SUMIF($C$8:$C$207,$C131,$P$8:$P$207))</f>
       </c>
       <c r="S131" s="27">
         <f>IF(OR($B131&lt;&gt;"Challan",$C131="",G131=0),"",IF(ROUND(G131-R131,2)=0,"Matches","Check Entries"))</f>
@@ -4678,7 +4737,7 @@
     </row>
     <row r="132" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A132" s="15">
-        <f>IF($B132="Entry",COUNTIF($B$6:$B132,"Entry"),"")</f>
+        <f>IF($B132="Entry",COUNTIF($B$8:$B132,"Entry"),"")</f>
       </c>
       <c r="B132" s="16"/>
       <c r="C132" s="17"/>
@@ -4697,7 +4756,7 @@
       <c r="P132" s="24"/>
       <c r="Q132" s="26"/>
       <c r="R132" s="27">
-        <f>IF($B132&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C132,$O$6:$O$205)+SUMIF($C$6:$C$205,$C132,$P$6:$P$205))</f>
+        <f>IF($B132&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C132,$O$8:$O$207)+SUMIF($C$8:$C$207,$C132,$P$8:$P$207))</f>
       </c>
       <c r="S132" s="27">
         <f>IF(OR($B132&lt;&gt;"Challan",$C132="",G132=0),"",IF(ROUND(G132-R132,2)=0,"Matches","Check Entries"))</f>
@@ -4705,7 +4764,7 @@
     </row>
     <row r="133" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A133" s="15">
-        <f>IF($B133="Entry",COUNTIF($B$6:$B133,"Entry"),"")</f>
+        <f>IF($B133="Entry",COUNTIF($B$8:$B133,"Entry"),"")</f>
       </c>
       <c r="B133" s="16"/>
       <c r="C133" s="17"/>
@@ -4724,7 +4783,7 @@
       <c r="P133" s="24"/>
       <c r="Q133" s="26"/>
       <c r="R133" s="27">
-        <f>IF($B133&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C133,$O$6:$O$205)+SUMIF($C$6:$C$205,$C133,$P$6:$P$205))</f>
+        <f>IF($B133&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C133,$O$8:$O$207)+SUMIF($C$8:$C$207,$C133,$P$8:$P$207))</f>
       </c>
       <c r="S133" s="27">
         <f>IF(OR($B133&lt;&gt;"Challan",$C133="",G133=0),"",IF(ROUND(G133-R133,2)=0,"Matches","Check Entries"))</f>
@@ -4732,7 +4791,7 @@
     </row>
     <row r="134" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A134" s="15">
-        <f>IF($B134="Entry",COUNTIF($B$6:$B134,"Entry"),"")</f>
+        <f>IF($B134="Entry",COUNTIF($B$8:$B134,"Entry"),"")</f>
       </c>
       <c r="B134" s="16"/>
       <c r="C134" s="17"/>
@@ -4751,7 +4810,7 @@
       <c r="P134" s="24"/>
       <c r="Q134" s="26"/>
       <c r="R134" s="27">
-        <f>IF($B134&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C134,$O$6:$O$205)+SUMIF($C$6:$C$205,$C134,$P$6:$P$205))</f>
+        <f>IF($B134&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C134,$O$8:$O$207)+SUMIF($C$8:$C$207,$C134,$P$8:$P$207))</f>
       </c>
       <c r="S134" s="27">
         <f>IF(OR($B134&lt;&gt;"Challan",$C134="",G134=0),"",IF(ROUND(G134-R134,2)=0,"Matches","Check Entries"))</f>
@@ -4759,7 +4818,7 @@
     </row>
     <row r="135" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A135" s="15">
-        <f>IF($B135="Entry",COUNTIF($B$6:$B135,"Entry"),"")</f>
+        <f>IF($B135="Entry",COUNTIF($B$8:$B135,"Entry"),"")</f>
       </c>
       <c r="B135" s="16"/>
       <c r="C135" s="17"/>
@@ -4778,7 +4837,7 @@
       <c r="P135" s="24"/>
       <c r="Q135" s="26"/>
       <c r="R135" s="27">
-        <f>IF($B135&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C135,$O$6:$O$205)+SUMIF($C$6:$C$205,$C135,$P$6:$P$205))</f>
+        <f>IF($B135&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C135,$O$8:$O$207)+SUMIF($C$8:$C$207,$C135,$P$8:$P$207))</f>
       </c>
       <c r="S135" s="27">
         <f>IF(OR($B135&lt;&gt;"Challan",$C135="",G135=0),"",IF(ROUND(G135-R135,2)=0,"Matches","Check Entries"))</f>
@@ -4786,7 +4845,7 @@
     </row>
     <row r="136" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A136" s="15">
-        <f>IF($B136="Entry",COUNTIF($B$6:$B136,"Entry"),"")</f>
+        <f>IF($B136="Entry",COUNTIF($B$8:$B136,"Entry"),"")</f>
       </c>
       <c r="B136" s="16"/>
       <c r="C136" s="17"/>
@@ -4805,7 +4864,7 @@
       <c r="P136" s="24"/>
       <c r="Q136" s="26"/>
       <c r="R136" s="27">
-        <f>IF($B136&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C136,$O$6:$O$205)+SUMIF($C$6:$C$205,$C136,$P$6:$P$205))</f>
+        <f>IF($B136&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C136,$O$8:$O$207)+SUMIF($C$8:$C$207,$C136,$P$8:$P$207))</f>
       </c>
       <c r="S136" s="27">
         <f>IF(OR($B136&lt;&gt;"Challan",$C136="",G136=0),"",IF(ROUND(G136-R136,2)=0,"Matches","Check Entries"))</f>
@@ -4813,7 +4872,7 @@
     </row>
     <row r="137" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A137" s="15">
-        <f>IF($B137="Entry",COUNTIF($B$6:$B137,"Entry"),"")</f>
+        <f>IF($B137="Entry",COUNTIF($B$8:$B137,"Entry"),"")</f>
       </c>
       <c r="B137" s="16"/>
       <c r="C137" s="17"/>
@@ -4832,7 +4891,7 @@
       <c r="P137" s="24"/>
       <c r="Q137" s="26"/>
       <c r="R137" s="27">
-        <f>IF($B137&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C137,$O$6:$O$205)+SUMIF($C$6:$C$205,$C137,$P$6:$P$205))</f>
+        <f>IF($B137&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C137,$O$8:$O$207)+SUMIF($C$8:$C$207,$C137,$P$8:$P$207))</f>
       </c>
       <c r="S137" s="27">
         <f>IF(OR($B137&lt;&gt;"Challan",$C137="",G137=0),"",IF(ROUND(G137-R137,2)=0,"Matches","Check Entries"))</f>
@@ -4840,7 +4899,7 @@
     </row>
     <row r="138" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A138" s="15">
-        <f>IF($B138="Entry",COUNTIF($B$6:$B138,"Entry"),"")</f>
+        <f>IF($B138="Entry",COUNTIF($B$8:$B138,"Entry"),"")</f>
       </c>
       <c r="B138" s="16"/>
       <c r="C138" s="17"/>
@@ -4859,7 +4918,7 @@
       <c r="P138" s="24"/>
       <c r="Q138" s="26"/>
       <c r="R138" s="27">
-        <f>IF($B138&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C138,$O$6:$O$205)+SUMIF($C$6:$C$205,$C138,$P$6:$P$205))</f>
+        <f>IF($B138&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C138,$O$8:$O$207)+SUMIF($C$8:$C$207,$C138,$P$8:$P$207))</f>
       </c>
       <c r="S138" s="27">
         <f>IF(OR($B138&lt;&gt;"Challan",$C138="",G138=0),"",IF(ROUND(G138-R138,2)=0,"Matches","Check Entries"))</f>
@@ -4867,7 +4926,7 @@
     </row>
     <row r="139" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A139" s="15">
-        <f>IF($B139="Entry",COUNTIF($B$6:$B139,"Entry"),"")</f>
+        <f>IF($B139="Entry",COUNTIF($B$8:$B139,"Entry"),"")</f>
       </c>
       <c r="B139" s="16"/>
       <c r="C139" s="17"/>
@@ -4886,7 +4945,7 @@
       <c r="P139" s="24"/>
       <c r="Q139" s="26"/>
       <c r="R139" s="27">
-        <f>IF($B139&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C139,$O$6:$O$205)+SUMIF($C$6:$C$205,$C139,$P$6:$P$205))</f>
+        <f>IF($B139&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C139,$O$8:$O$207)+SUMIF($C$8:$C$207,$C139,$P$8:$P$207))</f>
       </c>
       <c r="S139" s="27">
         <f>IF(OR($B139&lt;&gt;"Challan",$C139="",G139=0),"",IF(ROUND(G139-R139,2)=0,"Matches","Check Entries"))</f>
@@ -4894,7 +4953,7 @@
     </row>
     <row r="140" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A140" s="15">
-        <f>IF($B140="Entry",COUNTIF($B$6:$B140,"Entry"),"")</f>
+        <f>IF($B140="Entry",COUNTIF($B$8:$B140,"Entry"),"")</f>
       </c>
       <c r="B140" s="16"/>
       <c r="C140" s="17"/>
@@ -4913,7 +4972,7 @@
       <c r="P140" s="24"/>
       <c r="Q140" s="26"/>
       <c r="R140" s="27">
-        <f>IF($B140&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C140,$O$6:$O$205)+SUMIF($C$6:$C$205,$C140,$P$6:$P$205))</f>
+        <f>IF($B140&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C140,$O$8:$O$207)+SUMIF($C$8:$C$207,$C140,$P$8:$P$207))</f>
       </c>
       <c r="S140" s="27">
         <f>IF(OR($B140&lt;&gt;"Challan",$C140="",G140=0),"",IF(ROUND(G140-R140,2)=0,"Matches","Check Entries"))</f>
@@ -4921,7 +4980,7 @@
     </row>
     <row r="141" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A141" s="15">
-        <f>IF($B141="Entry",COUNTIF($B$6:$B141,"Entry"),"")</f>
+        <f>IF($B141="Entry",COUNTIF($B$8:$B141,"Entry"),"")</f>
       </c>
       <c r="B141" s="16"/>
       <c r="C141" s="17"/>
@@ -4940,7 +4999,7 @@
       <c r="P141" s="24"/>
       <c r="Q141" s="26"/>
       <c r="R141" s="27">
-        <f>IF($B141&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C141,$O$6:$O$205)+SUMIF($C$6:$C$205,$C141,$P$6:$P$205))</f>
+        <f>IF($B141&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C141,$O$8:$O$207)+SUMIF($C$8:$C$207,$C141,$P$8:$P$207))</f>
       </c>
       <c r="S141" s="27">
         <f>IF(OR($B141&lt;&gt;"Challan",$C141="",G141=0),"",IF(ROUND(G141-R141,2)=0,"Matches","Check Entries"))</f>
@@ -4948,7 +5007,7 @@
     </row>
     <row r="142" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A142" s="15">
-        <f>IF($B142="Entry",COUNTIF($B$6:$B142,"Entry"),"")</f>
+        <f>IF($B142="Entry",COUNTIF($B$8:$B142,"Entry"),"")</f>
       </c>
       <c r="B142" s="16"/>
       <c r="C142" s="17"/>
@@ -4967,7 +5026,7 @@
       <c r="P142" s="24"/>
       <c r="Q142" s="26"/>
       <c r="R142" s="27">
-        <f>IF($B142&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C142,$O$6:$O$205)+SUMIF($C$6:$C$205,$C142,$P$6:$P$205))</f>
+        <f>IF($B142&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C142,$O$8:$O$207)+SUMIF($C$8:$C$207,$C142,$P$8:$P$207))</f>
       </c>
       <c r="S142" s="27">
         <f>IF(OR($B142&lt;&gt;"Challan",$C142="",G142=0),"",IF(ROUND(G142-R142,2)=0,"Matches","Check Entries"))</f>
@@ -4975,7 +5034,7 @@
     </row>
     <row r="143" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A143" s="15">
-        <f>IF($B143="Entry",COUNTIF($B$6:$B143,"Entry"),"")</f>
+        <f>IF($B143="Entry",COUNTIF($B$8:$B143,"Entry"),"")</f>
       </c>
       <c r="B143" s="16"/>
       <c r="C143" s="17"/>
@@ -4994,7 +5053,7 @@
       <c r="P143" s="24"/>
       <c r="Q143" s="26"/>
       <c r="R143" s="27">
-        <f>IF($B143&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C143,$O$6:$O$205)+SUMIF($C$6:$C$205,$C143,$P$6:$P$205))</f>
+        <f>IF($B143&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C143,$O$8:$O$207)+SUMIF($C$8:$C$207,$C143,$P$8:$P$207))</f>
       </c>
       <c r="S143" s="27">
         <f>IF(OR($B143&lt;&gt;"Challan",$C143="",G143=0),"",IF(ROUND(G143-R143,2)=0,"Matches","Check Entries"))</f>
@@ -5002,7 +5061,7 @@
     </row>
     <row r="144" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A144" s="15">
-        <f>IF($B144="Entry",COUNTIF($B$6:$B144,"Entry"),"")</f>
+        <f>IF($B144="Entry",COUNTIF($B$8:$B144,"Entry"),"")</f>
       </c>
       <c r="B144" s="16"/>
       <c r="C144" s="17"/>
@@ -5021,7 +5080,7 @@
       <c r="P144" s="24"/>
       <c r="Q144" s="26"/>
       <c r="R144" s="27">
-        <f>IF($B144&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C144,$O$6:$O$205)+SUMIF($C$6:$C$205,$C144,$P$6:$P$205))</f>
+        <f>IF($B144&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C144,$O$8:$O$207)+SUMIF($C$8:$C$207,$C144,$P$8:$P$207))</f>
       </c>
       <c r="S144" s="27">
         <f>IF(OR($B144&lt;&gt;"Challan",$C144="",G144=0),"",IF(ROUND(G144-R144,2)=0,"Matches","Check Entries"))</f>
@@ -5029,7 +5088,7 @@
     </row>
     <row r="145" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A145" s="15">
-        <f>IF($B145="Entry",COUNTIF($B$6:$B145,"Entry"),"")</f>
+        <f>IF($B145="Entry",COUNTIF($B$8:$B145,"Entry"),"")</f>
       </c>
       <c r="B145" s="16"/>
       <c r="C145" s="17"/>
@@ -5048,7 +5107,7 @@
       <c r="P145" s="24"/>
       <c r="Q145" s="26"/>
       <c r="R145" s="27">
-        <f>IF($B145&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C145,$O$6:$O$205)+SUMIF($C$6:$C$205,$C145,$P$6:$P$205))</f>
+        <f>IF($B145&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C145,$O$8:$O$207)+SUMIF($C$8:$C$207,$C145,$P$8:$P$207))</f>
       </c>
       <c r="S145" s="27">
         <f>IF(OR($B145&lt;&gt;"Challan",$C145="",G145=0),"",IF(ROUND(G145-R145,2)=0,"Matches","Check Entries"))</f>
@@ -5056,7 +5115,7 @@
     </row>
     <row r="146" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A146" s="15">
-        <f>IF($B146="Entry",COUNTIF($B$6:$B146,"Entry"),"")</f>
+        <f>IF($B146="Entry",COUNTIF($B$8:$B146,"Entry"),"")</f>
       </c>
       <c r="B146" s="16"/>
       <c r="C146" s="17"/>
@@ -5075,7 +5134,7 @@
       <c r="P146" s="24"/>
       <c r="Q146" s="26"/>
       <c r="R146" s="27">
-        <f>IF($B146&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C146,$O$6:$O$205)+SUMIF($C$6:$C$205,$C146,$P$6:$P$205))</f>
+        <f>IF($B146&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C146,$O$8:$O$207)+SUMIF($C$8:$C$207,$C146,$P$8:$P$207))</f>
       </c>
       <c r="S146" s="27">
         <f>IF(OR($B146&lt;&gt;"Challan",$C146="",G146=0),"",IF(ROUND(G146-R146,2)=0,"Matches","Check Entries"))</f>
@@ -5083,7 +5142,7 @@
     </row>
     <row r="147" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A147" s="15">
-        <f>IF($B147="Entry",COUNTIF($B$6:$B147,"Entry"),"")</f>
+        <f>IF($B147="Entry",COUNTIF($B$8:$B147,"Entry"),"")</f>
       </c>
       <c r="B147" s="16"/>
       <c r="C147" s="17"/>
@@ -5102,7 +5161,7 @@
       <c r="P147" s="24"/>
       <c r="Q147" s="26"/>
       <c r="R147" s="27">
-        <f>IF($B147&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C147,$O$6:$O$205)+SUMIF($C$6:$C$205,$C147,$P$6:$P$205))</f>
+        <f>IF($B147&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C147,$O$8:$O$207)+SUMIF($C$8:$C$207,$C147,$P$8:$P$207))</f>
       </c>
       <c r="S147" s="27">
         <f>IF(OR($B147&lt;&gt;"Challan",$C147="",G147=0),"",IF(ROUND(G147-R147,2)=0,"Matches","Check Entries"))</f>
@@ -5110,7 +5169,7 @@
     </row>
     <row r="148" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A148" s="15">
-        <f>IF($B148="Entry",COUNTIF($B$6:$B148,"Entry"),"")</f>
+        <f>IF($B148="Entry",COUNTIF($B$8:$B148,"Entry"),"")</f>
       </c>
       <c r="B148" s="16"/>
       <c r="C148" s="17"/>
@@ -5129,7 +5188,7 @@
       <c r="P148" s="24"/>
       <c r="Q148" s="26"/>
       <c r="R148" s="27">
-        <f>IF($B148&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C148,$O$6:$O$205)+SUMIF($C$6:$C$205,$C148,$P$6:$P$205))</f>
+        <f>IF($B148&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C148,$O$8:$O$207)+SUMIF($C$8:$C$207,$C148,$P$8:$P$207))</f>
       </c>
       <c r="S148" s="27">
         <f>IF(OR($B148&lt;&gt;"Challan",$C148="",G148=0),"",IF(ROUND(G148-R148,2)=0,"Matches","Check Entries"))</f>
@@ -5137,7 +5196,7 @@
     </row>
     <row r="149" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A149" s="15">
-        <f>IF($B149="Entry",COUNTIF($B$6:$B149,"Entry"),"")</f>
+        <f>IF($B149="Entry",COUNTIF($B$8:$B149,"Entry"),"")</f>
       </c>
       <c r="B149" s="16"/>
       <c r="C149" s="17"/>
@@ -5156,7 +5215,7 @@
       <c r="P149" s="24"/>
       <c r="Q149" s="26"/>
       <c r="R149" s="27">
-        <f>IF($B149&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C149,$O$6:$O$205)+SUMIF($C$6:$C$205,$C149,$P$6:$P$205))</f>
+        <f>IF($B149&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C149,$O$8:$O$207)+SUMIF($C$8:$C$207,$C149,$P$8:$P$207))</f>
       </c>
       <c r="S149" s="27">
         <f>IF(OR($B149&lt;&gt;"Challan",$C149="",G149=0),"",IF(ROUND(G149-R149,2)=0,"Matches","Check Entries"))</f>
@@ -5164,7 +5223,7 @@
     </row>
     <row r="150" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A150" s="15">
-        <f>IF($B150="Entry",COUNTIF($B$6:$B150,"Entry"),"")</f>
+        <f>IF($B150="Entry",COUNTIF($B$8:$B150,"Entry"),"")</f>
       </c>
       <c r="B150" s="16"/>
       <c r="C150" s="17"/>
@@ -5183,7 +5242,7 @@
       <c r="P150" s="24"/>
       <c r="Q150" s="26"/>
       <c r="R150" s="27">
-        <f>IF($B150&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C150,$O$6:$O$205)+SUMIF($C$6:$C$205,$C150,$P$6:$P$205))</f>
+        <f>IF($B150&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C150,$O$8:$O$207)+SUMIF($C$8:$C$207,$C150,$P$8:$P$207))</f>
       </c>
       <c r="S150" s="27">
         <f>IF(OR($B150&lt;&gt;"Challan",$C150="",G150=0),"",IF(ROUND(G150-R150,2)=0,"Matches","Check Entries"))</f>
@@ -5191,7 +5250,7 @@
     </row>
     <row r="151" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A151" s="15">
-        <f>IF($B151="Entry",COUNTIF($B$6:$B151,"Entry"),"")</f>
+        <f>IF($B151="Entry",COUNTIF($B$8:$B151,"Entry"),"")</f>
       </c>
       <c r="B151" s="16"/>
       <c r="C151" s="17"/>
@@ -5210,7 +5269,7 @@
       <c r="P151" s="24"/>
       <c r="Q151" s="26"/>
       <c r="R151" s="27">
-        <f>IF($B151&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C151,$O$6:$O$205)+SUMIF($C$6:$C$205,$C151,$P$6:$P$205))</f>
+        <f>IF($B151&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C151,$O$8:$O$207)+SUMIF($C$8:$C$207,$C151,$P$8:$P$207))</f>
       </c>
       <c r="S151" s="27">
         <f>IF(OR($B151&lt;&gt;"Challan",$C151="",G151=0),"",IF(ROUND(G151-R151,2)=0,"Matches","Check Entries"))</f>
@@ -5218,7 +5277,7 @@
     </row>
     <row r="152" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A152" s="15">
-        <f>IF($B152="Entry",COUNTIF($B$6:$B152,"Entry"),"")</f>
+        <f>IF($B152="Entry",COUNTIF($B$8:$B152,"Entry"),"")</f>
       </c>
       <c r="B152" s="16"/>
       <c r="C152" s="17"/>
@@ -5237,7 +5296,7 @@
       <c r="P152" s="24"/>
       <c r="Q152" s="26"/>
       <c r="R152" s="27">
-        <f>IF($B152&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C152,$O$6:$O$205)+SUMIF($C$6:$C$205,$C152,$P$6:$P$205))</f>
+        <f>IF($B152&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C152,$O$8:$O$207)+SUMIF($C$8:$C$207,$C152,$P$8:$P$207))</f>
       </c>
       <c r="S152" s="27">
         <f>IF(OR($B152&lt;&gt;"Challan",$C152="",G152=0),"",IF(ROUND(G152-R152,2)=0,"Matches","Check Entries"))</f>
@@ -5245,7 +5304,7 @@
     </row>
     <row r="153" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A153" s="15">
-        <f>IF($B153="Entry",COUNTIF($B$6:$B153,"Entry"),"")</f>
+        <f>IF($B153="Entry",COUNTIF($B$8:$B153,"Entry"),"")</f>
       </c>
       <c r="B153" s="16"/>
       <c r="C153" s="17"/>
@@ -5264,7 +5323,7 @@
       <c r="P153" s="24"/>
       <c r="Q153" s="26"/>
       <c r="R153" s="27">
-        <f>IF($B153&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C153,$O$6:$O$205)+SUMIF($C$6:$C$205,$C153,$P$6:$P$205))</f>
+        <f>IF($B153&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C153,$O$8:$O$207)+SUMIF($C$8:$C$207,$C153,$P$8:$P$207))</f>
       </c>
       <c r="S153" s="27">
         <f>IF(OR($B153&lt;&gt;"Challan",$C153="",G153=0),"",IF(ROUND(G153-R153,2)=0,"Matches","Check Entries"))</f>
@@ -5272,7 +5331,7 @@
     </row>
     <row r="154" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A154" s="15">
-        <f>IF($B154="Entry",COUNTIF($B$6:$B154,"Entry"),"")</f>
+        <f>IF($B154="Entry",COUNTIF($B$8:$B154,"Entry"),"")</f>
       </c>
       <c r="B154" s="16"/>
       <c r="C154" s="17"/>
@@ -5291,7 +5350,7 @@
       <c r="P154" s="24"/>
       <c r="Q154" s="26"/>
       <c r="R154" s="27">
-        <f>IF($B154&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C154,$O$6:$O$205)+SUMIF($C$6:$C$205,$C154,$P$6:$P$205))</f>
+        <f>IF($B154&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C154,$O$8:$O$207)+SUMIF($C$8:$C$207,$C154,$P$8:$P$207))</f>
       </c>
       <c r="S154" s="27">
         <f>IF(OR($B154&lt;&gt;"Challan",$C154="",G154=0),"",IF(ROUND(G154-R154,2)=0,"Matches","Check Entries"))</f>
@@ -5299,7 +5358,7 @@
     </row>
     <row r="155" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A155" s="15">
-        <f>IF($B155="Entry",COUNTIF($B$6:$B155,"Entry"),"")</f>
+        <f>IF($B155="Entry",COUNTIF($B$8:$B155,"Entry"),"")</f>
       </c>
       <c r="B155" s="16"/>
       <c r="C155" s="17"/>
@@ -5318,7 +5377,7 @@
       <c r="P155" s="24"/>
       <c r="Q155" s="26"/>
       <c r="R155" s="27">
-        <f>IF($B155&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C155,$O$6:$O$205)+SUMIF($C$6:$C$205,$C155,$P$6:$P$205))</f>
+        <f>IF($B155&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C155,$O$8:$O$207)+SUMIF($C$8:$C$207,$C155,$P$8:$P$207))</f>
       </c>
       <c r="S155" s="27">
         <f>IF(OR($B155&lt;&gt;"Challan",$C155="",G155=0),"",IF(ROUND(G155-R155,2)=0,"Matches","Check Entries"))</f>
@@ -5326,7 +5385,7 @@
     </row>
     <row r="156" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A156" s="15">
-        <f>IF($B156="Entry",COUNTIF($B$6:$B156,"Entry"),"")</f>
+        <f>IF($B156="Entry",COUNTIF($B$8:$B156,"Entry"),"")</f>
       </c>
       <c r="B156" s="16"/>
       <c r="C156" s="17"/>
@@ -5345,7 +5404,7 @@
       <c r="P156" s="24"/>
       <c r="Q156" s="26"/>
       <c r="R156" s="27">
-        <f>IF($B156&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C156,$O$6:$O$205)+SUMIF($C$6:$C$205,$C156,$P$6:$P$205))</f>
+        <f>IF($B156&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C156,$O$8:$O$207)+SUMIF($C$8:$C$207,$C156,$P$8:$P$207))</f>
       </c>
       <c r="S156" s="27">
         <f>IF(OR($B156&lt;&gt;"Challan",$C156="",G156=0),"",IF(ROUND(G156-R156,2)=0,"Matches","Check Entries"))</f>
@@ -5353,7 +5412,7 @@
     </row>
     <row r="157" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A157" s="15">
-        <f>IF($B157="Entry",COUNTIF($B$6:$B157,"Entry"),"")</f>
+        <f>IF($B157="Entry",COUNTIF($B$8:$B157,"Entry"),"")</f>
       </c>
       <c r="B157" s="16"/>
       <c r="C157" s="17"/>
@@ -5372,7 +5431,7 @@
       <c r="P157" s="24"/>
       <c r="Q157" s="26"/>
       <c r="R157" s="27">
-        <f>IF($B157&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C157,$O$6:$O$205)+SUMIF($C$6:$C$205,$C157,$P$6:$P$205))</f>
+        <f>IF($B157&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C157,$O$8:$O$207)+SUMIF($C$8:$C$207,$C157,$P$8:$P$207))</f>
       </c>
       <c r="S157" s="27">
         <f>IF(OR($B157&lt;&gt;"Challan",$C157="",G157=0),"",IF(ROUND(G157-R157,2)=0,"Matches","Check Entries"))</f>
@@ -5380,7 +5439,7 @@
     </row>
     <row r="158" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A158" s="15">
-        <f>IF($B158="Entry",COUNTIF($B$6:$B158,"Entry"),"")</f>
+        <f>IF($B158="Entry",COUNTIF($B$8:$B158,"Entry"),"")</f>
       </c>
       <c r="B158" s="16"/>
       <c r="C158" s="17"/>
@@ -5399,7 +5458,7 @@
       <c r="P158" s="24"/>
       <c r="Q158" s="26"/>
       <c r="R158" s="27">
-        <f>IF($B158&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C158,$O$6:$O$205)+SUMIF($C$6:$C$205,$C158,$P$6:$P$205))</f>
+        <f>IF($B158&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C158,$O$8:$O$207)+SUMIF($C$8:$C$207,$C158,$P$8:$P$207))</f>
       </c>
       <c r="S158" s="27">
         <f>IF(OR($B158&lt;&gt;"Challan",$C158="",G158=0),"",IF(ROUND(G158-R158,2)=0,"Matches","Check Entries"))</f>
@@ -5407,7 +5466,7 @@
     </row>
     <row r="159" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A159" s="15">
-        <f>IF($B159="Entry",COUNTIF($B$6:$B159,"Entry"),"")</f>
+        <f>IF($B159="Entry",COUNTIF($B$8:$B159,"Entry"),"")</f>
       </c>
       <c r="B159" s="16"/>
       <c r="C159" s="17"/>
@@ -5426,7 +5485,7 @@
       <c r="P159" s="24"/>
       <c r="Q159" s="26"/>
       <c r="R159" s="27">
-        <f>IF($B159&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C159,$O$6:$O$205)+SUMIF($C$6:$C$205,$C159,$P$6:$P$205))</f>
+        <f>IF($B159&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C159,$O$8:$O$207)+SUMIF($C$8:$C$207,$C159,$P$8:$P$207))</f>
       </c>
       <c r="S159" s="27">
         <f>IF(OR($B159&lt;&gt;"Challan",$C159="",G159=0),"",IF(ROUND(G159-R159,2)=0,"Matches","Check Entries"))</f>
@@ -5434,7 +5493,7 @@
     </row>
     <row r="160" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A160" s="15">
-        <f>IF($B160="Entry",COUNTIF($B$6:$B160,"Entry"),"")</f>
+        <f>IF($B160="Entry",COUNTIF($B$8:$B160,"Entry"),"")</f>
       </c>
       <c r="B160" s="16"/>
       <c r="C160" s="17"/>
@@ -5453,7 +5512,7 @@
       <c r="P160" s="24"/>
       <c r="Q160" s="26"/>
       <c r="R160" s="27">
-        <f>IF($B160&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C160,$O$6:$O$205)+SUMIF($C$6:$C$205,$C160,$P$6:$P$205))</f>
+        <f>IF($B160&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C160,$O$8:$O$207)+SUMIF($C$8:$C$207,$C160,$P$8:$P$207))</f>
       </c>
       <c r="S160" s="27">
         <f>IF(OR($B160&lt;&gt;"Challan",$C160="",G160=0),"",IF(ROUND(G160-R160,2)=0,"Matches","Check Entries"))</f>
@@ -5461,7 +5520,7 @@
     </row>
     <row r="161" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A161" s="15">
-        <f>IF($B161="Entry",COUNTIF($B$6:$B161,"Entry"),"")</f>
+        <f>IF($B161="Entry",COUNTIF($B$8:$B161,"Entry"),"")</f>
       </c>
       <c r="B161" s="16"/>
       <c r="C161" s="17"/>
@@ -5480,7 +5539,7 @@
       <c r="P161" s="24"/>
       <c r="Q161" s="26"/>
       <c r="R161" s="27">
-        <f>IF($B161&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C161,$O$6:$O$205)+SUMIF($C$6:$C$205,$C161,$P$6:$P$205))</f>
+        <f>IF($B161&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C161,$O$8:$O$207)+SUMIF($C$8:$C$207,$C161,$P$8:$P$207))</f>
       </c>
       <c r="S161" s="27">
         <f>IF(OR($B161&lt;&gt;"Challan",$C161="",G161=0),"",IF(ROUND(G161-R161,2)=0,"Matches","Check Entries"))</f>
@@ -5488,7 +5547,7 @@
     </row>
     <row r="162" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A162" s="15">
-        <f>IF($B162="Entry",COUNTIF($B$6:$B162,"Entry"),"")</f>
+        <f>IF($B162="Entry",COUNTIF($B$8:$B162,"Entry"),"")</f>
       </c>
       <c r="B162" s="16"/>
       <c r="C162" s="17"/>
@@ -5507,7 +5566,7 @@
       <c r="P162" s="24"/>
       <c r="Q162" s="26"/>
       <c r="R162" s="27">
-        <f>IF($B162&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C162,$O$6:$O$205)+SUMIF($C$6:$C$205,$C162,$P$6:$P$205))</f>
+        <f>IF($B162&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C162,$O$8:$O$207)+SUMIF($C$8:$C$207,$C162,$P$8:$P$207))</f>
       </c>
       <c r="S162" s="27">
         <f>IF(OR($B162&lt;&gt;"Challan",$C162="",G162=0),"",IF(ROUND(G162-R162,2)=0,"Matches","Check Entries"))</f>
@@ -5515,7 +5574,7 @@
     </row>
     <row r="163" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A163" s="15">
-        <f>IF($B163="Entry",COUNTIF($B$6:$B163,"Entry"),"")</f>
+        <f>IF($B163="Entry",COUNTIF($B$8:$B163,"Entry"),"")</f>
       </c>
       <c r="B163" s="16"/>
       <c r="C163" s="17"/>
@@ -5534,7 +5593,7 @@
       <c r="P163" s="24"/>
       <c r="Q163" s="26"/>
       <c r="R163" s="27">
-        <f>IF($B163&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C163,$O$6:$O$205)+SUMIF($C$6:$C$205,$C163,$P$6:$P$205))</f>
+        <f>IF($B163&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C163,$O$8:$O$207)+SUMIF($C$8:$C$207,$C163,$P$8:$P$207))</f>
       </c>
       <c r="S163" s="27">
         <f>IF(OR($B163&lt;&gt;"Challan",$C163="",G163=0),"",IF(ROUND(G163-R163,2)=0,"Matches","Check Entries"))</f>
@@ -5542,7 +5601,7 @@
     </row>
     <row r="164" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A164" s="15">
-        <f>IF($B164="Entry",COUNTIF($B$6:$B164,"Entry"),"")</f>
+        <f>IF($B164="Entry",COUNTIF($B$8:$B164,"Entry"),"")</f>
       </c>
       <c r="B164" s="16"/>
       <c r="C164" s="17"/>
@@ -5561,7 +5620,7 @@
       <c r="P164" s="24"/>
       <c r="Q164" s="26"/>
       <c r="R164" s="27">
-        <f>IF($B164&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C164,$O$6:$O$205)+SUMIF($C$6:$C$205,$C164,$P$6:$P$205))</f>
+        <f>IF($B164&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C164,$O$8:$O$207)+SUMIF($C$8:$C$207,$C164,$P$8:$P$207))</f>
       </c>
       <c r="S164" s="27">
         <f>IF(OR($B164&lt;&gt;"Challan",$C164="",G164=0),"",IF(ROUND(G164-R164,2)=0,"Matches","Check Entries"))</f>
@@ -5569,7 +5628,7 @@
     </row>
     <row r="165" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A165" s="15">
-        <f>IF($B165="Entry",COUNTIF($B$6:$B165,"Entry"),"")</f>
+        <f>IF($B165="Entry",COUNTIF($B$8:$B165,"Entry"),"")</f>
       </c>
       <c r="B165" s="16"/>
       <c r="C165" s="17"/>
@@ -5588,7 +5647,7 @@
       <c r="P165" s="24"/>
       <c r="Q165" s="26"/>
       <c r="R165" s="27">
-        <f>IF($B165&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C165,$O$6:$O$205)+SUMIF($C$6:$C$205,$C165,$P$6:$P$205))</f>
+        <f>IF($B165&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C165,$O$8:$O$207)+SUMIF($C$8:$C$207,$C165,$P$8:$P$207))</f>
       </c>
       <c r="S165" s="27">
         <f>IF(OR($B165&lt;&gt;"Challan",$C165="",G165=0),"",IF(ROUND(G165-R165,2)=0,"Matches","Check Entries"))</f>
@@ -5596,7 +5655,7 @@
     </row>
     <row r="166" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A166" s="15">
-        <f>IF($B166="Entry",COUNTIF($B$6:$B166,"Entry"),"")</f>
+        <f>IF($B166="Entry",COUNTIF($B$8:$B166,"Entry"),"")</f>
       </c>
       <c r="B166" s="16"/>
       <c r="C166" s="17"/>
@@ -5615,7 +5674,7 @@
       <c r="P166" s="24"/>
       <c r="Q166" s="26"/>
       <c r="R166" s="27">
-        <f>IF($B166&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C166,$O$6:$O$205)+SUMIF($C$6:$C$205,$C166,$P$6:$P$205))</f>
+        <f>IF($B166&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C166,$O$8:$O$207)+SUMIF($C$8:$C$207,$C166,$P$8:$P$207))</f>
       </c>
       <c r="S166" s="27">
         <f>IF(OR($B166&lt;&gt;"Challan",$C166="",G166=0),"",IF(ROUND(G166-R166,2)=0,"Matches","Check Entries"))</f>
@@ -5623,7 +5682,7 @@
     </row>
     <row r="167" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A167" s="15">
-        <f>IF($B167="Entry",COUNTIF($B$6:$B167,"Entry"),"")</f>
+        <f>IF($B167="Entry",COUNTIF($B$8:$B167,"Entry"),"")</f>
       </c>
       <c r="B167" s="16"/>
       <c r="C167" s="17"/>
@@ -5642,7 +5701,7 @@
       <c r="P167" s="24"/>
       <c r="Q167" s="26"/>
       <c r="R167" s="27">
-        <f>IF($B167&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C167,$O$6:$O$205)+SUMIF($C$6:$C$205,$C167,$P$6:$P$205))</f>
+        <f>IF($B167&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C167,$O$8:$O$207)+SUMIF($C$8:$C$207,$C167,$P$8:$P$207))</f>
       </c>
       <c r="S167" s="27">
         <f>IF(OR($B167&lt;&gt;"Challan",$C167="",G167=0),"",IF(ROUND(G167-R167,2)=0,"Matches","Check Entries"))</f>
@@ -5650,7 +5709,7 @@
     </row>
     <row r="168" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A168" s="15">
-        <f>IF($B168="Entry",COUNTIF($B$6:$B168,"Entry"),"")</f>
+        <f>IF($B168="Entry",COUNTIF($B$8:$B168,"Entry"),"")</f>
       </c>
       <c r="B168" s="16"/>
       <c r="C168" s="17"/>
@@ -5669,7 +5728,7 @@
       <c r="P168" s="24"/>
       <c r="Q168" s="26"/>
       <c r="R168" s="27">
-        <f>IF($B168&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C168,$O$6:$O$205)+SUMIF($C$6:$C$205,$C168,$P$6:$P$205))</f>
+        <f>IF($B168&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C168,$O$8:$O$207)+SUMIF($C$8:$C$207,$C168,$P$8:$P$207))</f>
       </c>
       <c r="S168" s="27">
         <f>IF(OR($B168&lt;&gt;"Challan",$C168="",G168=0),"",IF(ROUND(G168-R168,2)=0,"Matches","Check Entries"))</f>
@@ -5677,7 +5736,7 @@
     </row>
     <row r="169" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A169" s="15">
-        <f>IF($B169="Entry",COUNTIF($B$6:$B169,"Entry"),"")</f>
+        <f>IF($B169="Entry",COUNTIF($B$8:$B169,"Entry"),"")</f>
       </c>
       <c r="B169" s="16"/>
       <c r="C169" s="17"/>
@@ -5696,7 +5755,7 @@
       <c r="P169" s="24"/>
       <c r="Q169" s="26"/>
       <c r="R169" s="27">
-        <f>IF($B169&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C169,$O$6:$O$205)+SUMIF($C$6:$C$205,$C169,$P$6:$P$205))</f>
+        <f>IF($B169&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C169,$O$8:$O$207)+SUMIF($C$8:$C$207,$C169,$P$8:$P$207))</f>
       </c>
       <c r="S169" s="27">
         <f>IF(OR($B169&lt;&gt;"Challan",$C169="",G169=0),"",IF(ROUND(G169-R169,2)=0,"Matches","Check Entries"))</f>
@@ -5704,7 +5763,7 @@
     </row>
     <row r="170" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A170" s="15">
-        <f>IF($B170="Entry",COUNTIF($B$6:$B170,"Entry"),"")</f>
+        <f>IF($B170="Entry",COUNTIF($B$8:$B170,"Entry"),"")</f>
       </c>
       <c r="B170" s="16"/>
       <c r="C170" s="17"/>
@@ -5723,7 +5782,7 @@
       <c r="P170" s="24"/>
       <c r="Q170" s="26"/>
       <c r="R170" s="27">
-        <f>IF($B170&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C170,$O$6:$O$205)+SUMIF($C$6:$C$205,$C170,$P$6:$P$205))</f>
+        <f>IF($B170&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C170,$O$8:$O$207)+SUMIF($C$8:$C$207,$C170,$P$8:$P$207))</f>
       </c>
       <c r="S170" s="27">
         <f>IF(OR($B170&lt;&gt;"Challan",$C170="",G170=0),"",IF(ROUND(G170-R170,2)=0,"Matches","Check Entries"))</f>
@@ -5731,7 +5790,7 @@
     </row>
     <row r="171" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A171" s="15">
-        <f>IF($B171="Entry",COUNTIF($B$6:$B171,"Entry"),"")</f>
+        <f>IF($B171="Entry",COUNTIF($B$8:$B171,"Entry"),"")</f>
       </c>
       <c r="B171" s="16"/>
       <c r="C171" s="17"/>
@@ -5750,7 +5809,7 @@
       <c r="P171" s="24"/>
       <c r="Q171" s="26"/>
       <c r="R171" s="27">
-        <f>IF($B171&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C171,$O$6:$O$205)+SUMIF($C$6:$C$205,$C171,$P$6:$P$205))</f>
+        <f>IF($B171&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C171,$O$8:$O$207)+SUMIF($C$8:$C$207,$C171,$P$8:$P$207))</f>
       </c>
       <c r="S171" s="27">
         <f>IF(OR($B171&lt;&gt;"Challan",$C171="",G171=0),"",IF(ROUND(G171-R171,2)=0,"Matches","Check Entries"))</f>
@@ -5758,7 +5817,7 @@
     </row>
     <row r="172" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A172" s="15">
-        <f>IF($B172="Entry",COUNTIF($B$6:$B172,"Entry"),"")</f>
+        <f>IF($B172="Entry",COUNTIF($B$8:$B172,"Entry"),"")</f>
       </c>
       <c r="B172" s="16"/>
       <c r="C172" s="17"/>
@@ -5777,7 +5836,7 @@
       <c r="P172" s="24"/>
       <c r="Q172" s="26"/>
       <c r="R172" s="27">
-        <f>IF($B172&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C172,$O$6:$O$205)+SUMIF($C$6:$C$205,$C172,$P$6:$P$205))</f>
+        <f>IF($B172&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C172,$O$8:$O$207)+SUMIF($C$8:$C$207,$C172,$P$8:$P$207))</f>
       </c>
       <c r="S172" s="27">
         <f>IF(OR($B172&lt;&gt;"Challan",$C172="",G172=0),"",IF(ROUND(G172-R172,2)=0,"Matches","Check Entries"))</f>
@@ -5785,7 +5844,7 @@
     </row>
     <row r="173" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A173" s="15">
-        <f>IF($B173="Entry",COUNTIF($B$6:$B173,"Entry"),"")</f>
+        <f>IF($B173="Entry",COUNTIF($B$8:$B173,"Entry"),"")</f>
       </c>
       <c r="B173" s="16"/>
       <c r="C173" s="17"/>
@@ -5804,7 +5863,7 @@
       <c r="P173" s="24"/>
       <c r="Q173" s="26"/>
       <c r="R173" s="27">
-        <f>IF($B173&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C173,$O$6:$O$205)+SUMIF($C$6:$C$205,$C173,$P$6:$P$205))</f>
+        <f>IF($B173&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C173,$O$8:$O$207)+SUMIF($C$8:$C$207,$C173,$P$8:$P$207))</f>
       </c>
       <c r="S173" s="27">
         <f>IF(OR($B173&lt;&gt;"Challan",$C173="",G173=0),"",IF(ROUND(G173-R173,2)=0,"Matches","Check Entries"))</f>
@@ -5812,7 +5871,7 @@
     </row>
     <row r="174" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A174" s="15">
-        <f>IF($B174="Entry",COUNTIF($B$6:$B174,"Entry"),"")</f>
+        <f>IF($B174="Entry",COUNTIF($B$8:$B174,"Entry"),"")</f>
       </c>
       <c r="B174" s="16"/>
       <c r="C174" s="17"/>
@@ -5831,7 +5890,7 @@
       <c r="P174" s="24"/>
       <c r="Q174" s="26"/>
       <c r="R174" s="27">
-        <f>IF($B174&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C174,$O$6:$O$205)+SUMIF($C$6:$C$205,$C174,$P$6:$P$205))</f>
+        <f>IF($B174&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C174,$O$8:$O$207)+SUMIF($C$8:$C$207,$C174,$P$8:$P$207))</f>
       </c>
       <c r="S174" s="27">
         <f>IF(OR($B174&lt;&gt;"Challan",$C174="",G174=0),"",IF(ROUND(G174-R174,2)=0,"Matches","Check Entries"))</f>
@@ -5839,7 +5898,7 @@
     </row>
     <row r="175" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A175" s="15">
-        <f>IF($B175="Entry",COUNTIF($B$6:$B175,"Entry"),"")</f>
+        <f>IF($B175="Entry",COUNTIF($B$8:$B175,"Entry"),"")</f>
       </c>
       <c r="B175" s="16"/>
       <c r="C175" s="17"/>
@@ -5858,7 +5917,7 @@
       <c r="P175" s="24"/>
       <c r="Q175" s="26"/>
       <c r="R175" s="27">
-        <f>IF($B175&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C175,$O$6:$O$205)+SUMIF($C$6:$C$205,$C175,$P$6:$P$205))</f>
+        <f>IF($B175&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C175,$O$8:$O$207)+SUMIF($C$8:$C$207,$C175,$P$8:$P$207))</f>
       </c>
       <c r="S175" s="27">
         <f>IF(OR($B175&lt;&gt;"Challan",$C175="",G175=0),"",IF(ROUND(G175-R175,2)=0,"Matches","Check Entries"))</f>
@@ -5866,7 +5925,7 @@
     </row>
     <row r="176" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A176" s="15">
-        <f>IF($B176="Entry",COUNTIF($B$6:$B176,"Entry"),"")</f>
+        <f>IF($B176="Entry",COUNTIF($B$8:$B176,"Entry"),"")</f>
       </c>
       <c r="B176" s="16"/>
       <c r="C176" s="17"/>
@@ -5885,7 +5944,7 @@
       <c r="P176" s="24"/>
       <c r="Q176" s="26"/>
       <c r="R176" s="27">
-        <f>IF($B176&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C176,$O$6:$O$205)+SUMIF($C$6:$C$205,$C176,$P$6:$P$205))</f>
+        <f>IF($B176&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C176,$O$8:$O$207)+SUMIF($C$8:$C$207,$C176,$P$8:$P$207))</f>
       </c>
       <c r="S176" s="27">
         <f>IF(OR($B176&lt;&gt;"Challan",$C176="",G176=0),"",IF(ROUND(G176-R176,2)=0,"Matches","Check Entries"))</f>
@@ -5893,7 +5952,7 @@
     </row>
     <row r="177" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A177" s="15">
-        <f>IF($B177="Entry",COUNTIF($B$6:$B177,"Entry"),"")</f>
+        <f>IF($B177="Entry",COUNTIF($B$8:$B177,"Entry"),"")</f>
       </c>
       <c r="B177" s="16"/>
       <c r="C177" s="17"/>
@@ -5912,7 +5971,7 @@
       <c r="P177" s="24"/>
       <c r="Q177" s="26"/>
       <c r="R177" s="27">
-        <f>IF($B177&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C177,$O$6:$O$205)+SUMIF($C$6:$C$205,$C177,$P$6:$P$205))</f>
+        <f>IF($B177&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C177,$O$8:$O$207)+SUMIF($C$8:$C$207,$C177,$P$8:$P$207))</f>
       </c>
       <c r="S177" s="27">
         <f>IF(OR($B177&lt;&gt;"Challan",$C177="",G177=0),"",IF(ROUND(G177-R177,2)=0,"Matches","Check Entries"))</f>
@@ -5920,7 +5979,7 @@
     </row>
     <row r="178" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A178" s="15">
-        <f>IF($B178="Entry",COUNTIF($B$6:$B178,"Entry"),"")</f>
+        <f>IF($B178="Entry",COUNTIF($B$8:$B178,"Entry"),"")</f>
       </c>
       <c r="B178" s="16"/>
       <c r="C178" s="17"/>
@@ -5939,7 +5998,7 @@
       <c r="P178" s="24"/>
       <c r="Q178" s="26"/>
       <c r="R178" s="27">
-        <f>IF($B178&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C178,$O$6:$O$205)+SUMIF($C$6:$C$205,$C178,$P$6:$P$205))</f>
+        <f>IF($B178&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C178,$O$8:$O$207)+SUMIF($C$8:$C$207,$C178,$P$8:$P$207))</f>
       </c>
       <c r="S178" s="27">
         <f>IF(OR($B178&lt;&gt;"Challan",$C178="",G178=0),"",IF(ROUND(G178-R178,2)=0,"Matches","Check Entries"))</f>
@@ -5947,7 +6006,7 @@
     </row>
     <row r="179" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A179" s="15">
-        <f>IF($B179="Entry",COUNTIF($B$6:$B179,"Entry"),"")</f>
+        <f>IF($B179="Entry",COUNTIF($B$8:$B179,"Entry"),"")</f>
       </c>
       <c r="B179" s="16"/>
       <c r="C179" s="17"/>
@@ -5966,7 +6025,7 @@
       <c r="P179" s="24"/>
       <c r="Q179" s="26"/>
       <c r="R179" s="27">
-        <f>IF($B179&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C179,$O$6:$O$205)+SUMIF($C$6:$C$205,$C179,$P$6:$P$205))</f>
+        <f>IF($B179&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C179,$O$8:$O$207)+SUMIF($C$8:$C$207,$C179,$P$8:$P$207))</f>
       </c>
       <c r="S179" s="27">
         <f>IF(OR($B179&lt;&gt;"Challan",$C179="",G179=0),"",IF(ROUND(G179-R179,2)=0,"Matches","Check Entries"))</f>
@@ -5974,7 +6033,7 @@
     </row>
     <row r="180" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A180" s="15">
-        <f>IF($B180="Entry",COUNTIF($B$6:$B180,"Entry"),"")</f>
+        <f>IF($B180="Entry",COUNTIF($B$8:$B180,"Entry"),"")</f>
       </c>
       <c r="B180" s="16"/>
       <c r="C180" s="17"/>
@@ -5993,7 +6052,7 @@
       <c r="P180" s="24"/>
       <c r="Q180" s="26"/>
       <c r="R180" s="27">
-        <f>IF($B180&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C180,$O$6:$O$205)+SUMIF($C$6:$C$205,$C180,$P$6:$P$205))</f>
+        <f>IF($B180&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C180,$O$8:$O$207)+SUMIF($C$8:$C$207,$C180,$P$8:$P$207))</f>
       </c>
       <c r="S180" s="27">
         <f>IF(OR($B180&lt;&gt;"Challan",$C180="",G180=0),"",IF(ROUND(G180-R180,2)=0,"Matches","Check Entries"))</f>
@@ -6001,7 +6060,7 @@
     </row>
     <row r="181" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A181" s="15">
-        <f>IF($B181="Entry",COUNTIF($B$6:$B181,"Entry"),"")</f>
+        <f>IF($B181="Entry",COUNTIF($B$8:$B181,"Entry"),"")</f>
       </c>
       <c r="B181" s="16"/>
       <c r="C181" s="17"/>
@@ -6020,7 +6079,7 @@
       <c r="P181" s="24"/>
       <c r="Q181" s="26"/>
       <c r="R181" s="27">
-        <f>IF($B181&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C181,$O$6:$O$205)+SUMIF($C$6:$C$205,$C181,$P$6:$P$205))</f>
+        <f>IF($B181&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C181,$O$8:$O$207)+SUMIF($C$8:$C$207,$C181,$P$8:$P$207))</f>
       </c>
       <c r="S181" s="27">
         <f>IF(OR($B181&lt;&gt;"Challan",$C181="",G181=0),"",IF(ROUND(G181-R181,2)=0,"Matches","Check Entries"))</f>
@@ -6028,7 +6087,7 @@
     </row>
     <row r="182" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A182" s="15">
-        <f>IF($B182="Entry",COUNTIF($B$6:$B182,"Entry"),"")</f>
+        <f>IF($B182="Entry",COUNTIF($B$8:$B182,"Entry"),"")</f>
       </c>
       <c r="B182" s="16"/>
       <c r="C182" s="17"/>
@@ -6047,7 +6106,7 @@
       <c r="P182" s="24"/>
       <c r="Q182" s="26"/>
       <c r="R182" s="27">
-        <f>IF($B182&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C182,$O$6:$O$205)+SUMIF($C$6:$C$205,$C182,$P$6:$P$205))</f>
+        <f>IF($B182&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C182,$O$8:$O$207)+SUMIF($C$8:$C$207,$C182,$P$8:$P$207))</f>
       </c>
       <c r="S182" s="27">
         <f>IF(OR($B182&lt;&gt;"Challan",$C182="",G182=0),"",IF(ROUND(G182-R182,2)=0,"Matches","Check Entries"))</f>
@@ -6055,7 +6114,7 @@
     </row>
     <row r="183" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A183" s="15">
-        <f>IF($B183="Entry",COUNTIF($B$6:$B183,"Entry"),"")</f>
+        <f>IF($B183="Entry",COUNTIF($B$8:$B183,"Entry"),"")</f>
       </c>
       <c r="B183" s="16"/>
       <c r="C183" s="17"/>
@@ -6074,7 +6133,7 @@
       <c r="P183" s="24"/>
       <c r="Q183" s="26"/>
       <c r="R183" s="27">
-        <f>IF($B183&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C183,$O$6:$O$205)+SUMIF($C$6:$C$205,$C183,$P$6:$P$205))</f>
+        <f>IF($B183&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C183,$O$8:$O$207)+SUMIF($C$8:$C$207,$C183,$P$8:$P$207))</f>
       </c>
       <c r="S183" s="27">
         <f>IF(OR($B183&lt;&gt;"Challan",$C183="",G183=0),"",IF(ROUND(G183-R183,2)=0,"Matches","Check Entries"))</f>
@@ -6082,7 +6141,7 @@
     </row>
     <row r="184" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A184" s="15">
-        <f>IF($B184="Entry",COUNTIF($B$6:$B184,"Entry"),"")</f>
+        <f>IF($B184="Entry",COUNTIF($B$8:$B184,"Entry"),"")</f>
       </c>
       <c r="B184" s="16"/>
       <c r="C184" s="17"/>
@@ -6101,7 +6160,7 @@
       <c r="P184" s="24"/>
       <c r="Q184" s="26"/>
       <c r="R184" s="27">
-        <f>IF($B184&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C184,$O$6:$O$205)+SUMIF($C$6:$C$205,$C184,$P$6:$P$205))</f>
+        <f>IF($B184&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C184,$O$8:$O$207)+SUMIF($C$8:$C$207,$C184,$P$8:$P$207))</f>
       </c>
       <c r="S184" s="27">
         <f>IF(OR($B184&lt;&gt;"Challan",$C184="",G184=0),"",IF(ROUND(G184-R184,2)=0,"Matches","Check Entries"))</f>
@@ -6109,7 +6168,7 @@
     </row>
     <row r="185" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A185" s="15">
-        <f>IF($B185="Entry",COUNTIF($B$6:$B185,"Entry"),"")</f>
+        <f>IF($B185="Entry",COUNTIF($B$8:$B185,"Entry"),"")</f>
       </c>
       <c r="B185" s="16"/>
       <c r="C185" s="17"/>
@@ -6128,7 +6187,7 @@
       <c r="P185" s="24"/>
       <c r="Q185" s="26"/>
       <c r="R185" s="27">
-        <f>IF($B185&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C185,$O$6:$O$205)+SUMIF($C$6:$C$205,$C185,$P$6:$P$205))</f>
+        <f>IF($B185&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C185,$O$8:$O$207)+SUMIF($C$8:$C$207,$C185,$P$8:$P$207))</f>
       </c>
       <c r="S185" s="27">
         <f>IF(OR($B185&lt;&gt;"Challan",$C185="",G185=0),"",IF(ROUND(G185-R185,2)=0,"Matches","Check Entries"))</f>
@@ -6136,7 +6195,7 @@
     </row>
     <row r="186" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A186" s="15">
-        <f>IF($B186="Entry",COUNTIF($B$6:$B186,"Entry"),"")</f>
+        <f>IF($B186="Entry",COUNTIF($B$8:$B186,"Entry"),"")</f>
       </c>
       <c r="B186" s="16"/>
       <c r="C186" s="17"/>
@@ -6155,7 +6214,7 @@
       <c r="P186" s="24"/>
       <c r="Q186" s="26"/>
       <c r="R186" s="27">
-        <f>IF($B186&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C186,$O$6:$O$205)+SUMIF($C$6:$C$205,$C186,$P$6:$P$205))</f>
+        <f>IF($B186&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C186,$O$8:$O$207)+SUMIF($C$8:$C$207,$C186,$P$8:$P$207))</f>
       </c>
       <c r="S186" s="27">
         <f>IF(OR($B186&lt;&gt;"Challan",$C186="",G186=0),"",IF(ROUND(G186-R186,2)=0,"Matches","Check Entries"))</f>
@@ -6163,7 +6222,7 @@
     </row>
     <row r="187" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A187" s="15">
-        <f>IF($B187="Entry",COUNTIF($B$6:$B187,"Entry"),"")</f>
+        <f>IF($B187="Entry",COUNTIF($B$8:$B187,"Entry"),"")</f>
       </c>
       <c r="B187" s="16"/>
       <c r="C187" s="17"/>
@@ -6182,7 +6241,7 @@
       <c r="P187" s="24"/>
       <c r="Q187" s="26"/>
       <c r="R187" s="27">
-        <f>IF($B187&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C187,$O$6:$O$205)+SUMIF($C$6:$C$205,$C187,$P$6:$P$205))</f>
+        <f>IF($B187&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C187,$O$8:$O$207)+SUMIF($C$8:$C$207,$C187,$P$8:$P$207))</f>
       </c>
       <c r="S187" s="27">
         <f>IF(OR($B187&lt;&gt;"Challan",$C187="",G187=0),"",IF(ROUND(G187-R187,2)=0,"Matches","Check Entries"))</f>
@@ -6190,7 +6249,7 @@
     </row>
     <row r="188" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A188" s="15">
-        <f>IF($B188="Entry",COUNTIF($B$6:$B188,"Entry"),"")</f>
+        <f>IF($B188="Entry",COUNTIF($B$8:$B188,"Entry"),"")</f>
       </c>
       <c r="B188" s="16"/>
       <c r="C188" s="17"/>
@@ -6209,7 +6268,7 @@
       <c r="P188" s="24"/>
       <c r="Q188" s="26"/>
       <c r="R188" s="27">
-        <f>IF($B188&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C188,$O$6:$O$205)+SUMIF($C$6:$C$205,$C188,$P$6:$P$205))</f>
+        <f>IF($B188&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C188,$O$8:$O$207)+SUMIF($C$8:$C$207,$C188,$P$8:$P$207))</f>
       </c>
       <c r="S188" s="27">
         <f>IF(OR($B188&lt;&gt;"Challan",$C188="",G188=0),"",IF(ROUND(G188-R188,2)=0,"Matches","Check Entries"))</f>
@@ -6217,7 +6276,7 @@
     </row>
     <row r="189" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A189" s="15">
-        <f>IF($B189="Entry",COUNTIF($B$6:$B189,"Entry"),"")</f>
+        <f>IF($B189="Entry",COUNTIF($B$8:$B189,"Entry"),"")</f>
       </c>
       <c r="B189" s="16"/>
       <c r="C189" s="17"/>
@@ -6236,7 +6295,7 @@
       <c r="P189" s="24"/>
       <c r="Q189" s="26"/>
       <c r="R189" s="27">
-        <f>IF($B189&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C189,$O$6:$O$205)+SUMIF($C$6:$C$205,$C189,$P$6:$P$205))</f>
+        <f>IF($B189&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C189,$O$8:$O$207)+SUMIF($C$8:$C$207,$C189,$P$8:$P$207))</f>
       </c>
       <c r="S189" s="27">
         <f>IF(OR($B189&lt;&gt;"Challan",$C189="",G189=0),"",IF(ROUND(G189-R189,2)=0,"Matches","Check Entries"))</f>
@@ -6244,7 +6303,7 @@
     </row>
     <row r="190" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A190" s="15">
-        <f>IF($B190="Entry",COUNTIF($B$6:$B190,"Entry"),"")</f>
+        <f>IF($B190="Entry",COUNTIF($B$8:$B190,"Entry"),"")</f>
       </c>
       <c r="B190" s="16"/>
       <c r="C190" s="17"/>
@@ -6263,7 +6322,7 @@
       <c r="P190" s="24"/>
       <c r="Q190" s="26"/>
       <c r="R190" s="27">
-        <f>IF($B190&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C190,$O$6:$O$205)+SUMIF($C$6:$C$205,$C190,$P$6:$P$205))</f>
+        <f>IF($B190&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C190,$O$8:$O$207)+SUMIF($C$8:$C$207,$C190,$P$8:$P$207))</f>
       </c>
       <c r="S190" s="27">
         <f>IF(OR($B190&lt;&gt;"Challan",$C190="",G190=0),"",IF(ROUND(G190-R190,2)=0,"Matches","Check Entries"))</f>
@@ -6271,7 +6330,7 @@
     </row>
     <row r="191" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
-        <f>IF($B191="Entry",COUNTIF($B$6:$B191,"Entry"),"")</f>
+        <f>IF($B191="Entry",COUNTIF($B$8:$B191,"Entry"),"")</f>
       </c>
       <c r="B191" s="16"/>
       <c r="C191" s="17"/>
@@ -6290,7 +6349,7 @@
       <c r="P191" s="24"/>
       <c r="Q191" s="26"/>
       <c r="R191" s="27">
-        <f>IF($B191&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C191,$O$6:$O$205)+SUMIF($C$6:$C$205,$C191,$P$6:$P$205))</f>
+        <f>IF($B191&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C191,$O$8:$O$207)+SUMIF($C$8:$C$207,$C191,$P$8:$P$207))</f>
       </c>
       <c r="S191" s="27">
         <f>IF(OR($B191&lt;&gt;"Challan",$C191="",G191=0),"",IF(ROUND(G191-R191,2)=0,"Matches","Check Entries"))</f>
@@ -6298,7 +6357,7 @@
     </row>
     <row r="192" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
-        <f>IF($B192="Entry",COUNTIF($B$6:$B192,"Entry"),"")</f>
+        <f>IF($B192="Entry",COUNTIF($B$8:$B192,"Entry"),"")</f>
       </c>
       <c r="B192" s="16"/>
       <c r="C192" s="17"/>
@@ -6317,7 +6376,7 @@
       <c r="P192" s="24"/>
       <c r="Q192" s="26"/>
       <c r="R192" s="27">
-        <f>IF($B192&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C192,$O$6:$O$205)+SUMIF($C$6:$C$205,$C192,$P$6:$P$205))</f>
+        <f>IF($B192&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C192,$O$8:$O$207)+SUMIF($C$8:$C$207,$C192,$P$8:$P$207))</f>
       </c>
       <c r="S192" s="27">
         <f>IF(OR($B192&lt;&gt;"Challan",$C192="",G192=0),"",IF(ROUND(G192-R192,2)=0,"Matches","Check Entries"))</f>
@@ -6325,7 +6384,7 @@
     </row>
     <row r="193" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
-        <f>IF($B193="Entry",COUNTIF($B$6:$B193,"Entry"),"")</f>
+        <f>IF($B193="Entry",COUNTIF($B$8:$B193,"Entry"),"")</f>
       </c>
       <c r="B193" s="16"/>
       <c r="C193" s="17"/>
@@ -6344,7 +6403,7 @@
       <c r="P193" s="24"/>
       <c r="Q193" s="26"/>
       <c r="R193" s="27">
-        <f>IF($B193&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C193,$O$6:$O$205)+SUMIF($C$6:$C$205,$C193,$P$6:$P$205))</f>
+        <f>IF($B193&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C193,$O$8:$O$207)+SUMIF($C$8:$C$207,$C193,$P$8:$P$207))</f>
       </c>
       <c r="S193" s="27">
         <f>IF(OR($B193&lt;&gt;"Challan",$C193="",G193=0),"",IF(ROUND(G193-R193,2)=0,"Matches","Check Entries"))</f>
@@ -6352,7 +6411,7 @@
     </row>
     <row r="194" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A194" s="15">
-        <f>IF($B194="Entry",COUNTIF($B$6:$B194,"Entry"),"")</f>
+        <f>IF($B194="Entry",COUNTIF($B$8:$B194,"Entry"),"")</f>
       </c>
       <c r="B194" s="16"/>
       <c r="C194" s="17"/>
@@ -6371,7 +6430,7 @@
       <c r="P194" s="24"/>
       <c r="Q194" s="26"/>
       <c r="R194" s="27">
-        <f>IF($B194&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C194,$O$6:$O$205)+SUMIF($C$6:$C$205,$C194,$P$6:$P$205))</f>
+        <f>IF($B194&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C194,$O$8:$O$207)+SUMIF($C$8:$C$207,$C194,$P$8:$P$207))</f>
       </c>
       <c r="S194" s="27">
         <f>IF(OR($B194&lt;&gt;"Challan",$C194="",G194=0),"",IF(ROUND(G194-R194,2)=0,"Matches","Check Entries"))</f>
@@ -6379,7 +6438,7 @@
     </row>
     <row r="195" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
-        <f>IF($B195="Entry",COUNTIF($B$6:$B195,"Entry"),"")</f>
+        <f>IF($B195="Entry",COUNTIF($B$8:$B195,"Entry"),"")</f>
       </c>
       <c r="B195" s="16"/>
       <c r="C195" s="17"/>
@@ -6398,7 +6457,7 @@
       <c r="P195" s="24"/>
       <c r="Q195" s="26"/>
       <c r="R195" s="27">
-        <f>IF($B195&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C195,$O$6:$O$205)+SUMIF($C$6:$C$205,$C195,$P$6:$P$205))</f>
+        <f>IF($B195&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C195,$O$8:$O$207)+SUMIF($C$8:$C$207,$C195,$P$8:$P$207))</f>
       </c>
       <c r="S195" s="27">
         <f>IF(OR($B195&lt;&gt;"Challan",$C195="",G195=0),"",IF(ROUND(G195-R195,2)=0,"Matches","Check Entries"))</f>
@@ -6406,7 +6465,7 @@
     </row>
     <row r="196" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
-        <f>IF($B196="Entry",COUNTIF($B$6:$B196,"Entry"),"")</f>
+        <f>IF($B196="Entry",COUNTIF($B$8:$B196,"Entry"),"")</f>
       </c>
       <c r="B196" s="16"/>
       <c r="C196" s="17"/>
@@ -6425,7 +6484,7 @@
       <c r="P196" s="24"/>
       <c r="Q196" s="26"/>
       <c r="R196" s="27">
-        <f>IF($B196&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C196,$O$6:$O$205)+SUMIF($C$6:$C$205,$C196,$P$6:$P$205))</f>
+        <f>IF($B196&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C196,$O$8:$O$207)+SUMIF($C$8:$C$207,$C196,$P$8:$P$207))</f>
       </c>
       <c r="S196" s="27">
         <f>IF(OR($B196&lt;&gt;"Challan",$C196="",G196=0),"",IF(ROUND(G196-R196,2)=0,"Matches","Check Entries"))</f>
@@ -6433,7 +6492,7 @@
     </row>
     <row r="197" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
-        <f>IF($B197="Entry",COUNTIF($B$6:$B197,"Entry"),"")</f>
+        <f>IF($B197="Entry",COUNTIF($B$8:$B197,"Entry"),"")</f>
       </c>
       <c r="B197" s="16"/>
       <c r="C197" s="17"/>
@@ -6452,7 +6511,7 @@
       <c r="P197" s="24"/>
       <c r="Q197" s="26"/>
       <c r="R197" s="27">
-        <f>IF($B197&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C197,$O$6:$O$205)+SUMIF($C$6:$C$205,$C197,$P$6:$P$205))</f>
+        <f>IF($B197&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C197,$O$8:$O$207)+SUMIF($C$8:$C$207,$C197,$P$8:$P$207))</f>
       </c>
       <c r="S197" s="27">
         <f>IF(OR($B197&lt;&gt;"Challan",$C197="",G197=0),"",IF(ROUND(G197-R197,2)=0,"Matches","Check Entries"))</f>
@@ -6460,7 +6519,7 @@
     </row>
     <row r="198" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A198" s="15">
-        <f>IF($B198="Entry",COUNTIF($B$6:$B198,"Entry"),"")</f>
+        <f>IF($B198="Entry",COUNTIF($B$8:$B198,"Entry"),"")</f>
       </c>
       <c r="B198" s="16"/>
       <c r="C198" s="17"/>
@@ -6479,7 +6538,7 @@
       <c r="P198" s="24"/>
       <c r="Q198" s="26"/>
       <c r="R198" s="27">
-        <f>IF($B198&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C198,$O$6:$O$205)+SUMIF($C$6:$C$205,$C198,$P$6:$P$205))</f>
+        <f>IF($B198&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C198,$O$8:$O$207)+SUMIF($C$8:$C$207,$C198,$P$8:$P$207))</f>
       </c>
       <c r="S198" s="27">
         <f>IF(OR($B198&lt;&gt;"Challan",$C198="",G198=0),"",IF(ROUND(G198-R198,2)=0,"Matches","Check Entries"))</f>
@@ -6487,7 +6546,7 @@
     </row>
     <row r="199" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A199" s="15">
-        <f>IF($B199="Entry",COUNTIF($B$6:$B199,"Entry"),"")</f>
+        <f>IF($B199="Entry",COUNTIF($B$8:$B199,"Entry"),"")</f>
       </c>
       <c r="B199" s="16"/>
       <c r="C199" s="17"/>
@@ -6506,7 +6565,7 @@
       <c r="P199" s="24"/>
       <c r="Q199" s="26"/>
       <c r="R199" s="27">
-        <f>IF($B199&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C199,$O$6:$O$205)+SUMIF($C$6:$C$205,$C199,$P$6:$P$205))</f>
+        <f>IF($B199&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C199,$O$8:$O$207)+SUMIF($C$8:$C$207,$C199,$P$8:$P$207))</f>
       </c>
       <c r="S199" s="27">
         <f>IF(OR($B199&lt;&gt;"Challan",$C199="",G199=0),"",IF(ROUND(G199-R199,2)=0,"Matches","Check Entries"))</f>
@@ -6514,7 +6573,7 @@
     </row>
     <row r="200" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
-        <f>IF($B200="Entry",COUNTIF($B$6:$B200,"Entry"),"")</f>
+        <f>IF($B200="Entry",COUNTIF($B$8:$B200,"Entry"),"")</f>
       </c>
       <c r="B200" s="16"/>
       <c r="C200" s="17"/>
@@ -6533,7 +6592,7 @@
       <c r="P200" s="24"/>
       <c r="Q200" s="26"/>
       <c r="R200" s="27">
-        <f>IF($B200&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C200,$O$6:$O$205)+SUMIF($C$6:$C$205,$C200,$P$6:$P$205))</f>
+        <f>IF($B200&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C200,$O$8:$O$207)+SUMIF($C$8:$C$207,$C200,$P$8:$P$207))</f>
       </c>
       <c r="S200" s="27">
         <f>IF(OR($B200&lt;&gt;"Challan",$C200="",G200=0),"",IF(ROUND(G200-R200,2)=0,"Matches","Check Entries"))</f>
@@ -6541,7 +6600,7 @@
     </row>
     <row r="201" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A201" s="15">
-        <f>IF($B201="Entry",COUNTIF($B$6:$B201,"Entry"),"")</f>
+        <f>IF($B201="Entry",COUNTIF($B$8:$B201,"Entry"),"")</f>
       </c>
       <c r="B201" s="16"/>
       <c r="C201" s="17"/>
@@ -6560,7 +6619,7 @@
       <c r="P201" s="24"/>
       <c r="Q201" s="26"/>
       <c r="R201" s="27">
-        <f>IF($B201&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C201,$O$6:$O$205)+SUMIF($C$6:$C$205,$C201,$P$6:$P$205))</f>
+        <f>IF($B201&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C201,$O$8:$O$207)+SUMIF($C$8:$C$207,$C201,$P$8:$P$207))</f>
       </c>
       <c r="S201" s="27">
         <f>IF(OR($B201&lt;&gt;"Challan",$C201="",G201=0),"",IF(ROUND(G201-R201,2)=0,"Matches","Check Entries"))</f>
@@ -6568,7 +6627,7 @@
     </row>
     <row r="202" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A202" s="15">
-        <f>IF($B202="Entry",COUNTIF($B$6:$B202,"Entry"),"")</f>
+        <f>IF($B202="Entry",COUNTIF($B$8:$B202,"Entry"),"")</f>
       </c>
       <c r="B202" s="16"/>
       <c r="C202" s="17"/>
@@ -6587,7 +6646,7 @@
       <c r="P202" s="24"/>
       <c r="Q202" s="26"/>
       <c r="R202" s="27">
-        <f>IF($B202&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C202,$O$6:$O$205)+SUMIF($C$6:$C$205,$C202,$P$6:$P$205))</f>
+        <f>IF($B202&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C202,$O$8:$O$207)+SUMIF($C$8:$C$207,$C202,$P$8:$P$207))</f>
       </c>
       <c r="S202" s="27">
         <f>IF(OR($B202&lt;&gt;"Challan",$C202="",G202=0),"",IF(ROUND(G202-R202,2)=0,"Matches","Check Entries"))</f>
@@ -6595,7 +6654,7 @@
     </row>
     <row r="203" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A203" s="15">
-        <f>IF($B203="Entry",COUNTIF($B$6:$B203,"Entry"),"")</f>
+        <f>IF($B203="Entry",COUNTIF($B$8:$B203,"Entry"),"")</f>
       </c>
       <c r="B203" s="16"/>
       <c r="C203" s="17"/>
@@ -6614,7 +6673,7 @@
       <c r="P203" s="24"/>
       <c r="Q203" s="26"/>
       <c r="R203" s="27">
-        <f>IF($B203&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C203,$O$6:$O$205)+SUMIF($C$6:$C$205,$C203,$P$6:$P$205))</f>
+        <f>IF($B203&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C203,$O$8:$O$207)+SUMIF($C$8:$C$207,$C203,$P$8:$P$207))</f>
       </c>
       <c r="S203" s="27">
         <f>IF(OR($B203&lt;&gt;"Challan",$C203="",G203=0),"",IF(ROUND(G203-R203,2)=0,"Matches","Check Entries"))</f>
@@ -6622,7 +6681,7 @@
     </row>
     <row r="204" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A204" s="15">
-        <f>IF($B204="Entry",COUNTIF($B$6:$B204,"Entry"),"")</f>
+        <f>IF($B204="Entry",COUNTIF($B$8:$B204,"Entry"),"")</f>
       </c>
       <c r="B204" s="16"/>
       <c r="C204" s="17"/>
@@ -6641,7 +6700,7 @@
       <c r="P204" s="24"/>
       <c r="Q204" s="26"/>
       <c r="R204" s="27">
-        <f>IF($B204&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C204,$O$6:$O$205)+SUMIF($C$6:$C$205,$C204,$P$6:$P$205))</f>
+        <f>IF($B204&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C204,$O$8:$O$207)+SUMIF($C$8:$C$207,$C204,$P$8:$P$207))</f>
       </c>
       <c r="S204" s="27">
         <f>IF(OR($B204&lt;&gt;"Challan",$C204="",G204=0),"",IF(ROUND(G204-R204,2)=0,"Matches","Check Entries"))</f>
@@ -6649,7 +6708,7 @@
     </row>
     <row r="205" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A205" s="15">
-        <f>IF($B205="Entry",COUNTIF($B$6:$B205,"Entry"),"")</f>
+        <f>IF($B205="Entry",COUNTIF($B$8:$B205,"Entry"),"")</f>
       </c>
       <c r="B205" s="16"/>
       <c r="C205" s="17"/>
@@ -6668,56 +6727,110 @@
       <c r="P205" s="24"/>
       <c r="Q205" s="26"/>
       <c r="R205" s="27">
-        <f>IF($B205&lt;&gt;"Challan","",SUMIF($C$6:$C$205,$C205,$O$6:$O$205)+SUMIF($C$6:$C$205,$C205,$P$6:$P$205))</f>
+        <f>IF($B205&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C205,$O$8:$O$207)+SUMIF($C$8:$C$207,$C205,$P$8:$P$207))</f>
       </c>
       <c r="S205" s="27">
         <f>IF(OR($B205&lt;&gt;"Challan",$C205="",G205=0),"",IF(ROUND(G205-R205,2)=0,"Matches","Check Entries"))</f>
+      </c>
+    </row>
+    <row r="206" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A206" s="15">
+        <f>IF($B206="Entry",COUNTIF($B$8:$B206,"Entry"),"")</f>
+      </c>
+      <c r="B206" s="16"/>
+      <c r="C206" s="17"/>
+      <c r="D206" s="18"/>
+      <c r="E206" s="18"/>
+      <c r="F206" s="19"/>
+      <c r="G206" s="20"/>
+      <c r="H206" s="21"/>
+      <c r="I206" s="22"/>
+      <c r="J206" s="22"/>
+      <c r="K206" s="22"/>
+      <c r="L206" s="23"/>
+      <c r="M206" s="24"/>
+      <c r="N206" s="25"/>
+      <c r="O206" s="24"/>
+      <c r="P206" s="24"/>
+      <c r="Q206" s="26"/>
+      <c r="R206" s="27">
+        <f>IF($B206&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C206,$O$8:$O$207)+SUMIF($C$8:$C$207,$C206,$P$8:$P$207))</f>
+      </c>
+      <c r="S206" s="27">
+        <f>IF(OR($B206&lt;&gt;"Challan",$C206="",G206=0),"",IF(ROUND(G206-R206,2)=0,"Matches","Check Entries"))</f>
+      </c>
+    </row>
+    <row r="207" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A207" s="15">
+        <f>IF($B207="Entry",COUNTIF($B$8:$B207,"Entry"),"")</f>
+      </c>
+      <c r="B207" s="16"/>
+      <c r="C207" s="17"/>
+      <c r="D207" s="18"/>
+      <c r="E207" s="18"/>
+      <c r="F207" s="19"/>
+      <c r="G207" s="20"/>
+      <c r="H207" s="21"/>
+      <c r="I207" s="22"/>
+      <c r="J207" s="22"/>
+      <c r="K207" s="22"/>
+      <c r="L207" s="23"/>
+      <c r="M207" s="24"/>
+      <c r="N207" s="25"/>
+      <c r="O207" s="24"/>
+      <c r="P207" s="24"/>
+      <c r="Q207" s="26"/>
+      <c r="R207" s="27">
+        <f>IF($B207&lt;&gt;"Challan","",SUMIF($C$8:$C$207,$C207,$O$8:$O$207)+SUMIF($C$8:$C$207,$C207,$P$8:$P$207))</f>
+      </c>
+      <c r="S207" s="27">
+        <f>IF(OR($B207&lt;&gt;"Challan",$C207="",G207=0),"",IF(ROUND(G207-R207,2)=0,"Matches","Check Entries"))</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:S1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:S205">
+  <conditionalFormatting sqref="A8:S207">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$B6="Challan"</formula>
+      <formula>$B8="Challan"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid Row Type" error="Pick either Challan or Entry from the dropdown." sqref="B6:B205">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid Row Type" error="Pick either Challan or Entry from the dropdown." sqref="B8:B207">
       <formula1>"Challan,Entry"</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="equal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid BSR Code" error="BSR Code must be exactly 7 characters." sqref="D6:D205">
+    <dataValidation type="textLength" operator="equal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid BSR Code" error="BSR Code must be exactly 7 characters." sqref="D8:D207">
       <formula1>7</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Date" error="Enter a real date (use the date picker), between 01-Apr-2020 and 31-Mar-2030." sqref="F6:F205">
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Date" error="Enter a real date (use the date picker), between 01-Apr-2020 and 31-Mar-2030." sqref="F8:F207">
       <formula1>43922</formula1>
       <formula2>47573</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Amount must be a number of 0 or more (no currency symbols or commas typed in)." sqref="G6:G205">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Amount must be a number of 0 or more (no currency symbols or commas typed in)." sqref="G8:G207">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Invalid PAN" error="PAN must be 5 letters + 4 digits + 1 letter, uppercase (e.g. AACCP6899F)." sqref="J6:J205">
-      <formula1>AND(LEN(J6)=10,CODE(MID(J6,1,1))&gt;=65,CODE(MID(J6,1,1))&lt;=90,CODE(MID(J6,2,1))&gt;=65,CODE(MID(J6,2,1))&lt;=90,CODE(MID(J6,3,1))&gt;=65,CODE(MID(J6,3,1))&lt;=90,CODE(MID(J6,4,1))&gt;=65,CODE(MID(J6,4,1))&lt;=90,CODE(MID(J6,5,1))&gt;=65,CODE(MID(J6,5,1))&lt;=90,CODE(MID(J6,6,1))&gt;=48,CODE(MID(J6,6,1))&lt;=57,CODE(MID(J6,7,1))&gt;=48,CODE(MID(J6,7,1))&lt;=57,CODE(MID(J6,8,1))&gt;=48,CODE(MID(J6,8,1))&lt;=57,CODE(MID(J6,9,1))&gt;=48,CODE(MID(J6,9,1))&lt;=57,CODE(MID(J6,10,1))&gt;=65,CODE(MID(J6,10,1))&lt;=90)</formula1>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Invalid PAN" error="PAN must be 5 letters + 4 digits + 1 letter, uppercase (e.g. AACCP6899F)." sqref="J8:J207">
+      <formula1>AND(LEN(J8)=10,CODE(MID(J8,1,1))&gt;=65,CODE(MID(J8,1,1))&lt;=90,CODE(MID(J8,2,1))&gt;=65,CODE(MID(J8,2,1))&lt;=90,CODE(MID(J8,3,1))&gt;=65,CODE(MID(J8,3,1))&lt;=90,CODE(MID(J8,4,1))&gt;=65,CODE(MID(J8,4,1))&lt;=90,CODE(MID(J8,5,1))&gt;=65,CODE(MID(J8,5,1))&lt;=90,CODE(MID(J8,6,1))&gt;=48,CODE(MID(J8,6,1))&lt;=57,CODE(MID(J8,7,1))&gt;=48,CODE(MID(J8,7,1))&lt;=57,CODE(MID(J8,8,1))&gt;=48,CODE(MID(J8,8,1))&lt;=57,CODE(MID(J8,9,1))&gt;=48,CODE(MID(J8,9,1))&lt;=57,CODE(MID(J8,10,1))&gt;=65,CODE(MID(J8,10,1))&lt;=90)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Section" error="Pick a section from the dropdown list." sqref="K6:K205">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Section" error="Pick a section from the dropdown list." sqref="K8:K207">
       <formula1>"192,194A,194C,194D,194H,194I,194IA,194IB,194J,194K,194M,194Q,206C"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Date" error="Enter a real date (use the date picker), between 01-Apr-2020 and 31-Mar-2030." sqref="L6:L205">
+    <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Date" error="Enter a real date (use the date picker), between 01-Apr-2020 and 31-Mar-2030." sqref="L8:L207">
       <formula1>43922</formula1>
       <formula2>47573</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Amount must be a number of 0 or more (no currency symbols or commas typed in)." sqref="M6:M205">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Amount must be a number of 0 or more (no currency symbols or commas typed in)." sqref="M8:M207">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Rate" error="Rate must be a number between 0 and 100 (e.g. enter 10 for 10%, not 0.10)." sqref="N6:N205">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Rate" error="Rate must be a number between 0 and 100 (e.g. enter 10 for 10%, not 0.10)." sqref="N8:N207">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid TDS Amount" error="TDS Amount must be a number of 0 or more." sqref="O6:O205">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid TDS Amount" error="TDS Amount must be a number of 0 or more." sqref="O8:O207">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Interest" error="Interest must be a number of 0 or more." sqref="P6:P205">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Interest" error="Interest must be a number of 0 or more." sqref="P8:P207">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(tds): Section 393/394 payment-code labels in the Data Entry template
- Section dropdown now shows "PaymentCode : [OldSection] : NewSectionCode
  - Description" for the ~15 sections verified against the user's own
  Income Tax Act 2025 reference table (K:\TDS.pdf)
- 194A/194C/194R bifurcated into lettered options (matching the existing
  194I(a)/(b), 194J(a)/(b) pattern) since the new Act's payment code is now
  the rate determinant, not just deductee type
- 194T added (previously missing from this template only)
- Every other section keeps its plain old-section label — two secondary
  web sources disagreed with each other and with the user's own PDF on at
  least one payment code, so unverified codes are not guessed
- Rate Lookup sheet is now also the Section dropdown's list source (a
  range reference, not an inline list — several new labels exceed Excel's
  255-char inline list limit)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/TDS_Data_Entry_Simple_Template.xlsx
+++ b/public/templates/TDS_Data_Entry_Simple_Template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="170">
   <si>
     <t>TDS Data Entry — Client Template</t>
   </si>
@@ -79,6 +79,18 @@
   </si>
   <si>
     <t>•  "Country of Residence" and the per-entry "Remarks" field are kept here for your own records, but a direct code check of the software found neither is actually used anywhere in that screen — they're declared in its data model but never read, written, or shown. Kept in this template anyway since they're useful, low-risk fields, not because the software actively uses them.</t>
+  </si>
+  <si>
+    <t>Section Codes — Income Tax Act 2025 (Section 393 reorganisation)</t>
+  </si>
+  <si>
+    <t>•  From 1-Apr-2026 (FY2026-27 onward), the old 194-series section numbers are being replaced by a numeric Payment Code and a new Section 392/393/394 citation. Wherever a verified mapping exists, the Section dropdown shows: PaymentCode : [OldSection] : NewSectionCode – Description — e.g. 1023 : [194C] : 393(1) [Table: S.N. 6(i).D(a)] – Payments to contractors and sub-contractors (Individual/HUF). This matches the software's own Section dropdown exactly.</t>
+  </si>
+  <si>
+    <t>•  194A, 194C and 194R are split into separate lettered options (194A(a)/(b)/(c), 194C(a)/(b), 194R(a)/(b)) because the new Act's Payment Code — not just the Deductee Type — now determines which citation and rate applies. Pick the option matching the actual payee/payment type; the Rate of TDS still fills in automatically.</t>
+  </si>
+  <si>
+    <t>•  Only the sections above have a verified Payment Code and new citation — sourced from a CBDT-derived reference table, cross-checked line by line. Every OTHER section (194B, 194BB, 194D, 194DA, 194G, 194IA, 194IB, 194IC, 194K, 194LA, 194LB, 194M, 194O, 194S, 195, 196A, 196D, 206C(1H)) still shows its plain old section code — two independent secondary sources checked for these gave conflicting payment codes for sections this template DOES have verified data for, so an unverified code is not shown rather than risk a wrong figure on an actual filing. These will be added once a verified source is available.</t>
   </si>
   <si>
     <t>Field Guide — Challan Rows (blue columns)</t>
@@ -182,7 +194,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Optional — this challan's predominant/default TDS section, for your reference. If a linked Entry's own Section differs, that Entry's Section cell is highlighted amber.</t>
+      <t>Optional — this challan's predominant/default TDS section, for your reference. If a linked Entry's own Section differs, that Entry's Section cell is highlighted amber. See "Section Codes" above for the PaymentCode : [OldSection] : NewSectionCode format.</t>
     </r>
   </si>
   <si>
@@ -508,7 +520,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
       </rPr>
-      <t>Pick from the dropdown — the TDS section under which this deduction was made. Highlighted amber if it differs from this entry's linked Challan's own Section.</t>
+      <t>Pick from the dropdown — the TDS section under which this deduction was made. Highlighted amber if it differs from this entry's linked Challan's own Section. See "Section Codes" above for the PaymentCode : [OldSection] : NewSectionCode format, and which sections have a verified new code.</t>
     </r>
   </si>
   <si>
@@ -790,16 +802,22 @@
     <t>192</t>
   </si>
   <si>
-    <t>192A</t>
+    <t>1004 : [192A] : 393(7) – Premature withdrawal from Employees' Provident Fund</t>
   </si>
   <si>
-    <t>193</t>
+    <t>1019 : [193] : 393(1) [Table: S.N. 5(i)] – Interest on securities</t>
   </si>
   <si>
-    <t>194</t>
+    <t>1029 : [194] : 393(1) [Table: S.N. 7] – Dividend</t>
   </si>
   <si>
-    <t>194A</t>
+    <t>1020 : [194A] : 393(1) [Table: S.N. 5(ii).D(a)] – Interest other than securities (Senior Citizens)</t>
+  </si>
+  <si>
+    <t>1021 : [194A] : 393(1) [Table: S.N. 5(ii).D(b)] – Interest other than securities (Other Individuals)</t>
+  </si>
+  <si>
+    <t>1022 : [194A] : 393(1) [Table: S.N. 5(iii)] – Interest other than securities (Others)</t>
   </si>
   <si>
     <t>194B</t>
@@ -808,7 +826,10 @@
     <t>194BB</t>
   </si>
   <si>
-    <t>194C</t>
+    <t>1023 : [194C] : 393(1) [Table: S.N. 6(i).D(a)] – Payments to contractors and sub-contractors (Individual/HUF)</t>
+  </si>
+  <si>
+    <t>1024 : [194C] : 393(1) [Table: S.N. 6(i).D(b)] – Payments to contractors and sub-contractors (Others)</t>
   </si>
   <si>
     <t>194D</t>
@@ -820,13 +841,13 @@
     <t>194G</t>
   </si>
   <si>
-    <t>194H</t>
+    <t>1006 : [194H] : 393(1) [Table: S.N. 1(ii)] – Commission or brokerage</t>
   </si>
   <si>
-    <t>194I(a)</t>
+    <t>1008 : [194I(a)] : 393(1) [Table: S.N. 2(ii).D(a)] – Rent – Plant &amp; Machinery</t>
   </si>
   <si>
-    <t>194I(b)</t>
+    <t>1009 : [194I(b)] : 393(1) [Table: S.N. 2(ii).D(b)] – Rent – Land/Building/Furniture</t>
   </si>
   <si>
     <t>194IA</t>
@@ -838,10 +859,10 @@
     <t>194IC</t>
   </si>
   <si>
-    <t>194J(a)</t>
+    <t>1027 : [194J(a)] : 393(1) [Table: S.N. 6(iii).D(b)] – Professional services / director remuneration</t>
   </si>
   <si>
-    <t>194J(b)</t>
+    <t>1026 : [194J(b)] : 393(1) [Table: S.N. 6(iii).D(a)] – Fees for technical services</t>
   </si>
   <si>
     <t>194K</t>
@@ -859,13 +880,19 @@
     <t>194O</t>
   </si>
   <si>
-    <t>194Q</t>
+    <t>1031 : [194Q] : 393(1) [Table: S.N. 8(ii)] – Purchase of goods (buyer TDS)</t>
   </si>
   <si>
-    <t>194R</t>
+    <t>1034 : [194R] : 393(1) [Table: S.N. 8(iv)] – Perquisite/benefit in business or profession (Cash)</t>
+  </si>
+  <si>
+    <t>1035 : [194R] : 393(1) [Table: S.N. 8(iv) Note 6] – Perquisite/benefit in business or profession (In Kind/Mixed)</t>
   </si>
   <si>
     <t>194S</t>
+  </si>
+  <si>
+    <t>1067 : [194T] : 393(3) [Table: S.N. 7] – Payment to partners of a firm (salary/remuneration/interest)</t>
   </si>
   <si>
     <t>195</t>
@@ -877,7 +904,7 @@
     <t>196D</t>
   </si>
   <si>
-    <t>206C(1)</t>
+    <t>1073 : [206C(1)] : 394(1) [Table: S.N. 4] – Sale of scrap (TCS)</t>
   </si>
   <si>
     <t>206C(1H)</t>
@@ -1727,7 +1754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A72"/>
+  <dimension ref="A1:A77"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -1848,212 +1875,212 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
+    <row r="28" ht="80" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="29" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+    <row r="29" ht="65" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
+    <row r="30" ht="110" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
+    <row r="33" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="33" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
+    <row r="34" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
+    <row r="35" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" s="5" t="s">
+    <row r="39" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="39" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="5" t="s">
+    <row r="40" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="40" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
+    <row r="41" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="41" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
+    <row r="45" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="45" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" s="5" t="s">
+    <row r="46" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" s="5" t="s">
+    <row r="47" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
+    <row r="48" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="49" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="50" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="51" ht="65" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="52" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" s="5" t="s">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
         <v>46</v>
-      </c>
-    </row>
-    <row r="53" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" s="5" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="54" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="55" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" s="5" t="s">
+    <row r="56" ht="65" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" s="5" t="s">
+    <row r="57" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="57" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" s="5" t="s">
+    <row r="58" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="58" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" s="5" t="s">
+    <row r="59" ht="65" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="59" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" s="5" t="s">
+    <row r="60" ht="50" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="60" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" s="5" t="s">
+    <row r="61" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="5" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="61" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" s="5" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="5" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="63" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" s="5" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="66" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="5" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="66" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" s="3" t="s">
+    <row r="69" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="70" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="71" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>64</v>
       </c>
@@ -2061,6 +2088,26 @@
     <row r="72" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="75" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="76" ht="35" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="5" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -2071,12 +2118,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -2090,7 +2137,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -2104,7 +2151,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -2118,7 +2165,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B4">
         <v>10</v>
@@ -2132,7 +2179,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B5">
         <v>10</v>
@@ -2146,69 +2193,69 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B6">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C6">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B7">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D7">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="D8">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="C9">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D9">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10">
         <v>20</v>
@@ -2216,7 +2263,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -2230,13 +2277,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D12">
         <v>20</v>
@@ -2244,7 +2291,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -2258,13 +2305,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B14">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C14">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D14">
         <v>20</v>
@@ -2272,13 +2319,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15">
         <v>20</v>
@@ -2286,13 +2333,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B16">
         <v>2</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D16">
         <v>20</v>
@@ -2300,7 +2347,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B17">
         <v>10</v>
@@ -2314,13 +2361,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B18">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C18">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D18">
         <v>20</v>
@@ -2328,13 +2375,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B19">
         <v>2</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D19">
         <v>20</v>
@@ -2342,7 +2389,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B20">
         <v>10</v>
@@ -2356,7 +2403,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B21">
         <v>10</v>
@@ -2370,13 +2417,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C22">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D22">
         <v>20</v>
@@ -2384,13 +2431,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D23">
         <v>20</v>
@@ -2398,13 +2445,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D24">
         <v>20</v>
@@ -2412,27 +2459,27 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B25">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="C25">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B26">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C26">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D26">
         <v>20</v>
@@ -2440,7 +2487,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B27">
         <v>1</v>
@@ -2454,21 +2501,21 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D28">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B29">
         <v>10</v>
@@ -2482,13 +2529,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B30">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C30">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D30">
         <v>20</v>
@@ -2496,7 +2543,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B31">
         <v>1</v>
@@ -2505,20 +2552,90 @@
         <v>1</v>
       </c>
       <c r="D31">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B32">
+        <v>10</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34">
+        <v>10</v>
+      </c>
+      <c r="C34">
+        <v>10</v>
+      </c>
+      <c r="D34">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35">
+        <v>20</v>
+      </c>
+      <c r="C35">
+        <v>20</v>
+      </c>
+      <c r="D35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>105</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>106</v>
+      </c>
+      <c r="B37">
         <v>0.1</v>
       </c>
-      <c r="C32">
+      <c r="C37">
         <v>0.1</v>
       </c>
-      <c r="D32">
+      <c r="D37">
         <v>1</v>
       </c>
     </row>
@@ -2537,10 +2654,14 @@
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="20" width="12" customWidth="1"/>
+    <col min="6" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="55" customWidth="1"/>
+    <col min="9" max="20" width="12" customWidth="1"/>
     <col min="21" max="21" width="18" customWidth="1"/>
     <col min="22" max="22" width="26" customWidth="1"/>
-    <col min="23" max="38" width="12" customWidth="1"/>
+    <col min="23" max="25" width="12" customWidth="1"/>
+    <col min="26" max="26" width="55" customWidth="1"/>
+    <col min="27" max="38" width="12" customWidth="1"/>
     <col min="39" max="39" width="18" customWidth="1"/>
     <col min="40" max="42" width="12" customWidth="1"/>
     <col min="43" max="44" width="12" hidden="1" customWidth="1"/>
@@ -2548,7 +2669,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2640,136 +2761,136 @@
     </row>
     <row r="3" ht="40" customHeight="1" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="U3" s="8" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="V3" s="8" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="W3" s="8" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="X3" s="8" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="Y3" s="8" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="Z3" s="8" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="AA3" s="8" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="AC3" s="8" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="AD3" s="8" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="AE3" s="8" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="AF3" s="8" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="AG3" s="8" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="AH3" s="8" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="AI3" s="8" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="AJ3" s="8" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="AK3" s="8" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="AL3" s="8" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="AM3" s="8" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="AN3" s="8" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="AO3" s="8" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="AP3" s="8" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="AQ3" s="8" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="AR3" s="8" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.25">
@@ -2777,13 +2898,13 @@
         <f>IF($B4="Entry",COUNTIF($B$4:$B4,"Entry"),"")</f>
       </c>
       <c r="B4" s="10" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="E4" s="12">
         <f>IF($B4&lt;&gt;"Challan","",IF(ROUND(AN4-AO4,2)&gt;0,"Over-applied",IF(ROUND(AN4-AO4,2)=0,"Fully Utilised","Unconsumed")))</f>
@@ -2792,10 +2913,10 @@
         <v>46177</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="I4" s="14">
         <v>6558</v>
@@ -2822,15 +2943,15 @@
         <f>IF($B4&lt;&gt;"Challan","",I4+J4+K4+L4+M4+N4)</f>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="S4" s="10"/>
       <c r="T4" s="10"/>
       <c r="U4" s="10" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="V4" s="10"/>
       <c r="W4" s="10"/>
@@ -2842,7 +2963,7 @@
       </c>
       <c r="Z4" s="10"/>
       <c r="AA4" s="16">
-        <f>IF($B4&lt;&gt;"Entry","",IF(Z4="","",IF(X4="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z4)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y4="Individual",Y4="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z4)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z4)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B4&lt;&gt;"Entry","",IF(Z4="","",IF(X4="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z4)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y4="Individual",Y4="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z4)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z4)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB4" s="13"/>
       <c r="AC4" s="14"/>
@@ -2887,11 +3008,11 @@
         <f>IF($B5="Entry",COUNTIF($B$4:$B5,"Entry"),"")</f>
       </c>
       <c r="B5" s="10" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="E5" s="12">
         <f>IF($B5&lt;&gt;"Challan","",IF(ROUND(AN5-AO5,2)&gt;0,"Over-applied",IF(ROUND(AN5-AO5,2)=0,"Fully Utilised","Unconsumed")))</f>
@@ -2915,10 +3036,10 @@
       <c r="T5" s="10"/>
       <c r="U5" s="10"/>
       <c r="V5" s="10" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="X5" s="12">
         <f>IF($B5&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W5)))=10,CODE(MID(TRIM(UPPER(W5)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),9,1))&lt;=57),"N","Y"))</f>
@@ -2927,10 +3048,10 @@
         <f>IF($B5&lt;&gt;"Entry","",IF(LEN(W5)&lt;4,"",IF(UPPER(MID(W5,4,1))="P","Individual",IF(UPPER(MID(W5,4,1))="H","HUF",IF(UPPER(MID(W5,4,1))="C","Company",IF(UPPER(MID(W5,4,1))="F","Firm",IF(UPPER(MID(W5,4,1))="L","LLP",IF(UPPER(MID(W5,4,1))="T","Trust",IF(UPPER(MID(W5,4,1))="A","AOP",""))))))))</f>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="AA5" s="16">
-        <f>IF($B5&lt;&gt;"Entry","",IF(Z5="","",IF(X5="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z5)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y5="Individual",Y5="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z5)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z5)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B5&lt;&gt;"Entry","",IF(Z5="","",IF(X5="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z5)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y5="Individual",Y5="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z5)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z5)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB5" s="13">
         <v>46173</v>
@@ -2954,17 +3075,17 @@
         <f>IF($B5&lt;&gt;"Entry","",0)</f>
       </c>
       <c r="AI5" s="10" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AJ5" s="10" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AK5" s="17" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AL5" s="10"/>
       <c r="AM5" s="10" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AN5" s="15">
         <f>IF($B5&lt;&gt;"Challan","",SUMIF($D$4:$D$207,D5,$AD$4:$AD$207)+SUMIF($D$4:$D$207,D5,$AG$4:$AG$207)+SUMIF($D$4:$D$207,D5,$AE$4:$AE$207))</f>
@@ -2987,11 +3108,11 @@
         <f>IF($B6="Entry",COUNTIF($B$4:$B6,"Entry"),"")</f>
       </c>
       <c r="B6" s="10" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="11" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="E6" s="12">
         <f>IF($B6&lt;&gt;"Challan","",IF(ROUND(AN6-AO6,2)&gt;0,"Over-applied",IF(ROUND(AN6-AO6,2)=0,"Fully Utilised","Unconsumed")))</f>
@@ -3015,10 +3136,10 @@
       <c r="T6" s="10"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="W6" s="10" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="X6" s="12">
         <f>IF($B6&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W6)))=10,CODE(MID(TRIM(UPPER(W6)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),9,1))&lt;=57),"N","Y"))</f>
@@ -3027,10 +3148,10 @@
         <f>IF($B6&lt;&gt;"Entry","",IF(LEN(W6)&lt;4,"",IF(UPPER(MID(W6,4,1))="P","Individual",IF(UPPER(MID(W6,4,1))="H","HUF",IF(UPPER(MID(W6,4,1))="C","Company",IF(UPPER(MID(W6,4,1))="F","Firm",IF(UPPER(MID(W6,4,1))="L","LLP",IF(UPPER(MID(W6,4,1))="T","Trust",IF(UPPER(MID(W6,4,1))="A","AOP",""))))))))</f>
       </c>
       <c r="Z6" s="10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="AA6" s="16">
-        <f>IF($B6&lt;&gt;"Entry","",IF(Z6="","",IF(X6="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z6)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y6="Individual",Y6="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z6)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z6)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B6&lt;&gt;"Entry","",IF(Z6="","",IF(X6="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z6)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y6="Individual",Y6="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z6)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z6)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB6" s="13">
         <v>46173</v>
@@ -3054,17 +3175,17 @@
         <f>IF($B6&lt;&gt;"Entry","",0)</f>
       </c>
       <c r="AI6" s="10" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AJ6" s="10" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AK6" s="17" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AL6" s="10"/>
       <c r="AM6" s="10" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="AN6" s="15">
         <f>IF($B6&lt;&gt;"Challan","",SUMIF($D$4:$D$207,D6,$AD$4:$AD$207)+SUMIF($D$4:$D$207,D6,$AG$4:$AG$207)+SUMIF($D$4:$D$207,D6,$AE$4:$AE$207))</f>
@@ -3087,11 +3208,11 @@
         <f>IF($B7="Entry",COUNTIF($B$4:$B7,"Entry"),"")</f>
       </c>
       <c r="B7" s="10" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="11" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="E7" s="12">
         <f>IF($B7&lt;&gt;"Challan","",IF(ROUND(AN7-AO7,2)&gt;0,"Over-applied",IF(ROUND(AN7-AO7,2)=0,"Fully Utilised","Unconsumed")))</f>
@@ -3115,10 +3236,10 @@
       <c r="T7" s="10"/>
       <c r="U7" s="10"/>
       <c r="V7" s="10" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="X7" s="12">
         <f>IF($B7&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W7)))=10,CODE(MID(TRIM(UPPER(W7)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),9,1))&lt;=57),"N","Y"))</f>
@@ -3127,10 +3248,10 @@
         <f>IF($B7&lt;&gt;"Entry","",IF(LEN(W7)&lt;4,"",IF(UPPER(MID(W7,4,1))="P","Individual",IF(UPPER(MID(W7,4,1))="H","HUF",IF(UPPER(MID(W7,4,1))="C","Company",IF(UPPER(MID(W7,4,1))="F","Firm",IF(UPPER(MID(W7,4,1))="L","LLP",IF(UPPER(MID(W7,4,1))="T","Trust",IF(UPPER(MID(W7,4,1))="A","AOP",""))))))))</f>
       </c>
       <c r="Z7" s="10" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="AA7" s="16">
-        <f>IF($B7&lt;&gt;"Entry","",IF(Z7="","",IF(X7="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z7)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y7="Individual",Y7="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z7)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z7)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B7&lt;&gt;"Entry","",IF(Z7="","",IF(X7="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z7)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y7="Individual",Y7="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z7)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z7)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB7" s="13">
         <v>46173</v>
@@ -3154,17 +3275,17 @@
         <f>IF($B7&lt;&gt;"Entry","",0)</f>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="AJ7" s="10" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="AK7" s="17">
         <v>0</v>
       </c>
       <c r="AL7" s="10"/>
       <c r="AM7" s="10" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="AN7" s="15">
         <f>IF($B7&lt;&gt;"Challan","",SUMIF($D$4:$D$207,D7,$AD$4:$AD$207)+SUMIF($D$4:$D$207,D7,$AG$4:$AG$207)+SUMIF($D$4:$D$207,D7,$AE$4:$AE$207))</f>
@@ -3220,7 +3341,7 @@
       </c>
       <c r="Z8" s="28"/>
       <c r="AA8" s="29">
-        <f>IF($B8&lt;&gt;"Entry","",IF(Z8="","",IF(X8="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z8)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y8="Individual",Y8="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z8)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z8)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B8&lt;&gt;"Entry","",IF(Z8="","",IF(X8="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z8)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y8="Individual",Y8="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z8)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z8)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB8" s="30"/>
       <c r="AC8" s="31"/>
@@ -3298,7 +3419,7 @@
       </c>
       <c r="Z9" s="28"/>
       <c r="AA9" s="29">
-        <f>IF($B9&lt;&gt;"Entry","",IF(Z9="","",IF(X9="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z9)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y9="Individual",Y9="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z9)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z9)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B9&lt;&gt;"Entry","",IF(Z9="","",IF(X9="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z9)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y9="Individual",Y9="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z9)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z9)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB9" s="30"/>
       <c r="AC9" s="31"/>
@@ -3376,7 +3497,7 @@
       </c>
       <c r="Z10" s="28"/>
       <c r="AA10" s="29">
-        <f>IF($B10&lt;&gt;"Entry","",IF(Z10="","",IF(X10="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z10)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y10="Individual",Y10="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z10)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z10)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B10&lt;&gt;"Entry","",IF(Z10="","",IF(X10="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z10)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y10="Individual",Y10="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z10)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z10)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB10" s="30"/>
       <c r="AC10" s="31"/>
@@ -3454,7 +3575,7 @@
       </c>
       <c r="Z11" s="28"/>
       <c r="AA11" s="29">
-        <f>IF($B11&lt;&gt;"Entry","",IF(Z11="","",IF(X11="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z11)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y11="Individual",Y11="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z11)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z11)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B11&lt;&gt;"Entry","",IF(Z11="","",IF(X11="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z11)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y11="Individual",Y11="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z11)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z11)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB11" s="30"/>
       <c r="AC11" s="31"/>
@@ -3532,7 +3653,7 @@
       </c>
       <c r="Z12" s="28"/>
       <c r="AA12" s="29">
-        <f>IF($B12&lt;&gt;"Entry","",IF(Z12="","",IF(X12="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z12)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y12="Individual",Y12="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z12)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z12)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B12&lt;&gt;"Entry","",IF(Z12="","",IF(X12="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z12)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y12="Individual",Y12="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z12)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z12)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB12" s="30"/>
       <c r="AC12" s="31"/>
@@ -3610,7 +3731,7 @@
       </c>
       <c r="Z13" s="28"/>
       <c r="AA13" s="29">
-        <f>IF($B13&lt;&gt;"Entry","",IF(Z13="","",IF(X13="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z13)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y13="Individual",Y13="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z13)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z13)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B13&lt;&gt;"Entry","",IF(Z13="","",IF(X13="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z13)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y13="Individual",Y13="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z13)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z13)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB13" s="30"/>
       <c r="AC13" s="31"/>
@@ -3688,7 +3809,7 @@
       </c>
       <c r="Z14" s="28"/>
       <c r="AA14" s="29">
-        <f>IF($B14&lt;&gt;"Entry","",IF(Z14="","",IF(X14="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z14)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y14="Individual",Y14="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z14)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z14)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B14&lt;&gt;"Entry","",IF(Z14="","",IF(X14="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z14)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y14="Individual",Y14="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z14)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z14)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB14" s="30"/>
       <c r="AC14" s="31"/>
@@ -3766,7 +3887,7 @@
       </c>
       <c r="Z15" s="28"/>
       <c r="AA15" s="29">
-        <f>IF($B15&lt;&gt;"Entry","",IF(Z15="","",IF(X15="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z15)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y15="Individual",Y15="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z15)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z15)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B15&lt;&gt;"Entry","",IF(Z15="","",IF(X15="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z15)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y15="Individual",Y15="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z15)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z15)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB15" s="30"/>
       <c r="AC15" s="31"/>
@@ -3844,7 +3965,7 @@
       </c>
       <c r="Z16" s="28"/>
       <c r="AA16" s="29">
-        <f>IF($B16&lt;&gt;"Entry","",IF(Z16="","",IF(X16="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z16)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y16="Individual",Y16="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z16)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z16)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B16&lt;&gt;"Entry","",IF(Z16="","",IF(X16="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z16)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y16="Individual",Y16="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z16)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z16)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB16" s="30"/>
       <c r="AC16" s="31"/>
@@ -3922,7 +4043,7 @@
       </c>
       <c r="Z17" s="28"/>
       <c r="AA17" s="29">
-        <f>IF($B17&lt;&gt;"Entry","",IF(Z17="","",IF(X17="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z17)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y17="Individual",Y17="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z17)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z17)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B17&lt;&gt;"Entry","",IF(Z17="","",IF(X17="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z17)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y17="Individual",Y17="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z17)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z17)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB17" s="30"/>
       <c r="AC17" s="31"/>
@@ -4000,7 +4121,7 @@
       </c>
       <c r="Z18" s="28"/>
       <c r="AA18" s="29">
-        <f>IF($B18&lt;&gt;"Entry","",IF(Z18="","",IF(X18="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z18)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y18="Individual",Y18="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z18)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z18)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B18&lt;&gt;"Entry","",IF(Z18="","",IF(X18="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z18)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y18="Individual",Y18="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z18)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z18)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB18" s="30"/>
       <c r="AC18" s="31"/>
@@ -4078,7 +4199,7 @@
       </c>
       <c r="Z19" s="28"/>
       <c r="AA19" s="29">
-        <f>IF($B19&lt;&gt;"Entry","",IF(Z19="","",IF(X19="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z19)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y19="Individual",Y19="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z19)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z19)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B19&lt;&gt;"Entry","",IF(Z19="","",IF(X19="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z19)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y19="Individual",Y19="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z19)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z19)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB19" s="30"/>
       <c r="AC19" s="31"/>
@@ -4156,7 +4277,7 @@
       </c>
       <c r="Z20" s="28"/>
       <c r="AA20" s="29">
-        <f>IF($B20&lt;&gt;"Entry","",IF(Z20="","",IF(X20="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z20)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y20="Individual",Y20="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z20)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z20)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B20&lt;&gt;"Entry","",IF(Z20="","",IF(X20="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z20)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y20="Individual",Y20="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z20)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z20)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB20" s="30"/>
       <c r="AC20" s="31"/>
@@ -4234,7 +4355,7 @@
       </c>
       <c r="Z21" s="28"/>
       <c r="AA21" s="29">
-        <f>IF($B21&lt;&gt;"Entry","",IF(Z21="","",IF(X21="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z21)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y21="Individual",Y21="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z21)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z21)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B21&lt;&gt;"Entry","",IF(Z21="","",IF(X21="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z21)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y21="Individual",Y21="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z21)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z21)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB21" s="30"/>
       <c r="AC21" s="31"/>
@@ -4312,7 +4433,7 @@
       </c>
       <c r="Z22" s="28"/>
       <c r="AA22" s="29">
-        <f>IF($B22&lt;&gt;"Entry","",IF(Z22="","",IF(X22="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z22)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y22="Individual",Y22="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z22)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z22)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B22&lt;&gt;"Entry","",IF(Z22="","",IF(X22="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z22)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y22="Individual",Y22="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z22)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z22)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB22" s="30"/>
       <c r="AC22" s="31"/>
@@ -4390,7 +4511,7 @@
       </c>
       <c r="Z23" s="28"/>
       <c r="AA23" s="29">
-        <f>IF($B23&lt;&gt;"Entry","",IF(Z23="","",IF(X23="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z23)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y23="Individual",Y23="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z23)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z23)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B23&lt;&gt;"Entry","",IF(Z23="","",IF(X23="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z23)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y23="Individual",Y23="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z23)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z23)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB23" s="30"/>
       <c r="AC23" s="31"/>
@@ -4468,7 +4589,7 @@
       </c>
       <c r="Z24" s="28"/>
       <c r="AA24" s="29">
-        <f>IF($B24&lt;&gt;"Entry","",IF(Z24="","",IF(X24="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z24)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y24="Individual",Y24="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z24)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z24)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B24&lt;&gt;"Entry","",IF(Z24="","",IF(X24="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z24)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y24="Individual",Y24="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z24)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z24)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB24" s="30"/>
       <c r="AC24" s="31"/>
@@ -4546,7 +4667,7 @@
       </c>
       <c r="Z25" s="28"/>
       <c r="AA25" s="29">
-        <f>IF($B25&lt;&gt;"Entry","",IF(Z25="","",IF(X25="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z25)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y25="Individual",Y25="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z25)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z25)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B25&lt;&gt;"Entry","",IF(Z25="","",IF(X25="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z25)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y25="Individual",Y25="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z25)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z25)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB25" s="30"/>
       <c r="AC25" s="31"/>
@@ -4624,7 +4745,7 @@
       </c>
       <c r="Z26" s="28"/>
       <c r="AA26" s="29">
-        <f>IF($B26&lt;&gt;"Entry","",IF(Z26="","",IF(X26="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z26)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y26="Individual",Y26="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z26)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z26)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B26&lt;&gt;"Entry","",IF(Z26="","",IF(X26="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z26)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y26="Individual",Y26="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z26)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z26)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB26" s="30"/>
       <c r="AC26" s="31"/>
@@ -4702,7 +4823,7 @@
       </c>
       <c r="Z27" s="28"/>
       <c r="AA27" s="29">
-        <f>IF($B27&lt;&gt;"Entry","",IF(Z27="","",IF(X27="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z27)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y27="Individual",Y27="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z27)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z27)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B27&lt;&gt;"Entry","",IF(Z27="","",IF(X27="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z27)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y27="Individual",Y27="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z27)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z27)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB27" s="30"/>
       <c r="AC27" s="31"/>
@@ -4780,7 +4901,7 @@
       </c>
       <c r="Z28" s="28"/>
       <c r="AA28" s="29">
-        <f>IF($B28&lt;&gt;"Entry","",IF(Z28="","",IF(X28="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z28)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y28="Individual",Y28="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z28)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z28)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B28&lt;&gt;"Entry","",IF(Z28="","",IF(X28="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z28)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y28="Individual",Y28="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z28)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z28)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB28" s="30"/>
       <c r="AC28" s="31"/>
@@ -4858,7 +4979,7 @@
       </c>
       <c r="Z29" s="28"/>
       <c r="AA29" s="29">
-        <f>IF($B29&lt;&gt;"Entry","",IF(Z29="","",IF(X29="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z29)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y29="Individual",Y29="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z29)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z29)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B29&lt;&gt;"Entry","",IF(Z29="","",IF(X29="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z29)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y29="Individual",Y29="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z29)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z29)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB29" s="30"/>
       <c r="AC29" s="31"/>
@@ -4936,7 +5057,7 @@
       </c>
       <c r="Z30" s="28"/>
       <c r="AA30" s="29">
-        <f>IF($B30&lt;&gt;"Entry","",IF(Z30="","",IF(X30="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z30)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y30="Individual",Y30="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z30)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z30)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B30&lt;&gt;"Entry","",IF(Z30="","",IF(X30="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z30)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y30="Individual",Y30="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z30)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z30)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB30" s="30"/>
       <c r="AC30" s="31"/>
@@ -5014,7 +5135,7 @@
       </c>
       <c r="Z31" s="28"/>
       <c r="AA31" s="29">
-        <f>IF($B31&lt;&gt;"Entry","",IF(Z31="","",IF(X31="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z31)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y31="Individual",Y31="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z31)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z31)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B31&lt;&gt;"Entry","",IF(Z31="","",IF(X31="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z31)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y31="Individual",Y31="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z31)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z31)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB31" s="30"/>
       <c r="AC31" s="31"/>
@@ -5092,7 +5213,7 @@
       </c>
       <c r="Z32" s="28"/>
       <c r="AA32" s="29">
-        <f>IF($B32&lt;&gt;"Entry","",IF(Z32="","",IF(X32="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z32)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y32="Individual",Y32="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z32)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z32)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B32&lt;&gt;"Entry","",IF(Z32="","",IF(X32="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z32)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y32="Individual",Y32="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z32)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z32)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB32" s="30"/>
       <c r="AC32" s="31"/>
@@ -5170,7 +5291,7 @@
       </c>
       <c r="Z33" s="28"/>
       <c r="AA33" s="29">
-        <f>IF($B33&lt;&gt;"Entry","",IF(Z33="","",IF(X33="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z33)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y33="Individual",Y33="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z33)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z33)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B33&lt;&gt;"Entry","",IF(Z33="","",IF(X33="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z33)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y33="Individual",Y33="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z33)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z33)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB33" s="30"/>
       <c r="AC33" s="31"/>
@@ -5248,7 +5369,7 @@
       </c>
       <c r="Z34" s="28"/>
       <c r="AA34" s="29">
-        <f>IF($B34&lt;&gt;"Entry","",IF(Z34="","",IF(X34="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z34)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y34="Individual",Y34="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z34)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z34)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B34&lt;&gt;"Entry","",IF(Z34="","",IF(X34="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z34)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y34="Individual",Y34="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z34)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z34)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB34" s="30"/>
       <c r="AC34" s="31"/>
@@ -5326,7 +5447,7 @@
       </c>
       <c r="Z35" s="28"/>
       <c r="AA35" s="29">
-        <f>IF($B35&lt;&gt;"Entry","",IF(Z35="","",IF(X35="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z35)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y35="Individual",Y35="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z35)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z35)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B35&lt;&gt;"Entry","",IF(Z35="","",IF(X35="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z35)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y35="Individual",Y35="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z35)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z35)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB35" s="30"/>
       <c r="AC35" s="31"/>
@@ -5404,7 +5525,7 @@
       </c>
       <c r="Z36" s="28"/>
       <c r="AA36" s="29">
-        <f>IF($B36&lt;&gt;"Entry","",IF(Z36="","",IF(X36="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z36)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y36="Individual",Y36="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z36)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z36)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B36&lt;&gt;"Entry","",IF(Z36="","",IF(X36="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z36)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y36="Individual",Y36="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z36)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z36)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB36" s="30"/>
       <c r="AC36" s="31"/>
@@ -5482,7 +5603,7 @@
       </c>
       <c r="Z37" s="28"/>
       <c r="AA37" s="29">
-        <f>IF($B37&lt;&gt;"Entry","",IF(Z37="","",IF(X37="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z37)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y37="Individual",Y37="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z37)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z37)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B37&lt;&gt;"Entry","",IF(Z37="","",IF(X37="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z37)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y37="Individual",Y37="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z37)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z37)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB37" s="30"/>
       <c r="AC37" s="31"/>
@@ -5560,7 +5681,7 @@
       </c>
       <c r="Z38" s="28"/>
       <c r="AA38" s="29">
-        <f>IF($B38&lt;&gt;"Entry","",IF(Z38="","",IF(X38="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z38)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y38="Individual",Y38="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z38)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z38)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B38&lt;&gt;"Entry","",IF(Z38="","",IF(X38="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z38)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y38="Individual",Y38="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z38)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z38)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB38" s="30"/>
       <c r="AC38" s="31"/>
@@ -5638,7 +5759,7 @@
       </c>
       <c r="Z39" s="28"/>
       <c r="AA39" s="29">
-        <f>IF($B39&lt;&gt;"Entry","",IF(Z39="","",IF(X39="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z39)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y39="Individual",Y39="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z39)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z39)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B39&lt;&gt;"Entry","",IF(Z39="","",IF(X39="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z39)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y39="Individual",Y39="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z39)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z39)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB39" s="30"/>
       <c r="AC39" s="31"/>
@@ -5716,7 +5837,7 @@
       </c>
       <c r="Z40" s="28"/>
       <c r="AA40" s="29">
-        <f>IF($B40&lt;&gt;"Entry","",IF(Z40="","",IF(X40="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z40)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y40="Individual",Y40="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z40)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z40)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B40&lt;&gt;"Entry","",IF(Z40="","",IF(X40="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z40)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y40="Individual",Y40="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z40)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z40)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB40" s="30"/>
       <c r="AC40" s="31"/>
@@ -5794,7 +5915,7 @@
       </c>
       <c r="Z41" s="28"/>
       <c r="AA41" s="29">
-        <f>IF($B41&lt;&gt;"Entry","",IF(Z41="","",IF(X41="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z41)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y41="Individual",Y41="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z41)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z41)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B41&lt;&gt;"Entry","",IF(Z41="","",IF(X41="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z41)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y41="Individual",Y41="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z41)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z41)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB41" s="30"/>
       <c r="AC41" s="31"/>
@@ -5872,7 +5993,7 @@
       </c>
       <c r="Z42" s="28"/>
       <c r="AA42" s="29">
-        <f>IF($B42&lt;&gt;"Entry","",IF(Z42="","",IF(X42="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z42)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y42="Individual",Y42="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z42)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z42)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B42&lt;&gt;"Entry","",IF(Z42="","",IF(X42="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z42)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y42="Individual",Y42="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z42)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z42)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB42" s="30"/>
       <c r="AC42" s="31"/>
@@ -5950,7 +6071,7 @@
       </c>
       <c r="Z43" s="28"/>
       <c r="AA43" s="29">
-        <f>IF($B43&lt;&gt;"Entry","",IF(Z43="","",IF(X43="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z43)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y43="Individual",Y43="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z43)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z43)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B43&lt;&gt;"Entry","",IF(Z43="","",IF(X43="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z43)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y43="Individual",Y43="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z43)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z43)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB43" s="30"/>
       <c r="AC43" s="31"/>
@@ -6028,7 +6149,7 @@
       </c>
       <c r="Z44" s="28"/>
       <c r="AA44" s="29">
-        <f>IF($B44&lt;&gt;"Entry","",IF(Z44="","",IF(X44="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z44)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y44="Individual",Y44="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z44)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z44)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B44&lt;&gt;"Entry","",IF(Z44="","",IF(X44="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z44)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y44="Individual",Y44="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z44)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z44)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB44" s="30"/>
       <c r="AC44" s="31"/>
@@ -6106,7 +6227,7 @@
       </c>
       <c r="Z45" s="28"/>
       <c r="AA45" s="29">
-        <f>IF($B45&lt;&gt;"Entry","",IF(Z45="","",IF(X45="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z45)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y45="Individual",Y45="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z45)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z45)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B45&lt;&gt;"Entry","",IF(Z45="","",IF(X45="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z45)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y45="Individual",Y45="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z45)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z45)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB45" s="30"/>
       <c r="AC45" s="31"/>
@@ -6184,7 +6305,7 @@
       </c>
       <c r="Z46" s="28"/>
       <c r="AA46" s="29">
-        <f>IF($B46&lt;&gt;"Entry","",IF(Z46="","",IF(X46="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z46)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y46="Individual",Y46="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z46)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z46)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B46&lt;&gt;"Entry","",IF(Z46="","",IF(X46="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z46)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y46="Individual",Y46="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z46)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z46)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB46" s="30"/>
       <c r="AC46" s="31"/>
@@ -6262,7 +6383,7 @@
       </c>
       <c r="Z47" s="28"/>
       <c r="AA47" s="29">
-        <f>IF($B47&lt;&gt;"Entry","",IF(Z47="","",IF(X47="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z47)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y47="Individual",Y47="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z47)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z47)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B47&lt;&gt;"Entry","",IF(Z47="","",IF(X47="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z47)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y47="Individual",Y47="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z47)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z47)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB47" s="30"/>
       <c r="AC47" s="31"/>
@@ -6340,7 +6461,7 @@
       </c>
       <c r="Z48" s="28"/>
       <c r="AA48" s="29">
-        <f>IF($B48&lt;&gt;"Entry","",IF(Z48="","",IF(X48="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z48)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y48="Individual",Y48="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z48)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z48)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B48&lt;&gt;"Entry","",IF(Z48="","",IF(X48="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z48)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y48="Individual",Y48="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z48)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z48)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB48" s="30"/>
       <c r="AC48" s="31"/>
@@ -6418,7 +6539,7 @@
       </c>
       <c r="Z49" s="28"/>
       <c r="AA49" s="29">
-        <f>IF($B49&lt;&gt;"Entry","",IF(Z49="","",IF(X49="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z49)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y49="Individual",Y49="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z49)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z49)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B49&lt;&gt;"Entry","",IF(Z49="","",IF(X49="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z49)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y49="Individual",Y49="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z49)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z49)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB49" s="30"/>
       <c r="AC49" s="31"/>
@@ -6496,7 +6617,7 @@
       </c>
       <c r="Z50" s="28"/>
       <c r="AA50" s="29">
-        <f>IF($B50&lt;&gt;"Entry","",IF(Z50="","",IF(X50="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z50)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y50="Individual",Y50="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z50)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z50)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B50&lt;&gt;"Entry","",IF(Z50="","",IF(X50="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z50)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y50="Individual",Y50="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z50)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z50)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB50" s="30"/>
       <c r="AC50" s="31"/>
@@ -6574,7 +6695,7 @@
       </c>
       <c r="Z51" s="28"/>
       <c r="AA51" s="29">
-        <f>IF($B51&lt;&gt;"Entry","",IF(Z51="","",IF(X51="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z51)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y51="Individual",Y51="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z51)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z51)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B51&lt;&gt;"Entry","",IF(Z51="","",IF(X51="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z51)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y51="Individual",Y51="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z51)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z51)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB51" s="30"/>
       <c r="AC51" s="31"/>
@@ -6652,7 +6773,7 @@
       </c>
       <c r="Z52" s="28"/>
       <c r="AA52" s="29">
-        <f>IF($B52&lt;&gt;"Entry","",IF(Z52="","",IF(X52="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z52)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y52="Individual",Y52="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z52)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z52)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B52&lt;&gt;"Entry","",IF(Z52="","",IF(X52="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z52)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y52="Individual",Y52="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z52)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z52)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB52" s="30"/>
       <c r="AC52" s="31"/>
@@ -6730,7 +6851,7 @@
       </c>
       <c r="Z53" s="28"/>
       <c r="AA53" s="29">
-        <f>IF($B53&lt;&gt;"Entry","",IF(Z53="","",IF(X53="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z53)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y53="Individual",Y53="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z53)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z53)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B53&lt;&gt;"Entry","",IF(Z53="","",IF(X53="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z53)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y53="Individual",Y53="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z53)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z53)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB53" s="30"/>
       <c r="AC53" s="31"/>
@@ -6808,7 +6929,7 @@
       </c>
       <c r="Z54" s="28"/>
       <c r="AA54" s="29">
-        <f>IF($B54&lt;&gt;"Entry","",IF(Z54="","",IF(X54="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z54)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y54="Individual",Y54="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z54)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z54)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B54&lt;&gt;"Entry","",IF(Z54="","",IF(X54="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z54)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y54="Individual",Y54="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z54)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z54)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB54" s="30"/>
       <c r="AC54" s="31"/>
@@ -6886,7 +7007,7 @@
       </c>
       <c r="Z55" s="28"/>
       <c r="AA55" s="29">
-        <f>IF($B55&lt;&gt;"Entry","",IF(Z55="","",IF(X55="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z55)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y55="Individual",Y55="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z55)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z55)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B55&lt;&gt;"Entry","",IF(Z55="","",IF(X55="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z55)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y55="Individual",Y55="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z55)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z55)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB55" s="30"/>
       <c r="AC55" s="31"/>
@@ -6964,7 +7085,7 @@
       </c>
       <c r="Z56" s="28"/>
       <c r="AA56" s="29">
-        <f>IF($B56&lt;&gt;"Entry","",IF(Z56="","",IF(X56="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z56)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y56="Individual",Y56="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z56)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z56)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B56&lt;&gt;"Entry","",IF(Z56="","",IF(X56="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z56)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y56="Individual",Y56="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z56)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z56)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB56" s="30"/>
       <c r="AC56" s="31"/>
@@ -7042,7 +7163,7 @@
       </c>
       <c r="Z57" s="28"/>
       <c r="AA57" s="29">
-        <f>IF($B57&lt;&gt;"Entry","",IF(Z57="","",IF(X57="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z57)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y57="Individual",Y57="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z57)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z57)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B57&lt;&gt;"Entry","",IF(Z57="","",IF(X57="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z57)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y57="Individual",Y57="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z57)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z57)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB57" s="30"/>
       <c r="AC57" s="31"/>
@@ -7120,7 +7241,7 @@
       </c>
       <c r="Z58" s="28"/>
       <c r="AA58" s="29">
-        <f>IF($B58&lt;&gt;"Entry","",IF(Z58="","",IF(X58="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z58)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y58="Individual",Y58="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z58)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z58)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B58&lt;&gt;"Entry","",IF(Z58="","",IF(X58="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z58)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y58="Individual",Y58="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z58)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z58)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB58" s="30"/>
       <c r="AC58" s="31"/>
@@ -7198,7 +7319,7 @@
       </c>
       <c r="Z59" s="28"/>
       <c r="AA59" s="29">
-        <f>IF($B59&lt;&gt;"Entry","",IF(Z59="","",IF(X59="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z59)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y59="Individual",Y59="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z59)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z59)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B59&lt;&gt;"Entry","",IF(Z59="","",IF(X59="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z59)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y59="Individual",Y59="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z59)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z59)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB59" s="30"/>
       <c r="AC59" s="31"/>
@@ -7276,7 +7397,7 @@
       </c>
       <c r="Z60" s="28"/>
       <c r="AA60" s="29">
-        <f>IF($B60&lt;&gt;"Entry","",IF(Z60="","",IF(X60="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z60)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y60="Individual",Y60="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z60)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z60)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B60&lt;&gt;"Entry","",IF(Z60="","",IF(X60="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z60)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y60="Individual",Y60="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z60)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z60)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB60" s="30"/>
       <c r="AC60" s="31"/>
@@ -7354,7 +7475,7 @@
       </c>
       <c r="Z61" s="28"/>
       <c r="AA61" s="29">
-        <f>IF($B61&lt;&gt;"Entry","",IF(Z61="","",IF(X61="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z61)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y61="Individual",Y61="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z61)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z61)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B61&lt;&gt;"Entry","",IF(Z61="","",IF(X61="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z61)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y61="Individual",Y61="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z61)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z61)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB61" s="30"/>
       <c r="AC61" s="31"/>
@@ -7432,7 +7553,7 @@
       </c>
       <c r="Z62" s="28"/>
       <c r="AA62" s="29">
-        <f>IF($B62&lt;&gt;"Entry","",IF(Z62="","",IF(X62="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z62)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y62="Individual",Y62="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z62)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z62)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B62&lt;&gt;"Entry","",IF(Z62="","",IF(X62="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z62)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y62="Individual",Y62="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z62)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z62)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB62" s="30"/>
       <c r="AC62" s="31"/>
@@ -7510,7 +7631,7 @@
       </c>
       <c r="Z63" s="28"/>
       <c r="AA63" s="29">
-        <f>IF($B63&lt;&gt;"Entry","",IF(Z63="","",IF(X63="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z63)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y63="Individual",Y63="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z63)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z63)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B63&lt;&gt;"Entry","",IF(Z63="","",IF(X63="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z63)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y63="Individual",Y63="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z63)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z63)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB63" s="30"/>
       <c r="AC63" s="31"/>
@@ -7588,7 +7709,7 @@
       </c>
       <c r="Z64" s="28"/>
       <c r="AA64" s="29">
-        <f>IF($B64&lt;&gt;"Entry","",IF(Z64="","",IF(X64="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z64)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y64="Individual",Y64="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z64)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z64)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B64&lt;&gt;"Entry","",IF(Z64="","",IF(X64="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z64)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y64="Individual",Y64="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z64)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z64)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB64" s="30"/>
       <c r="AC64" s="31"/>
@@ -7666,7 +7787,7 @@
       </c>
       <c r="Z65" s="28"/>
       <c r="AA65" s="29">
-        <f>IF($B65&lt;&gt;"Entry","",IF(Z65="","",IF(X65="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z65)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y65="Individual",Y65="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z65)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z65)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B65&lt;&gt;"Entry","",IF(Z65="","",IF(X65="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z65)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y65="Individual",Y65="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z65)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z65)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB65" s="30"/>
       <c r="AC65" s="31"/>
@@ -7744,7 +7865,7 @@
       </c>
       <c r="Z66" s="28"/>
       <c r="AA66" s="29">
-        <f>IF($B66&lt;&gt;"Entry","",IF(Z66="","",IF(X66="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z66)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y66="Individual",Y66="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z66)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z66)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B66&lt;&gt;"Entry","",IF(Z66="","",IF(X66="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z66)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y66="Individual",Y66="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z66)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z66)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB66" s="30"/>
       <c r="AC66" s="31"/>
@@ -7822,7 +7943,7 @@
       </c>
       <c r="Z67" s="28"/>
       <c r="AA67" s="29">
-        <f>IF($B67&lt;&gt;"Entry","",IF(Z67="","",IF(X67="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z67)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y67="Individual",Y67="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z67)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z67)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B67&lt;&gt;"Entry","",IF(Z67="","",IF(X67="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z67)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y67="Individual",Y67="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z67)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z67)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB67" s="30"/>
       <c r="AC67" s="31"/>
@@ -7900,7 +8021,7 @@
       </c>
       <c r="Z68" s="28"/>
       <c r="AA68" s="29">
-        <f>IF($B68&lt;&gt;"Entry","",IF(Z68="","",IF(X68="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z68)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y68="Individual",Y68="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z68)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z68)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B68&lt;&gt;"Entry","",IF(Z68="","",IF(X68="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z68)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y68="Individual",Y68="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z68)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z68)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB68" s="30"/>
       <c r="AC68" s="31"/>
@@ -7978,7 +8099,7 @@
       </c>
       <c r="Z69" s="28"/>
       <c r="AA69" s="29">
-        <f>IF($B69&lt;&gt;"Entry","",IF(Z69="","",IF(X69="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z69)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y69="Individual",Y69="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z69)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z69)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B69&lt;&gt;"Entry","",IF(Z69="","",IF(X69="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z69)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y69="Individual",Y69="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z69)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z69)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB69" s="30"/>
       <c r="AC69" s="31"/>
@@ -8056,7 +8177,7 @@
       </c>
       <c r="Z70" s="28"/>
       <c r="AA70" s="29">
-        <f>IF($B70&lt;&gt;"Entry","",IF(Z70="","",IF(X70="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z70)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y70="Individual",Y70="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z70)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z70)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B70&lt;&gt;"Entry","",IF(Z70="","",IF(X70="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z70)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y70="Individual",Y70="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z70)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z70)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB70" s="30"/>
       <c r="AC70" s="31"/>
@@ -8134,7 +8255,7 @@
       </c>
       <c r="Z71" s="28"/>
       <c r="AA71" s="29">
-        <f>IF($B71&lt;&gt;"Entry","",IF(Z71="","",IF(X71="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z71)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y71="Individual",Y71="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z71)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z71)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B71&lt;&gt;"Entry","",IF(Z71="","",IF(X71="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z71)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y71="Individual",Y71="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z71)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z71)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB71" s="30"/>
       <c r="AC71" s="31"/>
@@ -8212,7 +8333,7 @@
       </c>
       <c r="Z72" s="28"/>
       <c r="AA72" s="29">
-        <f>IF($B72&lt;&gt;"Entry","",IF(Z72="","",IF(X72="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z72)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y72="Individual",Y72="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z72)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z72)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B72&lt;&gt;"Entry","",IF(Z72="","",IF(X72="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z72)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y72="Individual",Y72="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z72)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z72)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB72" s="30"/>
       <c r="AC72" s="31"/>
@@ -8290,7 +8411,7 @@
       </c>
       <c r="Z73" s="28"/>
       <c r="AA73" s="29">
-        <f>IF($B73&lt;&gt;"Entry","",IF(Z73="","",IF(X73="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z73)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y73="Individual",Y73="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z73)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z73)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B73&lt;&gt;"Entry","",IF(Z73="","",IF(X73="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z73)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y73="Individual",Y73="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z73)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z73)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB73" s="30"/>
       <c r="AC73" s="31"/>
@@ -8368,7 +8489,7 @@
       </c>
       <c r="Z74" s="28"/>
       <c r="AA74" s="29">
-        <f>IF($B74&lt;&gt;"Entry","",IF(Z74="","",IF(X74="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z74)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y74="Individual",Y74="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z74)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z74)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B74&lt;&gt;"Entry","",IF(Z74="","",IF(X74="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z74)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y74="Individual",Y74="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z74)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z74)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB74" s="30"/>
       <c r="AC74" s="31"/>
@@ -8446,7 +8567,7 @@
       </c>
       <c r="Z75" s="28"/>
       <c r="AA75" s="29">
-        <f>IF($B75&lt;&gt;"Entry","",IF(Z75="","",IF(X75="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z75)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y75="Individual",Y75="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z75)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z75)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B75&lt;&gt;"Entry","",IF(Z75="","",IF(X75="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z75)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y75="Individual",Y75="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z75)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z75)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB75" s="30"/>
       <c r="AC75" s="31"/>
@@ -8524,7 +8645,7 @@
       </c>
       <c r="Z76" s="28"/>
       <c r="AA76" s="29">
-        <f>IF($B76&lt;&gt;"Entry","",IF(Z76="","",IF(X76="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z76)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y76="Individual",Y76="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z76)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z76)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B76&lt;&gt;"Entry","",IF(Z76="","",IF(X76="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z76)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y76="Individual",Y76="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z76)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z76)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB76" s="30"/>
       <c r="AC76" s="31"/>
@@ -8602,7 +8723,7 @@
       </c>
       <c r="Z77" s="28"/>
       <c r="AA77" s="29">
-        <f>IF($B77&lt;&gt;"Entry","",IF(Z77="","",IF(X77="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z77)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y77="Individual",Y77="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z77)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z77)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B77&lt;&gt;"Entry","",IF(Z77="","",IF(X77="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z77)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y77="Individual",Y77="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z77)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z77)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB77" s="30"/>
       <c r="AC77" s="31"/>
@@ -8680,7 +8801,7 @@
       </c>
       <c r="Z78" s="28"/>
       <c r="AA78" s="29">
-        <f>IF($B78&lt;&gt;"Entry","",IF(Z78="","",IF(X78="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z78)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y78="Individual",Y78="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z78)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z78)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B78&lt;&gt;"Entry","",IF(Z78="","",IF(X78="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z78)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y78="Individual",Y78="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z78)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z78)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB78" s="30"/>
       <c r="AC78" s="31"/>
@@ -8758,7 +8879,7 @@
       </c>
       <c r="Z79" s="28"/>
       <c r="AA79" s="29">
-        <f>IF($B79&lt;&gt;"Entry","",IF(Z79="","",IF(X79="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z79)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y79="Individual",Y79="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z79)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z79)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B79&lt;&gt;"Entry","",IF(Z79="","",IF(X79="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z79)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y79="Individual",Y79="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z79)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z79)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB79" s="30"/>
       <c r="AC79" s="31"/>
@@ -8836,7 +8957,7 @@
       </c>
       <c r="Z80" s="28"/>
       <c r="AA80" s="29">
-        <f>IF($B80&lt;&gt;"Entry","",IF(Z80="","",IF(X80="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z80)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y80="Individual",Y80="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z80)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z80)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B80&lt;&gt;"Entry","",IF(Z80="","",IF(X80="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z80)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y80="Individual",Y80="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z80)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z80)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB80" s="30"/>
       <c r="AC80" s="31"/>
@@ -8914,7 +9035,7 @@
       </c>
       <c r="Z81" s="28"/>
       <c r="AA81" s="29">
-        <f>IF($B81&lt;&gt;"Entry","",IF(Z81="","",IF(X81="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z81)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y81="Individual",Y81="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z81)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z81)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B81&lt;&gt;"Entry","",IF(Z81="","",IF(X81="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z81)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y81="Individual",Y81="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z81)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z81)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB81" s="30"/>
       <c r="AC81" s="31"/>
@@ -8992,7 +9113,7 @@
       </c>
       <c r="Z82" s="28"/>
       <c r="AA82" s="29">
-        <f>IF($B82&lt;&gt;"Entry","",IF(Z82="","",IF(X82="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z82)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y82="Individual",Y82="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z82)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z82)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B82&lt;&gt;"Entry","",IF(Z82="","",IF(X82="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z82)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y82="Individual",Y82="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z82)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z82)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB82" s="30"/>
       <c r="AC82" s="31"/>
@@ -9070,7 +9191,7 @@
       </c>
       <c r="Z83" s="28"/>
       <c r="AA83" s="29">
-        <f>IF($B83&lt;&gt;"Entry","",IF(Z83="","",IF(X83="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z83)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y83="Individual",Y83="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z83)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z83)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B83&lt;&gt;"Entry","",IF(Z83="","",IF(X83="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z83)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y83="Individual",Y83="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z83)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z83)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB83" s="30"/>
       <c r="AC83" s="31"/>
@@ -9148,7 +9269,7 @@
       </c>
       <c r="Z84" s="28"/>
       <c r="AA84" s="29">
-        <f>IF($B84&lt;&gt;"Entry","",IF(Z84="","",IF(X84="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z84)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y84="Individual",Y84="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z84)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z84)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B84&lt;&gt;"Entry","",IF(Z84="","",IF(X84="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z84)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y84="Individual",Y84="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z84)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z84)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB84" s="30"/>
       <c r="AC84" s="31"/>
@@ -9226,7 +9347,7 @@
       </c>
       <c r="Z85" s="28"/>
       <c r="AA85" s="29">
-        <f>IF($B85&lt;&gt;"Entry","",IF(Z85="","",IF(X85="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z85)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y85="Individual",Y85="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z85)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z85)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B85&lt;&gt;"Entry","",IF(Z85="","",IF(X85="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z85)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y85="Individual",Y85="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z85)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z85)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB85" s="30"/>
       <c r="AC85" s="31"/>
@@ -9304,7 +9425,7 @@
       </c>
       <c r="Z86" s="28"/>
       <c r="AA86" s="29">
-        <f>IF($B86&lt;&gt;"Entry","",IF(Z86="","",IF(X86="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z86)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y86="Individual",Y86="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z86)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z86)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B86&lt;&gt;"Entry","",IF(Z86="","",IF(X86="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z86)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y86="Individual",Y86="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z86)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z86)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB86" s="30"/>
       <c r="AC86" s="31"/>
@@ -9382,7 +9503,7 @@
       </c>
       <c r="Z87" s="28"/>
       <c r="AA87" s="29">
-        <f>IF($B87&lt;&gt;"Entry","",IF(Z87="","",IF(X87="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z87)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y87="Individual",Y87="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z87)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z87)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B87&lt;&gt;"Entry","",IF(Z87="","",IF(X87="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z87)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y87="Individual",Y87="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z87)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z87)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB87" s="30"/>
       <c r="AC87" s="31"/>
@@ -9460,7 +9581,7 @@
       </c>
       <c r="Z88" s="28"/>
       <c r="AA88" s="29">
-        <f>IF($B88&lt;&gt;"Entry","",IF(Z88="","",IF(X88="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z88)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y88="Individual",Y88="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z88)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z88)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B88&lt;&gt;"Entry","",IF(Z88="","",IF(X88="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z88)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y88="Individual",Y88="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z88)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z88)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB88" s="30"/>
       <c r="AC88" s="31"/>
@@ -9538,7 +9659,7 @@
       </c>
       <c r="Z89" s="28"/>
       <c r="AA89" s="29">
-        <f>IF($B89&lt;&gt;"Entry","",IF(Z89="","",IF(X89="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z89)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y89="Individual",Y89="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z89)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z89)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B89&lt;&gt;"Entry","",IF(Z89="","",IF(X89="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z89)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y89="Individual",Y89="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z89)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z89)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB89" s="30"/>
       <c r="AC89" s="31"/>
@@ -9616,7 +9737,7 @@
       </c>
       <c r="Z90" s="28"/>
       <c r="AA90" s="29">
-        <f>IF($B90&lt;&gt;"Entry","",IF(Z90="","",IF(X90="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z90)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y90="Individual",Y90="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z90)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z90)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B90&lt;&gt;"Entry","",IF(Z90="","",IF(X90="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z90)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y90="Individual",Y90="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z90)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z90)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB90" s="30"/>
       <c r="AC90" s="31"/>
@@ -9694,7 +9815,7 @@
       </c>
       <c r="Z91" s="28"/>
       <c r="AA91" s="29">
-        <f>IF($B91&lt;&gt;"Entry","",IF(Z91="","",IF(X91="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z91)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y91="Individual",Y91="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z91)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z91)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B91&lt;&gt;"Entry","",IF(Z91="","",IF(X91="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z91)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y91="Individual",Y91="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z91)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z91)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB91" s="30"/>
       <c r="AC91" s="31"/>
@@ -9772,7 +9893,7 @@
       </c>
       <c r="Z92" s="28"/>
       <c r="AA92" s="29">
-        <f>IF($B92&lt;&gt;"Entry","",IF(Z92="","",IF(X92="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z92)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y92="Individual",Y92="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z92)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z92)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B92&lt;&gt;"Entry","",IF(Z92="","",IF(X92="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z92)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y92="Individual",Y92="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z92)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z92)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB92" s="30"/>
       <c r="AC92" s="31"/>
@@ -9850,7 +9971,7 @@
       </c>
       <c r="Z93" s="28"/>
       <c r="AA93" s="29">
-        <f>IF($B93&lt;&gt;"Entry","",IF(Z93="","",IF(X93="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z93)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y93="Individual",Y93="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z93)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z93)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B93&lt;&gt;"Entry","",IF(Z93="","",IF(X93="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z93)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y93="Individual",Y93="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z93)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z93)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB93" s="30"/>
       <c r="AC93" s="31"/>
@@ -9928,7 +10049,7 @@
       </c>
       <c r="Z94" s="28"/>
       <c r="AA94" s="29">
-        <f>IF($B94&lt;&gt;"Entry","",IF(Z94="","",IF(X94="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z94)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y94="Individual",Y94="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z94)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z94)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B94&lt;&gt;"Entry","",IF(Z94="","",IF(X94="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z94)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y94="Individual",Y94="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z94)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z94)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB94" s="30"/>
       <c r="AC94" s="31"/>
@@ -10006,7 +10127,7 @@
       </c>
       <c r="Z95" s="28"/>
       <c r="AA95" s="29">
-        <f>IF($B95&lt;&gt;"Entry","",IF(Z95="","",IF(X95="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z95)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y95="Individual",Y95="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z95)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z95)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B95&lt;&gt;"Entry","",IF(Z95="","",IF(X95="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z95)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y95="Individual",Y95="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z95)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z95)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB95" s="30"/>
       <c r="AC95" s="31"/>
@@ -10084,7 +10205,7 @@
       </c>
       <c r="Z96" s="28"/>
       <c r="AA96" s="29">
-        <f>IF($B96&lt;&gt;"Entry","",IF(Z96="","",IF(X96="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z96)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y96="Individual",Y96="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z96)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z96)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B96&lt;&gt;"Entry","",IF(Z96="","",IF(X96="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z96)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y96="Individual",Y96="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z96)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z96)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB96" s="30"/>
       <c r="AC96" s="31"/>
@@ -10162,7 +10283,7 @@
       </c>
       <c r="Z97" s="28"/>
       <c r="AA97" s="29">
-        <f>IF($B97&lt;&gt;"Entry","",IF(Z97="","",IF(X97="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z97)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y97="Individual",Y97="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z97)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z97)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B97&lt;&gt;"Entry","",IF(Z97="","",IF(X97="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z97)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y97="Individual",Y97="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z97)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z97)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB97" s="30"/>
       <c r="AC97" s="31"/>
@@ -10240,7 +10361,7 @@
       </c>
       <c r="Z98" s="28"/>
       <c r="AA98" s="29">
-        <f>IF($B98&lt;&gt;"Entry","",IF(Z98="","",IF(X98="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z98)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y98="Individual",Y98="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z98)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z98)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B98&lt;&gt;"Entry","",IF(Z98="","",IF(X98="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z98)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y98="Individual",Y98="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z98)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z98)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB98" s="30"/>
       <c r="AC98" s="31"/>
@@ -10318,7 +10439,7 @@
       </c>
       <c r="Z99" s="28"/>
       <c r="AA99" s="29">
-        <f>IF($B99&lt;&gt;"Entry","",IF(Z99="","",IF(X99="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z99)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y99="Individual",Y99="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z99)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z99)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B99&lt;&gt;"Entry","",IF(Z99="","",IF(X99="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z99)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y99="Individual",Y99="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z99)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z99)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB99" s="30"/>
       <c r="AC99" s="31"/>
@@ -10396,7 +10517,7 @@
       </c>
       <c r="Z100" s="28"/>
       <c r="AA100" s="29">
-        <f>IF($B100&lt;&gt;"Entry","",IF(Z100="","",IF(X100="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z100)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y100="Individual",Y100="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z100)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z100)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B100&lt;&gt;"Entry","",IF(Z100="","",IF(X100="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z100)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y100="Individual",Y100="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z100)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z100)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB100" s="30"/>
       <c r="AC100" s="31"/>
@@ -10474,7 +10595,7 @@
       </c>
       <c r="Z101" s="28"/>
       <c r="AA101" s="29">
-        <f>IF($B101&lt;&gt;"Entry","",IF(Z101="","",IF(X101="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z101)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y101="Individual",Y101="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z101)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z101)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B101&lt;&gt;"Entry","",IF(Z101="","",IF(X101="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z101)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y101="Individual",Y101="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z101)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z101)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB101" s="30"/>
       <c r="AC101" s="31"/>
@@ -10552,7 +10673,7 @@
       </c>
       <c r="Z102" s="28"/>
       <c r="AA102" s="29">
-        <f>IF($B102&lt;&gt;"Entry","",IF(Z102="","",IF(X102="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z102)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y102="Individual",Y102="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z102)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z102)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B102&lt;&gt;"Entry","",IF(Z102="","",IF(X102="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z102)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y102="Individual",Y102="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z102)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z102)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB102" s="30"/>
       <c r="AC102" s="31"/>
@@ -10630,7 +10751,7 @@
       </c>
       <c r="Z103" s="28"/>
       <c r="AA103" s="29">
-        <f>IF($B103&lt;&gt;"Entry","",IF(Z103="","",IF(X103="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z103)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y103="Individual",Y103="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z103)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z103)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B103&lt;&gt;"Entry","",IF(Z103="","",IF(X103="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z103)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y103="Individual",Y103="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z103)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z103)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB103" s="30"/>
       <c r="AC103" s="31"/>
@@ -10708,7 +10829,7 @@
       </c>
       <c r="Z104" s="28"/>
       <c r="AA104" s="29">
-        <f>IF($B104&lt;&gt;"Entry","",IF(Z104="","",IF(X104="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z104)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y104="Individual",Y104="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z104)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z104)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B104&lt;&gt;"Entry","",IF(Z104="","",IF(X104="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z104)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y104="Individual",Y104="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z104)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z104)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB104" s="30"/>
       <c r="AC104" s="31"/>
@@ -10786,7 +10907,7 @@
       </c>
       <c r="Z105" s="28"/>
       <c r="AA105" s="29">
-        <f>IF($B105&lt;&gt;"Entry","",IF(Z105="","",IF(X105="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z105)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y105="Individual",Y105="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z105)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z105)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B105&lt;&gt;"Entry","",IF(Z105="","",IF(X105="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z105)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y105="Individual",Y105="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z105)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z105)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB105" s="30"/>
       <c r="AC105" s="31"/>
@@ -10864,7 +10985,7 @@
       </c>
       <c r="Z106" s="28"/>
       <c r="AA106" s="29">
-        <f>IF($B106&lt;&gt;"Entry","",IF(Z106="","",IF(X106="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z106)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y106="Individual",Y106="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z106)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z106)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B106&lt;&gt;"Entry","",IF(Z106="","",IF(X106="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z106)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y106="Individual",Y106="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z106)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z106)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB106" s="30"/>
       <c r="AC106" s="31"/>
@@ -10942,7 +11063,7 @@
       </c>
       <c r="Z107" s="28"/>
       <c r="AA107" s="29">
-        <f>IF($B107&lt;&gt;"Entry","",IF(Z107="","",IF(X107="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z107)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y107="Individual",Y107="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z107)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z107)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B107&lt;&gt;"Entry","",IF(Z107="","",IF(X107="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z107)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y107="Individual",Y107="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z107)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z107)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB107" s="30"/>
       <c r="AC107" s="31"/>
@@ -11020,7 +11141,7 @@
       </c>
       <c r="Z108" s="28"/>
       <c r="AA108" s="29">
-        <f>IF($B108&lt;&gt;"Entry","",IF(Z108="","",IF(X108="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z108)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y108="Individual",Y108="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z108)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z108)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B108&lt;&gt;"Entry","",IF(Z108="","",IF(X108="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z108)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y108="Individual",Y108="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z108)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z108)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB108" s="30"/>
       <c r="AC108" s="31"/>
@@ -11098,7 +11219,7 @@
       </c>
       <c r="Z109" s="28"/>
       <c r="AA109" s="29">
-        <f>IF($B109&lt;&gt;"Entry","",IF(Z109="","",IF(X109="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z109)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y109="Individual",Y109="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z109)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z109)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B109&lt;&gt;"Entry","",IF(Z109="","",IF(X109="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z109)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y109="Individual",Y109="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z109)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z109)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB109" s="30"/>
       <c r="AC109" s="31"/>
@@ -11176,7 +11297,7 @@
       </c>
       <c r="Z110" s="28"/>
       <c r="AA110" s="29">
-        <f>IF($B110&lt;&gt;"Entry","",IF(Z110="","",IF(X110="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z110)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y110="Individual",Y110="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z110)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z110)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B110&lt;&gt;"Entry","",IF(Z110="","",IF(X110="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z110)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y110="Individual",Y110="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z110)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z110)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB110" s="30"/>
       <c r="AC110" s="31"/>
@@ -11254,7 +11375,7 @@
       </c>
       <c r="Z111" s="28"/>
       <c r="AA111" s="29">
-        <f>IF($B111&lt;&gt;"Entry","",IF(Z111="","",IF(X111="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z111)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y111="Individual",Y111="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z111)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z111)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B111&lt;&gt;"Entry","",IF(Z111="","",IF(X111="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z111)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y111="Individual",Y111="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z111)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z111)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB111" s="30"/>
       <c r="AC111" s="31"/>
@@ -11332,7 +11453,7 @@
       </c>
       <c r="Z112" s="28"/>
       <c r="AA112" s="29">
-        <f>IF($B112&lt;&gt;"Entry","",IF(Z112="","",IF(X112="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z112)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y112="Individual",Y112="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z112)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z112)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B112&lt;&gt;"Entry","",IF(Z112="","",IF(X112="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z112)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y112="Individual",Y112="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z112)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z112)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB112" s="30"/>
       <c r="AC112" s="31"/>
@@ -11410,7 +11531,7 @@
       </c>
       <c r="Z113" s="28"/>
       <c r="AA113" s="29">
-        <f>IF($B113&lt;&gt;"Entry","",IF(Z113="","",IF(X113="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z113)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y113="Individual",Y113="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z113)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z113)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B113&lt;&gt;"Entry","",IF(Z113="","",IF(X113="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z113)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y113="Individual",Y113="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z113)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z113)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB113" s="30"/>
       <c r="AC113" s="31"/>
@@ -11488,7 +11609,7 @@
       </c>
       <c r="Z114" s="28"/>
       <c r="AA114" s="29">
-        <f>IF($B114&lt;&gt;"Entry","",IF(Z114="","",IF(X114="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z114)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y114="Individual",Y114="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z114)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z114)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B114&lt;&gt;"Entry","",IF(Z114="","",IF(X114="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z114)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y114="Individual",Y114="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z114)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z114)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB114" s="30"/>
       <c r="AC114" s="31"/>
@@ -11566,7 +11687,7 @@
       </c>
       <c r="Z115" s="28"/>
       <c r="AA115" s="29">
-        <f>IF($B115&lt;&gt;"Entry","",IF(Z115="","",IF(X115="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z115)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y115="Individual",Y115="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z115)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z115)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B115&lt;&gt;"Entry","",IF(Z115="","",IF(X115="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z115)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y115="Individual",Y115="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z115)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z115)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB115" s="30"/>
       <c r="AC115" s="31"/>
@@ -11644,7 +11765,7 @@
       </c>
       <c r="Z116" s="28"/>
       <c r="AA116" s="29">
-        <f>IF($B116&lt;&gt;"Entry","",IF(Z116="","",IF(X116="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z116)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y116="Individual",Y116="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z116)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z116)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B116&lt;&gt;"Entry","",IF(Z116="","",IF(X116="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z116)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y116="Individual",Y116="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z116)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z116)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB116" s="30"/>
       <c r="AC116" s="31"/>
@@ -11722,7 +11843,7 @@
       </c>
       <c r="Z117" s="28"/>
       <c r="AA117" s="29">
-        <f>IF($B117&lt;&gt;"Entry","",IF(Z117="","",IF(X117="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z117)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y117="Individual",Y117="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z117)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z117)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B117&lt;&gt;"Entry","",IF(Z117="","",IF(X117="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z117)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y117="Individual",Y117="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z117)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z117)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB117" s="30"/>
       <c r="AC117" s="31"/>
@@ -11800,7 +11921,7 @@
       </c>
       <c r="Z118" s="28"/>
       <c r="AA118" s="29">
-        <f>IF($B118&lt;&gt;"Entry","",IF(Z118="","",IF(X118="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z118)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y118="Individual",Y118="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z118)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z118)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B118&lt;&gt;"Entry","",IF(Z118="","",IF(X118="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z118)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y118="Individual",Y118="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z118)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z118)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB118" s="30"/>
       <c r="AC118" s="31"/>
@@ -11878,7 +11999,7 @@
       </c>
       <c r="Z119" s="28"/>
       <c r="AA119" s="29">
-        <f>IF($B119&lt;&gt;"Entry","",IF(Z119="","",IF(X119="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z119)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y119="Individual",Y119="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z119)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z119)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B119&lt;&gt;"Entry","",IF(Z119="","",IF(X119="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z119)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y119="Individual",Y119="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z119)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z119)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB119" s="30"/>
       <c r="AC119" s="31"/>
@@ -11956,7 +12077,7 @@
       </c>
       <c r="Z120" s="28"/>
       <c r="AA120" s="29">
-        <f>IF($B120&lt;&gt;"Entry","",IF(Z120="","",IF(X120="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z120)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y120="Individual",Y120="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z120)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z120)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B120&lt;&gt;"Entry","",IF(Z120="","",IF(X120="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z120)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y120="Individual",Y120="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z120)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z120)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB120" s="30"/>
       <c r="AC120" s="31"/>
@@ -12034,7 +12155,7 @@
       </c>
       <c r="Z121" s="28"/>
       <c r="AA121" s="29">
-        <f>IF($B121&lt;&gt;"Entry","",IF(Z121="","",IF(X121="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z121)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y121="Individual",Y121="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z121)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z121)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B121&lt;&gt;"Entry","",IF(Z121="","",IF(X121="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z121)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y121="Individual",Y121="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z121)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z121)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB121" s="30"/>
       <c r="AC121" s="31"/>
@@ -12112,7 +12233,7 @@
       </c>
       <c r="Z122" s="28"/>
       <c r="AA122" s="29">
-        <f>IF($B122&lt;&gt;"Entry","",IF(Z122="","",IF(X122="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z122)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y122="Individual",Y122="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z122)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z122)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B122&lt;&gt;"Entry","",IF(Z122="","",IF(X122="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z122)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y122="Individual",Y122="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z122)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z122)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB122" s="30"/>
       <c r="AC122" s="31"/>
@@ -12190,7 +12311,7 @@
       </c>
       <c r="Z123" s="28"/>
       <c r="AA123" s="29">
-        <f>IF($B123&lt;&gt;"Entry","",IF(Z123="","",IF(X123="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z123)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y123="Individual",Y123="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z123)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z123)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B123&lt;&gt;"Entry","",IF(Z123="","",IF(X123="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z123)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y123="Individual",Y123="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z123)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z123)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB123" s="30"/>
       <c r="AC123" s="31"/>
@@ -12268,7 +12389,7 @@
       </c>
       <c r="Z124" s="28"/>
       <c r="AA124" s="29">
-        <f>IF($B124&lt;&gt;"Entry","",IF(Z124="","",IF(X124="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z124)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y124="Individual",Y124="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z124)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z124)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B124&lt;&gt;"Entry","",IF(Z124="","",IF(X124="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z124)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y124="Individual",Y124="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z124)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z124)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB124" s="30"/>
       <c r="AC124" s="31"/>
@@ -12346,7 +12467,7 @@
       </c>
       <c r="Z125" s="28"/>
       <c r="AA125" s="29">
-        <f>IF($B125&lt;&gt;"Entry","",IF(Z125="","",IF(X125="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z125)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y125="Individual",Y125="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z125)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z125)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B125&lt;&gt;"Entry","",IF(Z125="","",IF(X125="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z125)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y125="Individual",Y125="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z125)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z125)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB125" s="30"/>
       <c r="AC125" s="31"/>
@@ -12424,7 +12545,7 @@
       </c>
       <c r="Z126" s="28"/>
       <c r="AA126" s="29">
-        <f>IF($B126&lt;&gt;"Entry","",IF(Z126="","",IF(X126="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z126)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y126="Individual",Y126="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z126)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z126)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B126&lt;&gt;"Entry","",IF(Z126="","",IF(X126="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z126)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y126="Individual",Y126="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z126)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z126)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB126" s="30"/>
       <c r="AC126" s="31"/>
@@ -12502,7 +12623,7 @@
       </c>
       <c r="Z127" s="28"/>
       <c r="AA127" s="29">
-        <f>IF($B127&lt;&gt;"Entry","",IF(Z127="","",IF(X127="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z127)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y127="Individual",Y127="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z127)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z127)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B127&lt;&gt;"Entry","",IF(Z127="","",IF(X127="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z127)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y127="Individual",Y127="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z127)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z127)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB127" s="30"/>
       <c r="AC127" s="31"/>
@@ -12580,7 +12701,7 @@
       </c>
       <c r="Z128" s="28"/>
       <c r="AA128" s="29">
-        <f>IF($B128&lt;&gt;"Entry","",IF(Z128="","",IF(X128="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z128)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y128="Individual",Y128="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z128)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z128)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B128&lt;&gt;"Entry","",IF(Z128="","",IF(X128="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z128)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y128="Individual",Y128="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z128)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z128)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB128" s="30"/>
       <c r="AC128" s="31"/>
@@ -12658,7 +12779,7 @@
       </c>
       <c r="Z129" s="28"/>
       <c r="AA129" s="29">
-        <f>IF($B129&lt;&gt;"Entry","",IF(Z129="","",IF(X129="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z129)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y129="Individual",Y129="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z129)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z129)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B129&lt;&gt;"Entry","",IF(Z129="","",IF(X129="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z129)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y129="Individual",Y129="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z129)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z129)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB129" s="30"/>
       <c r="AC129" s="31"/>
@@ -12736,7 +12857,7 @@
       </c>
       <c r="Z130" s="28"/>
       <c r="AA130" s="29">
-        <f>IF($B130&lt;&gt;"Entry","",IF(Z130="","",IF(X130="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z130)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y130="Individual",Y130="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z130)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z130)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B130&lt;&gt;"Entry","",IF(Z130="","",IF(X130="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z130)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y130="Individual",Y130="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z130)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z130)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB130" s="30"/>
       <c r="AC130" s="31"/>
@@ -12814,7 +12935,7 @@
       </c>
       <c r="Z131" s="28"/>
       <c r="AA131" s="29">
-        <f>IF($B131&lt;&gt;"Entry","",IF(Z131="","",IF(X131="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z131)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y131="Individual",Y131="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z131)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z131)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B131&lt;&gt;"Entry","",IF(Z131="","",IF(X131="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z131)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y131="Individual",Y131="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z131)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z131)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB131" s="30"/>
       <c r="AC131" s="31"/>
@@ -12892,7 +13013,7 @@
       </c>
       <c r="Z132" s="28"/>
       <c r="AA132" s="29">
-        <f>IF($B132&lt;&gt;"Entry","",IF(Z132="","",IF(X132="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z132)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y132="Individual",Y132="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z132)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z132)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B132&lt;&gt;"Entry","",IF(Z132="","",IF(X132="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z132)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y132="Individual",Y132="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z132)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z132)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB132" s="30"/>
       <c r="AC132" s="31"/>
@@ -12970,7 +13091,7 @@
       </c>
       <c r="Z133" s="28"/>
       <c r="AA133" s="29">
-        <f>IF($B133&lt;&gt;"Entry","",IF(Z133="","",IF(X133="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z133)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y133="Individual",Y133="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z133)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z133)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B133&lt;&gt;"Entry","",IF(Z133="","",IF(X133="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z133)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y133="Individual",Y133="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z133)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z133)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB133" s="30"/>
       <c r="AC133" s="31"/>
@@ -13048,7 +13169,7 @@
       </c>
       <c r="Z134" s="28"/>
       <c r="AA134" s="29">
-        <f>IF($B134&lt;&gt;"Entry","",IF(Z134="","",IF(X134="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z134)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y134="Individual",Y134="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z134)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z134)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B134&lt;&gt;"Entry","",IF(Z134="","",IF(X134="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z134)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y134="Individual",Y134="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z134)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z134)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB134" s="30"/>
       <c r="AC134" s="31"/>
@@ -13126,7 +13247,7 @@
       </c>
       <c r="Z135" s="28"/>
       <c r="AA135" s="29">
-        <f>IF($B135&lt;&gt;"Entry","",IF(Z135="","",IF(X135="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z135)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y135="Individual",Y135="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z135)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z135)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B135&lt;&gt;"Entry","",IF(Z135="","",IF(X135="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z135)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y135="Individual",Y135="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z135)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z135)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB135" s="30"/>
       <c r="AC135" s="31"/>
@@ -13204,7 +13325,7 @@
       </c>
       <c r="Z136" s="28"/>
       <c r="AA136" s="29">
-        <f>IF($B136&lt;&gt;"Entry","",IF(Z136="","",IF(X136="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z136)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y136="Individual",Y136="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z136)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z136)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B136&lt;&gt;"Entry","",IF(Z136="","",IF(X136="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z136)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y136="Individual",Y136="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z136)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z136)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB136" s="30"/>
       <c r="AC136" s="31"/>
@@ -13282,7 +13403,7 @@
       </c>
       <c r="Z137" s="28"/>
       <c r="AA137" s="29">
-        <f>IF($B137&lt;&gt;"Entry","",IF(Z137="","",IF(X137="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z137)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y137="Individual",Y137="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z137)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z137)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B137&lt;&gt;"Entry","",IF(Z137="","",IF(X137="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z137)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y137="Individual",Y137="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z137)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z137)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB137" s="30"/>
       <c r="AC137" s="31"/>
@@ -13360,7 +13481,7 @@
       </c>
       <c r="Z138" s="28"/>
       <c r="AA138" s="29">
-        <f>IF($B138&lt;&gt;"Entry","",IF(Z138="","",IF(X138="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z138)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y138="Individual",Y138="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z138)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z138)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B138&lt;&gt;"Entry","",IF(Z138="","",IF(X138="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z138)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y138="Individual",Y138="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z138)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z138)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB138" s="30"/>
       <c r="AC138" s="31"/>
@@ -13438,7 +13559,7 @@
       </c>
       <c r="Z139" s="28"/>
       <c r="AA139" s="29">
-        <f>IF($B139&lt;&gt;"Entry","",IF(Z139="","",IF(X139="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z139)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y139="Individual",Y139="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z139)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z139)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B139&lt;&gt;"Entry","",IF(Z139="","",IF(X139="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z139)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y139="Individual",Y139="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z139)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z139)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB139" s="30"/>
       <c r="AC139" s="31"/>
@@ -13516,7 +13637,7 @@
       </c>
       <c r="Z140" s="28"/>
       <c r="AA140" s="29">
-        <f>IF($B140&lt;&gt;"Entry","",IF(Z140="","",IF(X140="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z140)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y140="Individual",Y140="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z140)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z140)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B140&lt;&gt;"Entry","",IF(Z140="","",IF(X140="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z140)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y140="Individual",Y140="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z140)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z140)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB140" s="30"/>
       <c r="AC140" s="31"/>
@@ -13594,7 +13715,7 @@
       </c>
       <c r="Z141" s="28"/>
       <c r="AA141" s="29">
-        <f>IF($B141&lt;&gt;"Entry","",IF(Z141="","",IF(X141="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z141)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y141="Individual",Y141="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z141)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z141)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B141&lt;&gt;"Entry","",IF(Z141="","",IF(X141="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z141)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y141="Individual",Y141="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z141)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z141)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB141" s="30"/>
       <c r="AC141" s="31"/>
@@ -13672,7 +13793,7 @@
       </c>
       <c r="Z142" s="28"/>
       <c r="AA142" s="29">
-        <f>IF($B142&lt;&gt;"Entry","",IF(Z142="","",IF(X142="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z142)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y142="Individual",Y142="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z142)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z142)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B142&lt;&gt;"Entry","",IF(Z142="","",IF(X142="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z142)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y142="Individual",Y142="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z142)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z142)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB142" s="30"/>
       <c r="AC142" s="31"/>
@@ -13750,7 +13871,7 @@
       </c>
       <c r="Z143" s="28"/>
       <c r="AA143" s="29">
-        <f>IF($B143&lt;&gt;"Entry","",IF(Z143="","",IF(X143="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z143)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y143="Individual",Y143="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z143)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z143)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B143&lt;&gt;"Entry","",IF(Z143="","",IF(X143="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z143)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y143="Individual",Y143="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z143)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z143)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB143" s="30"/>
       <c r="AC143" s="31"/>
@@ -13828,7 +13949,7 @@
       </c>
       <c r="Z144" s="28"/>
       <c r="AA144" s="29">
-        <f>IF($B144&lt;&gt;"Entry","",IF(Z144="","",IF(X144="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z144)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y144="Individual",Y144="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z144)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z144)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B144&lt;&gt;"Entry","",IF(Z144="","",IF(X144="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z144)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y144="Individual",Y144="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z144)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z144)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB144" s="30"/>
       <c r="AC144" s="31"/>
@@ -13906,7 +14027,7 @@
       </c>
       <c r="Z145" s="28"/>
       <c r="AA145" s="29">
-        <f>IF($B145&lt;&gt;"Entry","",IF(Z145="","",IF(X145="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z145)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y145="Individual",Y145="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z145)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z145)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B145&lt;&gt;"Entry","",IF(Z145="","",IF(X145="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z145)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y145="Individual",Y145="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z145)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z145)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB145" s="30"/>
       <c r="AC145" s="31"/>
@@ -13984,7 +14105,7 @@
       </c>
       <c r="Z146" s="28"/>
       <c r="AA146" s="29">
-        <f>IF($B146&lt;&gt;"Entry","",IF(Z146="","",IF(X146="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z146)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y146="Individual",Y146="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z146)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z146)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B146&lt;&gt;"Entry","",IF(Z146="","",IF(X146="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z146)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y146="Individual",Y146="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z146)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z146)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB146" s="30"/>
       <c r="AC146" s="31"/>
@@ -14062,7 +14183,7 @@
       </c>
       <c r="Z147" s="28"/>
       <c r="AA147" s="29">
-        <f>IF($B147&lt;&gt;"Entry","",IF(Z147="","",IF(X147="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z147)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y147="Individual",Y147="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z147)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z147)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B147&lt;&gt;"Entry","",IF(Z147="","",IF(X147="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z147)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y147="Individual",Y147="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z147)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z147)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB147" s="30"/>
       <c r="AC147" s="31"/>
@@ -14140,7 +14261,7 @@
       </c>
       <c r="Z148" s="28"/>
       <c r="AA148" s="29">
-        <f>IF($B148&lt;&gt;"Entry","",IF(Z148="","",IF(X148="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z148)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y148="Individual",Y148="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z148)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z148)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B148&lt;&gt;"Entry","",IF(Z148="","",IF(X148="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z148)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y148="Individual",Y148="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z148)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z148)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB148" s="30"/>
       <c r="AC148" s="31"/>
@@ -14218,7 +14339,7 @@
       </c>
       <c r="Z149" s="28"/>
       <c r="AA149" s="29">
-        <f>IF($B149&lt;&gt;"Entry","",IF(Z149="","",IF(X149="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z149)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y149="Individual",Y149="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z149)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z149)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B149&lt;&gt;"Entry","",IF(Z149="","",IF(X149="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z149)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y149="Individual",Y149="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z149)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z149)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB149" s="30"/>
       <c r="AC149" s="31"/>
@@ -14296,7 +14417,7 @@
       </c>
       <c r="Z150" s="28"/>
       <c r="AA150" s="29">
-        <f>IF($B150&lt;&gt;"Entry","",IF(Z150="","",IF(X150="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z150)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y150="Individual",Y150="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z150)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z150)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B150&lt;&gt;"Entry","",IF(Z150="","",IF(X150="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z150)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y150="Individual",Y150="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z150)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z150)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB150" s="30"/>
       <c r="AC150" s="31"/>
@@ -14374,7 +14495,7 @@
       </c>
       <c r="Z151" s="28"/>
       <c r="AA151" s="29">
-        <f>IF($B151&lt;&gt;"Entry","",IF(Z151="","",IF(X151="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z151)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y151="Individual",Y151="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z151)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z151)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B151&lt;&gt;"Entry","",IF(Z151="","",IF(X151="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z151)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y151="Individual",Y151="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z151)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z151)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB151" s="30"/>
       <c r="AC151" s="31"/>
@@ -14452,7 +14573,7 @@
       </c>
       <c r="Z152" s="28"/>
       <c r="AA152" s="29">
-        <f>IF($B152&lt;&gt;"Entry","",IF(Z152="","",IF(X152="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z152)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y152="Individual",Y152="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z152)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z152)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B152&lt;&gt;"Entry","",IF(Z152="","",IF(X152="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z152)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y152="Individual",Y152="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z152)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z152)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB152" s="30"/>
       <c r="AC152" s="31"/>
@@ -14530,7 +14651,7 @@
       </c>
       <c r="Z153" s="28"/>
       <c r="AA153" s="29">
-        <f>IF($B153&lt;&gt;"Entry","",IF(Z153="","",IF(X153="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z153)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y153="Individual",Y153="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z153)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z153)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B153&lt;&gt;"Entry","",IF(Z153="","",IF(X153="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z153)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y153="Individual",Y153="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z153)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z153)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB153" s="30"/>
       <c r="AC153" s="31"/>
@@ -14608,7 +14729,7 @@
       </c>
       <c r="Z154" s="28"/>
       <c r="AA154" s="29">
-        <f>IF($B154&lt;&gt;"Entry","",IF(Z154="","",IF(X154="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z154)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y154="Individual",Y154="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z154)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z154)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B154&lt;&gt;"Entry","",IF(Z154="","",IF(X154="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z154)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y154="Individual",Y154="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z154)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z154)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB154" s="30"/>
       <c r="AC154" s="31"/>
@@ -14686,7 +14807,7 @@
       </c>
       <c r="Z155" s="28"/>
       <c r="AA155" s="29">
-        <f>IF($B155&lt;&gt;"Entry","",IF(Z155="","",IF(X155="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z155)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y155="Individual",Y155="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z155)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z155)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B155&lt;&gt;"Entry","",IF(Z155="","",IF(X155="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z155)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y155="Individual",Y155="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z155)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z155)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB155" s="30"/>
       <c r="AC155" s="31"/>
@@ -14764,7 +14885,7 @@
       </c>
       <c r="Z156" s="28"/>
       <c r="AA156" s="29">
-        <f>IF($B156&lt;&gt;"Entry","",IF(Z156="","",IF(X156="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z156)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y156="Individual",Y156="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z156)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z156)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B156&lt;&gt;"Entry","",IF(Z156="","",IF(X156="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z156)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y156="Individual",Y156="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z156)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z156)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB156" s="30"/>
       <c r="AC156" s="31"/>
@@ -14842,7 +14963,7 @@
       </c>
       <c r="Z157" s="28"/>
       <c r="AA157" s="29">
-        <f>IF($B157&lt;&gt;"Entry","",IF(Z157="","",IF(X157="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z157)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y157="Individual",Y157="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z157)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z157)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B157&lt;&gt;"Entry","",IF(Z157="","",IF(X157="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z157)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y157="Individual",Y157="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z157)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z157)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB157" s="30"/>
       <c r="AC157" s="31"/>
@@ -14920,7 +15041,7 @@
       </c>
       <c r="Z158" s="28"/>
       <c r="AA158" s="29">
-        <f>IF($B158&lt;&gt;"Entry","",IF(Z158="","",IF(X158="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z158)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y158="Individual",Y158="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z158)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z158)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B158&lt;&gt;"Entry","",IF(Z158="","",IF(X158="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z158)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y158="Individual",Y158="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z158)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z158)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB158" s="30"/>
       <c r="AC158" s="31"/>
@@ -14998,7 +15119,7 @@
       </c>
       <c r="Z159" s="28"/>
       <c r="AA159" s="29">
-        <f>IF($B159&lt;&gt;"Entry","",IF(Z159="","",IF(X159="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z159)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y159="Individual",Y159="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z159)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z159)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B159&lt;&gt;"Entry","",IF(Z159="","",IF(X159="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z159)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y159="Individual",Y159="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z159)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z159)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB159" s="30"/>
       <c r="AC159" s="31"/>
@@ -15076,7 +15197,7 @@
       </c>
       <c r="Z160" s="28"/>
       <c r="AA160" s="29">
-        <f>IF($B160&lt;&gt;"Entry","",IF(Z160="","",IF(X160="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z160)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y160="Individual",Y160="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z160)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z160)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B160&lt;&gt;"Entry","",IF(Z160="","",IF(X160="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z160)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y160="Individual",Y160="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z160)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z160)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB160" s="30"/>
       <c r="AC160" s="31"/>
@@ -15154,7 +15275,7 @@
       </c>
       <c r="Z161" s="28"/>
       <c r="AA161" s="29">
-        <f>IF($B161&lt;&gt;"Entry","",IF(Z161="","",IF(X161="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z161)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y161="Individual",Y161="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z161)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z161)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B161&lt;&gt;"Entry","",IF(Z161="","",IF(X161="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z161)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y161="Individual",Y161="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z161)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z161)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB161" s="30"/>
       <c r="AC161" s="31"/>
@@ -15232,7 +15353,7 @@
       </c>
       <c r="Z162" s="28"/>
       <c r="AA162" s="29">
-        <f>IF($B162&lt;&gt;"Entry","",IF(Z162="","",IF(X162="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z162)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y162="Individual",Y162="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z162)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z162)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B162&lt;&gt;"Entry","",IF(Z162="","",IF(X162="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z162)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y162="Individual",Y162="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z162)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z162)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB162" s="30"/>
       <c r="AC162" s="31"/>
@@ -15310,7 +15431,7 @@
       </c>
       <c r="Z163" s="28"/>
       <c r="AA163" s="29">
-        <f>IF($B163&lt;&gt;"Entry","",IF(Z163="","",IF(X163="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z163)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y163="Individual",Y163="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z163)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z163)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B163&lt;&gt;"Entry","",IF(Z163="","",IF(X163="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z163)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y163="Individual",Y163="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z163)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z163)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB163" s="30"/>
       <c r="AC163" s="31"/>
@@ -15388,7 +15509,7 @@
       </c>
       <c r="Z164" s="28"/>
       <c r="AA164" s="29">
-        <f>IF($B164&lt;&gt;"Entry","",IF(Z164="","",IF(X164="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z164)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y164="Individual",Y164="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z164)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z164)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B164&lt;&gt;"Entry","",IF(Z164="","",IF(X164="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z164)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y164="Individual",Y164="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z164)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z164)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB164" s="30"/>
       <c r="AC164" s="31"/>
@@ -15466,7 +15587,7 @@
       </c>
       <c r="Z165" s="28"/>
       <c r="AA165" s="29">
-        <f>IF($B165&lt;&gt;"Entry","",IF(Z165="","",IF(X165="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z165)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y165="Individual",Y165="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z165)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z165)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B165&lt;&gt;"Entry","",IF(Z165="","",IF(X165="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z165)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y165="Individual",Y165="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z165)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z165)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB165" s="30"/>
       <c r="AC165" s="31"/>
@@ -15544,7 +15665,7 @@
       </c>
       <c r="Z166" s="28"/>
       <c r="AA166" s="29">
-        <f>IF($B166&lt;&gt;"Entry","",IF(Z166="","",IF(X166="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z166)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y166="Individual",Y166="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z166)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z166)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B166&lt;&gt;"Entry","",IF(Z166="","",IF(X166="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z166)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y166="Individual",Y166="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z166)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z166)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB166" s="30"/>
       <c r="AC166" s="31"/>
@@ -15622,7 +15743,7 @@
       </c>
       <c r="Z167" s="28"/>
       <c r="AA167" s="29">
-        <f>IF($B167&lt;&gt;"Entry","",IF(Z167="","",IF(X167="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z167)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y167="Individual",Y167="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z167)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z167)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B167&lt;&gt;"Entry","",IF(Z167="","",IF(X167="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z167)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y167="Individual",Y167="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z167)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z167)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB167" s="30"/>
       <c r="AC167" s="31"/>
@@ -15700,7 +15821,7 @@
       </c>
       <c r="Z168" s="28"/>
       <c r="AA168" s="29">
-        <f>IF($B168&lt;&gt;"Entry","",IF(Z168="","",IF(X168="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z168)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y168="Individual",Y168="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z168)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z168)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B168&lt;&gt;"Entry","",IF(Z168="","",IF(X168="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z168)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y168="Individual",Y168="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z168)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z168)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB168" s="30"/>
       <c r="AC168" s="31"/>
@@ -15778,7 +15899,7 @@
       </c>
       <c r="Z169" s="28"/>
       <c r="AA169" s="29">
-        <f>IF($B169&lt;&gt;"Entry","",IF(Z169="","",IF(X169="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z169)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y169="Individual",Y169="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z169)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z169)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B169&lt;&gt;"Entry","",IF(Z169="","",IF(X169="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z169)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y169="Individual",Y169="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z169)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z169)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB169" s="30"/>
       <c r="AC169" s="31"/>
@@ -15856,7 +15977,7 @@
       </c>
       <c r="Z170" s="28"/>
       <c r="AA170" s="29">
-        <f>IF($B170&lt;&gt;"Entry","",IF(Z170="","",IF(X170="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z170)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y170="Individual",Y170="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z170)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z170)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B170&lt;&gt;"Entry","",IF(Z170="","",IF(X170="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z170)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y170="Individual",Y170="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z170)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z170)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB170" s="30"/>
       <c r="AC170" s="31"/>
@@ -15934,7 +16055,7 @@
       </c>
       <c r="Z171" s="28"/>
       <c r="AA171" s="29">
-        <f>IF($B171&lt;&gt;"Entry","",IF(Z171="","",IF(X171="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z171)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y171="Individual",Y171="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z171)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z171)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B171&lt;&gt;"Entry","",IF(Z171="","",IF(X171="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z171)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y171="Individual",Y171="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z171)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z171)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB171" s="30"/>
       <c r="AC171" s="31"/>
@@ -16012,7 +16133,7 @@
       </c>
       <c r="Z172" s="28"/>
       <c r="AA172" s="29">
-        <f>IF($B172&lt;&gt;"Entry","",IF(Z172="","",IF(X172="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z172)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y172="Individual",Y172="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z172)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z172)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B172&lt;&gt;"Entry","",IF(Z172="","",IF(X172="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z172)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y172="Individual",Y172="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z172)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z172)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB172" s="30"/>
       <c r="AC172" s="31"/>
@@ -16090,7 +16211,7 @@
       </c>
       <c r="Z173" s="28"/>
       <c r="AA173" s="29">
-        <f>IF($B173&lt;&gt;"Entry","",IF(Z173="","",IF(X173="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z173)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y173="Individual",Y173="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z173)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z173)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B173&lt;&gt;"Entry","",IF(Z173="","",IF(X173="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z173)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y173="Individual",Y173="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z173)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z173)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB173" s="30"/>
       <c r="AC173" s="31"/>
@@ -16168,7 +16289,7 @@
       </c>
       <c r="Z174" s="28"/>
       <c r="AA174" s="29">
-        <f>IF($B174&lt;&gt;"Entry","",IF(Z174="","",IF(X174="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z174)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y174="Individual",Y174="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z174)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z174)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B174&lt;&gt;"Entry","",IF(Z174="","",IF(X174="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z174)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y174="Individual",Y174="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z174)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z174)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB174" s="30"/>
       <c r="AC174" s="31"/>
@@ -16246,7 +16367,7 @@
       </c>
       <c r="Z175" s="28"/>
       <c r="AA175" s="29">
-        <f>IF($B175&lt;&gt;"Entry","",IF(Z175="","",IF(X175="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z175)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y175="Individual",Y175="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z175)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z175)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B175&lt;&gt;"Entry","",IF(Z175="","",IF(X175="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z175)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y175="Individual",Y175="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z175)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z175)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB175" s="30"/>
       <c r="AC175" s="31"/>
@@ -16324,7 +16445,7 @@
       </c>
       <c r="Z176" s="28"/>
       <c r="AA176" s="29">
-        <f>IF($B176&lt;&gt;"Entry","",IF(Z176="","",IF(X176="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z176)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y176="Individual",Y176="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z176)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z176)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B176&lt;&gt;"Entry","",IF(Z176="","",IF(X176="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z176)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y176="Individual",Y176="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z176)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z176)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB176" s="30"/>
       <c r="AC176" s="31"/>
@@ -16402,7 +16523,7 @@
       </c>
       <c r="Z177" s="28"/>
       <c r="AA177" s="29">
-        <f>IF($B177&lt;&gt;"Entry","",IF(Z177="","",IF(X177="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z177)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y177="Individual",Y177="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z177)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z177)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B177&lt;&gt;"Entry","",IF(Z177="","",IF(X177="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z177)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y177="Individual",Y177="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z177)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z177)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB177" s="30"/>
       <c r="AC177" s="31"/>
@@ -16480,7 +16601,7 @@
       </c>
       <c r="Z178" s="28"/>
       <c r="AA178" s="29">
-        <f>IF($B178&lt;&gt;"Entry","",IF(Z178="","",IF(X178="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z178)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y178="Individual",Y178="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z178)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z178)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B178&lt;&gt;"Entry","",IF(Z178="","",IF(X178="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z178)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y178="Individual",Y178="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z178)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z178)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB178" s="30"/>
       <c r="AC178" s="31"/>
@@ -16558,7 +16679,7 @@
       </c>
       <c r="Z179" s="28"/>
       <c r="AA179" s="29">
-        <f>IF($B179&lt;&gt;"Entry","",IF(Z179="","",IF(X179="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z179)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y179="Individual",Y179="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z179)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z179)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B179&lt;&gt;"Entry","",IF(Z179="","",IF(X179="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z179)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y179="Individual",Y179="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z179)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z179)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB179" s="30"/>
       <c r="AC179" s="31"/>
@@ -16636,7 +16757,7 @@
       </c>
       <c r="Z180" s="28"/>
       <c r="AA180" s="29">
-        <f>IF($B180&lt;&gt;"Entry","",IF(Z180="","",IF(X180="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z180)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y180="Individual",Y180="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z180)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z180)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B180&lt;&gt;"Entry","",IF(Z180="","",IF(X180="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z180)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y180="Individual",Y180="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z180)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z180)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB180" s="30"/>
       <c r="AC180" s="31"/>
@@ -16714,7 +16835,7 @@
       </c>
       <c r="Z181" s="28"/>
       <c r="AA181" s="29">
-        <f>IF($B181&lt;&gt;"Entry","",IF(Z181="","",IF(X181="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z181)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y181="Individual",Y181="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z181)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z181)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B181&lt;&gt;"Entry","",IF(Z181="","",IF(X181="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z181)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y181="Individual",Y181="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z181)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z181)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB181" s="30"/>
       <c r="AC181" s="31"/>
@@ -16792,7 +16913,7 @@
       </c>
       <c r="Z182" s="28"/>
       <c r="AA182" s="29">
-        <f>IF($B182&lt;&gt;"Entry","",IF(Z182="","",IF(X182="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z182)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y182="Individual",Y182="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z182)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z182)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B182&lt;&gt;"Entry","",IF(Z182="","",IF(X182="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z182)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y182="Individual",Y182="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z182)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z182)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB182" s="30"/>
       <c r="AC182" s="31"/>
@@ -16870,7 +16991,7 @@
       </c>
       <c r="Z183" s="28"/>
       <c r="AA183" s="29">
-        <f>IF($B183&lt;&gt;"Entry","",IF(Z183="","",IF(X183="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z183)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y183="Individual",Y183="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z183)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z183)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B183&lt;&gt;"Entry","",IF(Z183="","",IF(X183="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z183)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y183="Individual",Y183="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z183)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z183)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB183" s="30"/>
       <c r="AC183" s="31"/>
@@ -16948,7 +17069,7 @@
       </c>
       <c r="Z184" s="28"/>
       <c r="AA184" s="29">
-        <f>IF($B184&lt;&gt;"Entry","",IF(Z184="","",IF(X184="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z184)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y184="Individual",Y184="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z184)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z184)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B184&lt;&gt;"Entry","",IF(Z184="","",IF(X184="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z184)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y184="Individual",Y184="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z184)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z184)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB184" s="30"/>
       <c r="AC184" s="31"/>
@@ -17026,7 +17147,7 @@
       </c>
       <c r="Z185" s="28"/>
       <c r="AA185" s="29">
-        <f>IF($B185&lt;&gt;"Entry","",IF(Z185="","",IF(X185="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z185)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y185="Individual",Y185="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z185)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z185)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B185&lt;&gt;"Entry","",IF(Z185="","",IF(X185="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z185)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y185="Individual",Y185="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z185)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z185)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB185" s="30"/>
       <c r="AC185" s="31"/>
@@ -17104,7 +17225,7 @@
       </c>
       <c r="Z186" s="28"/>
       <c r="AA186" s="29">
-        <f>IF($B186&lt;&gt;"Entry","",IF(Z186="","",IF(X186="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z186)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y186="Individual",Y186="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z186)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z186)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B186&lt;&gt;"Entry","",IF(Z186="","",IF(X186="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z186)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y186="Individual",Y186="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z186)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z186)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB186" s="30"/>
       <c r="AC186" s="31"/>
@@ -17182,7 +17303,7 @@
       </c>
       <c r="Z187" s="28"/>
       <c r="AA187" s="29">
-        <f>IF($B187&lt;&gt;"Entry","",IF(Z187="","",IF(X187="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z187)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y187="Individual",Y187="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z187)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z187)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B187&lt;&gt;"Entry","",IF(Z187="","",IF(X187="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z187)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y187="Individual",Y187="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z187)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z187)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB187" s="30"/>
       <c r="AC187" s="31"/>
@@ -17260,7 +17381,7 @@
       </c>
       <c r="Z188" s="28"/>
       <c r="AA188" s="29">
-        <f>IF($B188&lt;&gt;"Entry","",IF(Z188="","",IF(X188="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z188)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y188="Individual",Y188="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z188)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z188)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B188&lt;&gt;"Entry","",IF(Z188="","",IF(X188="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z188)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y188="Individual",Y188="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z188)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z188)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB188" s="30"/>
       <c r="AC188" s="31"/>
@@ -17338,7 +17459,7 @@
       </c>
       <c r="Z189" s="28"/>
       <c r="AA189" s="29">
-        <f>IF($B189&lt;&gt;"Entry","",IF(Z189="","",IF(X189="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z189)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y189="Individual",Y189="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z189)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z189)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B189&lt;&gt;"Entry","",IF(Z189="","",IF(X189="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z189)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y189="Individual",Y189="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z189)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z189)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB189" s="30"/>
       <c r="AC189" s="31"/>
@@ -17416,7 +17537,7 @@
       </c>
       <c r="Z190" s="28"/>
       <c r="AA190" s="29">
-        <f>IF($B190&lt;&gt;"Entry","",IF(Z190="","",IF(X190="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z190)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y190="Individual",Y190="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z190)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z190)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B190&lt;&gt;"Entry","",IF(Z190="","",IF(X190="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z190)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y190="Individual",Y190="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z190)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z190)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB190" s="30"/>
       <c r="AC190" s="31"/>
@@ -17494,7 +17615,7 @@
       </c>
       <c r="Z191" s="28"/>
       <c r="AA191" s="29">
-        <f>IF($B191&lt;&gt;"Entry","",IF(Z191="","",IF(X191="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z191)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y191="Individual",Y191="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z191)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z191)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B191&lt;&gt;"Entry","",IF(Z191="","",IF(X191="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z191)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y191="Individual",Y191="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z191)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z191)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB191" s="30"/>
       <c r="AC191" s="31"/>
@@ -17572,7 +17693,7 @@
       </c>
       <c r="Z192" s="28"/>
       <c r="AA192" s="29">
-        <f>IF($B192&lt;&gt;"Entry","",IF(Z192="","",IF(X192="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z192)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y192="Individual",Y192="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z192)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z192)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B192&lt;&gt;"Entry","",IF(Z192="","",IF(X192="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z192)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y192="Individual",Y192="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z192)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z192)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB192" s="30"/>
       <c r="AC192" s="31"/>
@@ -17650,7 +17771,7 @@
       </c>
       <c r="Z193" s="28"/>
       <c r="AA193" s="29">
-        <f>IF($B193&lt;&gt;"Entry","",IF(Z193="","",IF(X193="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z193)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y193="Individual",Y193="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z193)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z193)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B193&lt;&gt;"Entry","",IF(Z193="","",IF(X193="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z193)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y193="Individual",Y193="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z193)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z193)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB193" s="30"/>
       <c r="AC193" s="31"/>
@@ -17728,7 +17849,7 @@
       </c>
       <c r="Z194" s="28"/>
       <c r="AA194" s="29">
-        <f>IF($B194&lt;&gt;"Entry","",IF(Z194="","",IF(X194="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z194)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y194="Individual",Y194="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z194)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z194)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B194&lt;&gt;"Entry","",IF(Z194="","",IF(X194="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z194)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y194="Individual",Y194="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z194)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z194)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB194" s="30"/>
       <c r="AC194" s="31"/>
@@ -17806,7 +17927,7 @@
       </c>
       <c r="Z195" s="28"/>
       <c r="AA195" s="29">
-        <f>IF($B195&lt;&gt;"Entry","",IF(Z195="","",IF(X195="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z195)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y195="Individual",Y195="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z195)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z195)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B195&lt;&gt;"Entry","",IF(Z195="","",IF(X195="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z195)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y195="Individual",Y195="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z195)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z195)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB195" s="30"/>
       <c r="AC195" s="31"/>
@@ -17884,7 +18005,7 @@
       </c>
       <c r="Z196" s="28"/>
       <c r="AA196" s="29">
-        <f>IF($B196&lt;&gt;"Entry","",IF(Z196="","",IF(X196="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z196)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y196="Individual",Y196="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z196)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z196)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B196&lt;&gt;"Entry","",IF(Z196="","",IF(X196="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z196)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y196="Individual",Y196="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z196)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z196)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB196" s="30"/>
       <c r="AC196" s="31"/>
@@ -17962,7 +18083,7 @@
       </c>
       <c r="Z197" s="28"/>
       <c r="AA197" s="29">
-        <f>IF($B197&lt;&gt;"Entry","",IF(Z197="","",IF(X197="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z197)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y197="Individual",Y197="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z197)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z197)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B197&lt;&gt;"Entry","",IF(Z197="","",IF(X197="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z197)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y197="Individual",Y197="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z197)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z197)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB197" s="30"/>
       <c r="AC197" s="31"/>
@@ -18040,7 +18161,7 @@
       </c>
       <c r="Z198" s="28"/>
       <c r="AA198" s="29">
-        <f>IF($B198&lt;&gt;"Entry","",IF(Z198="","",IF(X198="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z198)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y198="Individual",Y198="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z198)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z198)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B198&lt;&gt;"Entry","",IF(Z198="","",IF(X198="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z198)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y198="Individual",Y198="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z198)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z198)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB198" s="30"/>
       <c r="AC198" s="31"/>
@@ -18118,7 +18239,7 @@
       </c>
       <c r="Z199" s="28"/>
       <c r="AA199" s="29">
-        <f>IF($B199&lt;&gt;"Entry","",IF(Z199="","",IF(X199="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z199)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y199="Individual",Y199="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z199)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z199)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B199&lt;&gt;"Entry","",IF(Z199="","",IF(X199="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z199)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y199="Individual",Y199="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z199)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z199)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB199" s="30"/>
       <c r="AC199" s="31"/>
@@ -18196,7 +18317,7 @@
       </c>
       <c r="Z200" s="28"/>
       <c r="AA200" s="29">
-        <f>IF($B200&lt;&gt;"Entry","",IF(Z200="","",IF(X200="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z200)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y200="Individual",Y200="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z200)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z200)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B200&lt;&gt;"Entry","",IF(Z200="","",IF(X200="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z200)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y200="Individual",Y200="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z200)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z200)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB200" s="30"/>
       <c r="AC200" s="31"/>
@@ -18274,7 +18395,7 @@
       </c>
       <c r="Z201" s="28"/>
       <c r="AA201" s="29">
-        <f>IF($B201&lt;&gt;"Entry","",IF(Z201="","",IF(X201="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z201)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y201="Individual",Y201="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z201)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z201)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B201&lt;&gt;"Entry","",IF(Z201="","",IF(X201="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z201)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y201="Individual",Y201="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z201)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z201)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB201" s="30"/>
       <c r="AC201" s="31"/>
@@ -18352,7 +18473,7 @@
       </c>
       <c r="Z202" s="28"/>
       <c r="AA202" s="29">
-        <f>IF($B202&lt;&gt;"Entry","",IF(Z202="","",IF(X202="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z202)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y202="Individual",Y202="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z202)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z202)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B202&lt;&gt;"Entry","",IF(Z202="","",IF(X202="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z202)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y202="Individual",Y202="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z202)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z202)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB202" s="30"/>
       <c r="AC202" s="31"/>
@@ -18430,7 +18551,7 @@
       </c>
       <c r="Z203" s="28"/>
       <c r="AA203" s="29">
-        <f>IF($B203&lt;&gt;"Entry","",IF(Z203="","",IF(X203="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z203)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y203="Individual",Y203="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z203)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z203)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B203&lt;&gt;"Entry","",IF(Z203="","",IF(X203="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z203)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y203="Individual",Y203="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z203)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z203)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB203" s="30"/>
       <c r="AC203" s="31"/>
@@ -18508,7 +18629,7 @@
       </c>
       <c r="Z204" s="28"/>
       <c r="AA204" s="29">
-        <f>IF($B204&lt;&gt;"Entry","",IF(Z204="","",IF(X204="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z204)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y204="Individual",Y204="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z204)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z204)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B204&lt;&gt;"Entry","",IF(Z204="","",IF(X204="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z204)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y204="Individual",Y204="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z204)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z204)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB204" s="30"/>
       <c r="AC204" s="31"/>
@@ -18586,7 +18707,7 @@
       </c>
       <c r="Z205" s="28"/>
       <c r="AA205" s="29">
-        <f>IF($B205&lt;&gt;"Entry","",IF(Z205="","",IF(X205="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z205)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y205="Individual",Y205="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z205)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z205)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B205&lt;&gt;"Entry","",IF(Z205="","",IF(X205="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z205)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y205="Individual",Y205="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z205)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z205)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB205" s="30"/>
       <c r="AC205" s="31"/>
@@ -18664,7 +18785,7 @@
       </c>
       <c r="Z206" s="28"/>
       <c r="AA206" s="29">
-        <f>IF($B206&lt;&gt;"Entry","",IF(Z206="","",IF(X206="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z206)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y206="Individual",Y206="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z206)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z206)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B206&lt;&gt;"Entry","",IF(Z206="","",IF(X206="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z206)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y206="Individual",Y206="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z206)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z206)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB206" s="30"/>
       <c r="AC206" s="31"/>
@@ -18742,7 +18863,7 @@
       </c>
       <c r="Z207" s="28"/>
       <c r="AA207" s="29">
-        <f>IF($B207&lt;&gt;"Entry","",IF(Z207="","",IF(X207="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z207)*'Rate Lookup'!$D$1:$D$32),IF(OR(Y207="Individual",Y207="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z207)*'Rate Lookup'!$B$1:$B$32),SUMPRODUCT(('Rate Lookup'!$A$1:$A$32=Z207)*'Rate Lookup'!$C$1:$C$32)))))</f>
+        <f>IF($B207&lt;&gt;"Entry","",IF(Z207="","",IF(X207="Y",SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z207)*'Rate Lookup'!$D$1:$D$37),IF(OR(Y207="Individual",Y207="HUF"),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z207)*'Rate Lookup'!$B$1:$B$37),SUMPRODUCT(('Rate Lookup'!$A$1:$A$37=Z207)*'Rate Lookup'!$C$1:$C$37)))))</f>
       </c>
       <c r="AB207" s="30"/>
       <c r="AC207" s="31"/>
@@ -18859,7 +18980,7 @@
       <formula1>"200,400"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Section" error="Pick a section from the dropdown list." sqref="H4:H207">
-      <formula1>"192,192A,193,194,194A,194B,194BB,194C,194D,194DA,194G,194H,194I(a),194I(b),194IA,194IB,194IC,194J(a),194J(b),194K,194LA,194LB,194M,194O,194Q,194R,194S,195,196A,196D,206C(1),206C(1H)"</formula1>
+      <formula1>'Rate Lookup'!$A$1:$A$37</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Amount" error="Must be a number of 0 or more." sqref="I4:I207">
       <formula1>0</formula1>
@@ -18889,7 +19010,7 @@
       <formula1>"Y,N"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Section" error="Pick a section from the dropdown list." sqref="Z4:Z207">
-      <formula1>"192,192A,193,194,194A,194B,194BB,194C,194D,194DA,194G,194H,194I(a),194I(b),194IA,194IB,194IC,194J(a),194J(b),194K,194LA,194LB,194M,194O,194Q,194R,194S,195,196A,196D,206C(1),206C(1H)"</formula1>
+      <formula1>'Rate Lookup'!$A$1:$A$37</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix(tds): every Section option now shows a description, not a bare code
The template's Section dropdown previously showed a bare code (e.g. "194IA")
for any section outside the ~15 verified against the Section 393 payment-
code source, making it hard to identify. Added a plain description to all
18 remaining sections, using the SAME nature_of_payment text the live
software already shows for these — no payment code fabricated, only a
description, matching what's already visible in the software.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/TDS_Data_Entry_Simple_Template.xlsx
+++ b/public/templates/TDS_Data_Entry_Simple_Template.xlsx
@@ -90,7 +90,7 @@
     <t>•  194A, 194C and 194R are split into separate lettered options (194A(a)/(b)/(c), 194C(a)/(b), 194R(a)/(b)) because the new Act's Payment Code — not just the Deductee Type — now determines which citation and rate applies. Pick the option matching the actual payee/payment type; the Rate of TDS still fills in automatically.</t>
   </si>
   <si>
-    <t>•  Only the sections above have a verified Payment Code and new citation — sourced from a CBDT-derived reference table, cross-checked line by line. Every OTHER section (194B, 194BB, 194D, 194DA, 194G, 194IA, 194IB, 194IC, 194K, 194LA, 194LB, 194M, 194O, 194S, 195, 196A, 196D, 206C(1H)) still shows its plain old section code — two independent secondary sources checked for these gave conflicting payment codes for sections this template DOES have verified data for, so an unverified code is not shown rather than risk a wrong figure on an actual filing. These will be added once a verified source is available.</t>
+    <t>•  Only the sections above have a verified Payment Code and new citation — sourced from a CBDT-derived reference table, cross-checked line by line. Every OTHER section (194B, 194BB, 194D, 194DA, 194G, 194IA, 194IB, 194IC, 194K, 194LA, 194LB, 194M, 194O, 194S, 195, 196A, 196D, 206C(1H)) still shows a plain description instead (e.g. 194IA — Immovable Property Purchase) — the SAME description text the software's own Section dropdown already shows for these — rather than a Payment Code: two independent secondary sources checked for these gave conflicting payment codes for sections this template DOES have verified data for, so an unverified numeric code is never shown, only a description that carries no compliance risk. Full Payment Codes will be added once a verified source confirms them.</t>
   </si>
   <si>
     <t>Field Guide — Challan Rows (blue columns)</t>
@@ -799,7 +799,7 @@
     </r>
   </si>
   <si>
-    <t>192</t>
+    <t>192 — Salary</t>
   </si>
   <si>
     <t>1004 : [192A] : 393(7) – Premature withdrawal from Employees' Provident Fund</t>
@@ -820,10 +820,10 @@
     <t>1022 : [194A] : 393(1) [Table: S.N. 5(iii)] – Interest other than securities (Others)</t>
   </si>
   <si>
-    <t>194B</t>
+    <t>194B — Lottery/Crossword</t>
   </si>
   <si>
-    <t>194BB</t>
+    <t>194BB — Horse Racing</t>
   </si>
   <si>
     <t>1023 : [194C] : 393(1) [Table: S.N. 6(i).D(a)] – Payments to contractors and sub-contractors (Individual/HUF)</t>
@@ -832,13 +832,13 @@
     <t>1024 : [194C] : 393(1) [Table: S.N. 6(i).D(b)] – Payments to contractors and sub-contractors (Others)</t>
   </si>
   <si>
-    <t>194D</t>
+    <t>194D — Insurance Commission</t>
   </si>
   <si>
-    <t>194DA</t>
+    <t>194DA — Life Insurance Payout</t>
   </si>
   <si>
-    <t>194G</t>
+    <t>194G — Lottery Agent Commission</t>
   </si>
   <si>
     <t>1006 : [194H] : 393(1) [Table: S.N. 1(ii)] – Commission or brokerage</t>
@@ -850,13 +850,13 @@
     <t>1009 : [194I(b)] : 393(1) [Table: S.N. 2(ii).D(b)] – Rent – Land/Building/Furniture</t>
   </si>
   <si>
-    <t>194IA</t>
+    <t>194IA — Immovable Property Purchase</t>
   </si>
   <si>
-    <t>194IB</t>
+    <t>194IB — Rent by Ind/HUF (&gt;50k/month)</t>
   </si>
   <si>
-    <t>194IC</t>
+    <t>194IC — Joint Dev Agreement</t>
   </si>
   <si>
     <t>1027 : [194J(a)] : 393(1) [Table: S.N. 6(iii).D(b)] – Professional services / director remuneration</t>
@@ -865,19 +865,19 @@
     <t>1026 : [194J(b)] : 393(1) [Table: S.N. 6(iii).D(a)] – Fees for technical services</t>
   </si>
   <si>
-    <t>194K</t>
+    <t>194K — MF/UTI Units Income</t>
   </si>
   <si>
-    <t>194LA</t>
+    <t>194LA — Compulsory Acquisition</t>
   </si>
   <si>
-    <t>194LB</t>
+    <t>194LB — Infrastructure Bond Interest</t>
   </si>
   <si>
-    <t>194M</t>
+    <t>194M — Contractor/Professional by Ind</t>
   </si>
   <si>
-    <t>194O</t>
+    <t>194O — E-Commerce</t>
   </si>
   <si>
     <t>1031 : [194Q] : 393(1) [Table: S.N. 8(ii)] – Purchase of goods (buyer TDS)</t>
@@ -889,25 +889,25 @@
     <t>1035 : [194R] : 393(1) [Table: S.N. 8(iv) Note 6] – Perquisite/benefit in business or profession (In Kind/Mixed)</t>
   </si>
   <si>
-    <t>194S</t>
+    <t>194S — Virtual Digital Asset</t>
   </si>
   <si>
     <t>1067 : [194T] : 393(3) [Table: S.N. 7] – Payment to partners of a firm (salary/remuneration/interest)</t>
   </si>
   <si>
-    <t>195</t>
+    <t>195 — Other Payments to NR</t>
   </si>
   <si>
-    <t>196A</t>
+    <t>196A — MF Income to NR</t>
   </si>
   <si>
-    <t>196D</t>
+    <t>196D — FII Securities</t>
   </si>
   <si>
     <t>1073 : [206C(1)] : 394(1) [Table: S.N. 4] – Sale of scrap (TCS)</t>
   </si>
   <si>
-    <t>206C(1H)</t>
+    <t>206C(1H) — Sale of Goods (TCS)</t>
   </si>
   <si>
     <t>TDS DATA  —  each Challan row's full details, followed by its Entry rows</t>
@@ -1885,7 +1885,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" ht="110" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" ht="140" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
fix(tds): hint when PAN is typed before Row Type is picked
PAN Not Available and Deductee Type correctly stay blank until Row Type is
set to "Entry" — confirmed working as designed, not a bug — but a blank
cell looked identical to a broken one. Both columns now show "Set Row
Type" instead of a silent blank when a PAN has been typed into a row whose
Row Type isn't set yet. The software has no equivalent confusion since it
has no "Row Type" concept at all (every row there IS an entry already).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/TDS_Data_Entry_Simple_Template.xlsx
+++ b/public/templates/TDS_Data_Entry_Simple_Template.xlsx
@@ -2956,10 +2956,10 @@
       <c r="V4" s="10"/>
       <c r="W4" s="10"/>
       <c r="X4" s="12">
-        <f>IF($B4&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W4)))=10,CODE(MID(TRIM(UPPER(W4)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W4)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W4)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W4)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B4="Entry",IF(AND(LEN(TRIM(UPPER(W4)))=10,CODE(MID(TRIM(UPPER(W4)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W4)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W4)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W4)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W4)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W4)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W4)),9,1))&lt;=57),"N","Y"),IF($B4="Challan","",IF(W4&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y4" s="12">
-        <f>IF($B4&lt;&gt;"Entry","",IF(LEN(W4)&lt;4,"",IF(UPPER(MID(W4,4,1))="P","Individual",IF(UPPER(MID(W4,4,1))="H","HUF",IF(UPPER(MID(W4,4,1))="C","Company",IF(UPPER(MID(W4,4,1))="F","Firm",IF(UPPER(MID(W4,4,1))="L","LLP",IF(UPPER(MID(W4,4,1))="T","Trust",IF(UPPER(MID(W4,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B4="Entry",IF(LEN(W4)&lt;4,"",IF(UPPER(MID(W4,4,1))="P","Individual",IF(UPPER(MID(W4,4,1))="H","HUF",IF(UPPER(MID(W4,4,1))="C","Company",IF(UPPER(MID(W4,4,1))="F","Firm",IF(UPPER(MID(W4,4,1))="L","LLP",IF(UPPER(MID(W4,4,1))="T","Trust",IF(UPPER(MID(W4,4,1))="A","AOP","")))))))),IF($B4="Challan","",IF(W4&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z4" s="10"/>
       <c r="AA4" s="16">
@@ -3042,10 +3042,10 @@
         <v>161</v>
       </c>
       <c r="X5" s="12">
-        <f>IF($B5&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W5)))=10,CODE(MID(TRIM(UPPER(W5)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B5="Entry",IF(AND(LEN(TRIM(UPPER(W5)))=10,CODE(MID(TRIM(UPPER(W5)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W5)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W5)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W5)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W5)),9,1))&lt;=57),"N","Y"),IF($B5="Challan","",IF(W5&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y5" s="12">
-        <f>IF($B5&lt;&gt;"Entry","",IF(LEN(W5)&lt;4,"",IF(UPPER(MID(W5,4,1))="P","Individual",IF(UPPER(MID(W5,4,1))="H","HUF",IF(UPPER(MID(W5,4,1))="C","Company",IF(UPPER(MID(W5,4,1))="F","Firm",IF(UPPER(MID(W5,4,1))="L","LLP",IF(UPPER(MID(W5,4,1))="T","Trust",IF(UPPER(MID(W5,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B5="Entry",IF(LEN(W5)&lt;4,"",IF(UPPER(MID(W5,4,1))="P","Individual",IF(UPPER(MID(W5,4,1))="H","HUF",IF(UPPER(MID(W5,4,1))="C","Company",IF(UPPER(MID(W5,4,1))="F","Firm",IF(UPPER(MID(W5,4,1))="L","LLP",IF(UPPER(MID(W5,4,1))="T","Trust",IF(UPPER(MID(W5,4,1))="A","AOP","")))))))),IF($B5="Challan","",IF(W5&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z5" s="10" t="s">
         <v>80</v>
@@ -3142,10 +3142,10 @@
         <v>164</v>
       </c>
       <c r="X6" s="12">
-        <f>IF($B6&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W6)))=10,CODE(MID(TRIM(UPPER(W6)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B6="Entry",IF(AND(LEN(TRIM(UPPER(W6)))=10,CODE(MID(TRIM(UPPER(W6)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W6)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W6)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W6)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W6)),9,1))&lt;=57),"N","Y"),IF($B6="Challan","",IF(W6&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y6" s="12">
-        <f>IF($B6&lt;&gt;"Entry","",IF(LEN(W6)&lt;4,"",IF(UPPER(MID(W6,4,1))="P","Individual",IF(UPPER(MID(W6,4,1))="H","HUF",IF(UPPER(MID(W6,4,1))="C","Company",IF(UPPER(MID(W6,4,1))="F","Firm",IF(UPPER(MID(W6,4,1))="L","LLP",IF(UPPER(MID(W6,4,1))="T","Trust",IF(UPPER(MID(W6,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B6="Entry",IF(LEN(W6)&lt;4,"",IF(UPPER(MID(W6,4,1))="P","Individual",IF(UPPER(MID(W6,4,1))="H","HUF",IF(UPPER(MID(W6,4,1))="C","Company",IF(UPPER(MID(W6,4,1))="F","Firm",IF(UPPER(MID(W6,4,1))="L","LLP",IF(UPPER(MID(W6,4,1))="T","Trust",IF(UPPER(MID(W6,4,1))="A","AOP","")))))))),IF($B6="Challan","",IF(W6&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z6" s="10" t="s">
         <v>80</v>
@@ -3242,10 +3242,10 @@
         <v>166</v>
       </c>
       <c r="X7" s="12">
-        <f>IF($B7&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W7)))=10,CODE(MID(TRIM(UPPER(W7)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B7="Entry",IF(AND(LEN(TRIM(UPPER(W7)))=10,CODE(MID(TRIM(UPPER(W7)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W7)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W7)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W7)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W7)),9,1))&lt;=57),"N","Y"),IF($B7="Challan","",IF(W7&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y7" s="12">
-        <f>IF($B7&lt;&gt;"Entry","",IF(LEN(W7)&lt;4,"",IF(UPPER(MID(W7,4,1))="P","Individual",IF(UPPER(MID(W7,4,1))="H","HUF",IF(UPPER(MID(W7,4,1))="C","Company",IF(UPPER(MID(W7,4,1))="F","Firm",IF(UPPER(MID(W7,4,1))="L","LLP",IF(UPPER(MID(W7,4,1))="T","Trust",IF(UPPER(MID(W7,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B7="Entry",IF(LEN(W7)&lt;4,"",IF(UPPER(MID(W7,4,1))="P","Individual",IF(UPPER(MID(W7,4,1))="H","HUF",IF(UPPER(MID(W7,4,1))="C","Company",IF(UPPER(MID(W7,4,1))="F","Firm",IF(UPPER(MID(W7,4,1))="L","LLP",IF(UPPER(MID(W7,4,1))="T","Trust",IF(UPPER(MID(W7,4,1))="A","AOP","")))))))),IF($B7="Challan","",IF(W7&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z7" s="10" t="s">
         <v>90</v>
@@ -3334,10 +3334,10 @@
       <c r="V8" s="28"/>
       <c r="W8" s="28"/>
       <c r="X8" s="23">
-        <f>IF($B8&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W8)))=10,CODE(MID(TRIM(UPPER(W8)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W8)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W8)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W8)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B8="Entry",IF(AND(LEN(TRIM(UPPER(W8)))=10,CODE(MID(TRIM(UPPER(W8)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W8)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W8)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W8)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W8)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W8)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W8)),9,1))&lt;=57),"N","Y"),IF($B8="Challan","",IF(W8&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y8" s="23">
-        <f>IF($B8&lt;&gt;"Entry","",IF(LEN(W8)&lt;4,"",IF(UPPER(MID(W8,4,1))="P","Individual",IF(UPPER(MID(W8,4,1))="H","HUF",IF(UPPER(MID(W8,4,1))="C","Company",IF(UPPER(MID(W8,4,1))="F","Firm",IF(UPPER(MID(W8,4,1))="L","LLP",IF(UPPER(MID(W8,4,1))="T","Trust",IF(UPPER(MID(W8,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B8="Entry",IF(LEN(W8)&lt;4,"",IF(UPPER(MID(W8,4,1))="P","Individual",IF(UPPER(MID(W8,4,1))="H","HUF",IF(UPPER(MID(W8,4,1))="C","Company",IF(UPPER(MID(W8,4,1))="F","Firm",IF(UPPER(MID(W8,4,1))="L","LLP",IF(UPPER(MID(W8,4,1))="T","Trust",IF(UPPER(MID(W8,4,1))="A","AOP","")))))))),IF($B8="Challan","",IF(W8&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z8" s="28"/>
       <c r="AA8" s="29">
@@ -3412,10 +3412,10 @@
       <c r="V9" s="28"/>
       <c r="W9" s="28"/>
       <c r="X9" s="23">
-        <f>IF($B9&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W9)))=10,CODE(MID(TRIM(UPPER(W9)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W9)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W9)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W9)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B9="Entry",IF(AND(LEN(TRIM(UPPER(W9)))=10,CODE(MID(TRIM(UPPER(W9)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W9)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W9)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W9)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W9)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W9)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W9)),9,1))&lt;=57),"N","Y"),IF($B9="Challan","",IF(W9&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y9" s="23">
-        <f>IF($B9&lt;&gt;"Entry","",IF(LEN(W9)&lt;4,"",IF(UPPER(MID(W9,4,1))="P","Individual",IF(UPPER(MID(W9,4,1))="H","HUF",IF(UPPER(MID(W9,4,1))="C","Company",IF(UPPER(MID(W9,4,1))="F","Firm",IF(UPPER(MID(W9,4,1))="L","LLP",IF(UPPER(MID(W9,4,1))="T","Trust",IF(UPPER(MID(W9,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B9="Entry",IF(LEN(W9)&lt;4,"",IF(UPPER(MID(W9,4,1))="P","Individual",IF(UPPER(MID(W9,4,1))="H","HUF",IF(UPPER(MID(W9,4,1))="C","Company",IF(UPPER(MID(W9,4,1))="F","Firm",IF(UPPER(MID(W9,4,1))="L","LLP",IF(UPPER(MID(W9,4,1))="T","Trust",IF(UPPER(MID(W9,4,1))="A","AOP","")))))))),IF($B9="Challan","",IF(W9&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z9" s="28"/>
       <c r="AA9" s="29">
@@ -3490,10 +3490,10 @@
       <c r="V10" s="28"/>
       <c r="W10" s="28"/>
       <c r="X10" s="23">
-        <f>IF($B10&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W10)))=10,CODE(MID(TRIM(UPPER(W10)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W10)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W10)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W10)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B10="Entry",IF(AND(LEN(TRIM(UPPER(W10)))=10,CODE(MID(TRIM(UPPER(W10)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W10)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W10)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W10)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W10)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W10)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W10)),9,1))&lt;=57),"N","Y"),IF($B10="Challan","",IF(W10&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y10" s="23">
-        <f>IF($B10&lt;&gt;"Entry","",IF(LEN(W10)&lt;4,"",IF(UPPER(MID(W10,4,1))="P","Individual",IF(UPPER(MID(W10,4,1))="H","HUF",IF(UPPER(MID(W10,4,1))="C","Company",IF(UPPER(MID(W10,4,1))="F","Firm",IF(UPPER(MID(W10,4,1))="L","LLP",IF(UPPER(MID(W10,4,1))="T","Trust",IF(UPPER(MID(W10,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B10="Entry",IF(LEN(W10)&lt;4,"",IF(UPPER(MID(W10,4,1))="P","Individual",IF(UPPER(MID(W10,4,1))="H","HUF",IF(UPPER(MID(W10,4,1))="C","Company",IF(UPPER(MID(W10,4,1))="F","Firm",IF(UPPER(MID(W10,4,1))="L","LLP",IF(UPPER(MID(W10,4,1))="T","Trust",IF(UPPER(MID(W10,4,1))="A","AOP","")))))))),IF($B10="Challan","",IF(W10&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z10" s="28"/>
       <c r="AA10" s="29">
@@ -3568,10 +3568,10 @@
       <c r="V11" s="28"/>
       <c r="W11" s="28"/>
       <c r="X11" s="23">
-        <f>IF($B11&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W11)))=10,CODE(MID(TRIM(UPPER(W11)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W11)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W11)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W11)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B11="Entry",IF(AND(LEN(TRIM(UPPER(W11)))=10,CODE(MID(TRIM(UPPER(W11)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W11)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W11)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W11)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W11)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W11)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W11)),9,1))&lt;=57),"N","Y"),IF($B11="Challan","",IF(W11&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y11" s="23">
-        <f>IF($B11&lt;&gt;"Entry","",IF(LEN(W11)&lt;4,"",IF(UPPER(MID(W11,4,1))="P","Individual",IF(UPPER(MID(W11,4,1))="H","HUF",IF(UPPER(MID(W11,4,1))="C","Company",IF(UPPER(MID(W11,4,1))="F","Firm",IF(UPPER(MID(W11,4,1))="L","LLP",IF(UPPER(MID(W11,4,1))="T","Trust",IF(UPPER(MID(W11,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B11="Entry",IF(LEN(W11)&lt;4,"",IF(UPPER(MID(W11,4,1))="P","Individual",IF(UPPER(MID(W11,4,1))="H","HUF",IF(UPPER(MID(W11,4,1))="C","Company",IF(UPPER(MID(W11,4,1))="F","Firm",IF(UPPER(MID(W11,4,1))="L","LLP",IF(UPPER(MID(W11,4,1))="T","Trust",IF(UPPER(MID(W11,4,1))="A","AOP","")))))))),IF($B11="Challan","",IF(W11&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z11" s="28"/>
       <c r="AA11" s="29">
@@ -3646,10 +3646,10 @@
       <c r="V12" s="28"/>
       <c r="W12" s="28"/>
       <c r="X12" s="23">
-        <f>IF($B12&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W12)))=10,CODE(MID(TRIM(UPPER(W12)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W12)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W12)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W12)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B12="Entry",IF(AND(LEN(TRIM(UPPER(W12)))=10,CODE(MID(TRIM(UPPER(W12)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W12)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W12)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W12)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W12)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W12)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W12)),9,1))&lt;=57),"N","Y"),IF($B12="Challan","",IF(W12&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y12" s="23">
-        <f>IF($B12&lt;&gt;"Entry","",IF(LEN(W12)&lt;4,"",IF(UPPER(MID(W12,4,1))="P","Individual",IF(UPPER(MID(W12,4,1))="H","HUF",IF(UPPER(MID(W12,4,1))="C","Company",IF(UPPER(MID(W12,4,1))="F","Firm",IF(UPPER(MID(W12,4,1))="L","LLP",IF(UPPER(MID(W12,4,1))="T","Trust",IF(UPPER(MID(W12,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B12="Entry",IF(LEN(W12)&lt;4,"",IF(UPPER(MID(W12,4,1))="P","Individual",IF(UPPER(MID(W12,4,1))="H","HUF",IF(UPPER(MID(W12,4,1))="C","Company",IF(UPPER(MID(W12,4,1))="F","Firm",IF(UPPER(MID(W12,4,1))="L","LLP",IF(UPPER(MID(W12,4,1))="T","Trust",IF(UPPER(MID(W12,4,1))="A","AOP","")))))))),IF($B12="Challan","",IF(W12&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z12" s="28"/>
       <c r="AA12" s="29">
@@ -3724,10 +3724,10 @@
       <c r="V13" s="28"/>
       <c r="W13" s="28"/>
       <c r="X13" s="23">
-        <f>IF($B13&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W13)))=10,CODE(MID(TRIM(UPPER(W13)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W13)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W13)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W13)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B13="Entry",IF(AND(LEN(TRIM(UPPER(W13)))=10,CODE(MID(TRIM(UPPER(W13)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W13)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W13)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W13)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W13)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W13)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W13)),9,1))&lt;=57),"N","Y"),IF($B13="Challan","",IF(W13&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y13" s="23">
-        <f>IF($B13&lt;&gt;"Entry","",IF(LEN(W13)&lt;4,"",IF(UPPER(MID(W13,4,1))="P","Individual",IF(UPPER(MID(W13,4,1))="H","HUF",IF(UPPER(MID(W13,4,1))="C","Company",IF(UPPER(MID(W13,4,1))="F","Firm",IF(UPPER(MID(W13,4,1))="L","LLP",IF(UPPER(MID(W13,4,1))="T","Trust",IF(UPPER(MID(W13,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B13="Entry",IF(LEN(W13)&lt;4,"",IF(UPPER(MID(W13,4,1))="P","Individual",IF(UPPER(MID(W13,4,1))="H","HUF",IF(UPPER(MID(W13,4,1))="C","Company",IF(UPPER(MID(W13,4,1))="F","Firm",IF(UPPER(MID(W13,4,1))="L","LLP",IF(UPPER(MID(W13,4,1))="T","Trust",IF(UPPER(MID(W13,4,1))="A","AOP","")))))))),IF($B13="Challan","",IF(W13&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z13" s="28"/>
       <c r="AA13" s="29">
@@ -3802,10 +3802,10 @@
       <c r="V14" s="28"/>
       <c r="W14" s="28"/>
       <c r="X14" s="23">
-        <f>IF($B14&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W14)))=10,CODE(MID(TRIM(UPPER(W14)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W14)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W14)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W14)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B14="Entry",IF(AND(LEN(TRIM(UPPER(W14)))=10,CODE(MID(TRIM(UPPER(W14)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W14)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W14)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W14)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W14)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W14)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W14)),9,1))&lt;=57),"N","Y"),IF($B14="Challan","",IF(W14&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y14" s="23">
-        <f>IF($B14&lt;&gt;"Entry","",IF(LEN(W14)&lt;4,"",IF(UPPER(MID(W14,4,1))="P","Individual",IF(UPPER(MID(W14,4,1))="H","HUF",IF(UPPER(MID(W14,4,1))="C","Company",IF(UPPER(MID(W14,4,1))="F","Firm",IF(UPPER(MID(W14,4,1))="L","LLP",IF(UPPER(MID(W14,4,1))="T","Trust",IF(UPPER(MID(W14,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B14="Entry",IF(LEN(W14)&lt;4,"",IF(UPPER(MID(W14,4,1))="P","Individual",IF(UPPER(MID(W14,4,1))="H","HUF",IF(UPPER(MID(W14,4,1))="C","Company",IF(UPPER(MID(W14,4,1))="F","Firm",IF(UPPER(MID(W14,4,1))="L","LLP",IF(UPPER(MID(W14,4,1))="T","Trust",IF(UPPER(MID(W14,4,1))="A","AOP","")))))))),IF($B14="Challan","",IF(W14&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z14" s="28"/>
       <c r="AA14" s="29">
@@ -3880,10 +3880,10 @@
       <c r="V15" s="28"/>
       <c r="W15" s="28"/>
       <c r="X15" s="23">
-        <f>IF($B15&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W15)))=10,CODE(MID(TRIM(UPPER(W15)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W15)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W15)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W15)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B15="Entry",IF(AND(LEN(TRIM(UPPER(W15)))=10,CODE(MID(TRIM(UPPER(W15)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W15)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W15)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W15)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W15)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W15)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W15)),9,1))&lt;=57),"N","Y"),IF($B15="Challan","",IF(W15&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y15" s="23">
-        <f>IF($B15&lt;&gt;"Entry","",IF(LEN(W15)&lt;4,"",IF(UPPER(MID(W15,4,1))="P","Individual",IF(UPPER(MID(W15,4,1))="H","HUF",IF(UPPER(MID(W15,4,1))="C","Company",IF(UPPER(MID(W15,4,1))="F","Firm",IF(UPPER(MID(W15,4,1))="L","LLP",IF(UPPER(MID(W15,4,1))="T","Trust",IF(UPPER(MID(W15,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B15="Entry",IF(LEN(W15)&lt;4,"",IF(UPPER(MID(W15,4,1))="P","Individual",IF(UPPER(MID(W15,4,1))="H","HUF",IF(UPPER(MID(W15,4,1))="C","Company",IF(UPPER(MID(W15,4,1))="F","Firm",IF(UPPER(MID(W15,4,1))="L","LLP",IF(UPPER(MID(W15,4,1))="T","Trust",IF(UPPER(MID(W15,4,1))="A","AOP","")))))))),IF($B15="Challan","",IF(W15&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z15" s="28"/>
       <c r="AA15" s="29">
@@ -3958,10 +3958,10 @@
       <c r="V16" s="28"/>
       <c r="W16" s="28"/>
       <c r="X16" s="23">
-        <f>IF($B16&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W16)))=10,CODE(MID(TRIM(UPPER(W16)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W16)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W16)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W16)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B16="Entry",IF(AND(LEN(TRIM(UPPER(W16)))=10,CODE(MID(TRIM(UPPER(W16)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W16)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W16)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W16)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W16)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W16)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W16)),9,1))&lt;=57),"N","Y"),IF($B16="Challan","",IF(W16&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y16" s="23">
-        <f>IF($B16&lt;&gt;"Entry","",IF(LEN(W16)&lt;4,"",IF(UPPER(MID(W16,4,1))="P","Individual",IF(UPPER(MID(W16,4,1))="H","HUF",IF(UPPER(MID(W16,4,1))="C","Company",IF(UPPER(MID(W16,4,1))="F","Firm",IF(UPPER(MID(W16,4,1))="L","LLP",IF(UPPER(MID(W16,4,1))="T","Trust",IF(UPPER(MID(W16,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B16="Entry",IF(LEN(W16)&lt;4,"",IF(UPPER(MID(W16,4,1))="P","Individual",IF(UPPER(MID(W16,4,1))="H","HUF",IF(UPPER(MID(W16,4,1))="C","Company",IF(UPPER(MID(W16,4,1))="F","Firm",IF(UPPER(MID(W16,4,1))="L","LLP",IF(UPPER(MID(W16,4,1))="T","Trust",IF(UPPER(MID(W16,4,1))="A","AOP","")))))))),IF($B16="Challan","",IF(W16&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z16" s="28"/>
       <c r="AA16" s="29">
@@ -4036,10 +4036,10 @@
       <c r="V17" s="28"/>
       <c r="W17" s="28"/>
       <c r="X17" s="23">
-        <f>IF($B17&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W17)))=10,CODE(MID(TRIM(UPPER(W17)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W17)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W17)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W17)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B17="Entry",IF(AND(LEN(TRIM(UPPER(W17)))=10,CODE(MID(TRIM(UPPER(W17)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W17)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W17)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W17)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W17)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W17)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W17)),9,1))&lt;=57),"N","Y"),IF($B17="Challan","",IF(W17&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y17" s="23">
-        <f>IF($B17&lt;&gt;"Entry","",IF(LEN(W17)&lt;4,"",IF(UPPER(MID(W17,4,1))="P","Individual",IF(UPPER(MID(W17,4,1))="H","HUF",IF(UPPER(MID(W17,4,1))="C","Company",IF(UPPER(MID(W17,4,1))="F","Firm",IF(UPPER(MID(W17,4,1))="L","LLP",IF(UPPER(MID(W17,4,1))="T","Trust",IF(UPPER(MID(W17,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B17="Entry",IF(LEN(W17)&lt;4,"",IF(UPPER(MID(W17,4,1))="P","Individual",IF(UPPER(MID(W17,4,1))="H","HUF",IF(UPPER(MID(W17,4,1))="C","Company",IF(UPPER(MID(W17,4,1))="F","Firm",IF(UPPER(MID(W17,4,1))="L","LLP",IF(UPPER(MID(W17,4,1))="T","Trust",IF(UPPER(MID(W17,4,1))="A","AOP","")))))))),IF($B17="Challan","",IF(W17&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z17" s="28"/>
       <c r="AA17" s="29">
@@ -4114,10 +4114,10 @@
       <c r="V18" s="28"/>
       <c r="W18" s="28"/>
       <c r="X18" s="23">
-        <f>IF($B18&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W18)))=10,CODE(MID(TRIM(UPPER(W18)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W18)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W18)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W18)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B18="Entry",IF(AND(LEN(TRIM(UPPER(W18)))=10,CODE(MID(TRIM(UPPER(W18)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W18)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W18)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W18)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W18)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W18)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W18)),9,1))&lt;=57),"N","Y"),IF($B18="Challan","",IF(W18&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y18" s="23">
-        <f>IF($B18&lt;&gt;"Entry","",IF(LEN(W18)&lt;4,"",IF(UPPER(MID(W18,4,1))="P","Individual",IF(UPPER(MID(W18,4,1))="H","HUF",IF(UPPER(MID(W18,4,1))="C","Company",IF(UPPER(MID(W18,4,1))="F","Firm",IF(UPPER(MID(W18,4,1))="L","LLP",IF(UPPER(MID(W18,4,1))="T","Trust",IF(UPPER(MID(W18,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B18="Entry",IF(LEN(W18)&lt;4,"",IF(UPPER(MID(W18,4,1))="P","Individual",IF(UPPER(MID(W18,4,1))="H","HUF",IF(UPPER(MID(W18,4,1))="C","Company",IF(UPPER(MID(W18,4,1))="F","Firm",IF(UPPER(MID(W18,4,1))="L","LLP",IF(UPPER(MID(W18,4,1))="T","Trust",IF(UPPER(MID(W18,4,1))="A","AOP","")))))))),IF($B18="Challan","",IF(W18&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z18" s="28"/>
       <c r="AA18" s="29">
@@ -4192,10 +4192,10 @@
       <c r="V19" s="28"/>
       <c r="W19" s="28"/>
       <c r="X19" s="23">
-        <f>IF($B19&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W19)))=10,CODE(MID(TRIM(UPPER(W19)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W19)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W19)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W19)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B19="Entry",IF(AND(LEN(TRIM(UPPER(W19)))=10,CODE(MID(TRIM(UPPER(W19)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W19)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W19)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W19)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W19)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W19)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W19)),9,1))&lt;=57),"N","Y"),IF($B19="Challan","",IF(W19&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y19" s="23">
-        <f>IF($B19&lt;&gt;"Entry","",IF(LEN(W19)&lt;4,"",IF(UPPER(MID(W19,4,1))="P","Individual",IF(UPPER(MID(W19,4,1))="H","HUF",IF(UPPER(MID(W19,4,1))="C","Company",IF(UPPER(MID(W19,4,1))="F","Firm",IF(UPPER(MID(W19,4,1))="L","LLP",IF(UPPER(MID(W19,4,1))="T","Trust",IF(UPPER(MID(W19,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B19="Entry",IF(LEN(W19)&lt;4,"",IF(UPPER(MID(W19,4,1))="P","Individual",IF(UPPER(MID(W19,4,1))="H","HUF",IF(UPPER(MID(W19,4,1))="C","Company",IF(UPPER(MID(W19,4,1))="F","Firm",IF(UPPER(MID(W19,4,1))="L","LLP",IF(UPPER(MID(W19,4,1))="T","Trust",IF(UPPER(MID(W19,4,1))="A","AOP","")))))))),IF($B19="Challan","",IF(W19&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z19" s="28"/>
       <c r="AA19" s="29">
@@ -4270,10 +4270,10 @@
       <c r="V20" s="28"/>
       <c r="W20" s="28"/>
       <c r="X20" s="23">
-        <f>IF($B20&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W20)))=10,CODE(MID(TRIM(UPPER(W20)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W20)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W20)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W20)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B20="Entry",IF(AND(LEN(TRIM(UPPER(W20)))=10,CODE(MID(TRIM(UPPER(W20)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W20)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W20)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W20)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W20)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W20)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W20)),9,1))&lt;=57),"N","Y"),IF($B20="Challan","",IF(W20&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y20" s="23">
-        <f>IF($B20&lt;&gt;"Entry","",IF(LEN(W20)&lt;4,"",IF(UPPER(MID(W20,4,1))="P","Individual",IF(UPPER(MID(W20,4,1))="H","HUF",IF(UPPER(MID(W20,4,1))="C","Company",IF(UPPER(MID(W20,4,1))="F","Firm",IF(UPPER(MID(W20,4,1))="L","LLP",IF(UPPER(MID(W20,4,1))="T","Trust",IF(UPPER(MID(W20,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B20="Entry",IF(LEN(W20)&lt;4,"",IF(UPPER(MID(W20,4,1))="P","Individual",IF(UPPER(MID(W20,4,1))="H","HUF",IF(UPPER(MID(W20,4,1))="C","Company",IF(UPPER(MID(W20,4,1))="F","Firm",IF(UPPER(MID(W20,4,1))="L","LLP",IF(UPPER(MID(W20,4,1))="T","Trust",IF(UPPER(MID(W20,4,1))="A","AOP","")))))))),IF($B20="Challan","",IF(W20&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z20" s="28"/>
       <c r="AA20" s="29">
@@ -4348,10 +4348,10 @@
       <c r="V21" s="28"/>
       <c r="W21" s="28"/>
       <c r="X21" s="23">
-        <f>IF($B21&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W21)))=10,CODE(MID(TRIM(UPPER(W21)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W21)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W21)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W21)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B21="Entry",IF(AND(LEN(TRIM(UPPER(W21)))=10,CODE(MID(TRIM(UPPER(W21)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W21)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W21)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W21)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W21)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W21)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W21)),9,1))&lt;=57),"N","Y"),IF($B21="Challan","",IF(W21&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y21" s="23">
-        <f>IF($B21&lt;&gt;"Entry","",IF(LEN(W21)&lt;4,"",IF(UPPER(MID(W21,4,1))="P","Individual",IF(UPPER(MID(W21,4,1))="H","HUF",IF(UPPER(MID(W21,4,1))="C","Company",IF(UPPER(MID(W21,4,1))="F","Firm",IF(UPPER(MID(W21,4,1))="L","LLP",IF(UPPER(MID(W21,4,1))="T","Trust",IF(UPPER(MID(W21,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B21="Entry",IF(LEN(W21)&lt;4,"",IF(UPPER(MID(W21,4,1))="P","Individual",IF(UPPER(MID(W21,4,1))="H","HUF",IF(UPPER(MID(W21,4,1))="C","Company",IF(UPPER(MID(W21,4,1))="F","Firm",IF(UPPER(MID(W21,4,1))="L","LLP",IF(UPPER(MID(W21,4,1))="T","Trust",IF(UPPER(MID(W21,4,1))="A","AOP","")))))))),IF($B21="Challan","",IF(W21&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z21" s="28"/>
       <c r="AA21" s="29">
@@ -4426,10 +4426,10 @@
       <c r="V22" s="28"/>
       <c r="W22" s="28"/>
       <c r="X22" s="23">
-        <f>IF($B22&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W22)))=10,CODE(MID(TRIM(UPPER(W22)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W22)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W22)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W22)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B22="Entry",IF(AND(LEN(TRIM(UPPER(W22)))=10,CODE(MID(TRIM(UPPER(W22)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W22)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W22)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W22)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W22)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W22)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W22)),9,1))&lt;=57),"N","Y"),IF($B22="Challan","",IF(W22&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y22" s="23">
-        <f>IF($B22&lt;&gt;"Entry","",IF(LEN(W22)&lt;4,"",IF(UPPER(MID(W22,4,1))="P","Individual",IF(UPPER(MID(W22,4,1))="H","HUF",IF(UPPER(MID(W22,4,1))="C","Company",IF(UPPER(MID(W22,4,1))="F","Firm",IF(UPPER(MID(W22,4,1))="L","LLP",IF(UPPER(MID(W22,4,1))="T","Trust",IF(UPPER(MID(W22,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B22="Entry",IF(LEN(W22)&lt;4,"",IF(UPPER(MID(W22,4,1))="P","Individual",IF(UPPER(MID(W22,4,1))="H","HUF",IF(UPPER(MID(W22,4,1))="C","Company",IF(UPPER(MID(W22,4,1))="F","Firm",IF(UPPER(MID(W22,4,1))="L","LLP",IF(UPPER(MID(W22,4,1))="T","Trust",IF(UPPER(MID(W22,4,1))="A","AOP","")))))))),IF($B22="Challan","",IF(W22&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z22" s="28"/>
       <c r="AA22" s="29">
@@ -4504,10 +4504,10 @@
       <c r="V23" s="28"/>
       <c r="W23" s="28"/>
       <c r="X23" s="23">
-        <f>IF($B23&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W23)))=10,CODE(MID(TRIM(UPPER(W23)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W23)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W23)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W23)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B23="Entry",IF(AND(LEN(TRIM(UPPER(W23)))=10,CODE(MID(TRIM(UPPER(W23)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W23)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W23)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W23)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W23)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W23)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W23)),9,1))&lt;=57),"N","Y"),IF($B23="Challan","",IF(W23&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y23" s="23">
-        <f>IF($B23&lt;&gt;"Entry","",IF(LEN(W23)&lt;4,"",IF(UPPER(MID(W23,4,1))="P","Individual",IF(UPPER(MID(W23,4,1))="H","HUF",IF(UPPER(MID(W23,4,1))="C","Company",IF(UPPER(MID(W23,4,1))="F","Firm",IF(UPPER(MID(W23,4,1))="L","LLP",IF(UPPER(MID(W23,4,1))="T","Trust",IF(UPPER(MID(W23,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B23="Entry",IF(LEN(W23)&lt;4,"",IF(UPPER(MID(W23,4,1))="P","Individual",IF(UPPER(MID(W23,4,1))="H","HUF",IF(UPPER(MID(W23,4,1))="C","Company",IF(UPPER(MID(W23,4,1))="F","Firm",IF(UPPER(MID(W23,4,1))="L","LLP",IF(UPPER(MID(W23,4,1))="T","Trust",IF(UPPER(MID(W23,4,1))="A","AOP","")))))))),IF($B23="Challan","",IF(W23&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z23" s="28"/>
       <c r="AA23" s="29">
@@ -4582,10 +4582,10 @@
       <c r="V24" s="28"/>
       <c r="W24" s="28"/>
       <c r="X24" s="23">
-        <f>IF($B24&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W24)))=10,CODE(MID(TRIM(UPPER(W24)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W24)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W24)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W24)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B24="Entry",IF(AND(LEN(TRIM(UPPER(W24)))=10,CODE(MID(TRIM(UPPER(W24)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W24)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W24)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W24)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W24)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W24)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W24)),9,1))&lt;=57),"N","Y"),IF($B24="Challan","",IF(W24&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y24" s="23">
-        <f>IF($B24&lt;&gt;"Entry","",IF(LEN(W24)&lt;4,"",IF(UPPER(MID(W24,4,1))="P","Individual",IF(UPPER(MID(W24,4,1))="H","HUF",IF(UPPER(MID(W24,4,1))="C","Company",IF(UPPER(MID(W24,4,1))="F","Firm",IF(UPPER(MID(W24,4,1))="L","LLP",IF(UPPER(MID(W24,4,1))="T","Trust",IF(UPPER(MID(W24,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B24="Entry",IF(LEN(W24)&lt;4,"",IF(UPPER(MID(W24,4,1))="P","Individual",IF(UPPER(MID(W24,4,1))="H","HUF",IF(UPPER(MID(W24,4,1))="C","Company",IF(UPPER(MID(W24,4,1))="F","Firm",IF(UPPER(MID(W24,4,1))="L","LLP",IF(UPPER(MID(W24,4,1))="T","Trust",IF(UPPER(MID(W24,4,1))="A","AOP","")))))))),IF($B24="Challan","",IF(W24&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z24" s="28"/>
       <c r="AA24" s="29">
@@ -4660,10 +4660,10 @@
       <c r="V25" s="28"/>
       <c r="W25" s="28"/>
       <c r="X25" s="23">
-        <f>IF($B25&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W25)))=10,CODE(MID(TRIM(UPPER(W25)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W25)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W25)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W25)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B25="Entry",IF(AND(LEN(TRIM(UPPER(W25)))=10,CODE(MID(TRIM(UPPER(W25)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W25)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W25)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W25)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W25)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W25)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W25)),9,1))&lt;=57),"N","Y"),IF($B25="Challan","",IF(W25&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y25" s="23">
-        <f>IF($B25&lt;&gt;"Entry","",IF(LEN(W25)&lt;4,"",IF(UPPER(MID(W25,4,1))="P","Individual",IF(UPPER(MID(W25,4,1))="H","HUF",IF(UPPER(MID(W25,4,1))="C","Company",IF(UPPER(MID(W25,4,1))="F","Firm",IF(UPPER(MID(W25,4,1))="L","LLP",IF(UPPER(MID(W25,4,1))="T","Trust",IF(UPPER(MID(W25,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B25="Entry",IF(LEN(W25)&lt;4,"",IF(UPPER(MID(W25,4,1))="P","Individual",IF(UPPER(MID(W25,4,1))="H","HUF",IF(UPPER(MID(W25,4,1))="C","Company",IF(UPPER(MID(W25,4,1))="F","Firm",IF(UPPER(MID(W25,4,1))="L","LLP",IF(UPPER(MID(W25,4,1))="T","Trust",IF(UPPER(MID(W25,4,1))="A","AOP","")))))))),IF($B25="Challan","",IF(W25&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z25" s="28"/>
       <c r="AA25" s="29">
@@ -4738,10 +4738,10 @@
       <c r="V26" s="28"/>
       <c r="W26" s="28"/>
       <c r="X26" s="23">
-        <f>IF($B26&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W26)))=10,CODE(MID(TRIM(UPPER(W26)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W26)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W26)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W26)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B26="Entry",IF(AND(LEN(TRIM(UPPER(W26)))=10,CODE(MID(TRIM(UPPER(W26)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W26)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W26)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W26)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W26)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W26)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W26)),9,1))&lt;=57),"N","Y"),IF($B26="Challan","",IF(W26&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y26" s="23">
-        <f>IF($B26&lt;&gt;"Entry","",IF(LEN(W26)&lt;4,"",IF(UPPER(MID(W26,4,1))="P","Individual",IF(UPPER(MID(W26,4,1))="H","HUF",IF(UPPER(MID(W26,4,1))="C","Company",IF(UPPER(MID(W26,4,1))="F","Firm",IF(UPPER(MID(W26,4,1))="L","LLP",IF(UPPER(MID(W26,4,1))="T","Trust",IF(UPPER(MID(W26,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B26="Entry",IF(LEN(W26)&lt;4,"",IF(UPPER(MID(W26,4,1))="P","Individual",IF(UPPER(MID(W26,4,1))="H","HUF",IF(UPPER(MID(W26,4,1))="C","Company",IF(UPPER(MID(W26,4,1))="F","Firm",IF(UPPER(MID(W26,4,1))="L","LLP",IF(UPPER(MID(W26,4,1))="T","Trust",IF(UPPER(MID(W26,4,1))="A","AOP","")))))))),IF($B26="Challan","",IF(W26&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z26" s="28"/>
       <c r="AA26" s="29">
@@ -4816,10 +4816,10 @@
       <c r="V27" s="28"/>
       <c r="W27" s="28"/>
       <c r="X27" s="23">
-        <f>IF($B27&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W27)))=10,CODE(MID(TRIM(UPPER(W27)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W27)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W27)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W27)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B27="Entry",IF(AND(LEN(TRIM(UPPER(W27)))=10,CODE(MID(TRIM(UPPER(W27)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W27)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W27)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W27)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W27)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W27)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W27)),9,1))&lt;=57),"N","Y"),IF($B27="Challan","",IF(W27&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y27" s="23">
-        <f>IF($B27&lt;&gt;"Entry","",IF(LEN(W27)&lt;4,"",IF(UPPER(MID(W27,4,1))="P","Individual",IF(UPPER(MID(W27,4,1))="H","HUF",IF(UPPER(MID(W27,4,1))="C","Company",IF(UPPER(MID(W27,4,1))="F","Firm",IF(UPPER(MID(W27,4,1))="L","LLP",IF(UPPER(MID(W27,4,1))="T","Trust",IF(UPPER(MID(W27,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B27="Entry",IF(LEN(W27)&lt;4,"",IF(UPPER(MID(W27,4,1))="P","Individual",IF(UPPER(MID(W27,4,1))="H","HUF",IF(UPPER(MID(W27,4,1))="C","Company",IF(UPPER(MID(W27,4,1))="F","Firm",IF(UPPER(MID(W27,4,1))="L","LLP",IF(UPPER(MID(W27,4,1))="T","Trust",IF(UPPER(MID(W27,4,1))="A","AOP","")))))))),IF($B27="Challan","",IF(W27&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z27" s="28"/>
       <c r="AA27" s="29">
@@ -4894,10 +4894,10 @@
       <c r="V28" s="28"/>
       <c r="W28" s="28"/>
       <c r="X28" s="23">
-        <f>IF($B28&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W28)))=10,CODE(MID(TRIM(UPPER(W28)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W28)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W28)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W28)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B28="Entry",IF(AND(LEN(TRIM(UPPER(W28)))=10,CODE(MID(TRIM(UPPER(W28)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W28)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W28)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W28)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W28)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W28)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W28)),9,1))&lt;=57),"N","Y"),IF($B28="Challan","",IF(W28&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y28" s="23">
-        <f>IF($B28&lt;&gt;"Entry","",IF(LEN(W28)&lt;4,"",IF(UPPER(MID(W28,4,1))="P","Individual",IF(UPPER(MID(W28,4,1))="H","HUF",IF(UPPER(MID(W28,4,1))="C","Company",IF(UPPER(MID(W28,4,1))="F","Firm",IF(UPPER(MID(W28,4,1))="L","LLP",IF(UPPER(MID(W28,4,1))="T","Trust",IF(UPPER(MID(W28,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B28="Entry",IF(LEN(W28)&lt;4,"",IF(UPPER(MID(W28,4,1))="P","Individual",IF(UPPER(MID(W28,4,1))="H","HUF",IF(UPPER(MID(W28,4,1))="C","Company",IF(UPPER(MID(W28,4,1))="F","Firm",IF(UPPER(MID(W28,4,1))="L","LLP",IF(UPPER(MID(W28,4,1))="T","Trust",IF(UPPER(MID(W28,4,1))="A","AOP","")))))))),IF($B28="Challan","",IF(W28&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z28" s="28"/>
       <c r="AA28" s="29">
@@ -4972,10 +4972,10 @@
       <c r="V29" s="28"/>
       <c r="W29" s="28"/>
       <c r="X29" s="23">
-        <f>IF($B29&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W29)))=10,CODE(MID(TRIM(UPPER(W29)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W29)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W29)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W29)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B29="Entry",IF(AND(LEN(TRIM(UPPER(W29)))=10,CODE(MID(TRIM(UPPER(W29)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W29)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W29)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W29)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W29)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W29)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W29)),9,1))&lt;=57),"N","Y"),IF($B29="Challan","",IF(W29&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y29" s="23">
-        <f>IF($B29&lt;&gt;"Entry","",IF(LEN(W29)&lt;4,"",IF(UPPER(MID(W29,4,1))="P","Individual",IF(UPPER(MID(W29,4,1))="H","HUF",IF(UPPER(MID(W29,4,1))="C","Company",IF(UPPER(MID(W29,4,1))="F","Firm",IF(UPPER(MID(W29,4,1))="L","LLP",IF(UPPER(MID(W29,4,1))="T","Trust",IF(UPPER(MID(W29,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B29="Entry",IF(LEN(W29)&lt;4,"",IF(UPPER(MID(W29,4,1))="P","Individual",IF(UPPER(MID(W29,4,1))="H","HUF",IF(UPPER(MID(W29,4,1))="C","Company",IF(UPPER(MID(W29,4,1))="F","Firm",IF(UPPER(MID(W29,4,1))="L","LLP",IF(UPPER(MID(W29,4,1))="T","Trust",IF(UPPER(MID(W29,4,1))="A","AOP","")))))))),IF($B29="Challan","",IF(W29&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z29" s="28"/>
       <c r="AA29" s="29">
@@ -5050,10 +5050,10 @@
       <c r="V30" s="28"/>
       <c r="W30" s="28"/>
       <c r="X30" s="23">
-        <f>IF($B30&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W30)))=10,CODE(MID(TRIM(UPPER(W30)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W30)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W30)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W30)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B30="Entry",IF(AND(LEN(TRIM(UPPER(W30)))=10,CODE(MID(TRIM(UPPER(W30)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W30)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W30)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W30)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W30)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W30)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W30)),9,1))&lt;=57),"N","Y"),IF($B30="Challan","",IF(W30&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y30" s="23">
-        <f>IF($B30&lt;&gt;"Entry","",IF(LEN(W30)&lt;4,"",IF(UPPER(MID(W30,4,1))="P","Individual",IF(UPPER(MID(W30,4,1))="H","HUF",IF(UPPER(MID(W30,4,1))="C","Company",IF(UPPER(MID(W30,4,1))="F","Firm",IF(UPPER(MID(W30,4,1))="L","LLP",IF(UPPER(MID(W30,4,1))="T","Trust",IF(UPPER(MID(W30,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B30="Entry",IF(LEN(W30)&lt;4,"",IF(UPPER(MID(W30,4,1))="P","Individual",IF(UPPER(MID(W30,4,1))="H","HUF",IF(UPPER(MID(W30,4,1))="C","Company",IF(UPPER(MID(W30,4,1))="F","Firm",IF(UPPER(MID(W30,4,1))="L","LLP",IF(UPPER(MID(W30,4,1))="T","Trust",IF(UPPER(MID(W30,4,1))="A","AOP","")))))))),IF($B30="Challan","",IF(W30&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z30" s="28"/>
       <c r="AA30" s="29">
@@ -5128,10 +5128,10 @@
       <c r="V31" s="28"/>
       <c r="W31" s="28"/>
       <c r="X31" s="23">
-        <f>IF($B31&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W31)))=10,CODE(MID(TRIM(UPPER(W31)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W31)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W31)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W31)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B31="Entry",IF(AND(LEN(TRIM(UPPER(W31)))=10,CODE(MID(TRIM(UPPER(W31)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W31)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W31)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W31)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W31)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W31)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W31)),9,1))&lt;=57),"N","Y"),IF($B31="Challan","",IF(W31&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y31" s="23">
-        <f>IF($B31&lt;&gt;"Entry","",IF(LEN(W31)&lt;4,"",IF(UPPER(MID(W31,4,1))="P","Individual",IF(UPPER(MID(W31,4,1))="H","HUF",IF(UPPER(MID(W31,4,1))="C","Company",IF(UPPER(MID(W31,4,1))="F","Firm",IF(UPPER(MID(W31,4,1))="L","LLP",IF(UPPER(MID(W31,4,1))="T","Trust",IF(UPPER(MID(W31,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B31="Entry",IF(LEN(W31)&lt;4,"",IF(UPPER(MID(W31,4,1))="P","Individual",IF(UPPER(MID(W31,4,1))="H","HUF",IF(UPPER(MID(W31,4,1))="C","Company",IF(UPPER(MID(W31,4,1))="F","Firm",IF(UPPER(MID(W31,4,1))="L","LLP",IF(UPPER(MID(W31,4,1))="T","Trust",IF(UPPER(MID(W31,4,1))="A","AOP","")))))))),IF($B31="Challan","",IF(W31&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z31" s="28"/>
       <c r="AA31" s="29">
@@ -5206,10 +5206,10 @@
       <c r="V32" s="28"/>
       <c r="W32" s="28"/>
       <c r="X32" s="23">
-        <f>IF($B32&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W32)))=10,CODE(MID(TRIM(UPPER(W32)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W32)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W32)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W32)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B32="Entry",IF(AND(LEN(TRIM(UPPER(W32)))=10,CODE(MID(TRIM(UPPER(W32)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W32)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W32)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W32)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W32)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W32)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W32)),9,1))&lt;=57),"N","Y"),IF($B32="Challan","",IF(W32&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y32" s="23">
-        <f>IF($B32&lt;&gt;"Entry","",IF(LEN(W32)&lt;4,"",IF(UPPER(MID(W32,4,1))="P","Individual",IF(UPPER(MID(W32,4,1))="H","HUF",IF(UPPER(MID(W32,4,1))="C","Company",IF(UPPER(MID(W32,4,1))="F","Firm",IF(UPPER(MID(W32,4,1))="L","LLP",IF(UPPER(MID(W32,4,1))="T","Trust",IF(UPPER(MID(W32,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B32="Entry",IF(LEN(W32)&lt;4,"",IF(UPPER(MID(W32,4,1))="P","Individual",IF(UPPER(MID(W32,4,1))="H","HUF",IF(UPPER(MID(W32,4,1))="C","Company",IF(UPPER(MID(W32,4,1))="F","Firm",IF(UPPER(MID(W32,4,1))="L","LLP",IF(UPPER(MID(W32,4,1))="T","Trust",IF(UPPER(MID(W32,4,1))="A","AOP","")))))))),IF($B32="Challan","",IF(W32&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z32" s="28"/>
       <c r="AA32" s="29">
@@ -5284,10 +5284,10 @@
       <c r="V33" s="28"/>
       <c r="W33" s="28"/>
       <c r="X33" s="23">
-        <f>IF($B33&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W33)))=10,CODE(MID(TRIM(UPPER(W33)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W33)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W33)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W33)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B33="Entry",IF(AND(LEN(TRIM(UPPER(W33)))=10,CODE(MID(TRIM(UPPER(W33)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W33)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W33)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W33)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W33)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W33)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W33)),9,1))&lt;=57),"N","Y"),IF($B33="Challan","",IF(W33&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y33" s="23">
-        <f>IF($B33&lt;&gt;"Entry","",IF(LEN(W33)&lt;4,"",IF(UPPER(MID(W33,4,1))="P","Individual",IF(UPPER(MID(W33,4,1))="H","HUF",IF(UPPER(MID(W33,4,1))="C","Company",IF(UPPER(MID(W33,4,1))="F","Firm",IF(UPPER(MID(W33,4,1))="L","LLP",IF(UPPER(MID(W33,4,1))="T","Trust",IF(UPPER(MID(W33,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B33="Entry",IF(LEN(W33)&lt;4,"",IF(UPPER(MID(W33,4,1))="P","Individual",IF(UPPER(MID(W33,4,1))="H","HUF",IF(UPPER(MID(W33,4,1))="C","Company",IF(UPPER(MID(W33,4,1))="F","Firm",IF(UPPER(MID(W33,4,1))="L","LLP",IF(UPPER(MID(W33,4,1))="T","Trust",IF(UPPER(MID(W33,4,1))="A","AOP","")))))))),IF($B33="Challan","",IF(W33&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z33" s="28"/>
       <c r="AA33" s="29">
@@ -5362,10 +5362,10 @@
       <c r="V34" s="28"/>
       <c r="W34" s="28"/>
       <c r="X34" s="23">
-        <f>IF($B34&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W34)))=10,CODE(MID(TRIM(UPPER(W34)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W34)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W34)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W34)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B34="Entry",IF(AND(LEN(TRIM(UPPER(W34)))=10,CODE(MID(TRIM(UPPER(W34)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W34)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W34)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W34)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W34)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W34)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W34)),9,1))&lt;=57),"N","Y"),IF($B34="Challan","",IF(W34&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y34" s="23">
-        <f>IF($B34&lt;&gt;"Entry","",IF(LEN(W34)&lt;4,"",IF(UPPER(MID(W34,4,1))="P","Individual",IF(UPPER(MID(W34,4,1))="H","HUF",IF(UPPER(MID(W34,4,1))="C","Company",IF(UPPER(MID(W34,4,1))="F","Firm",IF(UPPER(MID(W34,4,1))="L","LLP",IF(UPPER(MID(W34,4,1))="T","Trust",IF(UPPER(MID(W34,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B34="Entry",IF(LEN(W34)&lt;4,"",IF(UPPER(MID(W34,4,1))="P","Individual",IF(UPPER(MID(W34,4,1))="H","HUF",IF(UPPER(MID(W34,4,1))="C","Company",IF(UPPER(MID(W34,4,1))="F","Firm",IF(UPPER(MID(W34,4,1))="L","LLP",IF(UPPER(MID(W34,4,1))="T","Trust",IF(UPPER(MID(W34,4,1))="A","AOP","")))))))),IF($B34="Challan","",IF(W34&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z34" s="28"/>
       <c r="AA34" s="29">
@@ -5440,10 +5440,10 @@
       <c r="V35" s="28"/>
       <c r="W35" s="28"/>
       <c r="X35" s="23">
-        <f>IF($B35&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W35)))=10,CODE(MID(TRIM(UPPER(W35)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W35)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W35)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W35)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B35="Entry",IF(AND(LEN(TRIM(UPPER(W35)))=10,CODE(MID(TRIM(UPPER(W35)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W35)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W35)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W35)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W35)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W35)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W35)),9,1))&lt;=57),"N","Y"),IF($B35="Challan","",IF(W35&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y35" s="23">
-        <f>IF($B35&lt;&gt;"Entry","",IF(LEN(W35)&lt;4,"",IF(UPPER(MID(W35,4,1))="P","Individual",IF(UPPER(MID(W35,4,1))="H","HUF",IF(UPPER(MID(W35,4,1))="C","Company",IF(UPPER(MID(W35,4,1))="F","Firm",IF(UPPER(MID(W35,4,1))="L","LLP",IF(UPPER(MID(W35,4,1))="T","Trust",IF(UPPER(MID(W35,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B35="Entry",IF(LEN(W35)&lt;4,"",IF(UPPER(MID(W35,4,1))="P","Individual",IF(UPPER(MID(W35,4,1))="H","HUF",IF(UPPER(MID(W35,4,1))="C","Company",IF(UPPER(MID(W35,4,1))="F","Firm",IF(UPPER(MID(W35,4,1))="L","LLP",IF(UPPER(MID(W35,4,1))="T","Trust",IF(UPPER(MID(W35,4,1))="A","AOP","")))))))),IF($B35="Challan","",IF(W35&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z35" s="28"/>
       <c r="AA35" s="29">
@@ -5518,10 +5518,10 @@
       <c r="V36" s="28"/>
       <c r="W36" s="28"/>
       <c r="X36" s="23">
-        <f>IF($B36&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W36)))=10,CODE(MID(TRIM(UPPER(W36)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W36)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W36)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W36)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B36="Entry",IF(AND(LEN(TRIM(UPPER(W36)))=10,CODE(MID(TRIM(UPPER(W36)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W36)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W36)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W36)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W36)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W36)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W36)),9,1))&lt;=57),"N","Y"),IF($B36="Challan","",IF(W36&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y36" s="23">
-        <f>IF($B36&lt;&gt;"Entry","",IF(LEN(W36)&lt;4,"",IF(UPPER(MID(W36,4,1))="P","Individual",IF(UPPER(MID(W36,4,1))="H","HUF",IF(UPPER(MID(W36,4,1))="C","Company",IF(UPPER(MID(W36,4,1))="F","Firm",IF(UPPER(MID(W36,4,1))="L","LLP",IF(UPPER(MID(W36,4,1))="T","Trust",IF(UPPER(MID(W36,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B36="Entry",IF(LEN(W36)&lt;4,"",IF(UPPER(MID(W36,4,1))="P","Individual",IF(UPPER(MID(W36,4,1))="H","HUF",IF(UPPER(MID(W36,4,1))="C","Company",IF(UPPER(MID(W36,4,1))="F","Firm",IF(UPPER(MID(W36,4,1))="L","LLP",IF(UPPER(MID(W36,4,1))="T","Trust",IF(UPPER(MID(W36,4,1))="A","AOP","")))))))),IF($B36="Challan","",IF(W36&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z36" s="28"/>
       <c r="AA36" s="29">
@@ -5596,10 +5596,10 @@
       <c r="V37" s="28"/>
       <c r="W37" s="28"/>
       <c r="X37" s="23">
-        <f>IF($B37&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W37)))=10,CODE(MID(TRIM(UPPER(W37)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W37)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W37)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W37)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B37="Entry",IF(AND(LEN(TRIM(UPPER(W37)))=10,CODE(MID(TRIM(UPPER(W37)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W37)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W37)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W37)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W37)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W37)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W37)),9,1))&lt;=57),"N","Y"),IF($B37="Challan","",IF(W37&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y37" s="23">
-        <f>IF($B37&lt;&gt;"Entry","",IF(LEN(W37)&lt;4,"",IF(UPPER(MID(W37,4,1))="P","Individual",IF(UPPER(MID(W37,4,1))="H","HUF",IF(UPPER(MID(W37,4,1))="C","Company",IF(UPPER(MID(W37,4,1))="F","Firm",IF(UPPER(MID(W37,4,1))="L","LLP",IF(UPPER(MID(W37,4,1))="T","Trust",IF(UPPER(MID(W37,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B37="Entry",IF(LEN(W37)&lt;4,"",IF(UPPER(MID(W37,4,1))="P","Individual",IF(UPPER(MID(W37,4,1))="H","HUF",IF(UPPER(MID(W37,4,1))="C","Company",IF(UPPER(MID(W37,4,1))="F","Firm",IF(UPPER(MID(W37,4,1))="L","LLP",IF(UPPER(MID(W37,4,1))="T","Trust",IF(UPPER(MID(W37,4,1))="A","AOP","")))))))),IF($B37="Challan","",IF(W37&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z37" s="28"/>
       <c r="AA37" s="29">
@@ -5674,10 +5674,10 @@
       <c r="V38" s="28"/>
       <c r="W38" s="28"/>
       <c r="X38" s="23">
-        <f>IF($B38&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W38)))=10,CODE(MID(TRIM(UPPER(W38)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W38)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W38)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W38)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B38="Entry",IF(AND(LEN(TRIM(UPPER(W38)))=10,CODE(MID(TRIM(UPPER(W38)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W38)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W38)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W38)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W38)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W38)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W38)),9,1))&lt;=57),"N","Y"),IF($B38="Challan","",IF(W38&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y38" s="23">
-        <f>IF($B38&lt;&gt;"Entry","",IF(LEN(W38)&lt;4,"",IF(UPPER(MID(W38,4,1))="P","Individual",IF(UPPER(MID(W38,4,1))="H","HUF",IF(UPPER(MID(W38,4,1))="C","Company",IF(UPPER(MID(W38,4,1))="F","Firm",IF(UPPER(MID(W38,4,1))="L","LLP",IF(UPPER(MID(W38,4,1))="T","Trust",IF(UPPER(MID(W38,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B38="Entry",IF(LEN(W38)&lt;4,"",IF(UPPER(MID(W38,4,1))="P","Individual",IF(UPPER(MID(W38,4,1))="H","HUF",IF(UPPER(MID(W38,4,1))="C","Company",IF(UPPER(MID(W38,4,1))="F","Firm",IF(UPPER(MID(W38,4,1))="L","LLP",IF(UPPER(MID(W38,4,1))="T","Trust",IF(UPPER(MID(W38,4,1))="A","AOP","")))))))),IF($B38="Challan","",IF(W38&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z38" s="28"/>
       <c r="AA38" s="29">
@@ -5752,10 +5752,10 @@
       <c r="V39" s="28"/>
       <c r="W39" s="28"/>
       <c r="X39" s="23">
-        <f>IF($B39&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W39)))=10,CODE(MID(TRIM(UPPER(W39)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W39)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W39)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W39)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B39="Entry",IF(AND(LEN(TRIM(UPPER(W39)))=10,CODE(MID(TRIM(UPPER(W39)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W39)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W39)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W39)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W39)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W39)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W39)),9,1))&lt;=57),"N","Y"),IF($B39="Challan","",IF(W39&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y39" s="23">
-        <f>IF($B39&lt;&gt;"Entry","",IF(LEN(W39)&lt;4,"",IF(UPPER(MID(W39,4,1))="P","Individual",IF(UPPER(MID(W39,4,1))="H","HUF",IF(UPPER(MID(W39,4,1))="C","Company",IF(UPPER(MID(W39,4,1))="F","Firm",IF(UPPER(MID(W39,4,1))="L","LLP",IF(UPPER(MID(W39,4,1))="T","Trust",IF(UPPER(MID(W39,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B39="Entry",IF(LEN(W39)&lt;4,"",IF(UPPER(MID(W39,4,1))="P","Individual",IF(UPPER(MID(W39,4,1))="H","HUF",IF(UPPER(MID(W39,4,1))="C","Company",IF(UPPER(MID(W39,4,1))="F","Firm",IF(UPPER(MID(W39,4,1))="L","LLP",IF(UPPER(MID(W39,4,1))="T","Trust",IF(UPPER(MID(W39,4,1))="A","AOP","")))))))),IF($B39="Challan","",IF(W39&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z39" s="28"/>
       <c r="AA39" s="29">
@@ -5830,10 +5830,10 @@
       <c r="V40" s="28"/>
       <c r="W40" s="28"/>
       <c r="X40" s="23">
-        <f>IF($B40&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W40)))=10,CODE(MID(TRIM(UPPER(W40)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W40)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W40)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W40)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B40="Entry",IF(AND(LEN(TRIM(UPPER(W40)))=10,CODE(MID(TRIM(UPPER(W40)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W40)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W40)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W40)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W40)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W40)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W40)),9,1))&lt;=57),"N","Y"),IF($B40="Challan","",IF(W40&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y40" s="23">
-        <f>IF($B40&lt;&gt;"Entry","",IF(LEN(W40)&lt;4,"",IF(UPPER(MID(W40,4,1))="P","Individual",IF(UPPER(MID(W40,4,1))="H","HUF",IF(UPPER(MID(W40,4,1))="C","Company",IF(UPPER(MID(W40,4,1))="F","Firm",IF(UPPER(MID(W40,4,1))="L","LLP",IF(UPPER(MID(W40,4,1))="T","Trust",IF(UPPER(MID(W40,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B40="Entry",IF(LEN(W40)&lt;4,"",IF(UPPER(MID(W40,4,1))="P","Individual",IF(UPPER(MID(W40,4,1))="H","HUF",IF(UPPER(MID(W40,4,1))="C","Company",IF(UPPER(MID(W40,4,1))="F","Firm",IF(UPPER(MID(W40,4,1))="L","LLP",IF(UPPER(MID(W40,4,1))="T","Trust",IF(UPPER(MID(W40,4,1))="A","AOP","")))))))),IF($B40="Challan","",IF(W40&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z40" s="28"/>
       <c r="AA40" s="29">
@@ -5908,10 +5908,10 @@
       <c r="V41" s="28"/>
       <c r="W41" s="28"/>
       <c r="X41" s="23">
-        <f>IF($B41&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W41)))=10,CODE(MID(TRIM(UPPER(W41)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W41)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W41)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W41)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B41="Entry",IF(AND(LEN(TRIM(UPPER(W41)))=10,CODE(MID(TRIM(UPPER(W41)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W41)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W41)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W41)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W41)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W41)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W41)),9,1))&lt;=57),"N","Y"),IF($B41="Challan","",IF(W41&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y41" s="23">
-        <f>IF($B41&lt;&gt;"Entry","",IF(LEN(W41)&lt;4,"",IF(UPPER(MID(W41,4,1))="P","Individual",IF(UPPER(MID(W41,4,1))="H","HUF",IF(UPPER(MID(W41,4,1))="C","Company",IF(UPPER(MID(W41,4,1))="F","Firm",IF(UPPER(MID(W41,4,1))="L","LLP",IF(UPPER(MID(W41,4,1))="T","Trust",IF(UPPER(MID(W41,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B41="Entry",IF(LEN(W41)&lt;4,"",IF(UPPER(MID(W41,4,1))="P","Individual",IF(UPPER(MID(W41,4,1))="H","HUF",IF(UPPER(MID(W41,4,1))="C","Company",IF(UPPER(MID(W41,4,1))="F","Firm",IF(UPPER(MID(W41,4,1))="L","LLP",IF(UPPER(MID(W41,4,1))="T","Trust",IF(UPPER(MID(W41,4,1))="A","AOP","")))))))),IF($B41="Challan","",IF(W41&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z41" s="28"/>
       <c r="AA41" s="29">
@@ -5986,10 +5986,10 @@
       <c r="V42" s="28"/>
       <c r="W42" s="28"/>
       <c r="X42" s="23">
-        <f>IF($B42&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W42)))=10,CODE(MID(TRIM(UPPER(W42)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W42)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W42)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W42)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B42="Entry",IF(AND(LEN(TRIM(UPPER(W42)))=10,CODE(MID(TRIM(UPPER(W42)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W42)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W42)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W42)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W42)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W42)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W42)),9,1))&lt;=57),"N","Y"),IF($B42="Challan","",IF(W42&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y42" s="23">
-        <f>IF($B42&lt;&gt;"Entry","",IF(LEN(W42)&lt;4,"",IF(UPPER(MID(W42,4,1))="P","Individual",IF(UPPER(MID(W42,4,1))="H","HUF",IF(UPPER(MID(W42,4,1))="C","Company",IF(UPPER(MID(W42,4,1))="F","Firm",IF(UPPER(MID(W42,4,1))="L","LLP",IF(UPPER(MID(W42,4,1))="T","Trust",IF(UPPER(MID(W42,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B42="Entry",IF(LEN(W42)&lt;4,"",IF(UPPER(MID(W42,4,1))="P","Individual",IF(UPPER(MID(W42,4,1))="H","HUF",IF(UPPER(MID(W42,4,1))="C","Company",IF(UPPER(MID(W42,4,1))="F","Firm",IF(UPPER(MID(W42,4,1))="L","LLP",IF(UPPER(MID(W42,4,1))="T","Trust",IF(UPPER(MID(W42,4,1))="A","AOP","")))))))),IF($B42="Challan","",IF(W42&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z42" s="28"/>
       <c r="AA42" s="29">
@@ -6064,10 +6064,10 @@
       <c r="V43" s="28"/>
       <c r="W43" s="28"/>
       <c r="X43" s="23">
-        <f>IF($B43&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W43)))=10,CODE(MID(TRIM(UPPER(W43)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W43)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W43)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W43)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B43="Entry",IF(AND(LEN(TRIM(UPPER(W43)))=10,CODE(MID(TRIM(UPPER(W43)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W43)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W43)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W43)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W43)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W43)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W43)),9,1))&lt;=57),"N","Y"),IF($B43="Challan","",IF(W43&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y43" s="23">
-        <f>IF($B43&lt;&gt;"Entry","",IF(LEN(W43)&lt;4,"",IF(UPPER(MID(W43,4,1))="P","Individual",IF(UPPER(MID(W43,4,1))="H","HUF",IF(UPPER(MID(W43,4,1))="C","Company",IF(UPPER(MID(W43,4,1))="F","Firm",IF(UPPER(MID(W43,4,1))="L","LLP",IF(UPPER(MID(W43,4,1))="T","Trust",IF(UPPER(MID(W43,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B43="Entry",IF(LEN(W43)&lt;4,"",IF(UPPER(MID(W43,4,1))="P","Individual",IF(UPPER(MID(W43,4,1))="H","HUF",IF(UPPER(MID(W43,4,1))="C","Company",IF(UPPER(MID(W43,4,1))="F","Firm",IF(UPPER(MID(W43,4,1))="L","LLP",IF(UPPER(MID(W43,4,1))="T","Trust",IF(UPPER(MID(W43,4,1))="A","AOP","")))))))),IF($B43="Challan","",IF(W43&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z43" s="28"/>
       <c r="AA43" s="29">
@@ -6142,10 +6142,10 @@
       <c r="V44" s="28"/>
       <c r="W44" s="28"/>
       <c r="X44" s="23">
-        <f>IF($B44&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W44)))=10,CODE(MID(TRIM(UPPER(W44)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W44)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W44)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W44)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B44="Entry",IF(AND(LEN(TRIM(UPPER(W44)))=10,CODE(MID(TRIM(UPPER(W44)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W44)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W44)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W44)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W44)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W44)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W44)),9,1))&lt;=57),"N","Y"),IF($B44="Challan","",IF(W44&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y44" s="23">
-        <f>IF($B44&lt;&gt;"Entry","",IF(LEN(W44)&lt;4,"",IF(UPPER(MID(W44,4,1))="P","Individual",IF(UPPER(MID(W44,4,1))="H","HUF",IF(UPPER(MID(W44,4,1))="C","Company",IF(UPPER(MID(W44,4,1))="F","Firm",IF(UPPER(MID(W44,4,1))="L","LLP",IF(UPPER(MID(W44,4,1))="T","Trust",IF(UPPER(MID(W44,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B44="Entry",IF(LEN(W44)&lt;4,"",IF(UPPER(MID(W44,4,1))="P","Individual",IF(UPPER(MID(W44,4,1))="H","HUF",IF(UPPER(MID(W44,4,1))="C","Company",IF(UPPER(MID(W44,4,1))="F","Firm",IF(UPPER(MID(W44,4,1))="L","LLP",IF(UPPER(MID(W44,4,1))="T","Trust",IF(UPPER(MID(W44,4,1))="A","AOP","")))))))),IF($B44="Challan","",IF(W44&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z44" s="28"/>
       <c r="AA44" s="29">
@@ -6220,10 +6220,10 @@
       <c r="V45" s="28"/>
       <c r="W45" s="28"/>
       <c r="X45" s="23">
-        <f>IF($B45&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W45)))=10,CODE(MID(TRIM(UPPER(W45)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W45)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W45)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W45)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B45="Entry",IF(AND(LEN(TRIM(UPPER(W45)))=10,CODE(MID(TRIM(UPPER(W45)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W45)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W45)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W45)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W45)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W45)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W45)),9,1))&lt;=57),"N","Y"),IF($B45="Challan","",IF(W45&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y45" s="23">
-        <f>IF($B45&lt;&gt;"Entry","",IF(LEN(W45)&lt;4,"",IF(UPPER(MID(W45,4,1))="P","Individual",IF(UPPER(MID(W45,4,1))="H","HUF",IF(UPPER(MID(W45,4,1))="C","Company",IF(UPPER(MID(W45,4,1))="F","Firm",IF(UPPER(MID(W45,4,1))="L","LLP",IF(UPPER(MID(W45,4,1))="T","Trust",IF(UPPER(MID(W45,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B45="Entry",IF(LEN(W45)&lt;4,"",IF(UPPER(MID(W45,4,1))="P","Individual",IF(UPPER(MID(W45,4,1))="H","HUF",IF(UPPER(MID(W45,4,1))="C","Company",IF(UPPER(MID(W45,4,1))="F","Firm",IF(UPPER(MID(W45,4,1))="L","LLP",IF(UPPER(MID(W45,4,1))="T","Trust",IF(UPPER(MID(W45,4,1))="A","AOP","")))))))),IF($B45="Challan","",IF(W45&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z45" s="28"/>
       <c r="AA45" s="29">
@@ -6298,10 +6298,10 @@
       <c r="V46" s="28"/>
       <c r="W46" s="28"/>
       <c r="X46" s="23">
-        <f>IF($B46&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W46)))=10,CODE(MID(TRIM(UPPER(W46)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W46)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W46)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W46)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B46="Entry",IF(AND(LEN(TRIM(UPPER(W46)))=10,CODE(MID(TRIM(UPPER(W46)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W46)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W46)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W46)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W46)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W46)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W46)),9,1))&lt;=57),"N","Y"),IF($B46="Challan","",IF(W46&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y46" s="23">
-        <f>IF($B46&lt;&gt;"Entry","",IF(LEN(W46)&lt;4,"",IF(UPPER(MID(W46,4,1))="P","Individual",IF(UPPER(MID(W46,4,1))="H","HUF",IF(UPPER(MID(W46,4,1))="C","Company",IF(UPPER(MID(W46,4,1))="F","Firm",IF(UPPER(MID(W46,4,1))="L","LLP",IF(UPPER(MID(W46,4,1))="T","Trust",IF(UPPER(MID(W46,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B46="Entry",IF(LEN(W46)&lt;4,"",IF(UPPER(MID(W46,4,1))="P","Individual",IF(UPPER(MID(W46,4,1))="H","HUF",IF(UPPER(MID(W46,4,1))="C","Company",IF(UPPER(MID(W46,4,1))="F","Firm",IF(UPPER(MID(W46,4,1))="L","LLP",IF(UPPER(MID(W46,4,1))="T","Trust",IF(UPPER(MID(W46,4,1))="A","AOP","")))))))),IF($B46="Challan","",IF(W46&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z46" s="28"/>
       <c r="AA46" s="29">
@@ -6376,10 +6376,10 @@
       <c r="V47" s="28"/>
       <c r="W47" s="28"/>
       <c r="X47" s="23">
-        <f>IF($B47&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W47)))=10,CODE(MID(TRIM(UPPER(W47)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W47)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W47)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W47)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B47="Entry",IF(AND(LEN(TRIM(UPPER(W47)))=10,CODE(MID(TRIM(UPPER(W47)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W47)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W47)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W47)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W47)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W47)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W47)),9,1))&lt;=57),"N","Y"),IF($B47="Challan","",IF(W47&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y47" s="23">
-        <f>IF($B47&lt;&gt;"Entry","",IF(LEN(W47)&lt;4,"",IF(UPPER(MID(W47,4,1))="P","Individual",IF(UPPER(MID(W47,4,1))="H","HUF",IF(UPPER(MID(W47,4,1))="C","Company",IF(UPPER(MID(W47,4,1))="F","Firm",IF(UPPER(MID(W47,4,1))="L","LLP",IF(UPPER(MID(W47,4,1))="T","Trust",IF(UPPER(MID(W47,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B47="Entry",IF(LEN(W47)&lt;4,"",IF(UPPER(MID(W47,4,1))="P","Individual",IF(UPPER(MID(W47,4,1))="H","HUF",IF(UPPER(MID(W47,4,1))="C","Company",IF(UPPER(MID(W47,4,1))="F","Firm",IF(UPPER(MID(W47,4,1))="L","LLP",IF(UPPER(MID(W47,4,1))="T","Trust",IF(UPPER(MID(W47,4,1))="A","AOP","")))))))),IF($B47="Challan","",IF(W47&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z47" s="28"/>
       <c r="AA47" s="29">
@@ -6454,10 +6454,10 @@
       <c r="V48" s="28"/>
       <c r="W48" s="28"/>
       <c r="X48" s="23">
-        <f>IF($B48&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W48)))=10,CODE(MID(TRIM(UPPER(W48)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W48)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W48)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W48)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B48="Entry",IF(AND(LEN(TRIM(UPPER(W48)))=10,CODE(MID(TRIM(UPPER(W48)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W48)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W48)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W48)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W48)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W48)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W48)),9,1))&lt;=57),"N","Y"),IF($B48="Challan","",IF(W48&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y48" s="23">
-        <f>IF($B48&lt;&gt;"Entry","",IF(LEN(W48)&lt;4,"",IF(UPPER(MID(W48,4,1))="P","Individual",IF(UPPER(MID(W48,4,1))="H","HUF",IF(UPPER(MID(W48,4,1))="C","Company",IF(UPPER(MID(W48,4,1))="F","Firm",IF(UPPER(MID(W48,4,1))="L","LLP",IF(UPPER(MID(W48,4,1))="T","Trust",IF(UPPER(MID(W48,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B48="Entry",IF(LEN(W48)&lt;4,"",IF(UPPER(MID(W48,4,1))="P","Individual",IF(UPPER(MID(W48,4,1))="H","HUF",IF(UPPER(MID(W48,4,1))="C","Company",IF(UPPER(MID(W48,4,1))="F","Firm",IF(UPPER(MID(W48,4,1))="L","LLP",IF(UPPER(MID(W48,4,1))="T","Trust",IF(UPPER(MID(W48,4,1))="A","AOP","")))))))),IF($B48="Challan","",IF(W48&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z48" s="28"/>
       <c r="AA48" s="29">
@@ -6532,10 +6532,10 @@
       <c r="V49" s="28"/>
       <c r="W49" s="28"/>
       <c r="X49" s="23">
-        <f>IF($B49&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W49)))=10,CODE(MID(TRIM(UPPER(W49)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W49)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W49)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W49)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B49="Entry",IF(AND(LEN(TRIM(UPPER(W49)))=10,CODE(MID(TRIM(UPPER(W49)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W49)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W49)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W49)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W49)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W49)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W49)),9,1))&lt;=57),"N","Y"),IF($B49="Challan","",IF(W49&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y49" s="23">
-        <f>IF($B49&lt;&gt;"Entry","",IF(LEN(W49)&lt;4,"",IF(UPPER(MID(W49,4,1))="P","Individual",IF(UPPER(MID(W49,4,1))="H","HUF",IF(UPPER(MID(W49,4,1))="C","Company",IF(UPPER(MID(W49,4,1))="F","Firm",IF(UPPER(MID(W49,4,1))="L","LLP",IF(UPPER(MID(W49,4,1))="T","Trust",IF(UPPER(MID(W49,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B49="Entry",IF(LEN(W49)&lt;4,"",IF(UPPER(MID(W49,4,1))="P","Individual",IF(UPPER(MID(W49,4,1))="H","HUF",IF(UPPER(MID(W49,4,1))="C","Company",IF(UPPER(MID(W49,4,1))="F","Firm",IF(UPPER(MID(W49,4,1))="L","LLP",IF(UPPER(MID(W49,4,1))="T","Trust",IF(UPPER(MID(W49,4,1))="A","AOP","")))))))),IF($B49="Challan","",IF(W49&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z49" s="28"/>
       <c r="AA49" s="29">
@@ -6610,10 +6610,10 @@
       <c r="V50" s="28"/>
       <c r="W50" s="28"/>
       <c r="X50" s="23">
-        <f>IF($B50&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W50)))=10,CODE(MID(TRIM(UPPER(W50)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W50)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W50)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W50)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B50="Entry",IF(AND(LEN(TRIM(UPPER(W50)))=10,CODE(MID(TRIM(UPPER(W50)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W50)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W50)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W50)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W50)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W50)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W50)),9,1))&lt;=57),"N","Y"),IF($B50="Challan","",IF(W50&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y50" s="23">
-        <f>IF($B50&lt;&gt;"Entry","",IF(LEN(W50)&lt;4,"",IF(UPPER(MID(W50,4,1))="P","Individual",IF(UPPER(MID(W50,4,1))="H","HUF",IF(UPPER(MID(W50,4,1))="C","Company",IF(UPPER(MID(W50,4,1))="F","Firm",IF(UPPER(MID(W50,4,1))="L","LLP",IF(UPPER(MID(W50,4,1))="T","Trust",IF(UPPER(MID(W50,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B50="Entry",IF(LEN(W50)&lt;4,"",IF(UPPER(MID(W50,4,1))="P","Individual",IF(UPPER(MID(W50,4,1))="H","HUF",IF(UPPER(MID(W50,4,1))="C","Company",IF(UPPER(MID(W50,4,1))="F","Firm",IF(UPPER(MID(W50,4,1))="L","LLP",IF(UPPER(MID(W50,4,1))="T","Trust",IF(UPPER(MID(W50,4,1))="A","AOP","")))))))),IF($B50="Challan","",IF(W50&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z50" s="28"/>
       <c r="AA50" s="29">
@@ -6688,10 +6688,10 @@
       <c r="V51" s="28"/>
       <c r="W51" s="28"/>
       <c r="X51" s="23">
-        <f>IF($B51&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W51)))=10,CODE(MID(TRIM(UPPER(W51)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W51)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W51)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W51)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B51="Entry",IF(AND(LEN(TRIM(UPPER(W51)))=10,CODE(MID(TRIM(UPPER(W51)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W51)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W51)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W51)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W51)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W51)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W51)),9,1))&lt;=57),"N","Y"),IF($B51="Challan","",IF(W51&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y51" s="23">
-        <f>IF($B51&lt;&gt;"Entry","",IF(LEN(W51)&lt;4,"",IF(UPPER(MID(W51,4,1))="P","Individual",IF(UPPER(MID(W51,4,1))="H","HUF",IF(UPPER(MID(W51,4,1))="C","Company",IF(UPPER(MID(W51,4,1))="F","Firm",IF(UPPER(MID(W51,4,1))="L","LLP",IF(UPPER(MID(W51,4,1))="T","Trust",IF(UPPER(MID(W51,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B51="Entry",IF(LEN(W51)&lt;4,"",IF(UPPER(MID(W51,4,1))="P","Individual",IF(UPPER(MID(W51,4,1))="H","HUF",IF(UPPER(MID(W51,4,1))="C","Company",IF(UPPER(MID(W51,4,1))="F","Firm",IF(UPPER(MID(W51,4,1))="L","LLP",IF(UPPER(MID(W51,4,1))="T","Trust",IF(UPPER(MID(W51,4,1))="A","AOP","")))))))),IF($B51="Challan","",IF(W51&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z51" s="28"/>
       <c r="AA51" s="29">
@@ -6766,10 +6766,10 @@
       <c r="V52" s="28"/>
       <c r="W52" s="28"/>
       <c r="X52" s="23">
-        <f>IF($B52&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W52)))=10,CODE(MID(TRIM(UPPER(W52)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W52)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W52)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W52)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B52="Entry",IF(AND(LEN(TRIM(UPPER(W52)))=10,CODE(MID(TRIM(UPPER(W52)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W52)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W52)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W52)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W52)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W52)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W52)),9,1))&lt;=57),"N","Y"),IF($B52="Challan","",IF(W52&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y52" s="23">
-        <f>IF($B52&lt;&gt;"Entry","",IF(LEN(W52)&lt;4,"",IF(UPPER(MID(W52,4,1))="P","Individual",IF(UPPER(MID(W52,4,1))="H","HUF",IF(UPPER(MID(W52,4,1))="C","Company",IF(UPPER(MID(W52,4,1))="F","Firm",IF(UPPER(MID(W52,4,1))="L","LLP",IF(UPPER(MID(W52,4,1))="T","Trust",IF(UPPER(MID(W52,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B52="Entry",IF(LEN(W52)&lt;4,"",IF(UPPER(MID(W52,4,1))="P","Individual",IF(UPPER(MID(W52,4,1))="H","HUF",IF(UPPER(MID(W52,4,1))="C","Company",IF(UPPER(MID(W52,4,1))="F","Firm",IF(UPPER(MID(W52,4,1))="L","LLP",IF(UPPER(MID(W52,4,1))="T","Trust",IF(UPPER(MID(W52,4,1))="A","AOP","")))))))),IF($B52="Challan","",IF(W52&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z52" s="28"/>
       <c r="AA52" s="29">
@@ -6844,10 +6844,10 @@
       <c r="V53" s="28"/>
       <c r="W53" s="28"/>
       <c r="X53" s="23">
-        <f>IF($B53&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W53)))=10,CODE(MID(TRIM(UPPER(W53)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W53)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W53)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W53)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B53="Entry",IF(AND(LEN(TRIM(UPPER(W53)))=10,CODE(MID(TRIM(UPPER(W53)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W53)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W53)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W53)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W53)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W53)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W53)),9,1))&lt;=57),"N","Y"),IF($B53="Challan","",IF(W53&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y53" s="23">
-        <f>IF($B53&lt;&gt;"Entry","",IF(LEN(W53)&lt;4,"",IF(UPPER(MID(W53,4,1))="P","Individual",IF(UPPER(MID(W53,4,1))="H","HUF",IF(UPPER(MID(W53,4,1))="C","Company",IF(UPPER(MID(W53,4,1))="F","Firm",IF(UPPER(MID(W53,4,1))="L","LLP",IF(UPPER(MID(W53,4,1))="T","Trust",IF(UPPER(MID(W53,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B53="Entry",IF(LEN(W53)&lt;4,"",IF(UPPER(MID(W53,4,1))="P","Individual",IF(UPPER(MID(W53,4,1))="H","HUF",IF(UPPER(MID(W53,4,1))="C","Company",IF(UPPER(MID(W53,4,1))="F","Firm",IF(UPPER(MID(W53,4,1))="L","LLP",IF(UPPER(MID(W53,4,1))="T","Trust",IF(UPPER(MID(W53,4,1))="A","AOP","")))))))),IF($B53="Challan","",IF(W53&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z53" s="28"/>
       <c r="AA53" s="29">
@@ -6922,10 +6922,10 @@
       <c r="V54" s="28"/>
       <c r="W54" s="28"/>
       <c r="X54" s="23">
-        <f>IF($B54&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W54)))=10,CODE(MID(TRIM(UPPER(W54)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W54)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W54)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W54)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B54="Entry",IF(AND(LEN(TRIM(UPPER(W54)))=10,CODE(MID(TRIM(UPPER(W54)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W54)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W54)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W54)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W54)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W54)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W54)),9,1))&lt;=57),"N","Y"),IF($B54="Challan","",IF(W54&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y54" s="23">
-        <f>IF($B54&lt;&gt;"Entry","",IF(LEN(W54)&lt;4,"",IF(UPPER(MID(W54,4,1))="P","Individual",IF(UPPER(MID(W54,4,1))="H","HUF",IF(UPPER(MID(W54,4,1))="C","Company",IF(UPPER(MID(W54,4,1))="F","Firm",IF(UPPER(MID(W54,4,1))="L","LLP",IF(UPPER(MID(W54,4,1))="T","Trust",IF(UPPER(MID(W54,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B54="Entry",IF(LEN(W54)&lt;4,"",IF(UPPER(MID(W54,4,1))="P","Individual",IF(UPPER(MID(W54,4,1))="H","HUF",IF(UPPER(MID(W54,4,1))="C","Company",IF(UPPER(MID(W54,4,1))="F","Firm",IF(UPPER(MID(W54,4,1))="L","LLP",IF(UPPER(MID(W54,4,1))="T","Trust",IF(UPPER(MID(W54,4,1))="A","AOP","")))))))),IF($B54="Challan","",IF(W54&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z54" s="28"/>
       <c r="AA54" s="29">
@@ -7000,10 +7000,10 @@
       <c r="V55" s="28"/>
       <c r="W55" s="28"/>
       <c r="X55" s="23">
-        <f>IF($B55&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W55)))=10,CODE(MID(TRIM(UPPER(W55)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W55)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W55)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W55)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B55="Entry",IF(AND(LEN(TRIM(UPPER(W55)))=10,CODE(MID(TRIM(UPPER(W55)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W55)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W55)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W55)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W55)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W55)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W55)),9,1))&lt;=57),"N","Y"),IF($B55="Challan","",IF(W55&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y55" s="23">
-        <f>IF($B55&lt;&gt;"Entry","",IF(LEN(W55)&lt;4,"",IF(UPPER(MID(W55,4,1))="P","Individual",IF(UPPER(MID(W55,4,1))="H","HUF",IF(UPPER(MID(W55,4,1))="C","Company",IF(UPPER(MID(W55,4,1))="F","Firm",IF(UPPER(MID(W55,4,1))="L","LLP",IF(UPPER(MID(W55,4,1))="T","Trust",IF(UPPER(MID(W55,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B55="Entry",IF(LEN(W55)&lt;4,"",IF(UPPER(MID(W55,4,1))="P","Individual",IF(UPPER(MID(W55,4,1))="H","HUF",IF(UPPER(MID(W55,4,1))="C","Company",IF(UPPER(MID(W55,4,1))="F","Firm",IF(UPPER(MID(W55,4,1))="L","LLP",IF(UPPER(MID(W55,4,1))="T","Trust",IF(UPPER(MID(W55,4,1))="A","AOP","")))))))),IF($B55="Challan","",IF(W55&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z55" s="28"/>
       <c r="AA55" s="29">
@@ -7078,10 +7078,10 @@
       <c r="V56" s="28"/>
       <c r="W56" s="28"/>
       <c r="X56" s="23">
-        <f>IF($B56&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W56)))=10,CODE(MID(TRIM(UPPER(W56)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W56)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W56)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W56)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B56="Entry",IF(AND(LEN(TRIM(UPPER(W56)))=10,CODE(MID(TRIM(UPPER(W56)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W56)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W56)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W56)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W56)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W56)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W56)),9,1))&lt;=57),"N","Y"),IF($B56="Challan","",IF(W56&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y56" s="23">
-        <f>IF($B56&lt;&gt;"Entry","",IF(LEN(W56)&lt;4,"",IF(UPPER(MID(W56,4,1))="P","Individual",IF(UPPER(MID(W56,4,1))="H","HUF",IF(UPPER(MID(W56,4,1))="C","Company",IF(UPPER(MID(W56,4,1))="F","Firm",IF(UPPER(MID(W56,4,1))="L","LLP",IF(UPPER(MID(W56,4,1))="T","Trust",IF(UPPER(MID(W56,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B56="Entry",IF(LEN(W56)&lt;4,"",IF(UPPER(MID(W56,4,1))="P","Individual",IF(UPPER(MID(W56,4,1))="H","HUF",IF(UPPER(MID(W56,4,1))="C","Company",IF(UPPER(MID(W56,4,1))="F","Firm",IF(UPPER(MID(W56,4,1))="L","LLP",IF(UPPER(MID(W56,4,1))="T","Trust",IF(UPPER(MID(W56,4,1))="A","AOP","")))))))),IF($B56="Challan","",IF(W56&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z56" s="28"/>
       <c r="AA56" s="29">
@@ -7156,10 +7156,10 @@
       <c r="V57" s="28"/>
       <c r="W57" s="28"/>
       <c r="X57" s="23">
-        <f>IF($B57&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W57)))=10,CODE(MID(TRIM(UPPER(W57)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W57)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W57)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W57)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B57="Entry",IF(AND(LEN(TRIM(UPPER(W57)))=10,CODE(MID(TRIM(UPPER(W57)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W57)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W57)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W57)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W57)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W57)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W57)),9,1))&lt;=57),"N","Y"),IF($B57="Challan","",IF(W57&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y57" s="23">
-        <f>IF($B57&lt;&gt;"Entry","",IF(LEN(W57)&lt;4,"",IF(UPPER(MID(W57,4,1))="P","Individual",IF(UPPER(MID(W57,4,1))="H","HUF",IF(UPPER(MID(W57,4,1))="C","Company",IF(UPPER(MID(W57,4,1))="F","Firm",IF(UPPER(MID(W57,4,1))="L","LLP",IF(UPPER(MID(W57,4,1))="T","Trust",IF(UPPER(MID(W57,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B57="Entry",IF(LEN(W57)&lt;4,"",IF(UPPER(MID(W57,4,1))="P","Individual",IF(UPPER(MID(W57,4,1))="H","HUF",IF(UPPER(MID(W57,4,1))="C","Company",IF(UPPER(MID(W57,4,1))="F","Firm",IF(UPPER(MID(W57,4,1))="L","LLP",IF(UPPER(MID(W57,4,1))="T","Trust",IF(UPPER(MID(W57,4,1))="A","AOP","")))))))),IF($B57="Challan","",IF(W57&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z57" s="28"/>
       <c r="AA57" s="29">
@@ -7234,10 +7234,10 @@
       <c r="V58" s="28"/>
       <c r="W58" s="28"/>
       <c r="X58" s="23">
-        <f>IF($B58&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W58)))=10,CODE(MID(TRIM(UPPER(W58)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W58)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W58)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W58)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B58="Entry",IF(AND(LEN(TRIM(UPPER(W58)))=10,CODE(MID(TRIM(UPPER(W58)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W58)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W58)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W58)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W58)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W58)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W58)),9,1))&lt;=57),"N","Y"),IF($B58="Challan","",IF(W58&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y58" s="23">
-        <f>IF($B58&lt;&gt;"Entry","",IF(LEN(W58)&lt;4,"",IF(UPPER(MID(W58,4,1))="P","Individual",IF(UPPER(MID(W58,4,1))="H","HUF",IF(UPPER(MID(W58,4,1))="C","Company",IF(UPPER(MID(W58,4,1))="F","Firm",IF(UPPER(MID(W58,4,1))="L","LLP",IF(UPPER(MID(W58,4,1))="T","Trust",IF(UPPER(MID(W58,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B58="Entry",IF(LEN(W58)&lt;4,"",IF(UPPER(MID(W58,4,1))="P","Individual",IF(UPPER(MID(W58,4,1))="H","HUF",IF(UPPER(MID(W58,4,1))="C","Company",IF(UPPER(MID(W58,4,1))="F","Firm",IF(UPPER(MID(W58,4,1))="L","LLP",IF(UPPER(MID(W58,4,1))="T","Trust",IF(UPPER(MID(W58,4,1))="A","AOP","")))))))),IF($B58="Challan","",IF(W58&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z58" s="28"/>
       <c r="AA58" s="29">
@@ -7312,10 +7312,10 @@
       <c r="V59" s="28"/>
       <c r="W59" s="28"/>
       <c r="X59" s="23">
-        <f>IF($B59&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W59)))=10,CODE(MID(TRIM(UPPER(W59)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W59)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W59)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W59)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B59="Entry",IF(AND(LEN(TRIM(UPPER(W59)))=10,CODE(MID(TRIM(UPPER(W59)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W59)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W59)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W59)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W59)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W59)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W59)),9,1))&lt;=57),"N","Y"),IF($B59="Challan","",IF(W59&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y59" s="23">
-        <f>IF($B59&lt;&gt;"Entry","",IF(LEN(W59)&lt;4,"",IF(UPPER(MID(W59,4,1))="P","Individual",IF(UPPER(MID(W59,4,1))="H","HUF",IF(UPPER(MID(W59,4,1))="C","Company",IF(UPPER(MID(W59,4,1))="F","Firm",IF(UPPER(MID(W59,4,1))="L","LLP",IF(UPPER(MID(W59,4,1))="T","Trust",IF(UPPER(MID(W59,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B59="Entry",IF(LEN(W59)&lt;4,"",IF(UPPER(MID(W59,4,1))="P","Individual",IF(UPPER(MID(W59,4,1))="H","HUF",IF(UPPER(MID(W59,4,1))="C","Company",IF(UPPER(MID(W59,4,1))="F","Firm",IF(UPPER(MID(W59,4,1))="L","LLP",IF(UPPER(MID(W59,4,1))="T","Trust",IF(UPPER(MID(W59,4,1))="A","AOP","")))))))),IF($B59="Challan","",IF(W59&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z59" s="28"/>
       <c r="AA59" s="29">
@@ -7390,10 +7390,10 @@
       <c r="V60" s="28"/>
       <c r="W60" s="28"/>
       <c r="X60" s="23">
-        <f>IF($B60&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W60)))=10,CODE(MID(TRIM(UPPER(W60)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W60)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W60)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W60)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B60="Entry",IF(AND(LEN(TRIM(UPPER(W60)))=10,CODE(MID(TRIM(UPPER(W60)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W60)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W60)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W60)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W60)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W60)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W60)),9,1))&lt;=57),"N","Y"),IF($B60="Challan","",IF(W60&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y60" s="23">
-        <f>IF($B60&lt;&gt;"Entry","",IF(LEN(W60)&lt;4,"",IF(UPPER(MID(W60,4,1))="P","Individual",IF(UPPER(MID(W60,4,1))="H","HUF",IF(UPPER(MID(W60,4,1))="C","Company",IF(UPPER(MID(W60,4,1))="F","Firm",IF(UPPER(MID(W60,4,1))="L","LLP",IF(UPPER(MID(W60,4,1))="T","Trust",IF(UPPER(MID(W60,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B60="Entry",IF(LEN(W60)&lt;4,"",IF(UPPER(MID(W60,4,1))="P","Individual",IF(UPPER(MID(W60,4,1))="H","HUF",IF(UPPER(MID(W60,4,1))="C","Company",IF(UPPER(MID(W60,4,1))="F","Firm",IF(UPPER(MID(W60,4,1))="L","LLP",IF(UPPER(MID(W60,4,1))="T","Trust",IF(UPPER(MID(W60,4,1))="A","AOP","")))))))),IF($B60="Challan","",IF(W60&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z60" s="28"/>
       <c r="AA60" s="29">
@@ -7468,10 +7468,10 @@
       <c r="V61" s="28"/>
       <c r="W61" s="28"/>
       <c r="X61" s="23">
-        <f>IF($B61&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W61)))=10,CODE(MID(TRIM(UPPER(W61)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W61)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W61)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W61)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B61="Entry",IF(AND(LEN(TRIM(UPPER(W61)))=10,CODE(MID(TRIM(UPPER(W61)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W61)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W61)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W61)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W61)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W61)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W61)),9,1))&lt;=57),"N","Y"),IF($B61="Challan","",IF(W61&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y61" s="23">
-        <f>IF($B61&lt;&gt;"Entry","",IF(LEN(W61)&lt;4,"",IF(UPPER(MID(W61,4,1))="P","Individual",IF(UPPER(MID(W61,4,1))="H","HUF",IF(UPPER(MID(W61,4,1))="C","Company",IF(UPPER(MID(W61,4,1))="F","Firm",IF(UPPER(MID(W61,4,1))="L","LLP",IF(UPPER(MID(W61,4,1))="T","Trust",IF(UPPER(MID(W61,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B61="Entry",IF(LEN(W61)&lt;4,"",IF(UPPER(MID(W61,4,1))="P","Individual",IF(UPPER(MID(W61,4,1))="H","HUF",IF(UPPER(MID(W61,4,1))="C","Company",IF(UPPER(MID(W61,4,1))="F","Firm",IF(UPPER(MID(W61,4,1))="L","LLP",IF(UPPER(MID(W61,4,1))="T","Trust",IF(UPPER(MID(W61,4,1))="A","AOP","")))))))),IF($B61="Challan","",IF(W61&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z61" s="28"/>
       <c r="AA61" s="29">
@@ -7546,10 +7546,10 @@
       <c r="V62" s="28"/>
       <c r="W62" s="28"/>
       <c r="X62" s="23">
-        <f>IF($B62&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W62)))=10,CODE(MID(TRIM(UPPER(W62)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W62)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W62)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W62)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B62="Entry",IF(AND(LEN(TRIM(UPPER(W62)))=10,CODE(MID(TRIM(UPPER(W62)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W62)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W62)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W62)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W62)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W62)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W62)),9,1))&lt;=57),"N","Y"),IF($B62="Challan","",IF(W62&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y62" s="23">
-        <f>IF($B62&lt;&gt;"Entry","",IF(LEN(W62)&lt;4,"",IF(UPPER(MID(W62,4,1))="P","Individual",IF(UPPER(MID(W62,4,1))="H","HUF",IF(UPPER(MID(W62,4,1))="C","Company",IF(UPPER(MID(W62,4,1))="F","Firm",IF(UPPER(MID(W62,4,1))="L","LLP",IF(UPPER(MID(W62,4,1))="T","Trust",IF(UPPER(MID(W62,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B62="Entry",IF(LEN(W62)&lt;4,"",IF(UPPER(MID(W62,4,1))="P","Individual",IF(UPPER(MID(W62,4,1))="H","HUF",IF(UPPER(MID(W62,4,1))="C","Company",IF(UPPER(MID(W62,4,1))="F","Firm",IF(UPPER(MID(W62,4,1))="L","LLP",IF(UPPER(MID(W62,4,1))="T","Trust",IF(UPPER(MID(W62,4,1))="A","AOP","")))))))),IF($B62="Challan","",IF(W62&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z62" s="28"/>
       <c r="AA62" s="29">
@@ -7624,10 +7624,10 @@
       <c r="V63" s="28"/>
       <c r="W63" s="28"/>
       <c r="X63" s="23">
-        <f>IF($B63&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W63)))=10,CODE(MID(TRIM(UPPER(W63)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W63)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W63)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W63)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B63="Entry",IF(AND(LEN(TRIM(UPPER(W63)))=10,CODE(MID(TRIM(UPPER(W63)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W63)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W63)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W63)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W63)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W63)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W63)),9,1))&lt;=57),"N","Y"),IF($B63="Challan","",IF(W63&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y63" s="23">
-        <f>IF($B63&lt;&gt;"Entry","",IF(LEN(W63)&lt;4,"",IF(UPPER(MID(W63,4,1))="P","Individual",IF(UPPER(MID(W63,4,1))="H","HUF",IF(UPPER(MID(W63,4,1))="C","Company",IF(UPPER(MID(W63,4,1))="F","Firm",IF(UPPER(MID(W63,4,1))="L","LLP",IF(UPPER(MID(W63,4,1))="T","Trust",IF(UPPER(MID(W63,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B63="Entry",IF(LEN(W63)&lt;4,"",IF(UPPER(MID(W63,4,1))="P","Individual",IF(UPPER(MID(W63,4,1))="H","HUF",IF(UPPER(MID(W63,4,1))="C","Company",IF(UPPER(MID(W63,4,1))="F","Firm",IF(UPPER(MID(W63,4,1))="L","LLP",IF(UPPER(MID(W63,4,1))="T","Trust",IF(UPPER(MID(W63,4,1))="A","AOP","")))))))),IF($B63="Challan","",IF(W63&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z63" s="28"/>
       <c r="AA63" s="29">
@@ -7702,10 +7702,10 @@
       <c r="V64" s="28"/>
       <c r="W64" s="28"/>
       <c r="X64" s="23">
-        <f>IF($B64&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W64)))=10,CODE(MID(TRIM(UPPER(W64)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W64)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W64)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W64)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B64="Entry",IF(AND(LEN(TRIM(UPPER(W64)))=10,CODE(MID(TRIM(UPPER(W64)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W64)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W64)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W64)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W64)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W64)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W64)),9,1))&lt;=57),"N","Y"),IF($B64="Challan","",IF(W64&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y64" s="23">
-        <f>IF($B64&lt;&gt;"Entry","",IF(LEN(W64)&lt;4,"",IF(UPPER(MID(W64,4,1))="P","Individual",IF(UPPER(MID(W64,4,1))="H","HUF",IF(UPPER(MID(W64,4,1))="C","Company",IF(UPPER(MID(W64,4,1))="F","Firm",IF(UPPER(MID(W64,4,1))="L","LLP",IF(UPPER(MID(W64,4,1))="T","Trust",IF(UPPER(MID(W64,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B64="Entry",IF(LEN(W64)&lt;4,"",IF(UPPER(MID(W64,4,1))="P","Individual",IF(UPPER(MID(W64,4,1))="H","HUF",IF(UPPER(MID(W64,4,1))="C","Company",IF(UPPER(MID(W64,4,1))="F","Firm",IF(UPPER(MID(W64,4,1))="L","LLP",IF(UPPER(MID(W64,4,1))="T","Trust",IF(UPPER(MID(W64,4,1))="A","AOP","")))))))),IF($B64="Challan","",IF(W64&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z64" s="28"/>
       <c r="AA64" s="29">
@@ -7780,10 +7780,10 @@
       <c r="V65" s="28"/>
       <c r="W65" s="28"/>
       <c r="X65" s="23">
-        <f>IF($B65&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W65)))=10,CODE(MID(TRIM(UPPER(W65)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W65)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W65)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W65)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B65="Entry",IF(AND(LEN(TRIM(UPPER(W65)))=10,CODE(MID(TRIM(UPPER(W65)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W65)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W65)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W65)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W65)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W65)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W65)),9,1))&lt;=57),"N","Y"),IF($B65="Challan","",IF(W65&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y65" s="23">
-        <f>IF($B65&lt;&gt;"Entry","",IF(LEN(W65)&lt;4,"",IF(UPPER(MID(W65,4,1))="P","Individual",IF(UPPER(MID(W65,4,1))="H","HUF",IF(UPPER(MID(W65,4,1))="C","Company",IF(UPPER(MID(W65,4,1))="F","Firm",IF(UPPER(MID(W65,4,1))="L","LLP",IF(UPPER(MID(W65,4,1))="T","Trust",IF(UPPER(MID(W65,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B65="Entry",IF(LEN(W65)&lt;4,"",IF(UPPER(MID(W65,4,1))="P","Individual",IF(UPPER(MID(W65,4,1))="H","HUF",IF(UPPER(MID(W65,4,1))="C","Company",IF(UPPER(MID(W65,4,1))="F","Firm",IF(UPPER(MID(W65,4,1))="L","LLP",IF(UPPER(MID(W65,4,1))="T","Trust",IF(UPPER(MID(W65,4,1))="A","AOP","")))))))),IF($B65="Challan","",IF(W65&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z65" s="28"/>
       <c r="AA65" s="29">
@@ -7858,10 +7858,10 @@
       <c r="V66" s="28"/>
       <c r="W66" s="28"/>
       <c r="X66" s="23">
-        <f>IF($B66&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W66)))=10,CODE(MID(TRIM(UPPER(W66)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W66)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W66)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W66)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B66="Entry",IF(AND(LEN(TRIM(UPPER(W66)))=10,CODE(MID(TRIM(UPPER(W66)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W66)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W66)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W66)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W66)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W66)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W66)),9,1))&lt;=57),"N","Y"),IF($B66="Challan","",IF(W66&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y66" s="23">
-        <f>IF($B66&lt;&gt;"Entry","",IF(LEN(W66)&lt;4,"",IF(UPPER(MID(W66,4,1))="P","Individual",IF(UPPER(MID(W66,4,1))="H","HUF",IF(UPPER(MID(W66,4,1))="C","Company",IF(UPPER(MID(W66,4,1))="F","Firm",IF(UPPER(MID(W66,4,1))="L","LLP",IF(UPPER(MID(W66,4,1))="T","Trust",IF(UPPER(MID(W66,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B66="Entry",IF(LEN(W66)&lt;4,"",IF(UPPER(MID(W66,4,1))="P","Individual",IF(UPPER(MID(W66,4,1))="H","HUF",IF(UPPER(MID(W66,4,1))="C","Company",IF(UPPER(MID(W66,4,1))="F","Firm",IF(UPPER(MID(W66,4,1))="L","LLP",IF(UPPER(MID(W66,4,1))="T","Trust",IF(UPPER(MID(W66,4,1))="A","AOP","")))))))),IF($B66="Challan","",IF(W66&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z66" s="28"/>
       <c r="AA66" s="29">
@@ -7936,10 +7936,10 @@
       <c r="V67" s="28"/>
       <c r="W67" s="28"/>
       <c r="X67" s="23">
-        <f>IF($B67&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W67)))=10,CODE(MID(TRIM(UPPER(W67)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W67)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W67)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W67)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B67="Entry",IF(AND(LEN(TRIM(UPPER(W67)))=10,CODE(MID(TRIM(UPPER(W67)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W67)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W67)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W67)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W67)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W67)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W67)),9,1))&lt;=57),"N","Y"),IF($B67="Challan","",IF(W67&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y67" s="23">
-        <f>IF($B67&lt;&gt;"Entry","",IF(LEN(W67)&lt;4,"",IF(UPPER(MID(W67,4,1))="P","Individual",IF(UPPER(MID(W67,4,1))="H","HUF",IF(UPPER(MID(W67,4,1))="C","Company",IF(UPPER(MID(W67,4,1))="F","Firm",IF(UPPER(MID(W67,4,1))="L","LLP",IF(UPPER(MID(W67,4,1))="T","Trust",IF(UPPER(MID(W67,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B67="Entry",IF(LEN(W67)&lt;4,"",IF(UPPER(MID(W67,4,1))="P","Individual",IF(UPPER(MID(W67,4,1))="H","HUF",IF(UPPER(MID(W67,4,1))="C","Company",IF(UPPER(MID(W67,4,1))="F","Firm",IF(UPPER(MID(W67,4,1))="L","LLP",IF(UPPER(MID(W67,4,1))="T","Trust",IF(UPPER(MID(W67,4,1))="A","AOP","")))))))),IF($B67="Challan","",IF(W67&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z67" s="28"/>
       <c r="AA67" s="29">
@@ -8014,10 +8014,10 @@
       <c r="V68" s="28"/>
       <c r="W68" s="28"/>
       <c r="X68" s="23">
-        <f>IF($B68&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W68)))=10,CODE(MID(TRIM(UPPER(W68)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W68)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W68)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W68)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B68="Entry",IF(AND(LEN(TRIM(UPPER(W68)))=10,CODE(MID(TRIM(UPPER(W68)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W68)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W68)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W68)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W68)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W68)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W68)),9,1))&lt;=57),"N","Y"),IF($B68="Challan","",IF(W68&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y68" s="23">
-        <f>IF($B68&lt;&gt;"Entry","",IF(LEN(W68)&lt;4,"",IF(UPPER(MID(W68,4,1))="P","Individual",IF(UPPER(MID(W68,4,1))="H","HUF",IF(UPPER(MID(W68,4,1))="C","Company",IF(UPPER(MID(W68,4,1))="F","Firm",IF(UPPER(MID(W68,4,1))="L","LLP",IF(UPPER(MID(W68,4,1))="T","Trust",IF(UPPER(MID(W68,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B68="Entry",IF(LEN(W68)&lt;4,"",IF(UPPER(MID(W68,4,1))="P","Individual",IF(UPPER(MID(W68,4,1))="H","HUF",IF(UPPER(MID(W68,4,1))="C","Company",IF(UPPER(MID(W68,4,1))="F","Firm",IF(UPPER(MID(W68,4,1))="L","LLP",IF(UPPER(MID(W68,4,1))="T","Trust",IF(UPPER(MID(W68,4,1))="A","AOP","")))))))),IF($B68="Challan","",IF(W68&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z68" s="28"/>
       <c r="AA68" s="29">
@@ -8092,10 +8092,10 @@
       <c r="V69" s="28"/>
       <c r="W69" s="28"/>
       <c r="X69" s="23">
-        <f>IF($B69&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W69)))=10,CODE(MID(TRIM(UPPER(W69)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W69)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W69)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W69)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B69="Entry",IF(AND(LEN(TRIM(UPPER(W69)))=10,CODE(MID(TRIM(UPPER(W69)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W69)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W69)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W69)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W69)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W69)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W69)),9,1))&lt;=57),"N","Y"),IF($B69="Challan","",IF(W69&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y69" s="23">
-        <f>IF($B69&lt;&gt;"Entry","",IF(LEN(W69)&lt;4,"",IF(UPPER(MID(W69,4,1))="P","Individual",IF(UPPER(MID(W69,4,1))="H","HUF",IF(UPPER(MID(W69,4,1))="C","Company",IF(UPPER(MID(W69,4,1))="F","Firm",IF(UPPER(MID(W69,4,1))="L","LLP",IF(UPPER(MID(W69,4,1))="T","Trust",IF(UPPER(MID(W69,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B69="Entry",IF(LEN(W69)&lt;4,"",IF(UPPER(MID(W69,4,1))="P","Individual",IF(UPPER(MID(W69,4,1))="H","HUF",IF(UPPER(MID(W69,4,1))="C","Company",IF(UPPER(MID(W69,4,1))="F","Firm",IF(UPPER(MID(W69,4,1))="L","LLP",IF(UPPER(MID(W69,4,1))="T","Trust",IF(UPPER(MID(W69,4,1))="A","AOP","")))))))),IF($B69="Challan","",IF(W69&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z69" s="28"/>
       <c r="AA69" s="29">
@@ -8170,10 +8170,10 @@
       <c r="V70" s="28"/>
       <c r="W70" s="28"/>
       <c r="X70" s="23">
-        <f>IF($B70&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W70)))=10,CODE(MID(TRIM(UPPER(W70)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W70)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W70)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W70)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B70="Entry",IF(AND(LEN(TRIM(UPPER(W70)))=10,CODE(MID(TRIM(UPPER(W70)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W70)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W70)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W70)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W70)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W70)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W70)),9,1))&lt;=57),"N","Y"),IF($B70="Challan","",IF(W70&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y70" s="23">
-        <f>IF($B70&lt;&gt;"Entry","",IF(LEN(W70)&lt;4,"",IF(UPPER(MID(W70,4,1))="P","Individual",IF(UPPER(MID(W70,4,1))="H","HUF",IF(UPPER(MID(W70,4,1))="C","Company",IF(UPPER(MID(W70,4,1))="F","Firm",IF(UPPER(MID(W70,4,1))="L","LLP",IF(UPPER(MID(W70,4,1))="T","Trust",IF(UPPER(MID(W70,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B70="Entry",IF(LEN(W70)&lt;4,"",IF(UPPER(MID(W70,4,1))="P","Individual",IF(UPPER(MID(W70,4,1))="H","HUF",IF(UPPER(MID(W70,4,1))="C","Company",IF(UPPER(MID(W70,4,1))="F","Firm",IF(UPPER(MID(W70,4,1))="L","LLP",IF(UPPER(MID(W70,4,1))="T","Trust",IF(UPPER(MID(W70,4,1))="A","AOP","")))))))),IF($B70="Challan","",IF(W70&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z70" s="28"/>
       <c r="AA70" s="29">
@@ -8248,10 +8248,10 @@
       <c r="V71" s="28"/>
       <c r="W71" s="28"/>
       <c r="X71" s="23">
-        <f>IF($B71&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W71)))=10,CODE(MID(TRIM(UPPER(W71)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W71)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W71)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W71)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B71="Entry",IF(AND(LEN(TRIM(UPPER(W71)))=10,CODE(MID(TRIM(UPPER(W71)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W71)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W71)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W71)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W71)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W71)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W71)),9,1))&lt;=57),"N","Y"),IF($B71="Challan","",IF(W71&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y71" s="23">
-        <f>IF($B71&lt;&gt;"Entry","",IF(LEN(W71)&lt;4,"",IF(UPPER(MID(W71,4,1))="P","Individual",IF(UPPER(MID(W71,4,1))="H","HUF",IF(UPPER(MID(W71,4,1))="C","Company",IF(UPPER(MID(W71,4,1))="F","Firm",IF(UPPER(MID(W71,4,1))="L","LLP",IF(UPPER(MID(W71,4,1))="T","Trust",IF(UPPER(MID(W71,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B71="Entry",IF(LEN(W71)&lt;4,"",IF(UPPER(MID(W71,4,1))="P","Individual",IF(UPPER(MID(W71,4,1))="H","HUF",IF(UPPER(MID(W71,4,1))="C","Company",IF(UPPER(MID(W71,4,1))="F","Firm",IF(UPPER(MID(W71,4,1))="L","LLP",IF(UPPER(MID(W71,4,1))="T","Trust",IF(UPPER(MID(W71,4,1))="A","AOP","")))))))),IF($B71="Challan","",IF(W71&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z71" s="28"/>
       <c r="AA71" s="29">
@@ -8326,10 +8326,10 @@
       <c r="V72" s="28"/>
       <c r="W72" s="28"/>
       <c r="X72" s="23">
-        <f>IF($B72&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W72)))=10,CODE(MID(TRIM(UPPER(W72)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W72)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W72)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W72)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B72="Entry",IF(AND(LEN(TRIM(UPPER(W72)))=10,CODE(MID(TRIM(UPPER(W72)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W72)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W72)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W72)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W72)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W72)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W72)),9,1))&lt;=57),"N","Y"),IF($B72="Challan","",IF(W72&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y72" s="23">
-        <f>IF($B72&lt;&gt;"Entry","",IF(LEN(W72)&lt;4,"",IF(UPPER(MID(W72,4,1))="P","Individual",IF(UPPER(MID(W72,4,1))="H","HUF",IF(UPPER(MID(W72,4,1))="C","Company",IF(UPPER(MID(W72,4,1))="F","Firm",IF(UPPER(MID(W72,4,1))="L","LLP",IF(UPPER(MID(W72,4,1))="T","Trust",IF(UPPER(MID(W72,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B72="Entry",IF(LEN(W72)&lt;4,"",IF(UPPER(MID(W72,4,1))="P","Individual",IF(UPPER(MID(W72,4,1))="H","HUF",IF(UPPER(MID(W72,4,1))="C","Company",IF(UPPER(MID(W72,4,1))="F","Firm",IF(UPPER(MID(W72,4,1))="L","LLP",IF(UPPER(MID(W72,4,1))="T","Trust",IF(UPPER(MID(W72,4,1))="A","AOP","")))))))),IF($B72="Challan","",IF(W72&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z72" s="28"/>
       <c r="AA72" s="29">
@@ -8404,10 +8404,10 @@
       <c r="V73" s="28"/>
       <c r="W73" s="28"/>
       <c r="X73" s="23">
-        <f>IF($B73&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W73)))=10,CODE(MID(TRIM(UPPER(W73)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W73)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W73)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W73)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B73="Entry",IF(AND(LEN(TRIM(UPPER(W73)))=10,CODE(MID(TRIM(UPPER(W73)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W73)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W73)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W73)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W73)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W73)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W73)),9,1))&lt;=57),"N","Y"),IF($B73="Challan","",IF(W73&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y73" s="23">
-        <f>IF($B73&lt;&gt;"Entry","",IF(LEN(W73)&lt;4,"",IF(UPPER(MID(W73,4,1))="P","Individual",IF(UPPER(MID(W73,4,1))="H","HUF",IF(UPPER(MID(W73,4,1))="C","Company",IF(UPPER(MID(W73,4,1))="F","Firm",IF(UPPER(MID(W73,4,1))="L","LLP",IF(UPPER(MID(W73,4,1))="T","Trust",IF(UPPER(MID(W73,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B73="Entry",IF(LEN(W73)&lt;4,"",IF(UPPER(MID(W73,4,1))="P","Individual",IF(UPPER(MID(W73,4,1))="H","HUF",IF(UPPER(MID(W73,4,1))="C","Company",IF(UPPER(MID(W73,4,1))="F","Firm",IF(UPPER(MID(W73,4,1))="L","LLP",IF(UPPER(MID(W73,4,1))="T","Trust",IF(UPPER(MID(W73,4,1))="A","AOP","")))))))),IF($B73="Challan","",IF(W73&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z73" s="28"/>
       <c r="AA73" s="29">
@@ -8482,10 +8482,10 @@
       <c r="V74" s="28"/>
       <c r="W74" s="28"/>
       <c r="X74" s="23">
-        <f>IF($B74&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W74)))=10,CODE(MID(TRIM(UPPER(W74)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W74)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W74)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W74)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B74="Entry",IF(AND(LEN(TRIM(UPPER(W74)))=10,CODE(MID(TRIM(UPPER(W74)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W74)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W74)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W74)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W74)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W74)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W74)),9,1))&lt;=57),"N","Y"),IF($B74="Challan","",IF(W74&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y74" s="23">
-        <f>IF($B74&lt;&gt;"Entry","",IF(LEN(W74)&lt;4,"",IF(UPPER(MID(W74,4,1))="P","Individual",IF(UPPER(MID(W74,4,1))="H","HUF",IF(UPPER(MID(W74,4,1))="C","Company",IF(UPPER(MID(W74,4,1))="F","Firm",IF(UPPER(MID(W74,4,1))="L","LLP",IF(UPPER(MID(W74,4,1))="T","Trust",IF(UPPER(MID(W74,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B74="Entry",IF(LEN(W74)&lt;4,"",IF(UPPER(MID(W74,4,1))="P","Individual",IF(UPPER(MID(W74,4,1))="H","HUF",IF(UPPER(MID(W74,4,1))="C","Company",IF(UPPER(MID(W74,4,1))="F","Firm",IF(UPPER(MID(W74,4,1))="L","LLP",IF(UPPER(MID(W74,4,1))="T","Trust",IF(UPPER(MID(W74,4,1))="A","AOP","")))))))),IF($B74="Challan","",IF(W74&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z74" s="28"/>
       <c r="AA74" s="29">
@@ -8560,10 +8560,10 @@
       <c r="V75" s="28"/>
       <c r="W75" s="28"/>
       <c r="X75" s="23">
-        <f>IF($B75&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W75)))=10,CODE(MID(TRIM(UPPER(W75)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W75)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W75)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W75)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B75="Entry",IF(AND(LEN(TRIM(UPPER(W75)))=10,CODE(MID(TRIM(UPPER(W75)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W75)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W75)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W75)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W75)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W75)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W75)),9,1))&lt;=57),"N","Y"),IF($B75="Challan","",IF(W75&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y75" s="23">
-        <f>IF($B75&lt;&gt;"Entry","",IF(LEN(W75)&lt;4,"",IF(UPPER(MID(W75,4,1))="P","Individual",IF(UPPER(MID(W75,4,1))="H","HUF",IF(UPPER(MID(W75,4,1))="C","Company",IF(UPPER(MID(W75,4,1))="F","Firm",IF(UPPER(MID(W75,4,1))="L","LLP",IF(UPPER(MID(W75,4,1))="T","Trust",IF(UPPER(MID(W75,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B75="Entry",IF(LEN(W75)&lt;4,"",IF(UPPER(MID(W75,4,1))="P","Individual",IF(UPPER(MID(W75,4,1))="H","HUF",IF(UPPER(MID(W75,4,1))="C","Company",IF(UPPER(MID(W75,4,1))="F","Firm",IF(UPPER(MID(W75,4,1))="L","LLP",IF(UPPER(MID(W75,4,1))="T","Trust",IF(UPPER(MID(W75,4,1))="A","AOP","")))))))),IF($B75="Challan","",IF(W75&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z75" s="28"/>
       <c r="AA75" s="29">
@@ -8638,10 +8638,10 @@
       <c r="V76" s="28"/>
       <c r="W76" s="28"/>
       <c r="X76" s="23">
-        <f>IF($B76&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W76)))=10,CODE(MID(TRIM(UPPER(W76)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W76)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W76)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W76)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B76="Entry",IF(AND(LEN(TRIM(UPPER(W76)))=10,CODE(MID(TRIM(UPPER(W76)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W76)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W76)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W76)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W76)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W76)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W76)),9,1))&lt;=57),"N","Y"),IF($B76="Challan","",IF(W76&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y76" s="23">
-        <f>IF($B76&lt;&gt;"Entry","",IF(LEN(W76)&lt;4,"",IF(UPPER(MID(W76,4,1))="P","Individual",IF(UPPER(MID(W76,4,1))="H","HUF",IF(UPPER(MID(W76,4,1))="C","Company",IF(UPPER(MID(W76,4,1))="F","Firm",IF(UPPER(MID(W76,4,1))="L","LLP",IF(UPPER(MID(W76,4,1))="T","Trust",IF(UPPER(MID(W76,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B76="Entry",IF(LEN(W76)&lt;4,"",IF(UPPER(MID(W76,4,1))="P","Individual",IF(UPPER(MID(W76,4,1))="H","HUF",IF(UPPER(MID(W76,4,1))="C","Company",IF(UPPER(MID(W76,4,1))="F","Firm",IF(UPPER(MID(W76,4,1))="L","LLP",IF(UPPER(MID(W76,4,1))="T","Trust",IF(UPPER(MID(W76,4,1))="A","AOP","")))))))),IF($B76="Challan","",IF(W76&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z76" s="28"/>
       <c r="AA76" s="29">
@@ -8716,10 +8716,10 @@
       <c r="V77" s="28"/>
       <c r="W77" s="28"/>
       <c r="X77" s="23">
-        <f>IF($B77&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W77)))=10,CODE(MID(TRIM(UPPER(W77)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W77)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W77)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W77)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B77="Entry",IF(AND(LEN(TRIM(UPPER(W77)))=10,CODE(MID(TRIM(UPPER(W77)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W77)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W77)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W77)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W77)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W77)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W77)),9,1))&lt;=57),"N","Y"),IF($B77="Challan","",IF(W77&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y77" s="23">
-        <f>IF($B77&lt;&gt;"Entry","",IF(LEN(W77)&lt;4,"",IF(UPPER(MID(W77,4,1))="P","Individual",IF(UPPER(MID(W77,4,1))="H","HUF",IF(UPPER(MID(W77,4,1))="C","Company",IF(UPPER(MID(W77,4,1))="F","Firm",IF(UPPER(MID(W77,4,1))="L","LLP",IF(UPPER(MID(W77,4,1))="T","Trust",IF(UPPER(MID(W77,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B77="Entry",IF(LEN(W77)&lt;4,"",IF(UPPER(MID(W77,4,1))="P","Individual",IF(UPPER(MID(W77,4,1))="H","HUF",IF(UPPER(MID(W77,4,1))="C","Company",IF(UPPER(MID(W77,4,1))="F","Firm",IF(UPPER(MID(W77,4,1))="L","LLP",IF(UPPER(MID(W77,4,1))="T","Trust",IF(UPPER(MID(W77,4,1))="A","AOP","")))))))),IF($B77="Challan","",IF(W77&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z77" s="28"/>
       <c r="AA77" s="29">
@@ -8794,10 +8794,10 @@
       <c r="V78" s="28"/>
       <c r="W78" s="28"/>
       <c r="X78" s="23">
-        <f>IF($B78&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W78)))=10,CODE(MID(TRIM(UPPER(W78)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W78)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W78)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W78)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B78="Entry",IF(AND(LEN(TRIM(UPPER(W78)))=10,CODE(MID(TRIM(UPPER(W78)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W78)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W78)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W78)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W78)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W78)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W78)),9,1))&lt;=57),"N","Y"),IF($B78="Challan","",IF(W78&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y78" s="23">
-        <f>IF($B78&lt;&gt;"Entry","",IF(LEN(W78)&lt;4,"",IF(UPPER(MID(W78,4,1))="P","Individual",IF(UPPER(MID(W78,4,1))="H","HUF",IF(UPPER(MID(W78,4,1))="C","Company",IF(UPPER(MID(W78,4,1))="F","Firm",IF(UPPER(MID(W78,4,1))="L","LLP",IF(UPPER(MID(W78,4,1))="T","Trust",IF(UPPER(MID(W78,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B78="Entry",IF(LEN(W78)&lt;4,"",IF(UPPER(MID(W78,4,1))="P","Individual",IF(UPPER(MID(W78,4,1))="H","HUF",IF(UPPER(MID(W78,4,1))="C","Company",IF(UPPER(MID(W78,4,1))="F","Firm",IF(UPPER(MID(W78,4,1))="L","LLP",IF(UPPER(MID(W78,4,1))="T","Trust",IF(UPPER(MID(W78,4,1))="A","AOP","")))))))),IF($B78="Challan","",IF(W78&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z78" s="28"/>
       <c r="AA78" s="29">
@@ -8872,10 +8872,10 @@
       <c r="V79" s="28"/>
       <c r="W79" s="28"/>
       <c r="X79" s="23">
-        <f>IF($B79&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W79)))=10,CODE(MID(TRIM(UPPER(W79)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W79)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W79)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W79)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B79="Entry",IF(AND(LEN(TRIM(UPPER(W79)))=10,CODE(MID(TRIM(UPPER(W79)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W79)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W79)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W79)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W79)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W79)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W79)),9,1))&lt;=57),"N","Y"),IF($B79="Challan","",IF(W79&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y79" s="23">
-        <f>IF($B79&lt;&gt;"Entry","",IF(LEN(W79)&lt;4,"",IF(UPPER(MID(W79,4,1))="P","Individual",IF(UPPER(MID(W79,4,1))="H","HUF",IF(UPPER(MID(W79,4,1))="C","Company",IF(UPPER(MID(W79,4,1))="F","Firm",IF(UPPER(MID(W79,4,1))="L","LLP",IF(UPPER(MID(W79,4,1))="T","Trust",IF(UPPER(MID(W79,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B79="Entry",IF(LEN(W79)&lt;4,"",IF(UPPER(MID(W79,4,1))="P","Individual",IF(UPPER(MID(W79,4,1))="H","HUF",IF(UPPER(MID(W79,4,1))="C","Company",IF(UPPER(MID(W79,4,1))="F","Firm",IF(UPPER(MID(W79,4,1))="L","LLP",IF(UPPER(MID(W79,4,1))="T","Trust",IF(UPPER(MID(W79,4,1))="A","AOP","")))))))),IF($B79="Challan","",IF(W79&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z79" s="28"/>
       <c r="AA79" s="29">
@@ -8950,10 +8950,10 @@
       <c r="V80" s="28"/>
       <c r="W80" s="28"/>
       <c r="X80" s="23">
-        <f>IF($B80&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W80)))=10,CODE(MID(TRIM(UPPER(W80)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W80)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W80)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W80)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B80="Entry",IF(AND(LEN(TRIM(UPPER(W80)))=10,CODE(MID(TRIM(UPPER(W80)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W80)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W80)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W80)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W80)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W80)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W80)),9,1))&lt;=57),"N","Y"),IF($B80="Challan","",IF(W80&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y80" s="23">
-        <f>IF($B80&lt;&gt;"Entry","",IF(LEN(W80)&lt;4,"",IF(UPPER(MID(W80,4,1))="P","Individual",IF(UPPER(MID(W80,4,1))="H","HUF",IF(UPPER(MID(W80,4,1))="C","Company",IF(UPPER(MID(W80,4,1))="F","Firm",IF(UPPER(MID(W80,4,1))="L","LLP",IF(UPPER(MID(W80,4,1))="T","Trust",IF(UPPER(MID(W80,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B80="Entry",IF(LEN(W80)&lt;4,"",IF(UPPER(MID(W80,4,1))="P","Individual",IF(UPPER(MID(W80,4,1))="H","HUF",IF(UPPER(MID(W80,4,1))="C","Company",IF(UPPER(MID(W80,4,1))="F","Firm",IF(UPPER(MID(W80,4,1))="L","LLP",IF(UPPER(MID(W80,4,1))="T","Trust",IF(UPPER(MID(W80,4,1))="A","AOP","")))))))),IF($B80="Challan","",IF(W80&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z80" s="28"/>
       <c r="AA80" s="29">
@@ -9028,10 +9028,10 @@
       <c r="V81" s="28"/>
       <c r="W81" s="28"/>
       <c r="X81" s="23">
-        <f>IF($B81&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W81)))=10,CODE(MID(TRIM(UPPER(W81)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W81)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W81)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W81)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B81="Entry",IF(AND(LEN(TRIM(UPPER(W81)))=10,CODE(MID(TRIM(UPPER(W81)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W81)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W81)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W81)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W81)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W81)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W81)),9,1))&lt;=57),"N","Y"),IF($B81="Challan","",IF(W81&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y81" s="23">
-        <f>IF($B81&lt;&gt;"Entry","",IF(LEN(W81)&lt;4,"",IF(UPPER(MID(W81,4,1))="P","Individual",IF(UPPER(MID(W81,4,1))="H","HUF",IF(UPPER(MID(W81,4,1))="C","Company",IF(UPPER(MID(W81,4,1))="F","Firm",IF(UPPER(MID(W81,4,1))="L","LLP",IF(UPPER(MID(W81,4,1))="T","Trust",IF(UPPER(MID(W81,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B81="Entry",IF(LEN(W81)&lt;4,"",IF(UPPER(MID(W81,4,1))="P","Individual",IF(UPPER(MID(W81,4,1))="H","HUF",IF(UPPER(MID(W81,4,1))="C","Company",IF(UPPER(MID(W81,4,1))="F","Firm",IF(UPPER(MID(W81,4,1))="L","LLP",IF(UPPER(MID(W81,4,1))="T","Trust",IF(UPPER(MID(W81,4,1))="A","AOP","")))))))),IF($B81="Challan","",IF(W81&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z81" s="28"/>
       <c r="AA81" s="29">
@@ -9106,10 +9106,10 @@
       <c r="V82" s="28"/>
       <c r="W82" s="28"/>
       <c r="X82" s="23">
-        <f>IF($B82&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W82)))=10,CODE(MID(TRIM(UPPER(W82)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W82)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W82)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W82)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B82="Entry",IF(AND(LEN(TRIM(UPPER(W82)))=10,CODE(MID(TRIM(UPPER(W82)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W82)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W82)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W82)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W82)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W82)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W82)),9,1))&lt;=57),"N","Y"),IF($B82="Challan","",IF(W82&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y82" s="23">
-        <f>IF($B82&lt;&gt;"Entry","",IF(LEN(W82)&lt;4,"",IF(UPPER(MID(W82,4,1))="P","Individual",IF(UPPER(MID(W82,4,1))="H","HUF",IF(UPPER(MID(W82,4,1))="C","Company",IF(UPPER(MID(W82,4,1))="F","Firm",IF(UPPER(MID(W82,4,1))="L","LLP",IF(UPPER(MID(W82,4,1))="T","Trust",IF(UPPER(MID(W82,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B82="Entry",IF(LEN(W82)&lt;4,"",IF(UPPER(MID(W82,4,1))="P","Individual",IF(UPPER(MID(W82,4,1))="H","HUF",IF(UPPER(MID(W82,4,1))="C","Company",IF(UPPER(MID(W82,4,1))="F","Firm",IF(UPPER(MID(W82,4,1))="L","LLP",IF(UPPER(MID(W82,4,1))="T","Trust",IF(UPPER(MID(W82,4,1))="A","AOP","")))))))),IF($B82="Challan","",IF(W82&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z82" s="28"/>
       <c r="AA82" s="29">
@@ -9184,10 +9184,10 @@
       <c r="V83" s="28"/>
       <c r="W83" s="28"/>
       <c r="X83" s="23">
-        <f>IF($B83&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W83)))=10,CODE(MID(TRIM(UPPER(W83)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W83)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W83)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W83)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B83="Entry",IF(AND(LEN(TRIM(UPPER(W83)))=10,CODE(MID(TRIM(UPPER(W83)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W83)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W83)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W83)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W83)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W83)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W83)),9,1))&lt;=57),"N","Y"),IF($B83="Challan","",IF(W83&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y83" s="23">
-        <f>IF($B83&lt;&gt;"Entry","",IF(LEN(W83)&lt;4,"",IF(UPPER(MID(W83,4,1))="P","Individual",IF(UPPER(MID(W83,4,1))="H","HUF",IF(UPPER(MID(W83,4,1))="C","Company",IF(UPPER(MID(W83,4,1))="F","Firm",IF(UPPER(MID(W83,4,1))="L","LLP",IF(UPPER(MID(W83,4,1))="T","Trust",IF(UPPER(MID(W83,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B83="Entry",IF(LEN(W83)&lt;4,"",IF(UPPER(MID(W83,4,1))="P","Individual",IF(UPPER(MID(W83,4,1))="H","HUF",IF(UPPER(MID(W83,4,1))="C","Company",IF(UPPER(MID(W83,4,1))="F","Firm",IF(UPPER(MID(W83,4,1))="L","LLP",IF(UPPER(MID(W83,4,1))="T","Trust",IF(UPPER(MID(W83,4,1))="A","AOP","")))))))),IF($B83="Challan","",IF(W83&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z83" s="28"/>
       <c r="AA83" s="29">
@@ -9262,10 +9262,10 @@
       <c r="V84" s="28"/>
       <c r="W84" s="28"/>
       <c r="X84" s="23">
-        <f>IF($B84&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W84)))=10,CODE(MID(TRIM(UPPER(W84)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W84)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W84)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W84)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B84="Entry",IF(AND(LEN(TRIM(UPPER(W84)))=10,CODE(MID(TRIM(UPPER(W84)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W84)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W84)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W84)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W84)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W84)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W84)),9,1))&lt;=57),"N","Y"),IF($B84="Challan","",IF(W84&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y84" s="23">
-        <f>IF($B84&lt;&gt;"Entry","",IF(LEN(W84)&lt;4,"",IF(UPPER(MID(W84,4,1))="P","Individual",IF(UPPER(MID(W84,4,1))="H","HUF",IF(UPPER(MID(W84,4,1))="C","Company",IF(UPPER(MID(W84,4,1))="F","Firm",IF(UPPER(MID(W84,4,1))="L","LLP",IF(UPPER(MID(W84,4,1))="T","Trust",IF(UPPER(MID(W84,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B84="Entry",IF(LEN(W84)&lt;4,"",IF(UPPER(MID(W84,4,1))="P","Individual",IF(UPPER(MID(W84,4,1))="H","HUF",IF(UPPER(MID(W84,4,1))="C","Company",IF(UPPER(MID(W84,4,1))="F","Firm",IF(UPPER(MID(W84,4,1))="L","LLP",IF(UPPER(MID(W84,4,1))="T","Trust",IF(UPPER(MID(W84,4,1))="A","AOP","")))))))),IF($B84="Challan","",IF(W84&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z84" s="28"/>
       <c r="AA84" s="29">
@@ -9340,10 +9340,10 @@
       <c r="V85" s="28"/>
       <c r="W85" s="28"/>
       <c r="X85" s="23">
-        <f>IF($B85&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W85)))=10,CODE(MID(TRIM(UPPER(W85)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W85)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W85)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W85)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B85="Entry",IF(AND(LEN(TRIM(UPPER(W85)))=10,CODE(MID(TRIM(UPPER(W85)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W85)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W85)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W85)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W85)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W85)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W85)),9,1))&lt;=57),"N","Y"),IF($B85="Challan","",IF(W85&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y85" s="23">
-        <f>IF($B85&lt;&gt;"Entry","",IF(LEN(W85)&lt;4,"",IF(UPPER(MID(W85,4,1))="P","Individual",IF(UPPER(MID(W85,4,1))="H","HUF",IF(UPPER(MID(W85,4,1))="C","Company",IF(UPPER(MID(W85,4,1))="F","Firm",IF(UPPER(MID(W85,4,1))="L","LLP",IF(UPPER(MID(W85,4,1))="T","Trust",IF(UPPER(MID(W85,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B85="Entry",IF(LEN(W85)&lt;4,"",IF(UPPER(MID(W85,4,1))="P","Individual",IF(UPPER(MID(W85,4,1))="H","HUF",IF(UPPER(MID(W85,4,1))="C","Company",IF(UPPER(MID(W85,4,1))="F","Firm",IF(UPPER(MID(W85,4,1))="L","LLP",IF(UPPER(MID(W85,4,1))="T","Trust",IF(UPPER(MID(W85,4,1))="A","AOP","")))))))),IF($B85="Challan","",IF(W85&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z85" s="28"/>
       <c r="AA85" s="29">
@@ -9418,10 +9418,10 @@
       <c r="V86" s="28"/>
       <c r="W86" s="28"/>
       <c r="X86" s="23">
-        <f>IF($B86&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W86)))=10,CODE(MID(TRIM(UPPER(W86)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W86)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W86)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W86)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B86="Entry",IF(AND(LEN(TRIM(UPPER(W86)))=10,CODE(MID(TRIM(UPPER(W86)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W86)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W86)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W86)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W86)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W86)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W86)),9,1))&lt;=57),"N","Y"),IF($B86="Challan","",IF(W86&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y86" s="23">
-        <f>IF($B86&lt;&gt;"Entry","",IF(LEN(W86)&lt;4,"",IF(UPPER(MID(W86,4,1))="P","Individual",IF(UPPER(MID(W86,4,1))="H","HUF",IF(UPPER(MID(W86,4,1))="C","Company",IF(UPPER(MID(W86,4,1))="F","Firm",IF(UPPER(MID(W86,4,1))="L","LLP",IF(UPPER(MID(W86,4,1))="T","Trust",IF(UPPER(MID(W86,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B86="Entry",IF(LEN(W86)&lt;4,"",IF(UPPER(MID(W86,4,1))="P","Individual",IF(UPPER(MID(W86,4,1))="H","HUF",IF(UPPER(MID(W86,4,1))="C","Company",IF(UPPER(MID(W86,4,1))="F","Firm",IF(UPPER(MID(W86,4,1))="L","LLP",IF(UPPER(MID(W86,4,1))="T","Trust",IF(UPPER(MID(W86,4,1))="A","AOP","")))))))),IF($B86="Challan","",IF(W86&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z86" s="28"/>
       <c r="AA86" s="29">
@@ -9496,10 +9496,10 @@
       <c r="V87" s="28"/>
       <c r="W87" s="28"/>
       <c r="X87" s="23">
-        <f>IF($B87&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W87)))=10,CODE(MID(TRIM(UPPER(W87)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W87)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W87)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W87)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B87="Entry",IF(AND(LEN(TRIM(UPPER(W87)))=10,CODE(MID(TRIM(UPPER(W87)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W87)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W87)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W87)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W87)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W87)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W87)),9,1))&lt;=57),"N","Y"),IF($B87="Challan","",IF(W87&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y87" s="23">
-        <f>IF($B87&lt;&gt;"Entry","",IF(LEN(W87)&lt;4,"",IF(UPPER(MID(W87,4,1))="P","Individual",IF(UPPER(MID(W87,4,1))="H","HUF",IF(UPPER(MID(W87,4,1))="C","Company",IF(UPPER(MID(W87,4,1))="F","Firm",IF(UPPER(MID(W87,4,1))="L","LLP",IF(UPPER(MID(W87,4,1))="T","Trust",IF(UPPER(MID(W87,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B87="Entry",IF(LEN(W87)&lt;4,"",IF(UPPER(MID(W87,4,1))="P","Individual",IF(UPPER(MID(W87,4,1))="H","HUF",IF(UPPER(MID(W87,4,1))="C","Company",IF(UPPER(MID(W87,4,1))="F","Firm",IF(UPPER(MID(W87,4,1))="L","LLP",IF(UPPER(MID(W87,4,1))="T","Trust",IF(UPPER(MID(W87,4,1))="A","AOP","")))))))),IF($B87="Challan","",IF(W87&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z87" s="28"/>
       <c r="AA87" s="29">
@@ -9574,10 +9574,10 @@
       <c r="V88" s="28"/>
       <c r="W88" s="28"/>
       <c r="X88" s="23">
-        <f>IF($B88&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W88)))=10,CODE(MID(TRIM(UPPER(W88)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W88)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W88)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W88)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B88="Entry",IF(AND(LEN(TRIM(UPPER(W88)))=10,CODE(MID(TRIM(UPPER(W88)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W88)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W88)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W88)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W88)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W88)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W88)),9,1))&lt;=57),"N","Y"),IF($B88="Challan","",IF(W88&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y88" s="23">
-        <f>IF($B88&lt;&gt;"Entry","",IF(LEN(W88)&lt;4,"",IF(UPPER(MID(W88,4,1))="P","Individual",IF(UPPER(MID(W88,4,1))="H","HUF",IF(UPPER(MID(W88,4,1))="C","Company",IF(UPPER(MID(W88,4,1))="F","Firm",IF(UPPER(MID(W88,4,1))="L","LLP",IF(UPPER(MID(W88,4,1))="T","Trust",IF(UPPER(MID(W88,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B88="Entry",IF(LEN(W88)&lt;4,"",IF(UPPER(MID(W88,4,1))="P","Individual",IF(UPPER(MID(W88,4,1))="H","HUF",IF(UPPER(MID(W88,4,1))="C","Company",IF(UPPER(MID(W88,4,1))="F","Firm",IF(UPPER(MID(W88,4,1))="L","LLP",IF(UPPER(MID(W88,4,1))="T","Trust",IF(UPPER(MID(W88,4,1))="A","AOP","")))))))),IF($B88="Challan","",IF(W88&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z88" s="28"/>
       <c r="AA88" s="29">
@@ -9652,10 +9652,10 @@
       <c r="V89" s="28"/>
       <c r="W89" s="28"/>
       <c r="X89" s="23">
-        <f>IF($B89&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W89)))=10,CODE(MID(TRIM(UPPER(W89)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W89)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W89)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W89)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B89="Entry",IF(AND(LEN(TRIM(UPPER(W89)))=10,CODE(MID(TRIM(UPPER(W89)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W89)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W89)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W89)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W89)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W89)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W89)),9,1))&lt;=57),"N","Y"),IF($B89="Challan","",IF(W89&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y89" s="23">
-        <f>IF($B89&lt;&gt;"Entry","",IF(LEN(W89)&lt;4,"",IF(UPPER(MID(W89,4,1))="P","Individual",IF(UPPER(MID(W89,4,1))="H","HUF",IF(UPPER(MID(W89,4,1))="C","Company",IF(UPPER(MID(W89,4,1))="F","Firm",IF(UPPER(MID(W89,4,1))="L","LLP",IF(UPPER(MID(W89,4,1))="T","Trust",IF(UPPER(MID(W89,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B89="Entry",IF(LEN(W89)&lt;4,"",IF(UPPER(MID(W89,4,1))="P","Individual",IF(UPPER(MID(W89,4,1))="H","HUF",IF(UPPER(MID(W89,4,1))="C","Company",IF(UPPER(MID(W89,4,1))="F","Firm",IF(UPPER(MID(W89,4,1))="L","LLP",IF(UPPER(MID(W89,4,1))="T","Trust",IF(UPPER(MID(W89,4,1))="A","AOP","")))))))),IF($B89="Challan","",IF(W89&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z89" s="28"/>
       <c r="AA89" s="29">
@@ -9730,10 +9730,10 @@
       <c r="V90" s="28"/>
       <c r="W90" s="28"/>
       <c r="X90" s="23">
-        <f>IF($B90&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W90)))=10,CODE(MID(TRIM(UPPER(W90)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W90)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W90)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W90)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B90="Entry",IF(AND(LEN(TRIM(UPPER(W90)))=10,CODE(MID(TRIM(UPPER(W90)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W90)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W90)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W90)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W90)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W90)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W90)),9,1))&lt;=57),"N","Y"),IF($B90="Challan","",IF(W90&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y90" s="23">
-        <f>IF($B90&lt;&gt;"Entry","",IF(LEN(W90)&lt;4,"",IF(UPPER(MID(W90,4,1))="P","Individual",IF(UPPER(MID(W90,4,1))="H","HUF",IF(UPPER(MID(W90,4,1))="C","Company",IF(UPPER(MID(W90,4,1))="F","Firm",IF(UPPER(MID(W90,4,1))="L","LLP",IF(UPPER(MID(W90,4,1))="T","Trust",IF(UPPER(MID(W90,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B90="Entry",IF(LEN(W90)&lt;4,"",IF(UPPER(MID(W90,4,1))="P","Individual",IF(UPPER(MID(W90,4,1))="H","HUF",IF(UPPER(MID(W90,4,1))="C","Company",IF(UPPER(MID(W90,4,1))="F","Firm",IF(UPPER(MID(W90,4,1))="L","LLP",IF(UPPER(MID(W90,4,1))="T","Trust",IF(UPPER(MID(W90,4,1))="A","AOP","")))))))),IF($B90="Challan","",IF(W90&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z90" s="28"/>
       <c r="AA90" s="29">
@@ -9808,10 +9808,10 @@
       <c r="V91" s="28"/>
       <c r="W91" s="28"/>
       <c r="X91" s="23">
-        <f>IF($B91&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W91)))=10,CODE(MID(TRIM(UPPER(W91)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W91)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W91)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W91)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B91="Entry",IF(AND(LEN(TRIM(UPPER(W91)))=10,CODE(MID(TRIM(UPPER(W91)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W91)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W91)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W91)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W91)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W91)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W91)),9,1))&lt;=57),"N","Y"),IF($B91="Challan","",IF(W91&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y91" s="23">
-        <f>IF($B91&lt;&gt;"Entry","",IF(LEN(W91)&lt;4,"",IF(UPPER(MID(W91,4,1))="P","Individual",IF(UPPER(MID(W91,4,1))="H","HUF",IF(UPPER(MID(W91,4,1))="C","Company",IF(UPPER(MID(W91,4,1))="F","Firm",IF(UPPER(MID(W91,4,1))="L","LLP",IF(UPPER(MID(W91,4,1))="T","Trust",IF(UPPER(MID(W91,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B91="Entry",IF(LEN(W91)&lt;4,"",IF(UPPER(MID(W91,4,1))="P","Individual",IF(UPPER(MID(W91,4,1))="H","HUF",IF(UPPER(MID(W91,4,1))="C","Company",IF(UPPER(MID(W91,4,1))="F","Firm",IF(UPPER(MID(W91,4,1))="L","LLP",IF(UPPER(MID(W91,4,1))="T","Trust",IF(UPPER(MID(W91,4,1))="A","AOP","")))))))),IF($B91="Challan","",IF(W91&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z91" s="28"/>
       <c r="AA91" s="29">
@@ -9886,10 +9886,10 @@
       <c r="V92" s="28"/>
       <c r="W92" s="28"/>
       <c r="X92" s="23">
-        <f>IF($B92&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W92)))=10,CODE(MID(TRIM(UPPER(W92)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W92)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W92)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W92)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B92="Entry",IF(AND(LEN(TRIM(UPPER(W92)))=10,CODE(MID(TRIM(UPPER(W92)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W92)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W92)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W92)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W92)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W92)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W92)),9,1))&lt;=57),"N","Y"),IF($B92="Challan","",IF(W92&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y92" s="23">
-        <f>IF($B92&lt;&gt;"Entry","",IF(LEN(W92)&lt;4,"",IF(UPPER(MID(W92,4,1))="P","Individual",IF(UPPER(MID(W92,4,1))="H","HUF",IF(UPPER(MID(W92,4,1))="C","Company",IF(UPPER(MID(W92,4,1))="F","Firm",IF(UPPER(MID(W92,4,1))="L","LLP",IF(UPPER(MID(W92,4,1))="T","Trust",IF(UPPER(MID(W92,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B92="Entry",IF(LEN(W92)&lt;4,"",IF(UPPER(MID(W92,4,1))="P","Individual",IF(UPPER(MID(W92,4,1))="H","HUF",IF(UPPER(MID(W92,4,1))="C","Company",IF(UPPER(MID(W92,4,1))="F","Firm",IF(UPPER(MID(W92,4,1))="L","LLP",IF(UPPER(MID(W92,4,1))="T","Trust",IF(UPPER(MID(W92,4,1))="A","AOP","")))))))),IF($B92="Challan","",IF(W92&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z92" s="28"/>
       <c r="AA92" s="29">
@@ -9964,10 +9964,10 @@
       <c r="V93" s="28"/>
       <c r="W93" s="28"/>
       <c r="X93" s="23">
-        <f>IF($B93&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W93)))=10,CODE(MID(TRIM(UPPER(W93)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W93)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W93)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W93)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B93="Entry",IF(AND(LEN(TRIM(UPPER(W93)))=10,CODE(MID(TRIM(UPPER(W93)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W93)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W93)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W93)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W93)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W93)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W93)),9,1))&lt;=57),"N","Y"),IF($B93="Challan","",IF(W93&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y93" s="23">
-        <f>IF($B93&lt;&gt;"Entry","",IF(LEN(W93)&lt;4,"",IF(UPPER(MID(W93,4,1))="P","Individual",IF(UPPER(MID(W93,4,1))="H","HUF",IF(UPPER(MID(W93,4,1))="C","Company",IF(UPPER(MID(W93,4,1))="F","Firm",IF(UPPER(MID(W93,4,1))="L","LLP",IF(UPPER(MID(W93,4,1))="T","Trust",IF(UPPER(MID(W93,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B93="Entry",IF(LEN(W93)&lt;4,"",IF(UPPER(MID(W93,4,1))="P","Individual",IF(UPPER(MID(W93,4,1))="H","HUF",IF(UPPER(MID(W93,4,1))="C","Company",IF(UPPER(MID(W93,4,1))="F","Firm",IF(UPPER(MID(W93,4,1))="L","LLP",IF(UPPER(MID(W93,4,1))="T","Trust",IF(UPPER(MID(W93,4,1))="A","AOP","")))))))),IF($B93="Challan","",IF(W93&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z93" s="28"/>
       <c r="AA93" s="29">
@@ -10042,10 +10042,10 @@
       <c r="V94" s="28"/>
       <c r="W94" s="28"/>
       <c r="X94" s="23">
-        <f>IF($B94&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W94)))=10,CODE(MID(TRIM(UPPER(W94)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W94)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W94)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W94)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B94="Entry",IF(AND(LEN(TRIM(UPPER(W94)))=10,CODE(MID(TRIM(UPPER(W94)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W94)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W94)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W94)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W94)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W94)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W94)),9,1))&lt;=57),"N","Y"),IF($B94="Challan","",IF(W94&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y94" s="23">
-        <f>IF($B94&lt;&gt;"Entry","",IF(LEN(W94)&lt;4,"",IF(UPPER(MID(W94,4,1))="P","Individual",IF(UPPER(MID(W94,4,1))="H","HUF",IF(UPPER(MID(W94,4,1))="C","Company",IF(UPPER(MID(W94,4,1))="F","Firm",IF(UPPER(MID(W94,4,1))="L","LLP",IF(UPPER(MID(W94,4,1))="T","Trust",IF(UPPER(MID(W94,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B94="Entry",IF(LEN(W94)&lt;4,"",IF(UPPER(MID(W94,4,1))="P","Individual",IF(UPPER(MID(W94,4,1))="H","HUF",IF(UPPER(MID(W94,4,1))="C","Company",IF(UPPER(MID(W94,4,1))="F","Firm",IF(UPPER(MID(W94,4,1))="L","LLP",IF(UPPER(MID(W94,4,1))="T","Trust",IF(UPPER(MID(W94,4,1))="A","AOP","")))))))),IF($B94="Challan","",IF(W94&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z94" s="28"/>
       <c r="AA94" s="29">
@@ -10120,10 +10120,10 @@
       <c r="V95" s="28"/>
       <c r="W95" s="28"/>
       <c r="X95" s="23">
-        <f>IF($B95&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W95)))=10,CODE(MID(TRIM(UPPER(W95)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W95)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W95)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W95)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B95="Entry",IF(AND(LEN(TRIM(UPPER(W95)))=10,CODE(MID(TRIM(UPPER(W95)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W95)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W95)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W95)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W95)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W95)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W95)),9,1))&lt;=57),"N","Y"),IF($B95="Challan","",IF(W95&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y95" s="23">
-        <f>IF($B95&lt;&gt;"Entry","",IF(LEN(W95)&lt;4,"",IF(UPPER(MID(W95,4,1))="P","Individual",IF(UPPER(MID(W95,4,1))="H","HUF",IF(UPPER(MID(W95,4,1))="C","Company",IF(UPPER(MID(W95,4,1))="F","Firm",IF(UPPER(MID(W95,4,1))="L","LLP",IF(UPPER(MID(W95,4,1))="T","Trust",IF(UPPER(MID(W95,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B95="Entry",IF(LEN(W95)&lt;4,"",IF(UPPER(MID(W95,4,1))="P","Individual",IF(UPPER(MID(W95,4,1))="H","HUF",IF(UPPER(MID(W95,4,1))="C","Company",IF(UPPER(MID(W95,4,1))="F","Firm",IF(UPPER(MID(W95,4,1))="L","LLP",IF(UPPER(MID(W95,4,1))="T","Trust",IF(UPPER(MID(W95,4,1))="A","AOP","")))))))),IF($B95="Challan","",IF(W95&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z95" s="28"/>
       <c r="AA95" s="29">
@@ -10198,10 +10198,10 @@
       <c r="V96" s="28"/>
       <c r="W96" s="28"/>
       <c r="X96" s="23">
-        <f>IF($B96&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W96)))=10,CODE(MID(TRIM(UPPER(W96)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W96)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W96)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W96)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B96="Entry",IF(AND(LEN(TRIM(UPPER(W96)))=10,CODE(MID(TRIM(UPPER(W96)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W96)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W96)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W96)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W96)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W96)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W96)),9,1))&lt;=57),"N","Y"),IF($B96="Challan","",IF(W96&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y96" s="23">
-        <f>IF($B96&lt;&gt;"Entry","",IF(LEN(W96)&lt;4,"",IF(UPPER(MID(W96,4,1))="P","Individual",IF(UPPER(MID(W96,4,1))="H","HUF",IF(UPPER(MID(W96,4,1))="C","Company",IF(UPPER(MID(W96,4,1))="F","Firm",IF(UPPER(MID(W96,4,1))="L","LLP",IF(UPPER(MID(W96,4,1))="T","Trust",IF(UPPER(MID(W96,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B96="Entry",IF(LEN(W96)&lt;4,"",IF(UPPER(MID(W96,4,1))="P","Individual",IF(UPPER(MID(W96,4,1))="H","HUF",IF(UPPER(MID(W96,4,1))="C","Company",IF(UPPER(MID(W96,4,1))="F","Firm",IF(UPPER(MID(W96,4,1))="L","LLP",IF(UPPER(MID(W96,4,1))="T","Trust",IF(UPPER(MID(W96,4,1))="A","AOP","")))))))),IF($B96="Challan","",IF(W96&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z96" s="28"/>
       <c r="AA96" s="29">
@@ -10276,10 +10276,10 @@
       <c r="V97" s="28"/>
       <c r="W97" s="28"/>
       <c r="X97" s="23">
-        <f>IF($B97&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W97)))=10,CODE(MID(TRIM(UPPER(W97)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W97)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W97)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W97)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B97="Entry",IF(AND(LEN(TRIM(UPPER(W97)))=10,CODE(MID(TRIM(UPPER(W97)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W97)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W97)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W97)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W97)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W97)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W97)),9,1))&lt;=57),"N","Y"),IF($B97="Challan","",IF(W97&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y97" s="23">
-        <f>IF($B97&lt;&gt;"Entry","",IF(LEN(W97)&lt;4,"",IF(UPPER(MID(W97,4,1))="P","Individual",IF(UPPER(MID(W97,4,1))="H","HUF",IF(UPPER(MID(W97,4,1))="C","Company",IF(UPPER(MID(W97,4,1))="F","Firm",IF(UPPER(MID(W97,4,1))="L","LLP",IF(UPPER(MID(W97,4,1))="T","Trust",IF(UPPER(MID(W97,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B97="Entry",IF(LEN(W97)&lt;4,"",IF(UPPER(MID(W97,4,1))="P","Individual",IF(UPPER(MID(W97,4,1))="H","HUF",IF(UPPER(MID(W97,4,1))="C","Company",IF(UPPER(MID(W97,4,1))="F","Firm",IF(UPPER(MID(W97,4,1))="L","LLP",IF(UPPER(MID(W97,4,1))="T","Trust",IF(UPPER(MID(W97,4,1))="A","AOP","")))))))),IF($B97="Challan","",IF(W97&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z97" s="28"/>
       <c r="AA97" s="29">
@@ -10354,10 +10354,10 @@
       <c r="V98" s="28"/>
       <c r="W98" s="28"/>
       <c r="X98" s="23">
-        <f>IF($B98&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W98)))=10,CODE(MID(TRIM(UPPER(W98)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W98)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W98)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W98)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B98="Entry",IF(AND(LEN(TRIM(UPPER(W98)))=10,CODE(MID(TRIM(UPPER(W98)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W98)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W98)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W98)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W98)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W98)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W98)),9,1))&lt;=57),"N","Y"),IF($B98="Challan","",IF(W98&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y98" s="23">
-        <f>IF($B98&lt;&gt;"Entry","",IF(LEN(W98)&lt;4,"",IF(UPPER(MID(W98,4,1))="P","Individual",IF(UPPER(MID(W98,4,1))="H","HUF",IF(UPPER(MID(W98,4,1))="C","Company",IF(UPPER(MID(W98,4,1))="F","Firm",IF(UPPER(MID(W98,4,1))="L","LLP",IF(UPPER(MID(W98,4,1))="T","Trust",IF(UPPER(MID(W98,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B98="Entry",IF(LEN(W98)&lt;4,"",IF(UPPER(MID(W98,4,1))="P","Individual",IF(UPPER(MID(W98,4,1))="H","HUF",IF(UPPER(MID(W98,4,1))="C","Company",IF(UPPER(MID(W98,4,1))="F","Firm",IF(UPPER(MID(W98,4,1))="L","LLP",IF(UPPER(MID(W98,4,1))="T","Trust",IF(UPPER(MID(W98,4,1))="A","AOP","")))))))),IF($B98="Challan","",IF(W98&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z98" s="28"/>
       <c r="AA98" s="29">
@@ -10432,10 +10432,10 @@
       <c r="V99" s="28"/>
       <c r="W99" s="28"/>
       <c r="X99" s="23">
-        <f>IF($B99&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W99)))=10,CODE(MID(TRIM(UPPER(W99)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W99)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W99)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W99)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B99="Entry",IF(AND(LEN(TRIM(UPPER(W99)))=10,CODE(MID(TRIM(UPPER(W99)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W99)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W99)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W99)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W99)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W99)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W99)),9,1))&lt;=57),"N","Y"),IF($B99="Challan","",IF(W99&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y99" s="23">
-        <f>IF($B99&lt;&gt;"Entry","",IF(LEN(W99)&lt;4,"",IF(UPPER(MID(W99,4,1))="P","Individual",IF(UPPER(MID(W99,4,1))="H","HUF",IF(UPPER(MID(W99,4,1))="C","Company",IF(UPPER(MID(W99,4,1))="F","Firm",IF(UPPER(MID(W99,4,1))="L","LLP",IF(UPPER(MID(W99,4,1))="T","Trust",IF(UPPER(MID(W99,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B99="Entry",IF(LEN(W99)&lt;4,"",IF(UPPER(MID(W99,4,1))="P","Individual",IF(UPPER(MID(W99,4,1))="H","HUF",IF(UPPER(MID(W99,4,1))="C","Company",IF(UPPER(MID(W99,4,1))="F","Firm",IF(UPPER(MID(W99,4,1))="L","LLP",IF(UPPER(MID(W99,4,1))="T","Trust",IF(UPPER(MID(W99,4,1))="A","AOP","")))))))),IF($B99="Challan","",IF(W99&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z99" s="28"/>
       <c r="AA99" s="29">
@@ -10510,10 +10510,10 @@
       <c r="V100" s="28"/>
       <c r="W100" s="28"/>
       <c r="X100" s="23">
-        <f>IF($B100&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W100)))=10,CODE(MID(TRIM(UPPER(W100)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W100)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W100)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W100)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B100="Entry",IF(AND(LEN(TRIM(UPPER(W100)))=10,CODE(MID(TRIM(UPPER(W100)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W100)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W100)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W100)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W100)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W100)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W100)),9,1))&lt;=57),"N","Y"),IF($B100="Challan","",IF(W100&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y100" s="23">
-        <f>IF($B100&lt;&gt;"Entry","",IF(LEN(W100)&lt;4,"",IF(UPPER(MID(W100,4,1))="P","Individual",IF(UPPER(MID(W100,4,1))="H","HUF",IF(UPPER(MID(W100,4,1))="C","Company",IF(UPPER(MID(W100,4,1))="F","Firm",IF(UPPER(MID(W100,4,1))="L","LLP",IF(UPPER(MID(W100,4,1))="T","Trust",IF(UPPER(MID(W100,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B100="Entry",IF(LEN(W100)&lt;4,"",IF(UPPER(MID(W100,4,1))="P","Individual",IF(UPPER(MID(W100,4,1))="H","HUF",IF(UPPER(MID(W100,4,1))="C","Company",IF(UPPER(MID(W100,4,1))="F","Firm",IF(UPPER(MID(W100,4,1))="L","LLP",IF(UPPER(MID(W100,4,1))="T","Trust",IF(UPPER(MID(W100,4,1))="A","AOP","")))))))),IF($B100="Challan","",IF(W100&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z100" s="28"/>
       <c r="AA100" s="29">
@@ -10588,10 +10588,10 @@
       <c r="V101" s="28"/>
       <c r="W101" s="28"/>
       <c r="X101" s="23">
-        <f>IF($B101&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W101)))=10,CODE(MID(TRIM(UPPER(W101)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W101)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W101)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W101)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B101="Entry",IF(AND(LEN(TRIM(UPPER(W101)))=10,CODE(MID(TRIM(UPPER(W101)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W101)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W101)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W101)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W101)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W101)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W101)),9,1))&lt;=57),"N","Y"),IF($B101="Challan","",IF(W101&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y101" s="23">
-        <f>IF($B101&lt;&gt;"Entry","",IF(LEN(W101)&lt;4,"",IF(UPPER(MID(W101,4,1))="P","Individual",IF(UPPER(MID(W101,4,1))="H","HUF",IF(UPPER(MID(W101,4,1))="C","Company",IF(UPPER(MID(W101,4,1))="F","Firm",IF(UPPER(MID(W101,4,1))="L","LLP",IF(UPPER(MID(W101,4,1))="T","Trust",IF(UPPER(MID(W101,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B101="Entry",IF(LEN(W101)&lt;4,"",IF(UPPER(MID(W101,4,1))="P","Individual",IF(UPPER(MID(W101,4,1))="H","HUF",IF(UPPER(MID(W101,4,1))="C","Company",IF(UPPER(MID(W101,4,1))="F","Firm",IF(UPPER(MID(W101,4,1))="L","LLP",IF(UPPER(MID(W101,4,1))="T","Trust",IF(UPPER(MID(W101,4,1))="A","AOP","")))))))),IF($B101="Challan","",IF(W101&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z101" s="28"/>
       <c r="AA101" s="29">
@@ -10666,10 +10666,10 @@
       <c r="V102" s="28"/>
       <c r="W102" s="28"/>
       <c r="X102" s="23">
-        <f>IF($B102&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W102)))=10,CODE(MID(TRIM(UPPER(W102)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W102)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W102)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W102)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B102="Entry",IF(AND(LEN(TRIM(UPPER(W102)))=10,CODE(MID(TRIM(UPPER(W102)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W102)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W102)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W102)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W102)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W102)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W102)),9,1))&lt;=57),"N","Y"),IF($B102="Challan","",IF(W102&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y102" s="23">
-        <f>IF($B102&lt;&gt;"Entry","",IF(LEN(W102)&lt;4,"",IF(UPPER(MID(W102,4,1))="P","Individual",IF(UPPER(MID(W102,4,1))="H","HUF",IF(UPPER(MID(W102,4,1))="C","Company",IF(UPPER(MID(W102,4,1))="F","Firm",IF(UPPER(MID(W102,4,1))="L","LLP",IF(UPPER(MID(W102,4,1))="T","Trust",IF(UPPER(MID(W102,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B102="Entry",IF(LEN(W102)&lt;4,"",IF(UPPER(MID(W102,4,1))="P","Individual",IF(UPPER(MID(W102,4,1))="H","HUF",IF(UPPER(MID(W102,4,1))="C","Company",IF(UPPER(MID(W102,4,1))="F","Firm",IF(UPPER(MID(W102,4,1))="L","LLP",IF(UPPER(MID(W102,4,1))="T","Trust",IF(UPPER(MID(W102,4,1))="A","AOP","")))))))),IF($B102="Challan","",IF(W102&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z102" s="28"/>
       <c r="AA102" s="29">
@@ -10744,10 +10744,10 @@
       <c r="V103" s="28"/>
       <c r="W103" s="28"/>
       <c r="X103" s="23">
-        <f>IF($B103&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W103)))=10,CODE(MID(TRIM(UPPER(W103)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W103)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W103)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W103)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B103="Entry",IF(AND(LEN(TRIM(UPPER(W103)))=10,CODE(MID(TRIM(UPPER(W103)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W103)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W103)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W103)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W103)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W103)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W103)),9,1))&lt;=57),"N","Y"),IF($B103="Challan","",IF(W103&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y103" s="23">
-        <f>IF($B103&lt;&gt;"Entry","",IF(LEN(W103)&lt;4,"",IF(UPPER(MID(W103,4,1))="P","Individual",IF(UPPER(MID(W103,4,1))="H","HUF",IF(UPPER(MID(W103,4,1))="C","Company",IF(UPPER(MID(W103,4,1))="F","Firm",IF(UPPER(MID(W103,4,1))="L","LLP",IF(UPPER(MID(W103,4,1))="T","Trust",IF(UPPER(MID(W103,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B103="Entry",IF(LEN(W103)&lt;4,"",IF(UPPER(MID(W103,4,1))="P","Individual",IF(UPPER(MID(W103,4,1))="H","HUF",IF(UPPER(MID(W103,4,1))="C","Company",IF(UPPER(MID(W103,4,1))="F","Firm",IF(UPPER(MID(W103,4,1))="L","LLP",IF(UPPER(MID(W103,4,1))="T","Trust",IF(UPPER(MID(W103,4,1))="A","AOP","")))))))),IF($B103="Challan","",IF(W103&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z103" s="28"/>
       <c r="AA103" s="29">
@@ -10822,10 +10822,10 @@
       <c r="V104" s="28"/>
       <c r="W104" s="28"/>
       <c r="X104" s="23">
-        <f>IF($B104&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W104)))=10,CODE(MID(TRIM(UPPER(W104)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W104)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W104)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W104)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B104="Entry",IF(AND(LEN(TRIM(UPPER(W104)))=10,CODE(MID(TRIM(UPPER(W104)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W104)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W104)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W104)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W104)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W104)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W104)),9,1))&lt;=57),"N","Y"),IF($B104="Challan","",IF(W104&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y104" s="23">
-        <f>IF($B104&lt;&gt;"Entry","",IF(LEN(W104)&lt;4,"",IF(UPPER(MID(W104,4,1))="P","Individual",IF(UPPER(MID(W104,4,1))="H","HUF",IF(UPPER(MID(W104,4,1))="C","Company",IF(UPPER(MID(W104,4,1))="F","Firm",IF(UPPER(MID(W104,4,1))="L","LLP",IF(UPPER(MID(W104,4,1))="T","Trust",IF(UPPER(MID(W104,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B104="Entry",IF(LEN(W104)&lt;4,"",IF(UPPER(MID(W104,4,1))="P","Individual",IF(UPPER(MID(W104,4,1))="H","HUF",IF(UPPER(MID(W104,4,1))="C","Company",IF(UPPER(MID(W104,4,1))="F","Firm",IF(UPPER(MID(W104,4,1))="L","LLP",IF(UPPER(MID(W104,4,1))="T","Trust",IF(UPPER(MID(W104,4,1))="A","AOP","")))))))),IF($B104="Challan","",IF(W104&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z104" s="28"/>
       <c r="AA104" s="29">
@@ -10900,10 +10900,10 @@
       <c r="V105" s="28"/>
       <c r="W105" s="28"/>
       <c r="X105" s="23">
-        <f>IF($B105&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W105)))=10,CODE(MID(TRIM(UPPER(W105)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W105)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W105)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W105)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B105="Entry",IF(AND(LEN(TRIM(UPPER(W105)))=10,CODE(MID(TRIM(UPPER(W105)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W105)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W105)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W105)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W105)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W105)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W105)),9,1))&lt;=57),"N","Y"),IF($B105="Challan","",IF(W105&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y105" s="23">
-        <f>IF($B105&lt;&gt;"Entry","",IF(LEN(W105)&lt;4,"",IF(UPPER(MID(W105,4,1))="P","Individual",IF(UPPER(MID(W105,4,1))="H","HUF",IF(UPPER(MID(W105,4,1))="C","Company",IF(UPPER(MID(W105,4,1))="F","Firm",IF(UPPER(MID(W105,4,1))="L","LLP",IF(UPPER(MID(W105,4,1))="T","Trust",IF(UPPER(MID(W105,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B105="Entry",IF(LEN(W105)&lt;4,"",IF(UPPER(MID(W105,4,1))="P","Individual",IF(UPPER(MID(W105,4,1))="H","HUF",IF(UPPER(MID(W105,4,1))="C","Company",IF(UPPER(MID(W105,4,1))="F","Firm",IF(UPPER(MID(W105,4,1))="L","LLP",IF(UPPER(MID(W105,4,1))="T","Trust",IF(UPPER(MID(W105,4,1))="A","AOP","")))))))),IF($B105="Challan","",IF(W105&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z105" s="28"/>
       <c r="AA105" s="29">
@@ -10978,10 +10978,10 @@
       <c r="V106" s="28"/>
       <c r="W106" s="28"/>
       <c r="X106" s="23">
-        <f>IF($B106&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W106)))=10,CODE(MID(TRIM(UPPER(W106)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W106)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W106)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W106)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B106="Entry",IF(AND(LEN(TRIM(UPPER(W106)))=10,CODE(MID(TRIM(UPPER(W106)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W106)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W106)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W106)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W106)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W106)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W106)),9,1))&lt;=57),"N","Y"),IF($B106="Challan","",IF(W106&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y106" s="23">
-        <f>IF($B106&lt;&gt;"Entry","",IF(LEN(W106)&lt;4,"",IF(UPPER(MID(W106,4,1))="P","Individual",IF(UPPER(MID(W106,4,1))="H","HUF",IF(UPPER(MID(W106,4,1))="C","Company",IF(UPPER(MID(W106,4,1))="F","Firm",IF(UPPER(MID(W106,4,1))="L","LLP",IF(UPPER(MID(W106,4,1))="T","Trust",IF(UPPER(MID(W106,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B106="Entry",IF(LEN(W106)&lt;4,"",IF(UPPER(MID(W106,4,1))="P","Individual",IF(UPPER(MID(W106,4,1))="H","HUF",IF(UPPER(MID(W106,4,1))="C","Company",IF(UPPER(MID(W106,4,1))="F","Firm",IF(UPPER(MID(W106,4,1))="L","LLP",IF(UPPER(MID(W106,4,1))="T","Trust",IF(UPPER(MID(W106,4,1))="A","AOP","")))))))),IF($B106="Challan","",IF(W106&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z106" s="28"/>
       <c r="AA106" s="29">
@@ -11056,10 +11056,10 @@
       <c r="V107" s="28"/>
       <c r="W107" s="28"/>
       <c r="X107" s="23">
-        <f>IF($B107&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W107)))=10,CODE(MID(TRIM(UPPER(W107)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W107)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W107)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W107)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B107="Entry",IF(AND(LEN(TRIM(UPPER(W107)))=10,CODE(MID(TRIM(UPPER(W107)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W107)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W107)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W107)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W107)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W107)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W107)),9,1))&lt;=57),"N","Y"),IF($B107="Challan","",IF(W107&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y107" s="23">
-        <f>IF($B107&lt;&gt;"Entry","",IF(LEN(W107)&lt;4,"",IF(UPPER(MID(W107,4,1))="P","Individual",IF(UPPER(MID(W107,4,1))="H","HUF",IF(UPPER(MID(W107,4,1))="C","Company",IF(UPPER(MID(W107,4,1))="F","Firm",IF(UPPER(MID(W107,4,1))="L","LLP",IF(UPPER(MID(W107,4,1))="T","Trust",IF(UPPER(MID(W107,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B107="Entry",IF(LEN(W107)&lt;4,"",IF(UPPER(MID(W107,4,1))="P","Individual",IF(UPPER(MID(W107,4,1))="H","HUF",IF(UPPER(MID(W107,4,1))="C","Company",IF(UPPER(MID(W107,4,1))="F","Firm",IF(UPPER(MID(W107,4,1))="L","LLP",IF(UPPER(MID(W107,4,1))="T","Trust",IF(UPPER(MID(W107,4,1))="A","AOP","")))))))),IF($B107="Challan","",IF(W107&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z107" s="28"/>
       <c r="AA107" s="29">
@@ -11134,10 +11134,10 @@
       <c r="V108" s="28"/>
       <c r="W108" s="28"/>
       <c r="X108" s="23">
-        <f>IF($B108&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W108)))=10,CODE(MID(TRIM(UPPER(W108)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W108)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W108)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W108)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B108="Entry",IF(AND(LEN(TRIM(UPPER(W108)))=10,CODE(MID(TRIM(UPPER(W108)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W108)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W108)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W108)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W108)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W108)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W108)),9,1))&lt;=57),"N","Y"),IF($B108="Challan","",IF(W108&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y108" s="23">
-        <f>IF($B108&lt;&gt;"Entry","",IF(LEN(W108)&lt;4,"",IF(UPPER(MID(W108,4,1))="P","Individual",IF(UPPER(MID(W108,4,1))="H","HUF",IF(UPPER(MID(W108,4,1))="C","Company",IF(UPPER(MID(W108,4,1))="F","Firm",IF(UPPER(MID(W108,4,1))="L","LLP",IF(UPPER(MID(W108,4,1))="T","Trust",IF(UPPER(MID(W108,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B108="Entry",IF(LEN(W108)&lt;4,"",IF(UPPER(MID(W108,4,1))="P","Individual",IF(UPPER(MID(W108,4,1))="H","HUF",IF(UPPER(MID(W108,4,1))="C","Company",IF(UPPER(MID(W108,4,1))="F","Firm",IF(UPPER(MID(W108,4,1))="L","LLP",IF(UPPER(MID(W108,4,1))="T","Trust",IF(UPPER(MID(W108,4,1))="A","AOP","")))))))),IF($B108="Challan","",IF(W108&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z108" s="28"/>
       <c r="AA108" s="29">
@@ -11212,10 +11212,10 @@
       <c r="V109" s="28"/>
       <c r="W109" s="28"/>
       <c r="X109" s="23">
-        <f>IF($B109&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W109)))=10,CODE(MID(TRIM(UPPER(W109)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W109)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W109)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W109)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B109="Entry",IF(AND(LEN(TRIM(UPPER(W109)))=10,CODE(MID(TRIM(UPPER(W109)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W109)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W109)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W109)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W109)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W109)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W109)),9,1))&lt;=57),"N","Y"),IF($B109="Challan","",IF(W109&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y109" s="23">
-        <f>IF($B109&lt;&gt;"Entry","",IF(LEN(W109)&lt;4,"",IF(UPPER(MID(W109,4,1))="P","Individual",IF(UPPER(MID(W109,4,1))="H","HUF",IF(UPPER(MID(W109,4,1))="C","Company",IF(UPPER(MID(W109,4,1))="F","Firm",IF(UPPER(MID(W109,4,1))="L","LLP",IF(UPPER(MID(W109,4,1))="T","Trust",IF(UPPER(MID(W109,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B109="Entry",IF(LEN(W109)&lt;4,"",IF(UPPER(MID(W109,4,1))="P","Individual",IF(UPPER(MID(W109,4,1))="H","HUF",IF(UPPER(MID(W109,4,1))="C","Company",IF(UPPER(MID(W109,4,1))="F","Firm",IF(UPPER(MID(W109,4,1))="L","LLP",IF(UPPER(MID(W109,4,1))="T","Trust",IF(UPPER(MID(W109,4,1))="A","AOP","")))))))),IF($B109="Challan","",IF(W109&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z109" s="28"/>
       <c r="AA109" s="29">
@@ -11290,10 +11290,10 @@
       <c r="V110" s="28"/>
       <c r="W110" s="28"/>
       <c r="X110" s="23">
-        <f>IF($B110&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W110)))=10,CODE(MID(TRIM(UPPER(W110)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W110)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W110)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W110)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B110="Entry",IF(AND(LEN(TRIM(UPPER(W110)))=10,CODE(MID(TRIM(UPPER(W110)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W110)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W110)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W110)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W110)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W110)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W110)),9,1))&lt;=57),"N","Y"),IF($B110="Challan","",IF(W110&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y110" s="23">
-        <f>IF($B110&lt;&gt;"Entry","",IF(LEN(W110)&lt;4,"",IF(UPPER(MID(W110,4,1))="P","Individual",IF(UPPER(MID(W110,4,1))="H","HUF",IF(UPPER(MID(W110,4,1))="C","Company",IF(UPPER(MID(W110,4,1))="F","Firm",IF(UPPER(MID(W110,4,1))="L","LLP",IF(UPPER(MID(W110,4,1))="T","Trust",IF(UPPER(MID(W110,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B110="Entry",IF(LEN(W110)&lt;4,"",IF(UPPER(MID(W110,4,1))="P","Individual",IF(UPPER(MID(W110,4,1))="H","HUF",IF(UPPER(MID(W110,4,1))="C","Company",IF(UPPER(MID(W110,4,1))="F","Firm",IF(UPPER(MID(W110,4,1))="L","LLP",IF(UPPER(MID(W110,4,1))="T","Trust",IF(UPPER(MID(W110,4,1))="A","AOP","")))))))),IF($B110="Challan","",IF(W110&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z110" s="28"/>
       <c r="AA110" s="29">
@@ -11368,10 +11368,10 @@
       <c r="V111" s="28"/>
       <c r="W111" s="28"/>
       <c r="X111" s="23">
-        <f>IF($B111&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W111)))=10,CODE(MID(TRIM(UPPER(W111)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W111)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W111)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W111)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B111="Entry",IF(AND(LEN(TRIM(UPPER(W111)))=10,CODE(MID(TRIM(UPPER(W111)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W111)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W111)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W111)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W111)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W111)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W111)),9,1))&lt;=57),"N","Y"),IF($B111="Challan","",IF(W111&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y111" s="23">
-        <f>IF($B111&lt;&gt;"Entry","",IF(LEN(W111)&lt;4,"",IF(UPPER(MID(W111,4,1))="P","Individual",IF(UPPER(MID(W111,4,1))="H","HUF",IF(UPPER(MID(W111,4,1))="C","Company",IF(UPPER(MID(W111,4,1))="F","Firm",IF(UPPER(MID(W111,4,1))="L","LLP",IF(UPPER(MID(W111,4,1))="T","Trust",IF(UPPER(MID(W111,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B111="Entry",IF(LEN(W111)&lt;4,"",IF(UPPER(MID(W111,4,1))="P","Individual",IF(UPPER(MID(W111,4,1))="H","HUF",IF(UPPER(MID(W111,4,1))="C","Company",IF(UPPER(MID(W111,4,1))="F","Firm",IF(UPPER(MID(W111,4,1))="L","LLP",IF(UPPER(MID(W111,4,1))="T","Trust",IF(UPPER(MID(W111,4,1))="A","AOP","")))))))),IF($B111="Challan","",IF(W111&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z111" s="28"/>
       <c r="AA111" s="29">
@@ -11446,10 +11446,10 @@
       <c r="V112" s="28"/>
       <c r="W112" s="28"/>
       <c r="X112" s="23">
-        <f>IF($B112&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W112)))=10,CODE(MID(TRIM(UPPER(W112)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W112)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W112)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W112)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B112="Entry",IF(AND(LEN(TRIM(UPPER(W112)))=10,CODE(MID(TRIM(UPPER(W112)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W112)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W112)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W112)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W112)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W112)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W112)),9,1))&lt;=57),"N","Y"),IF($B112="Challan","",IF(W112&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y112" s="23">
-        <f>IF($B112&lt;&gt;"Entry","",IF(LEN(W112)&lt;4,"",IF(UPPER(MID(W112,4,1))="P","Individual",IF(UPPER(MID(W112,4,1))="H","HUF",IF(UPPER(MID(W112,4,1))="C","Company",IF(UPPER(MID(W112,4,1))="F","Firm",IF(UPPER(MID(W112,4,1))="L","LLP",IF(UPPER(MID(W112,4,1))="T","Trust",IF(UPPER(MID(W112,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B112="Entry",IF(LEN(W112)&lt;4,"",IF(UPPER(MID(W112,4,1))="P","Individual",IF(UPPER(MID(W112,4,1))="H","HUF",IF(UPPER(MID(W112,4,1))="C","Company",IF(UPPER(MID(W112,4,1))="F","Firm",IF(UPPER(MID(W112,4,1))="L","LLP",IF(UPPER(MID(W112,4,1))="T","Trust",IF(UPPER(MID(W112,4,1))="A","AOP","")))))))),IF($B112="Challan","",IF(W112&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z112" s="28"/>
       <c r="AA112" s="29">
@@ -11524,10 +11524,10 @@
       <c r="V113" s="28"/>
       <c r="W113" s="28"/>
       <c r="X113" s="23">
-        <f>IF($B113&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W113)))=10,CODE(MID(TRIM(UPPER(W113)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W113)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W113)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W113)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B113="Entry",IF(AND(LEN(TRIM(UPPER(W113)))=10,CODE(MID(TRIM(UPPER(W113)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W113)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W113)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W113)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W113)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W113)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W113)),9,1))&lt;=57),"N","Y"),IF($B113="Challan","",IF(W113&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y113" s="23">
-        <f>IF($B113&lt;&gt;"Entry","",IF(LEN(W113)&lt;4,"",IF(UPPER(MID(W113,4,1))="P","Individual",IF(UPPER(MID(W113,4,1))="H","HUF",IF(UPPER(MID(W113,4,1))="C","Company",IF(UPPER(MID(W113,4,1))="F","Firm",IF(UPPER(MID(W113,4,1))="L","LLP",IF(UPPER(MID(W113,4,1))="T","Trust",IF(UPPER(MID(W113,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B113="Entry",IF(LEN(W113)&lt;4,"",IF(UPPER(MID(W113,4,1))="P","Individual",IF(UPPER(MID(W113,4,1))="H","HUF",IF(UPPER(MID(W113,4,1))="C","Company",IF(UPPER(MID(W113,4,1))="F","Firm",IF(UPPER(MID(W113,4,1))="L","LLP",IF(UPPER(MID(W113,4,1))="T","Trust",IF(UPPER(MID(W113,4,1))="A","AOP","")))))))),IF($B113="Challan","",IF(W113&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z113" s="28"/>
       <c r="AA113" s="29">
@@ -11602,10 +11602,10 @@
       <c r="V114" s="28"/>
       <c r="W114" s="28"/>
       <c r="X114" s="23">
-        <f>IF($B114&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W114)))=10,CODE(MID(TRIM(UPPER(W114)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W114)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W114)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W114)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B114="Entry",IF(AND(LEN(TRIM(UPPER(W114)))=10,CODE(MID(TRIM(UPPER(W114)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W114)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W114)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W114)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W114)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W114)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W114)),9,1))&lt;=57),"N","Y"),IF($B114="Challan","",IF(W114&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y114" s="23">
-        <f>IF($B114&lt;&gt;"Entry","",IF(LEN(W114)&lt;4,"",IF(UPPER(MID(W114,4,1))="P","Individual",IF(UPPER(MID(W114,4,1))="H","HUF",IF(UPPER(MID(W114,4,1))="C","Company",IF(UPPER(MID(W114,4,1))="F","Firm",IF(UPPER(MID(W114,4,1))="L","LLP",IF(UPPER(MID(W114,4,1))="T","Trust",IF(UPPER(MID(W114,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B114="Entry",IF(LEN(W114)&lt;4,"",IF(UPPER(MID(W114,4,1))="P","Individual",IF(UPPER(MID(W114,4,1))="H","HUF",IF(UPPER(MID(W114,4,1))="C","Company",IF(UPPER(MID(W114,4,1))="F","Firm",IF(UPPER(MID(W114,4,1))="L","LLP",IF(UPPER(MID(W114,4,1))="T","Trust",IF(UPPER(MID(W114,4,1))="A","AOP","")))))))),IF($B114="Challan","",IF(W114&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z114" s="28"/>
       <c r="AA114" s="29">
@@ -11680,10 +11680,10 @@
       <c r="V115" s="28"/>
       <c r="W115" s="28"/>
       <c r="X115" s="23">
-        <f>IF($B115&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W115)))=10,CODE(MID(TRIM(UPPER(W115)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W115)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W115)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W115)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B115="Entry",IF(AND(LEN(TRIM(UPPER(W115)))=10,CODE(MID(TRIM(UPPER(W115)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W115)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W115)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W115)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W115)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W115)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W115)),9,1))&lt;=57),"N","Y"),IF($B115="Challan","",IF(W115&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y115" s="23">
-        <f>IF($B115&lt;&gt;"Entry","",IF(LEN(W115)&lt;4,"",IF(UPPER(MID(W115,4,1))="P","Individual",IF(UPPER(MID(W115,4,1))="H","HUF",IF(UPPER(MID(W115,4,1))="C","Company",IF(UPPER(MID(W115,4,1))="F","Firm",IF(UPPER(MID(W115,4,1))="L","LLP",IF(UPPER(MID(W115,4,1))="T","Trust",IF(UPPER(MID(W115,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B115="Entry",IF(LEN(W115)&lt;4,"",IF(UPPER(MID(W115,4,1))="P","Individual",IF(UPPER(MID(W115,4,1))="H","HUF",IF(UPPER(MID(W115,4,1))="C","Company",IF(UPPER(MID(W115,4,1))="F","Firm",IF(UPPER(MID(W115,4,1))="L","LLP",IF(UPPER(MID(W115,4,1))="T","Trust",IF(UPPER(MID(W115,4,1))="A","AOP","")))))))),IF($B115="Challan","",IF(W115&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z115" s="28"/>
       <c r="AA115" s="29">
@@ -11758,10 +11758,10 @@
       <c r="V116" s="28"/>
       <c r="W116" s="28"/>
       <c r="X116" s="23">
-        <f>IF($B116&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W116)))=10,CODE(MID(TRIM(UPPER(W116)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W116)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W116)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W116)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B116="Entry",IF(AND(LEN(TRIM(UPPER(W116)))=10,CODE(MID(TRIM(UPPER(W116)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W116)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W116)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W116)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W116)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W116)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W116)),9,1))&lt;=57),"N","Y"),IF($B116="Challan","",IF(W116&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y116" s="23">
-        <f>IF($B116&lt;&gt;"Entry","",IF(LEN(W116)&lt;4,"",IF(UPPER(MID(W116,4,1))="P","Individual",IF(UPPER(MID(W116,4,1))="H","HUF",IF(UPPER(MID(W116,4,1))="C","Company",IF(UPPER(MID(W116,4,1))="F","Firm",IF(UPPER(MID(W116,4,1))="L","LLP",IF(UPPER(MID(W116,4,1))="T","Trust",IF(UPPER(MID(W116,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B116="Entry",IF(LEN(W116)&lt;4,"",IF(UPPER(MID(W116,4,1))="P","Individual",IF(UPPER(MID(W116,4,1))="H","HUF",IF(UPPER(MID(W116,4,1))="C","Company",IF(UPPER(MID(W116,4,1))="F","Firm",IF(UPPER(MID(W116,4,1))="L","LLP",IF(UPPER(MID(W116,4,1))="T","Trust",IF(UPPER(MID(W116,4,1))="A","AOP","")))))))),IF($B116="Challan","",IF(W116&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z116" s="28"/>
       <c r="AA116" s="29">
@@ -11836,10 +11836,10 @@
       <c r="V117" s="28"/>
       <c r="W117" s="28"/>
       <c r="X117" s="23">
-        <f>IF($B117&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W117)))=10,CODE(MID(TRIM(UPPER(W117)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W117)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W117)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W117)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B117="Entry",IF(AND(LEN(TRIM(UPPER(W117)))=10,CODE(MID(TRIM(UPPER(W117)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W117)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W117)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W117)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W117)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W117)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W117)),9,1))&lt;=57),"N","Y"),IF($B117="Challan","",IF(W117&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y117" s="23">
-        <f>IF($B117&lt;&gt;"Entry","",IF(LEN(W117)&lt;4,"",IF(UPPER(MID(W117,4,1))="P","Individual",IF(UPPER(MID(W117,4,1))="H","HUF",IF(UPPER(MID(W117,4,1))="C","Company",IF(UPPER(MID(W117,4,1))="F","Firm",IF(UPPER(MID(W117,4,1))="L","LLP",IF(UPPER(MID(W117,4,1))="T","Trust",IF(UPPER(MID(W117,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B117="Entry",IF(LEN(W117)&lt;4,"",IF(UPPER(MID(W117,4,1))="P","Individual",IF(UPPER(MID(W117,4,1))="H","HUF",IF(UPPER(MID(W117,4,1))="C","Company",IF(UPPER(MID(W117,4,1))="F","Firm",IF(UPPER(MID(W117,4,1))="L","LLP",IF(UPPER(MID(W117,4,1))="T","Trust",IF(UPPER(MID(W117,4,1))="A","AOP","")))))))),IF($B117="Challan","",IF(W117&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z117" s="28"/>
       <c r="AA117" s="29">
@@ -11914,10 +11914,10 @@
       <c r="V118" s="28"/>
       <c r="W118" s="28"/>
       <c r="X118" s="23">
-        <f>IF($B118&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W118)))=10,CODE(MID(TRIM(UPPER(W118)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W118)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W118)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W118)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B118="Entry",IF(AND(LEN(TRIM(UPPER(W118)))=10,CODE(MID(TRIM(UPPER(W118)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W118)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W118)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W118)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W118)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W118)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W118)),9,1))&lt;=57),"N","Y"),IF($B118="Challan","",IF(W118&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y118" s="23">
-        <f>IF($B118&lt;&gt;"Entry","",IF(LEN(W118)&lt;4,"",IF(UPPER(MID(W118,4,1))="P","Individual",IF(UPPER(MID(W118,4,1))="H","HUF",IF(UPPER(MID(W118,4,1))="C","Company",IF(UPPER(MID(W118,4,1))="F","Firm",IF(UPPER(MID(W118,4,1))="L","LLP",IF(UPPER(MID(W118,4,1))="T","Trust",IF(UPPER(MID(W118,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B118="Entry",IF(LEN(W118)&lt;4,"",IF(UPPER(MID(W118,4,1))="P","Individual",IF(UPPER(MID(W118,4,1))="H","HUF",IF(UPPER(MID(W118,4,1))="C","Company",IF(UPPER(MID(W118,4,1))="F","Firm",IF(UPPER(MID(W118,4,1))="L","LLP",IF(UPPER(MID(W118,4,1))="T","Trust",IF(UPPER(MID(W118,4,1))="A","AOP","")))))))),IF($B118="Challan","",IF(W118&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z118" s="28"/>
       <c r="AA118" s="29">
@@ -11992,10 +11992,10 @@
       <c r="V119" s="28"/>
       <c r="W119" s="28"/>
       <c r="X119" s="23">
-        <f>IF($B119&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W119)))=10,CODE(MID(TRIM(UPPER(W119)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W119)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W119)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W119)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B119="Entry",IF(AND(LEN(TRIM(UPPER(W119)))=10,CODE(MID(TRIM(UPPER(W119)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W119)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W119)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W119)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W119)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W119)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W119)),9,1))&lt;=57),"N","Y"),IF($B119="Challan","",IF(W119&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y119" s="23">
-        <f>IF($B119&lt;&gt;"Entry","",IF(LEN(W119)&lt;4,"",IF(UPPER(MID(W119,4,1))="P","Individual",IF(UPPER(MID(W119,4,1))="H","HUF",IF(UPPER(MID(W119,4,1))="C","Company",IF(UPPER(MID(W119,4,1))="F","Firm",IF(UPPER(MID(W119,4,1))="L","LLP",IF(UPPER(MID(W119,4,1))="T","Trust",IF(UPPER(MID(W119,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B119="Entry",IF(LEN(W119)&lt;4,"",IF(UPPER(MID(W119,4,1))="P","Individual",IF(UPPER(MID(W119,4,1))="H","HUF",IF(UPPER(MID(W119,4,1))="C","Company",IF(UPPER(MID(W119,4,1))="F","Firm",IF(UPPER(MID(W119,4,1))="L","LLP",IF(UPPER(MID(W119,4,1))="T","Trust",IF(UPPER(MID(W119,4,1))="A","AOP","")))))))),IF($B119="Challan","",IF(W119&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z119" s="28"/>
       <c r="AA119" s="29">
@@ -12070,10 +12070,10 @@
       <c r="V120" s="28"/>
       <c r="W120" s="28"/>
       <c r="X120" s="23">
-        <f>IF($B120&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W120)))=10,CODE(MID(TRIM(UPPER(W120)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W120)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W120)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W120)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B120="Entry",IF(AND(LEN(TRIM(UPPER(W120)))=10,CODE(MID(TRIM(UPPER(W120)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W120)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W120)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W120)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W120)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W120)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W120)),9,1))&lt;=57),"N","Y"),IF($B120="Challan","",IF(W120&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y120" s="23">
-        <f>IF($B120&lt;&gt;"Entry","",IF(LEN(W120)&lt;4,"",IF(UPPER(MID(W120,4,1))="P","Individual",IF(UPPER(MID(W120,4,1))="H","HUF",IF(UPPER(MID(W120,4,1))="C","Company",IF(UPPER(MID(W120,4,1))="F","Firm",IF(UPPER(MID(W120,4,1))="L","LLP",IF(UPPER(MID(W120,4,1))="T","Trust",IF(UPPER(MID(W120,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B120="Entry",IF(LEN(W120)&lt;4,"",IF(UPPER(MID(W120,4,1))="P","Individual",IF(UPPER(MID(W120,4,1))="H","HUF",IF(UPPER(MID(W120,4,1))="C","Company",IF(UPPER(MID(W120,4,1))="F","Firm",IF(UPPER(MID(W120,4,1))="L","LLP",IF(UPPER(MID(W120,4,1))="T","Trust",IF(UPPER(MID(W120,4,1))="A","AOP","")))))))),IF($B120="Challan","",IF(W120&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z120" s="28"/>
       <c r="AA120" s="29">
@@ -12148,10 +12148,10 @@
       <c r="V121" s="28"/>
       <c r="W121" s="28"/>
       <c r="X121" s="23">
-        <f>IF($B121&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W121)))=10,CODE(MID(TRIM(UPPER(W121)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W121)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W121)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W121)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B121="Entry",IF(AND(LEN(TRIM(UPPER(W121)))=10,CODE(MID(TRIM(UPPER(W121)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W121)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W121)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W121)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W121)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W121)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W121)),9,1))&lt;=57),"N","Y"),IF($B121="Challan","",IF(W121&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y121" s="23">
-        <f>IF($B121&lt;&gt;"Entry","",IF(LEN(W121)&lt;4,"",IF(UPPER(MID(W121,4,1))="P","Individual",IF(UPPER(MID(W121,4,1))="H","HUF",IF(UPPER(MID(W121,4,1))="C","Company",IF(UPPER(MID(W121,4,1))="F","Firm",IF(UPPER(MID(W121,4,1))="L","LLP",IF(UPPER(MID(W121,4,1))="T","Trust",IF(UPPER(MID(W121,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B121="Entry",IF(LEN(W121)&lt;4,"",IF(UPPER(MID(W121,4,1))="P","Individual",IF(UPPER(MID(W121,4,1))="H","HUF",IF(UPPER(MID(W121,4,1))="C","Company",IF(UPPER(MID(W121,4,1))="F","Firm",IF(UPPER(MID(W121,4,1))="L","LLP",IF(UPPER(MID(W121,4,1))="T","Trust",IF(UPPER(MID(W121,4,1))="A","AOP","")))))))),IF($B121="Challan","",IF(W121&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z121" s="28"/>
       <c r="AA121" s="29">
@@ -12226,10 +12226,10 @@
       <c r="V122" s="28"/>
       <c r="W122" s="28"/>
       <c r="X122" s="23">
-        <f>IF($B122&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W122)))=10,CODE(MID(TRIM(UPPER(W122)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W122)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W122)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W122)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B122="Entry",IF(AND(LEN(TRIM(UPPER(W122)))=10,CODE(MID(TRIM(UPPER(W122)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W122)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W122)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W122)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W122)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W122)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W122)),9,1))&lt;=57),"N","Y"),IF($B122="Challan","",IF(W122&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y122" s="23">
-        <f>IF($B122&lt;&gt;"Entry","",IF(LEN(W122)&lt;4,"",IF(UPPER(MID(W122,4,1))="P","Individual",IF(UPPER(MID(W122,4,1))="H","HUF",IF(UPPER(MID(W122,4,1))="C","Company",IF(UPPER(MID(W122,4,1))="F","Firm",IF(UPPER(MID(W122,4,1))="L","LLP",IF(UPPER(MID(W122,4,1))="T","Trust",IF(UPPER(MID(W122,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B122="Entry",IF(LEN(W122)&lt;4,"",IF(UPPER(MID(W122,4,1))="P","Individual",IF(UPPER(MID(W122,4,1))="H","HUF",IF(UPPER(MID(W122,4,1))="C","Company",IF(UPPER(MID(W122,4,1))="F","Firm",IF(UPPER(MID(W122,4,1))="L","LLP",IF(UPPER(MID(W122,4,1))="T","Trust",IF(UPPER(MID(W122,4,1))="A","AOP","")))))))),IF($B122="Challan","",IF(W122&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z122" s="28"/>
       <c r="AA122" s="29">
@@ -12304,10 +12304,10 @@
       <c r="V123" s="28"/>
       <c r="W123" s="28"/>
       <c r="X123" s="23">
-        <f>IF($B123&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W123)))=10,CODE(MID(TRIM(UPPER(W123)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W123)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W123)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W123)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B123="Entry",IF(AND(LEN(TRIM(UPPER(W123)))=10,CODE(MID(TRIM(UPPER(W123)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W123)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W123)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W123)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W123)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W123)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W123)),9,1))&lt;=57),"N","Y"),IF($B123="Challan","",IF(W123&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y123" s="23">
-        <f>IF($B123&lt;&gt;"Entry","",IF(LEN(W123)&lt;4,"",IF(UPPER(MID(W123,4,1))="P","Individual",IF(UPPER(MID(W123,4,1))="H","HUF",IF(UPPER(MID(W123,4,1))="C","Company",IF(UPPER(MID(W123,4,1))="F","Firm",IF(UPPER(MID(W123,4,1))="L","LLP",IF(UPPER(MID(W123,4,1))="T","Trust",IF(UPPER(MID(W123,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B123="Entry",IF(LEN(W123)&lt;4,"",IF(UPPER(MID(W123,4,1))="P","Individual",IF(UPPER(MID(W123,4,1))="H","HUF",IF(UPPER(MID(W123,4,1))="C","Company",IF(UPPER(MID(W123,4,1))="F","Firm",IF(UPPER(MID(W123,4,1))="L","LLP",IF(UPPER(MID(W123,4,1))="T","Trust",IF(UPPER(MID(W123,4,1))="A","AOP","")))))))),IF($B123="Challan","",IF(W123&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z123" s="28"/>
       <c r="AA123" s="29">
@@ -12382,10 +12382,10 @@
       <c r="V124" s="28"/>
       <c r="W124" s="28"/>
       <c r="X124" s="23">
-        <f>IF($B124&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W124)))=10,CODE(MID(TRIM(UPPER(W124)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W124)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W124)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W124)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B124="Entry",IF(AND(LEN(TRIM(UPPER(W124)))=10,CODE(MID(TRIM(UPPER(W124)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W124)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W124)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W124)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W124)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W124)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W124)),9,1))&lt;=57),"N","Y"),IF($B124="Challan","",IF(W124&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y124" s="23">
-        <f>IF($B124&lt;&gt;"Entry","",IF(LEN(W124)&lt;4,"",IF(UPPER(MID(W124,4,1))="P","Individual",IF(UPPER(MID(W124,4,1))="H","HUF",IF(UPPER(MID(W124,4,1))="C","Company",IF(UPPER(MID(W124,4,1))="F","Firm",IF(UPPER(MID(W124,4,1))="L","LLP",IF(UPPER(MID(W124,4,1))="T","Trust",IF(UPPER(MID(W124,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B124="Entry",IF(LEN(W124)&lt;4,"",IF(UPPER(MID(W124,4,1))="P","Individual",IF(UPPER(MID(W124,4,1))="H","HUF",IF(UPPER(MID(W124,4,1))="C","Company",IF(UPPER(MID(W124,4,1))="F","Firm",IF(UPPER(MID(W124,4,1))="L","LLP",IF(UPPER(MID(W124,4,1))="T","Trust",IF(UPPER(MID(W124,4,1))="A","AOP","")))))))),IF($B124="Challan","",IF(W124&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z124" s="28"/>
       <c r="AA124" s="29">
@@ -12460,10 +12460,10 @@
       <c r="V125" s="28"/>
       <c r="W125" s="28"/>
       <c r="X125" s="23">
-        <f>IF($B125&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W125)))=10,CODE(MID(TRIM(UPPER(W125)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W125)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W125)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W125)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B125="Entry",IF(AND(LEN(TRIM(UPPER(W125)))=10,CODE(MID(TRIM(UPPER(W125)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W125)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W125)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W125)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W125)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W125)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W125)),9,1))&lt;=57),"N","Y"),IF($B125="Challan","",IF(W125&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y125" s="23">
-        <f>IF($B125&lt;&gt;"Entry","",IF(LEN(W125)&lt;4,"",IF(UPPER(MID(W125,4,1))="P","Individual",IF(UPPER(MID(W125,4,1))="H","HUF",IF(UPPER(MID(W125,4,1))="C","Company",IF(UPPER(MID(W125,4,1))="F","Firm",IF(UPPER(MID(W125,4,1))="L","LLP",IF(UPPER(MID(W125,4,1))="T","Trust",IF(UPPER(MID(W125,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B125="Entry",IF(LEN(W125)&lt;4,"",IF(UPPER(MID(W125,4,1))="P","Individual",IF(UPPER(MID(W125,4,1))="H","HUF",IF(UPPER(MID(W125,4,1))="C","Company",IF(UPPER(MID(W125,4,1))="F","Firm",IF(UPPER(MID(W125,4,1))="L","LLP",IF(UPPER(MID(W125,4,1))="T","Trust",IF(UPPER(MID(W125,4,1))="A","AOP","")))))))),IF($B125="Challan","",IF(W125&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z125" s="28"/>
       <c r="AA125" s="29">
@@ -12538,10 +12538,10 @@
       <c r="V126" s="28"/>
       <c r="W126" s="28"/>
       <c r="X126" s="23">
-        <f>IF($B126&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W126)))=10,CODE(MID(TRIM(UPPER(W126)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W126)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W126)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W126)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B126="Entry",IF(AND(LEN(TRIM(UPPER(W126)))=10,CODE(MID(TRIM(UPPER(W126)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W126)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W126)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W126)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W126)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W126)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W126)),9,1))&lt;=57),"N","Y"),IF($B126="Challan","",IF(W126&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y126" s="23">
-        <f>IF($B126&lt;&gt;"Entry","",IF(LEN(W126)&lt;4,"",IF(UPPER(MID(W126,4,1))="P","Individual",IF(UPPER(MID(W126,4,1))="H","HUF",IF(UPPER(MID(W126,4,1))="C","Company",IF(UPPER(MID(W126,4,1))="F","Firm",IF(UPPER(MID(W126,4,1))="L","LLP",IF(UPPER(MID(W126,4,1))="T","Trust",IF(UPPER(MID(W126,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B126="Entry",IF(LEN(W126)&lt;4,"",IF(UPPER(MID(W126,4,1))="P","Individual",IF(UPPER(MID(W126,4,1))="H","HUF",IF(UPPER(MID(W126,4,1))="C","Company",IF(UPPER(MID(W126,4,1))="F","Firm",IF(UPPER(MID(W126,4,1))="L","LLP",IF(UPPER(MID(W126,4,1))="T","Trust",IF(UPPER(MID(W126,4,1))="A","AOP","")))))))),IF($B126="Challan","",IF(W126&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z126" s="28"/>
       <c r="AA126" s="29">
@@ -12616,10 +12616,10 @@
       <c r="V127" s="28"/>
       <c r="W127" s="28"/>
       <c r="X127" s="23">
-        <f>IF($B127&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W127)))=10,CODE(MID(TRIM(UPPER(W127)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W127)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W127)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W127)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B127="Entry",IF(AND(LEN(TRIM(UPPER(W127)))=10,CODE(MID(TRIM(UPPER(W127)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W127)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W127)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W127)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W127)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W127)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W127)),9,1))&lt;=57),"N","Y"),IF($B127="Challan","",IF(W127&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y127" s="23">
-        <f>IF($B127&lt;&gt;"Entry","",IF(LEN(W127)&lt;4,"",IF(UPPER(MID(W127,4,1))="P","Individual",IF(UPPER(MID(W127,4,1))="H","HUF",IF(UPPER(MID(W127,4,1))="C","Company",IF(UPPER(MID(W127,4,1))="F","Firm",IF(UPPER(MID(W127,4,1))="L","LLP",IF(UPPER(MID(W127,4,1))="T","Trust",IF(UPPER(MID(W127,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B127="Entry",IF(LEN(W127)&lt;4,"",IF(UPPER(MID(W127,4,1))="P","Individual",IF(UPPER(MID(W127,4,1))="H","HUF",IF(UPPER(MID(W127,4,1))="C","Company",IF(UPPER(MID(W127,4,1))="F","Firm",IF(UPPER(MID(W127,4,1))="L","LLP",IF(UPPER(MID(W127,4,1))="T","Trust",IF(UPPER(MID(W127,4,1))="A","AOP","")))))))),IF($B127="Challan","",IF(W127&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z127" s="28"/>
       <c r="AA127" s="29">
@@ -12694,10 +12694,10 @@
       <c r="V128" s="28"/>
       <c r="W128" s="28"/>
       <c r="X128" s="23">
-        <f>IF($B128&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W128)))=10,CODE(MID(TRIM(UPPER(W128)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W128)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W128)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W128)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B128="Entry",IF(AND(LEN(TRIM(UPPER(W128)))=10,CODE(MID(TRIM(UPPER(W128)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W128)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W128)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W128)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W128)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W128)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W128)),9,1))&lt;=57),"N","Y"),IF($B128="Challan","",IF(W128&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y128" s="23">
-        <f>IF($B128&lt;&gt;"Entry","",IF(LEN(W128)&lt;4,"",IF(UPPER(MID(W128,4,1))="P","Individual",IF(UPPER(MID(W128,4,1))="H","HUF",IF(UPPER(MID(W128,4,1))="C","Company",IF(UPPER(MID(W128,4,1))="F","Firm",IF(UPPER(MID(W128,4,1))="L","LLP",IF(UPPER(MID(W128,4,1))="T","Trust",IF(UPPER(MID(W128,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B128="Entry",IF(LEN(W128)&lt;4,"",IF(UPPER(MID(W128,4,1))="P","Individual",IF(UPPER(MID(W128,4,1))="H","HUF",IF(UPPER(MID(W128,4,1))="C","Company",IF(UPPER(MID(W128,4,1))="F","Firm",IF(UPPER(MID(W128,4,1))="L","LLP",IF(UPPER(MID(W128,4,1))="T","Trust",IF(UPPER(MID(W128,4,1))="A","AOP","")))))))),IF($B128="Challan","",IF(W128&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z128" s="28"/>
       <c r="AA128" s="29">
@@ -12772,10 +12772,10 @@
       <c r="V129" s="28"/>
       <c r="W129" s="28"/>
       <c r="X129" s="23">
-        <f>IF($B129&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W129)))=10,CODE(MID(TRIM(UPPER(W129)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W129)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W129)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W129)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B129="Entry",IF(AND(LEN(TRIM(UPPER(W129)))=10,CODE(MID(TRIM(UPPER(W129)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W129)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W129)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W129)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W129)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W129)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W129)),9,1))&lt;=57),"N","Y"),IF($B129="Challan","",IF(W129&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y129" s="23">
-        <f>IF($B129&lt;&gt;"Entry","",IF(LEN(W129)&lt;4,"",IF(UPPER(MID(W129,4,1))="P","Individual",IF(UPPER(MID(W129,4,1))="H","HUF",IF(UPPER(MID(W129,4,1))="C","Company",IF(UPPER(MID(W129,4,1))="F","Firm",IF(UPPER(MID(W129,4,1))="L","LLP",IF(UPPER(MID(W129,4,1))="T","Trust",IF(UPPER(MID(W129,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B129="Entry",IF(LEN(W129)&lt;4,"",IF(UPPER(MID(W129,4,1))="P","Individual",IF(UPPER(MID(W129,4,1))="H","HUF",IF(UPPER(MID(W129,4,1))="C","Company",IF(UPPER(MID(W129,4,1))="F","Firm",IF(UPPER(MID(W129,4,1))="L","LLP",IF(UPPER(MID(W129,4,1))="T","Trust",IF(UPPER(MID(W129,4,1))="A","AOP","")))))))),IF($B129="Challan","",IF(W129&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z129" s="28"/>
       <c r="AA129" s="29">
@@ -12850,10 +12850,10 @@
       <c r="V130" s="28"/>
       <c r="W130" s="28"/>
       <c r="X130" s="23">
-        <f>IF($B130&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W130)))=10,CODE(MID(TRIM(UPPER(W130)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W130)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W130)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W130)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B130="Entry",IF(AND(LEN(TRIM(UPPER(W130)))=10,CODE(MID(TRIM(UPPER(W130)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W130)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W130)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W130)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W130)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W130)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W130)),9,1))&lt;=57),"N","Y"),IF($B130="Challan","",IF(W130&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y130" s="23">
-        <f>IF($B130&lt;&gt;"Entry","",IF(LEN(W130)&lt;4,"",IF(UPPER(MID(W130,4,1))="P","Individual",IF(UPPER(MID(W130,4,1))="H","HUF",IF(UPPER(MID(W130,4,1))="C","Company",IF(UPPER(MID(W130,4,1))="F","Firm",IF(UPPER(MID(W130,4,1))="L","LLP",IF(UPPER(MID(W130,4,1))="T","Trust",IF(UPPER(MID(W130,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B130="Entry",IF(LEN(W130)&lt;4,"",IF(UPPER(MID(W130,4,1))="P","Individual",IF(UPPER(MID(W130,4,1))="H","HUF",IF(UPPER(MID(W130,4,1))="C","Company",IF(UPPER(MID(W130,4,1))="F","Firm",IF(UPPER(MID(W130,4,1))="L","LLP",IF(UPPER(MID(W130,4,1))="T","Trust",IF(UPPER(MID(W130,4,1))="A","AOP","")))))))),IF($B130="Challan","",IF(W130&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z130" s="28"/>
       <c r="AA130" s="29">
@@ -12928,10 +12928,10 @@
       <c r="V131" s="28"/>
       <c r="W131" s="28"/>
       <c r="X131" s="23">
-        <f>IF($B131&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W131)))=10,CODE(MID(TRIM(UPPER(W131)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W131)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W131)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W131)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B131="Entry",IF(AND(LEN(TRIM(UPPER(W131)))=10,CODE(MID(TRIM(UPPER(W131)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W131)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W131)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W131)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W131)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W131)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W131)),9,1))&lt;=57),"N","Y"),IF($B131="Challan","",IF(W131&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y131" s="23">
-        <f>IF($B131&lt;&gt;"Entry","",IF(LEN(W131)&lt;4,"",IF(UPPER(MID(W131,4,1))="P","Individual",IF(UPPER(MID(W131,4,1))="H","HUF",IF(UPPER(MID(W131,4,1))="C","Company",IF(UPPER(MID(W131,4,1))="F","Firm",IF(UPPER(MID(W131,4,1))="L","LLP",IF(UPPER(MID(W131,4,1))="T","Trust",IF(UPPER(MID(W131,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B131="Entry",IF(LEN(W131)&lt;4,"",IF(UPPER(MID(W131,4,1))="P","Individual",IF(UPPER(MID(W131,4,1))="H","HUF",IF(UPPER(MID(W131,4,1))="C","Company",IF(UPPER(MID(W131,4,1))="F","Firm",IF(UPPER(MID(W131,4,1))="L","LLP",IF(UPPER(MID(W131,4,1))="T","Trust",IF(UPPER(MID(W131,4,1))="A","AOP","")))))))),IF($B131="Challan","",IF(W131&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z131" s="28"/>
       <c r="AA131" s="29">
@@ -13006,10 +13006,10 @@
       <c r="V132" s="28"/>
       <c r="W132" s="28"/>
       <c r="X132" s="23">
-        <f>IF($B132&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W132)))=10,CODE(MID(TRIM(UPPER(W132)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W132)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W132)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W132)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B132="Entry",IF(AND(LEN(TRIM(UPPER(W132)))=10,CODE(MID(TRIM(UPPER(W132)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W132)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W132)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W132)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W132)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W132)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W132)),9,1))&lt;=57),"N","Y"),IF($B132="Challan","",IF(W132&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y132" s="23">
-        <f>IF($B132&lt;&gt;"Entry","",IF(LEN(W132)&lt;4,"",IF(UPPER(MID(W132,4,1))="P","Individual",IF(UPPER(MID(W132,4,1))="H","HUF",IF(UPPER(MID(W132,4,1))="C","Company",IF(UPPER(MID(W132,4,1))="F","Firm",IF(UPPER(MID(W132,4,1))="L","LLP",IF(UPPER(MID(W132,4,1))="T","Trust",IF(UPPER(MID(W132,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B132="Entry",IF(LEN(W132)&lt;4,"",IF(UPPER(MID(W132,4,1))="P","Individual",IF(UPPER(MID(W132,4,1))="H","HUF",IF(UPPER(MID(W132,4,1))="C","Company",IF(UPPER(MID(W132,4,1))="F","Firm",IF(UPPER(MID(W132,4,1))="L","LLP",IF(UPPER(MID(W132,4,1))="T","Trust",IF(UPPER(MID(W132,4,1))="A","AOP","")))))))),IF($B132="Challan","",IF(W132&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z132" s="28"/>
       <c r="AA132" s="29">
@@ -13084,10 +13084,10 @@
       <c r="V133" s="28"/>
       <c r="W133" s="28"/>
       <c r="X133" s="23">
-        <f>IF($B133&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W133)))=10,CODE(MID(TRIM(UPPER(W133)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W133)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W133)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W133)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B133="Entry",IF(AND(LEN(TRIM(UPPER(W133)))=10,CODE(MID(TRIM(UPPER(W133)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W133)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W133)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W133)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W133)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W133)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W133)),9,1))&lt;=57),"N","Y"),IF($B133="Challan","",IF(W133&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y133" s="23">
-        <f>IF($B133&lt;&gt;"Entry","",IF(LEN(W133)&lt;4,"",IF(UPPER(MID(W133,4,1))="P","Individual",IF(UPPER(MID(W133,4,1))="H","HUF",IF(UPPER(MID(W133,4,1))="C","Company",IF(UPPER(MID(W133,4,1))="F","Firm",IF(UPPER(MID(W133,4,1))="L","LLP",IF(UPPER(MID(W133,4,1))="T","Trust",IF(UPPER(MID(W133,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B133="Entry",IF(LEN(W133)&lt;4,"",IF(UPPER(MID(W133,4,1))="P","Individual",IF(UPPER(MID(W133,4,1))="H","HUF",IF(UPPER(MID(W133,4,1))="C","Company",IF(UPPER(MID(W133,4,1))="F","Firm",IF(UPPER(MID(W133,4,1))="L","LLP",IF(UPPER(MID(W133,4,1))="T","Trust",IF(UPPER(MID(W133,4,1))="A","AOP","")))))))),IF($B133="Challan","",IF(W133&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z133" s="28"/>
       <c r="AA133" s="29">
@@ -13162,10 +13162,10 @@
       <c r="V134" s="28"/>
       <c r="W134" s="28"/>
       <c r="X134" s="23">
-        <f>IF($B134&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W134)))=10,CODE(MID(TRIM(UPPER(W134)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W134)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W134)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W134)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B134="Entry",IF(AND(LEN(TRIM(UPPER(W134)))=10,CODE(MID(TRIM(UPPER(W134)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W134)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W134)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W134)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W134)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W134)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W134)),9,1))&lt;=57),"N","Y"),IF($B134="Challan","",IF(W134&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y134" s="23">
-        <f>IF($B134&lt;&gt;"Entry","",IF(LEN(W134)&lt;4,"",IF(UPPER(MID(W134,4,1))="P","Individual",IF(UPPER(MID(W134,4,1))="H","HUF",IF(UPPER(MID(W134,4,1))="C","Company",IF(UPPER(MID(W134,4,1))="F","Firm",IF(UPPER(MID(W134,4,1))="L","LLP",IF(UPPER(MID(W134,4,1))="T","Trust",IF(UPPER(MID(W134,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B134="Entry",IF(LEN(W134)&lt;4,"",IF(UPPER(MID(W134,4,1))="P","Individual",IF(UPPER(MID(W134,4,1))="H","HUF",IF(UPPER(MID(W134,4,1))="C","Company",IF(UPPER(MID(W134,4,1))="F","Firm",IF(UPPER(MID(W134,4,1))="L","LLP",IF(UPPER(MID(W134,4,1))="T","Trust",IF(UPPER(MID(W134,4,1))="A","AOP","")))))))),IF($B134="Challan","",IF(W134&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z134" s="28"/>
       <c r="AA134" s="29">
@@ -13240,10 +13240,10 @@
       <c r="V135" s="28"/>
       <c r="W135" s="28"/>
       <c r="X135" s="23">
-        <f>IF($B135&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W135)))=10,CODE(MID(TRIM(UPPER(W135)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W135)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W135)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W135)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B135="Entry",IF(AND(LEN(TRIM(UPPER(W135)))=10,CODE(MID(TRIM(UPPER(W135)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W135)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W135)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W135)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W135)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W135)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W135)),9,1))&lt;=57),"N","Y"),IF($B135="Challan","",IF(W135&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y135" s="23">
-        <f>IF($B135&lt;&gt;"Entry","",IF(LEN(W135)&lt;4,"",IF(UPPER(MID(W135,4,1))="P","Individual",IF(UPPER(MID(W135,4,1))="H","HUF",IF(UPPER(MID(W135,4,1))="C","Company",IF(UPPER(MID(W135,4,1))="F","Firm",IF(UPPER(MID(W135,4,1))="L","LLP",IF(UPPER(MID(W135,4,1))="T","Trust",IF(UPPER(MID(W135,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B135="Entry",IF(LEN(W135)&lt;4,"",IF(UPPER(MID(W135,4,1))="P","Individual",IF(UPPER(MID(W135,4,1))="H","HUF",IF(UPPER(MID(W135,4,1))="C","Company",IF(UPPER(MID(W135,4,1))="F","Firm",IF(UPPER(MID(W135,4,1))="L","LLP",IF(UPPER(MID(W135,4,1))="T","Trust",IF(UPPER(MID(W135,4,1))="A","AOP","")))))))),IF($B135="Challan","",IF(W135&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z135" s="28"/>
       <c r="AA135" s="29">
@@ -13318,10 +13318,10 @@
       <c r="V136" s="28"/>
       <c r="W136" s="28"/>
       <c r="X136" s="23">
-        <f>IF($B136&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W136)))=10,CODE(MID(TRIM(UPPER(W136)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W136)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W136)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W136)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B136="Entry",IF(AND(LEN(TRIM(UPPER(W136)))=10,CODE(MID(TRIM(UPPER(W136)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W136)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W136)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W136)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W136)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W136)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W136)),9,1))&lt;=57),"N","Y"),IF($B136="Challan","",IF(W136&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y136" s="23">
-        <f>IF($B136&lt;&gt;"Entry","",IF(LEN(W136)&lt;4,"",IF(UPPER(MID(W136,4,1))="P","Individual",IF(UPPER(MID(W136,4,1))="H","HUF",IF(UPPER(MID(W136,4,1))="C","Company",IF(UPPER(MID(W136,4,1))="F","Firm",IF(UPPER(MID(W136,4,1))="L","LLP",IF(UPPER(MID(W136,4,1))="T","Trust",IF(UPPER(MID(W136,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B136="Entry",IF(LEN(W136)&lt;4,"",IF(UPPER(MID(W136,4,1))="P","Individual",IF(UPPER(MID(W136,4,1))="H","HUF",IF(UPPER(MID(W136,4,1))="C","Company",IF(UPPER(MID(W136,4,1))="F","Firm",IF(UPPER(MID(W136,4,1))="L","LLP",IF(UPPER(MID(W136,4,1))="T","Trust",IF(UPPER(MID(W136,4,1))="A","AOP","")))))))),IF($B136="Challan","",IF(W136&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z136" s="28"/>
       <c r="AA136" s="29">
@@ -13396,10 +13396,10 @@
       <c r="V137" s="28"/>
       <c r="W137" s="28"/>
       <c r="X137" s="23">
-        <f>IF($B137&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W137)))=10,CODE(MID(TRIM(UPPER(W137)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W137)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W137)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W137)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B137="Entry",IF(AND(LEN(TRIM(UPPER(W137)))=10,CODE(MID(TRIM(UPPER(W137)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W137)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W137)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W137)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W137)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W137)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W137)),9,1))&lt;=57),"N","Y"),IF($B137="Challan","",IF(W137&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y137" s="23">
-        <f>IF($B137&lt;&gt;"Entry","",IF(LEN(W137)&lt;4,"",IF(UPPER(MID(W137,4,1))="P","Individual",IF(UPPER(MID(W137,4,1))="H","HUF",IF(UPPER(MID(W137,4,1))="C","Company",IF(UPPER(MID(W137,4,1))="F","Firm",IF(UPPER(MID(W137,4,1))="L","LLP",IF(UPPER(MID(W137,4,1))="T","Trust",IF(UPPER(MID(W137,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B137="Entry",IF(LEN(W137)&lt;4,"",IF(UPPER(MID(W137,4,1))="P","Individual",IF(UPPER(MID(W137,4,1))="H","HUF",IF(UPPER(MID(W137,4,1))="C","Company",IF(UPPER(MID(W137,4,1))="F","Firm",IF(UPPER(MID(W137,4,1))="L","LLP",IF(UPPER(MID(W137,4,1))="T","Trust",IF(UPPER(MID(W137,4,1))="A","AOP","")))))))),IF($B137="Challan","",IF(W137&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z137" s="28"/>
       <c r="AA137" s="29">
@@ -13474,10 +13474,10 @@
       <c r="V138" s="28"/>
       <c r="W138" s="28"/>
       <c r="X138" s="23">
-        <f>IF($B138&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W138)))=10,CODE(MID(TRIM(UPPER(W138)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W138)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W138)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W138)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B138="Entry",IF(AND(LEN(TRIM(UPPER(W138)))=10,CODE(MID(TRIM(UPPER(W138)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W138)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W138)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W138)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W138)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W138)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W138)),9,1))&lt;=57),"N","Y"),IF($B138="Challan","",IF(W138&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y138" s="23">
-        <f>IF($B138&lt;&gt;"Entry","",IF(LEN(W138)&lt;4,"",IF(UPPER(MID(W138,4,1))="P","Individual",IF(UPPER(MID(W138,4,1))="H","HUF",IF(UPPER(MID(W138,4,1))="C","Company",IF(UPPER(MID(W138,4,1))="F","Firm",IF(UPPER(MID(W138,4,1))="L","LLP",IF(UPPER(MID(W138,4,1))="T","Trust",IF(UPPER(MID(W138,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B138="Entry",IF(LEN(W138)&lt;4,"",IF(UPPER(MID(W138,4,1))="P","Individual",IF(UPPER(MID(W138,4,1))="H","HUF",IF(UPPER(MID(W138,4,1))="C","Company",IF(UPPER(MID(W138,4,1))="F","Firm",IF(UPPER(MID(W138,4,1))="L","LLP",IF(UPPER(MID(W138,4,1))="T","Trust",IF(UPPER(MID(W138,4,1))="A","AOP","")))))))),IF($B138="Challan","",IF(W138&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z138" s="28"/>
       <c r="AA138" s="29">
@@ -13552,10 +13552,10 @@
       <c r="V139" s="28"/>
       <c r="W139" s="28"/>
       <c r="X139" s="23">
-        <f>IF($B139&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W139)))=10,CODE(MID(TRIM(UPPER(W139)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W139)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W139)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W139)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B139="Entry",IF(AND(LEN(TRIM(UPPER(W139)))=10,CODE(MID(TRIM(UPPER(W139)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W139)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W139)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W139)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W139)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W139)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W139)),9,1))&lt;=57),"N","Y"),IF($B139="Challan","",IF(W139&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y139" s="23">
-        <f>IF($B139&lt;&gt;"Entry","",IF(LEN(W139)&lt;4,"",IF(UPPER(MID(W139,4,1))="P","Individual",IF(UPPER(MID(W139,4,1))="H","HUF",IF(UPPER(MID(W139,4,1))="C","Company",IF(UPPER(MID(W139,4,1))="F","Firm",IF(UPPER(MID(W139,4,1))="L","LLP",IF(UPPER(MID(W139,4,1))="T","Trust",IF(UPPER(MID(W139,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B139="Entry",IF(LEN(W139)&lt;4,"",IF(UPPER(MID(W139,4,1))="P","Individual",IF(UPPER(MID(W139,4,1))="H","HUF",IF(UPPER(MID(W139,4,1))="C","Company",IF(UPPER(MID(W139,4,1))="F","Firm",IF(UPPER(MID(W139,4,1))="L","LLP",IF(UPPER(MID(W139,4,1))="T","Trust",IF(UPPER(MID(W139,4,1))="A","AOP","")))))))),IF($B139="Challan","",IF(W139&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z139" s="28"/>
       <c r="AA139" s="29">
@@ -13630,10 +13630,10 @@
       <c r="V140" s="28"/>
       <c r="W140" s="28"/>
       <c r="X140" s="23">
-        <f>IF($B140&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W140)))=10,CODE(MID(TRIM(UPPER(W140)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W140)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W140)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W140)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B140="Entry",IF(AND(LEN(TRIM(UPPER(W140)))=10,CODE(MID(TRIM(UPPER(W140)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W140)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W140)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W140)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W140)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W140)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W140)),9,1))&lt;=57),"N","Y"),IF($B140="Challan","",IF(W140&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y140" s="23">
-        <f>IF($B140&lt;&gt;"Entry","",IF(LEN(W140)&lt;4,"",IF(UPPER(MID(W140,4,1))="P","Individual",IF(UPPER(MID(W140,4,1))="H","HUF",IF(UPPER(MID(W140,4,1))="C","Company",IF(UPPER(MID(W140,4,1))="F","Firm",IF(UPPER(MID(W140,4,1))="L","LLP",IF(UPPER(MID(W140,4,1))="T","Trust",IF(UPPER(MID(W140,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B140="Entry",IF(LEN(W140)&lt;4,"",IF(UPPER(MID(W140,4,1))="P","Individual",IF(UPPER(MID(W140,4,1))="H","HUF",IF(UPPER(MID(W140,4,1))="C","Company",IF(UPPER(MID(W140,4,1))="F","Firm",IF(UPPER(MID(W140,4,1))="L","LLP",IF(UPPER(MID(W140,4,1))="T","Trust",IF(UPPER(MID(W140,4,1))="A","AOP","")))))))),IF($B140="Challan","",IF(W140&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z140" s="28"/>
       <c r="AA140" s="29">
@@ -13708,10 +13708,10 @@
       <c r="V141" s="28"/>
       <c r="W141" s="28"/>
       <c r="X141" s="23">
-        <f>IF($B141&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W141)))=10,CODE(MID(TRIM(UPPER(W141)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W141)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W141)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W141)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B141="Entry",IF(AND(LEN(TRIM(UPPER(W141)))=10,CODE(MID(TRIM(UPPER(W141)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W141)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W141)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W141)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W141)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W141)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W141)),9,1))&lt;=57),"N","Y"),IF($B141="Challan","",IF(W141&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y141" s="23">
-        <f>IF($B141&lt;&gt;"Entry","",IF(LEN(W141)&lt;4,"",IF(UPPER(MID(W141,4,1))="P","Individual",IF(UPPER(MID(W141,4,1))="H","HUF",IF(UPPER(MID(W141,4,1))="C","Company",IF(UPPER(MID(W141,4,1))="F","Firm",IF(UPPER(MID(W141,4,1))="L","LLP",IF(UPPER(MID(W141,4,1))="T","Trust",IF(UPPER(MID(W141,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B141="Entry",IF(LEN(W141)&lt;4,"",IF(UPPER(MID(W141,4,1))="P","Individual",IF(UPPER(MID(W141,4,1))="H","HUF",IF(UPPER(MID(W141,4,1))="C","Company",IF(UPPER(MID(W141,4,1))="F","Firm",IF(UPPER(MID(W141,4,1))="L","LLP",IF(UPPER(MID(W141,4,1))="T","Trust",IF(UPPER(MID(W141,4,1))="A","AOP","")))))))),IF($B141="Challan","",IF(W141&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z141" s="28"/>
       <c r="AA141" s="29">
@@ -13786,10 +13786,10 @@
       <c r="V142" s="28"/>
       <c r="W142" s="28"/>
       <c r="X142" s="23">
-        <f>IF($B142&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W142)))=10,CODE(MID(TRIM(UPPER(W142)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W142)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W142)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W142)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B142="Entry",IF(AND(LEN(TRIM(UPPER(W142)))=10,CODE(MID(TRIM(UPPER(W142)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W142)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W142)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W142)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W142)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W142)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W142)),9,1))&lt;=57),"N","Y"),IF($B142="Challan","",IF(W142&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y142" s="23">
-        <f>IF($B142&lt;&gt;"Entry","",IF(LEN(W142)&lt;4,"",IF(UPPER(MID(W142,4,1))="P","Individual",IF(UPPER(MID(W142,4,1))="H","HUF",IF(UPPER(MID(W142,4,1))="C","Company",IF(UPPER(MID(W142,4,1))="F","Firm",IF(UPPER(MID(W142,4,1))="L","LLP",IF(UPPER(MID(W142,4,1))="T","Trust",IF(UPPER(MID(W142,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B142="Entry",IF(LEN(W142)&lt;4,"",IF(UPPER(MID(W142,4,1))="P","Individual",IF(UPPER(MID(W142,4,1))="H","HUF",IF(UPPER(MID(W142,4,1))="C","Company",IF(UPPER(MID(W142,4,1))="F","Firm",IF(UPPER(MID(W142,4,1))="L","LLP",IF(UPPER(MID(W142,4,1))="T","Trust",IF(UPPER(MID(W142,4,1))="A","AOP","")))))))),IF($B142="Challan","",IF(W142&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z142" s="28"/>
       <c r="AA142" s="29">
@@ -13864,10 +13864,10 @@
       <c r="V143" s="28"/>
       <c r="W143" s="28"/>
       <c r="X143" s="23">
-        <f>IF($B143&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W143)))=10,CODE(MID(TRIM(UPPER(W143)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W143)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W143)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W143)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B143="Entry",IF(AND(LEN(TRIM(UPPER(W143)))=10,CODE(MID(TRIM(UPPER(W143)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W143)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W143)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W143)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W143)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W143)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W143)),9,1))&lt;=57),"N","Y"),IF($B143="Challan","",IF(W143&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y143" s="23">
-        <f>IF($B143&lt;&gt;"Entry","",IF(LEN(W143)&lt;4,"",IF(UPPER(MID(W143,4,1))="P","Individual",IF(UPPER(MID(W143,4,1))="H","HUF",IF(UPPER(MID(W143,4,1))="C","Company",IF(UPPER(MID(W143,4,1))="F","Firm",IF(UPPER(MID(W143,4,1))="L","LLP",IF(UPPER(MID(W143,4,1))="T","Trust",IF(UPPER(MID(W143,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B143="Entry",IF(LEN(W143)&lt;4,"",IF(UPPER(MID(W143,4,1))="P","Individual",IF(UPPER(MID(W143,4,1))="H","HUF",IF(UPPER(MID(W143,4,1))="C","Company",IF(UPPER(MID(W143,4,1))="F","Firm",IF(UPPER(MID(W143,4,1))="L","LLP",IF(UPPER(MID(W143,4,1))="T","Trust",IF(UPPER(MID(W143,4,1))="A","AOP","")))))))),IF($B143="Challan","",IF(W143&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z143" s="28"/>
       <c r="AA143" s="29">
@@ -13942,10 +13942,10 @@
       <c r="V144" s="28"/>
       <c r="W144" s="28"/>
       <c r="X144" s="23">
-        <f>IF($B144&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W144)))=10,CODE(MID(TRIM(UPPER(W144)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W144)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W144)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W144)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B144="Entry",IF(AND(LEN(TRIM(UPPER(W144)))=10,CODE(MID(TRIM(UPPER(W144)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W144)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W144)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W144)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W144)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W144)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W144)),9,1))&lt;=57),"N","Y"),IF($B144="Challan","",IF(W144&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y144" s="23">
-        <f>IF($B144&lt;&gt;"Entry","",IF(LEN(W144)&lt;4,"",IF(UPPER(MID(W144,4,1))="P","Individual",IF(UPPER(MID(W144,4,1))="H","HUF",IF(UPPER(MID(W144,4,1))="C","Company",IF(UPPER(MID(W144,4,1))="F","Firm",IF(UPPER(MID(W144,4,1))="L","LLP",IF(UPPER(MID(W144,4,1))="T","Trust",IF(UPPER(MID(W144,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B144="Entry",IF(LEN(W144)&lt;4,"",IF(UPPER(MID(W144,4,1))="P","Individual",IF(UPPER(MID(W144,4,1))="H","HUF",IF(UPPER(MID(W144,4,1))="C","Company",IF(UPPER(MID(W144,4,1))="F","Firm",IF(UPPER(MID(W144,4,1))="L","LLP",IF(UPPER(MID(W144,4,1))="T","Trust",IF(UPPER(MID(W144,4,1))="A","AOP","")))))))),IF($B144="Challan","",IF(W144&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z144" s="28"/>
       <c r="AA144" s="29">
@@ -14020,10 +14020,10 @@
       <c r="V145" s="28"/>
       <c r="W145" s="28"/>
       <c r="X145" s="23">
-        <f>IF($B145&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W145)))=10,CODE(MID(TRIM(UPPER(W145)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W145)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W145)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W145)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B145="Entry",IF(AND(LEN(TRIM(UPPER(W145)))=10,CODE(MID(TRIM(UPPER(W145)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W145)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W145)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W145)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W145)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W145)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W145)),9,1))&lt;=57),"N","Y"),IF($B145="Challan","",IF(W145&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y145" s="23">
-        <f>IF($B145&lt;&gt;"Entry","",IF(LEN(W145)&lt;4,"",IF(UPPER(MID(W145,4,1))="P","Individual",IF(UPPER(MID(W145,4,1))="H","HUF",IF(UPPER(MID(W145,4,1))="C","Company",IF(UPPER(MID(W145,4,1))="F","Firm",IF(UPPER(MID(W145,4,1))="L","LLP",IF(UPPER(MID(W145,4,1))="T","Trust",IF(UPPER(MID(W145,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B145="Entry",IF(LEN(W145)&lt;4,"",IF(UPPER(MID(W145,4,1))="P","Individual",IF(UPPER(MID(W145,4,1))="H","HUF",IF(UPPER(MID(W145,4,1))="C","Company",IF(UPPER(MID(W145,4,1))="F","Firm",IF(UPPER(MID(W145,4,1))="L","LLP",IF(UPPER(MID(W145,4,1))="T","Trust",IF(UPPER(MID(W145,4,1))="A","AOP","")))))))),IF($B145="Challan","",IF(W145&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z145" s="28"/>
       <c r="AA145" s="29">
@@ -14098,10 +14098,10 @@
       <c r="V146" s="28"/>
       <c r="W146" s="28"/>
       <c r="X146" s="23">
-        <f>IF($B146&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W146)))=10,CODE(MID(TRIM(UPPER(W146)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W146)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W146)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W146)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B146="Entry",IF(AND(LEN(TRIM(UPPER(W146)))=10,CODE(MID(TRIM(UPPER(W146)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W146)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W146)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W146)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W146)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W146)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W146)),9,1))&lt;=57),"N","Y"),IF($B146="Challan","",IF(W146&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y146" s="23">
-        <f>IF($B146&lt;&gt;"Entry","",IF(LEN(W146)&lt;4,"",IF(UPPER(MID(W146,4,1))="P","Individual",IF(UPPER(MID(W146,4,1))="H","HUF",IF(UPPER(MID(W146,4,1))="C","Company",IF(UPPER(MID(W146,4,1))="F","Firm",IF(UPPER(MID(W146,4,1))="L","LLP",IF(UPPER(MID(W146,4,1))="T","Trust",IF(UPPER(MID(W146,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B146="Entry",IF(LEN(W146)&lt;4,"",IF(UPPER(MID(W146,4,1))="P","Individual",IF(UPPER(MID(W146,4,1))="H","HUF",IF(UPPER(MID(W146,4,1))="C","Company",IF(UPPER(MID(W146,4,1))="F","Firm",IF(UPPER(MID(W146,4,1))="L","LLP",IF(UPPER(MID(W146,4,1))="T","Trust",IF(UPPER(MID(W146,4,1))="A","AOP","")))))))),IF($B146="Challan","",IF(W146&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z146" s="28"/>
       <c r="AA146" s="29">
@@ -14176,10 +14176,10 @@
       <c r="V147" s="28"/>
       <c r="W147" s="28"/>
       <c r="X147" s="23">
-        <f>IF($B147&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W147)))=10,CODE(MID(TRIM(UPPER(W147)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W147)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W147)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W147)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B147="Entry",IF(AND(LEN(TRIM(UPPER(W147)))=10,CODE(MID(TRIM(UPPER(W147)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W147)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W147)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W147)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W147)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W147)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W147)),9,1))&lt;=57),"N","Y"),IF($B147="Challan","",IF(W147&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y147" s="23">
-        <f>IF($B147&lt;&gt;"Entry","",IF(LEN(W147)&lt;4,"",IF(UPPER(MID(W147,4,1))="P","Individual",IF(UPPER(MID(W147,4,1))="H","HUF",IF(UPPER(MID(W147,4,1))="C","Company",IF(UPPER(MID(W147,4,1))="F","Firm",IF(UPPER(MID(W147,4,1))="L","LLP",IF(UPPER(MID(W147,4,1))="T","Trust",IF(UPPER(MID(W147,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B147="Entry",IF(LEN(W147)&lt;4,"",IF(UPPER(MID(W147,4,1))="P","Individual",IF(UPPER(MID(W147,4,1))="H","HUF",IF(UPPER(MID(W147,4,1))="C","Company",IF(UPPER(MID(W147,4,1))="F","Firm",IF(UPPER(MID(W147,4,1))="L","LLP",IF(UPPER(MID(W147,4,1))="T","Trust",IF(UPPER(MID(W147,4,1))="A","AOP","")))))))),IF($B147="Challan","",IF(W147&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z147" s="28"/>
       <c r="AA147" s="29">
@@ -14254,10 +14254,10 @@
       <c r="V148" s="28"/>
       <c r="W148" s="28"/>
       <c r="X148" s="23">
-        <f>IF($B148&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W148)))=10,CODE(MID(TRIM(UPPER(W148)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W148)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W148)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W148)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B148="Entry",IF(AND(LEN(TRIM(UPPER(W148)))=10,CODE(MID(TRIM(UPPER(W148)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W148)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W148)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W148)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W148)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W148)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W148)),9,1))&lt;=57),"N","Y"),IF($B148="Challan","",IF(W148&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y148" s="23">
-        <f>IF($B148&lt;&gt;"Entry","",IF(LEN(W148)&lt;4,"",IF(UPPER(MID(W148,4,1))="P","Individual",IF(UPPER(MID(W148,4,1))="H","HUF",IF(UPPER(MID(W148,4,1))="C","Company",IF(UPPER(MID(W148,4,1))="F","Firm",IF(UPPER(MID(W148,4,1))="L","LLP",IF(UPPER(MID(W148,4,1))="T","Trust",IF(UPPER(MID(W148,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B148="Entry",IF(LEN(W148)&lt;4,"",IF(UPPER(MID(W148,4,1))="P","Individual",IF(UPPER(MID(W148,4,1))="H","HUF",IF(UPPER(MID(W148,4,1))="C","Company",IF(UPPER(MID(W148,4,1))="F","Firm",IF(UPPER(MID(W148,4,1))="L","LLP",IF(UPPER(MID(W148,4,1))="T","Trust",IF(UPPER(MID(W148,4,1))="A","AOP","")))))))),IF($B148="Challan","",IF(W148&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z148" s="28"/>
       <c r="AA148" s="29">
@@ -14332,10 +14332,10 @@
       <c r="V149" s="28"/>
       <c r="W149" s="28"/>
       <c r="X149" s="23">
-        <f>IF($B149&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W149)))=10,CODE(MID(TRIM(UPPER(W149)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W149)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W149)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W149)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B149="Entry",IF(AND(LEN(TRIM(UPPER(W149)))=10,CODE(MID(TRIM(UPPER(W149)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W149)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W149)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W149)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W149)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W149)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W149)),9,1))&lt;=57),"N","Y"),IF($B149="Challan","",IF(W149&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y149" s="23">
-        <f>IF($B149&lt;&gt;"Entry","",IF(LEN(W149)&lt;4,"",IF(UPPER(MID(W149,4,1))="P","Individual",IF(UPPER(MID(W149,4,1))="H","HUF",IF(UPPER(MID(W149,4,1))="C","Company",IF(UPPER(MID(W149,4,1))="F","Firm",IF(UPPER(MID(W149,4,1))="L","LLP",IF(UPPER(MID(W149,4,1))="T","Trust",IF(UPPER(MID(W149,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B149="Entry",IF(LEN(W149)&lt;4,"",IF(UPPER(MID(W149,4,1))="P","Individual",IF(UPPER(MID(W149,4,1))="H","HUF",IF(UPPER(MID(W149,4,1))="C","Company",IF(UPPER(MID(W149,4,1))="F","Firm",IF(UPPER(MID(W149,4,1))="L","LLP",IF(UPPER(MID(W149,4,1))="T","Trust",IF(UPPER(MID(W149,4,1))="A","AOP","")))))))),IF($B149="Challan","",IF(W149&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z149" s="28"/>
       <c r="AA149" s="29">
@@ -14410,10 +14410,10 @@
       <c r="V150" s="28"/>
       <c r="W150" s="28"/>
       <c r="X150" s="23">
-        <f>IF($B150&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W150)))=10,CODE(MID(TRIM(UPPER(W150)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W150)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W150)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W150)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B150="Entry",IF(AND(LEN(TRIM(UPPER(W150)))=10,CODE(MID(TRIM(UPPER(W150)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W150)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W150)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W150)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W150)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W150)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W150)),9,1))&lt;=57),"N","Y"),IF($B150="Challan","",IF(W150&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y150" s="23">
-        <f>IF($B150&lt;&gt;"Entry","",IF(LEN(W150)&lt;4,"",IF(UPPER(MID(W150,4,1))="P","Individual",IF(UPPER(MID(W150,4,1))="H","HUF",IF(UPPER(MID(W150,4,1))="C","Company",IF(UPPER(MID(W150,4,1))="F","Firm",IF(UPPER(MID(W150,4,1))="L","LLP",IF(UPPER(MID(W150,4,1))="T","Trust",IF(UPPER(MID(W150,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B150="Entry",IF(LEN(W150)&lt;4,"",IF(UPPER(MID(W150,4,1))="P","Individual",IF(UPPER(MID(W150,4,1))="H","HUF",IF(UPPER(MID(W150,4,1))="C","Company",IF(UPPER(MID(W150,4,1))="F","Firm",IF(UPPER(MID(W150,4,1))="L","LLP",IF(UPPER(MID(W150,4,1))="T","Trust",IF(UPPER(MID(W150,4,1))="A","AOP","")))))))),IF($B150="Challan","",IF(W150&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z150" s="28"/>
       <c r="AA150" s="29">
@@ -14488,10 +14488,10 @@
       <c r="V151" s="28"/>
       <c r="W151" s="28"/>
       <c r="X151" s="23">
-        <f>IF($B151&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W151)))=10,CODE(MID(TRIM(UPPER(W151)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W151)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W151)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W151)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B151="Entry",IF(AND(LEN(TRIM(UPPER(W151)))=10,CODE(MID(TRIM(UPPER(W151)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W151)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W151)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W151)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W151)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W151)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W151)),9,1))&lt;=57),"N","Y"),IF($B151="Challan","",IF(W151&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y151" s="23">
-        <f>IF($B151&lt;&gt;"Entry","",IF(LEN(W151)&lt;4,"",IF(UPPER(MID(W151,4,1))="P","Individual",IF(UPPER(MID(W151,4,1))="H","HUF",IF(UPPER(MID(W151,4,1))="C","Company",IF(UPPER(MID(W151,4,1))="F","Firm",IF(UPPER(MID(W151,4,1))="L","LLP",IF(UPPER(MID(W151,4,1))="T","Trust",IF(UPPER(MID(W151,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B151="Entry",IF(LEN(W151)&lt;4,"",IF(UPPER(MID(W151,4,1))="P","Individual",IF(UPPER(MID(W151,4,1))="H","HUF",IF(UPPER(MID(W151,4,1))="C","Company",IF(UPPER(MID(W151,4,1))="F","Firm",IF(UPPER(MID(W151,4,1))="L","LLP",IF(UPPER(MID(W151,4,1))="T","Trust",IF(UPPER(MID(W151,4,1))="A","AOP","")))))))),IF($B151="Challan","",IF(W151&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z151" s="28"/>
       <c r="AA151" s="29">
@@ -14566,10 +14566,10 @@
       <c r="V152" s="28"/>
       <c r="W152" s="28"/>
       <c r="X152" s="23">
-        <f>IF($B152&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W152)))=10,CODE(MID(TRIM(UPPER(W152)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W152)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W152)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W152)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B152="Entry",IF(AND(LEN(TRIM(UPPER(W152)))=10,CODE(MID(TRIM(UPPER(W152)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W152)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W152)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W152)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W152)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W152)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W152)),9,1))&lt;=57),"N","Y"),IF($B152="Challan","",IF(W152&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y152" s="23">
-        <f>IF($B152&lt;&gt;"Entry","",IF(LEN(W152)&lt;4,"",IF(UPPER(MID(W152,4,1))="P","Individual",IF(UPPER(MID(W152,4,1))="H","HUF",IF(UPPER(MID(W152,4,1))="C","Company",IF(UPPER(MID(W152,4,1))="F","Firm",IF(UPPER(MID(W152,4,1))="L","LLP",IF(UPPER(MID(W152,4,1))="T","Trust",IF(UPPER(MID(W152,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B152="Entry",IF(LEN(W152)&lt;4,"",IF(UPPER(MID(W152,4,1))="P","Individual",IF(UPPER(MID(W152,4,1))="H","HUF",IF(UPPER(MID(W152,4,1))="C","Company",IF(UPPER(MID(W152,4,1))="F","Firm",IF(UPPER(MID(W152,4,1))="L","LLP",IF(UPPER(MID(W152,4,1))="T","Trust",IF(UPPER(MID(W152,4,1))="A","AOP","")))))))),IF($B152="Challan","",IF(W152&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z152" s="28"/>
       <c r="AA152" s="29">
@@ -14644,10 +14644,10 @@
       <c r="V153" s="28"/>
       <c r="W153" s="28"/>
       <c r="X153" s="23">
-        <f>IF($B153&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W153)))=10,CODE(MID(TRIM(UPPER(W153)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W153)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W153)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W153)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B153="Entry",IF(AND(LEN(TRIM(UPPER(W153)))=10,CODE(MID(TRIM(UPPER(W153)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W153)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W153)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W153)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W153)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W153)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W153)),9,1))&lt;=57),"N","Y"),IF($B153="Challan","",IF(W153&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y153" s="23">
-        <f>IF($B153&lt;&gt;"Entry","",IF(LEN(W153)&lt;4,"",IF(UPPER(MID(W153,4,1))="P","Individual",IF(UPPER(MID(W153,4,1))="H","HUF",IF(UPPER(MID(W153,4,1))="C","Company",IF(UPPER(MID(W153,4,1))="F","Firm",IF(UPPER(MID(W153,4,1))="L","LLP",IF(UPPER(MID(W153,4,1))="T","Trust",IF(UPPER(MID(W153,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B153="Entry",IF(LEN(W153)&lt;4,"",IF(UPPER(MID(W153,4,1))="P","Individual",IF(UPPER(MID(W153,4,1))="H","HUF",IF(UPPER(MID(W153,4,1))="C","Company",IF(UPPER(MID(W153,4,1))="F","Firm",IF(UPPER(MID(W153,4,1))="L","LLP",IF(UPPER(MID(W153,4,1))="T","Trust",IF(UPPER(MID(W153,4,1))="A","AOP","")))))))),IF($B153="Challan","",IF(W153&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z153" s="28"/>
       <c r="AA153" s="29">
@@ -14722,10 +14722,10 @@
       <c r="V154" s="28"/>
       <c r="W154" s="28"/>
       <c r="X154" s="23">
-        <f>IF($B154&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W154)))=10,CODE(MID(TRIM(UPPER(W154)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W154)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W154)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W154)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B154="Entry",IF(AND(LEN(TRIM(UPPER(W154)))=10,CODE(MID(TRIM(UPPER(W154)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W154)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W154)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W154)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W154)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W154)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W154)),9,1))&lt;=57),"N","Y"),IF($B154="Challan","",IF(W154&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y154" s="23">
-        <f>IF($B154&lt;&gt;"Entry","",IF(LEN(W154)&lt;4,"",IF(UPPER(MID(W154,4,1))="P","Individual",IF(UPPER(MID(W154,4,1))="H","HUF",IF(UPPER(MID(W154,4,1))="C","Company",IF(UPPER(MID(W154,4,1))="F","Firm",IF(UPPER(MID(W154,4,1))="L","LLP",IF(UPPER(MID(W154,4,1))="T","Trust",IF(UPPER(MID(W154,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B154="Entry",IF(LEN(W154)&lt;4,"",IF(UPPER(MID(W154,4,1))="P","Individual",IF(UPPER(MID(W154,4,1))="H","HUF",IF(UPPER(MID(W154,4,1))="C","Company",IF(UPPER(MID(W154,4,1))="F","Firm",IF(UPPER(MID(W154,4,1))="L","LLP",IF(UPPER(MID(W154,4,1))="T","Trust",IF(UPPER(MID(W154,4,1))="A","AOP","")))))))),IF($B154="Challan","",IF(W154&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z154" s="28"/>
       <c r="AA154" s="29">
@@ -14800,10 +14800,10 @@
       <c r="V155" s="28"/>
       <c r="W155" s="28"/>
       <c r="X155" s="23">
-        <f>IF($B155&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W155)))=10,CODE(MID(TRIM(UPPER(W155)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W155)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W155)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W155)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B155="Entry",IF(AND(LEN(TRIM(UPPER(W155)))=10,CODE(MID(TRIM(UPPER(W155)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W155)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W155)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W155)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W155)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W155)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W155)),9,1))&lt;=57),"N","Y"),IF($B155="Challan","",IF(W155&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y155" s="23">
-        <f>IF($B155&lt;&gt;"Entry","",IF(LEN(W155)&lt;4,"",IF(UPPER(MID(W155,4,1))="P","Individual",IF(UPPER(MID(W155,4,1))="H","HUF",IF(UPPER(MID(W155,4,1))="C","Company",IF(UPPER(MID(W155,4,1))="F","Firm",IF(UPPER(MID(W155,4,1))="L","LLP",IF(UPPER(MID(W155,4,1))="T","Trust",IF(UPPER(MID(W155,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B155="Entry",IF(LEN(W155)&lt;4,"",IF(UPPER(MID(W155,4,1))="P","Individual",IF(UPPER(MID(W155,4,1))="H","HUF",IF(UPPER(MID(W155,4,1))="C","Company",IF(UPPER(MID(W155,4,1))="F","Firm",IF(UPPER(MID(W155,4,1))="L","LLP",IF(UPPER(MID(W155,4,1))="T","Trust",IF(UPPER(MID(W155,4,1))="A","AOP","")))))))),IF($B155="Challan","",IF(W155&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z155" s="28"/>
       <c r="AA155" s="29">
@@ -14878,10 +14878,10 @@
       <c r="V156" s="28"/>
       <c r="W156" s="28"/>
       <c r="X156" s="23">
-        <f>IF($B156&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W156)))=10,CODE(MID(TRIM(UPPER(W156)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W156)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W156)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W156)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B156="Entry",IF(AND(LEN(TRIM(UPPER(W156)))=10,CODE(MID(TRIM(UPPER(W156)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W156)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W156)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W156)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W156)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W156)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W156)),9,1))&lt;=57),"N","Y"),IF($B156="Challan","",IF(W156&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y156" s="23">
-        <f>IF($B156&lt;&gt;"Entry","",IF(LEN(W156)&lt;4,"",IF(UPPER(MID(W156,4,1))="P","Individual",IF(UPPER(MID(W156,4,1))="H","HUF",IF(UPPER(MID(W156,4,1))="C","Company",IF(UPPER(MID(W156,4,1))="F","Firm",IF(UPPER(MID(W156,4,1))="L","LLP",IF(UPPER(MID(W156,4,1))="T","Trust",IF(UPPER(MID(W156,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B156="Entry",IF(LEN(W156)&lt;4,"",IF(UPPER(MID(W156,4,1))="P","Individual",IF(UPPER(MID(W156,4,1))="H","HUF",IF(UPPER(MID(W156,4,1))="C","Company",IF(UPPER(MID(W156,4,1))="F","Firm",IF(UPPER(MID(W156,4,1))="L","LLP",IF(UPPER(MID(W156,4,1))="T","Trust",IF(UPPER(MID(W156,4,1))="A","AOP","")))))))),IF($B156="Challan","",IF(W156&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z156" s="28"/>
       <c r="AA156" s="29">
@@ -14956,10 +14956,10 @@
       <c r="V157" s="28"/>
       <c r="W157" s="28"/>
       <c r="X157" s="23">
-        <f>IF($B157&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W157)))=10,CODE(MID(TRIM(UPPER(W157)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W157)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W157)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W157)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B157="Entry",IF(AND(LEN(TRIM(UPPER(W157)))=10,CODE(MID(TRIM(UPPER(W157)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W157)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W157)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W157)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W157)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W157)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W157)),9,1))&lt;=57),"N","Y"),IF($B157="Challan","",IF(W157&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y157" s="23">
-        <f>IF($B157&lt;&gt;"Entry","",IF(LEN(W157)&lt;4,"",IF(UPPER(MID(W157,4,1))="P","Individual",IF(UPPER(MID(W157,4,1))="H","HUF",IF(UPPER(MID(W157,4,1))="C","Company",IF(UPPER(MID(W157,4,1))="F","Firm",IF(UPPER(MID(W157,4,1))="L","LLP",IF(UPPER(MID(W157,4,1))="T","Trust",IF(UPPER(MID(W157,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B157="Entry",IF(LEN(W157)&lt;4,"",IF(UPPER(MID(W157,4,1))="P","Individual",IF(UPPER(MID(W157,4,1))="H","HUF",IF(UPPER(MID(W157,4,1))="C","Company",IF(UPPER(MID(W157,4,1))="F","Firm",IF(UPPER(MID(W157,4,1))="L","LLP",IF(UPPER(MID(W157,4,1))="T","Trust",IF(UPPER(MID(W157,4,1))="A","AOP","")))))))),IF($B157="Challan","",IF(W157&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z157" s="28"/>
       <c r="AA157" s="29">
@@ -15034,10 +15034,10 @@
       <c r="V158" s="28"/>
       <c r="W158" s="28"/>
       <c r="X158" s="23">
-        <f>IF($B158&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W158)))=10,CODE(MID(TRIM(UPPER(W158)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W158)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W158)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W158)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B158="Entry",IF(AND(LEN(TRIM(UPPER(W158)))=10,CODE(MID(TRIM(UPPER(W158)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W158)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W158)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W158)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W158)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W158)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W158)),9,1))&lt;=57),"N","Y"),IF($B158="Challan","",IF(W158&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y158" s="23">
-        <f>IF($B158&lt;&gt;"Entry","",IF(LEN(W158)&lt;4,"",IF(UPPER(MID(W158,4,1))="P","Individual",IF(UPPER(MID(W158,4,1))="H","HUF",IF(UPPER(MID(W158,4,1))="C","Company",IF(UPPER(MID(W158,4,1))="F","Firm",IF(UPPER(MID(W158,4,1))="L","LLP",IF(UPPER(MID(W158,4,1))="T","Trust",IF(UPPER(MID(W158,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B158="Entry",IF(LEN(W158)&lt;4,"",IF(UPPER(MID(W158,4,1))="P","Individual",IF(UPPER(MID(W158,4,1))="H","HUF",IF(UPPER(MID(W158,4,1))="C","Company",IF(UPPER(MID(W158,4,1))="F","Firm",IF(UPPER(MID(W158,4,1))="L","LLP",IF(UPPER(MID(W158,4,1))="T","Trust",IF(UPPER(MID(W158,4,1))="A","AOP","")))))))),IF($B158="Challan","",IF(W158&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z158" s="28"/>
       <c r="AA158" s="29">
@@ -15112,10 +15112,10 @@
       <c r="V159" s="28"/>
       <c r="W159" s="28"/>
       <c r="X159" s="23">
-        <f>IF($B159&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W159)))=10,CODE(MID(TRIM(UPPER(W159)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W159)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W159)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W159)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B159="Entry",IF(AND(LEN(TRIM(UPPER(W159)))=10,CODE(MID(TRIM(UPPER(W159)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W159)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W159)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W159)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W159)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W159)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W159)),9,1))&lt;=57),"N","Y"),IF($B159="Challan","",IF(W159&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y159" s="23">
-        <f>IF($B159&lt;&gt;"Entry","",IF(LEN(W159)&lt;4,"",IF(UPPER(MID(W159,4,1))="P","Individual",IF(UPPER(MID(W159,4,1))="H","HUF",IF(UPPER(MID(W159,4,1))="C","Company",IF(UPPER(MID(W159,4,1))="F","Firm",IF(UPPER(MID(W159,4,1))="L","LLP",IF(UPPER(MID(W159,4,1))="T","Trust",IF(UPPER(MID(W159,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B159="Entry",IF(LEN(W159)&lt;4,"",IF(UPPER(MID(W159,4,1))="P","Individual",IF(UPPER(MID(W159,4,1))="H","HUF",IF(UPPER(MID(W159,4,1))="C","Company",IF(UPPER(MID(W159,4,1))="F","Firm",IF(UPPER(MID(W159,4,1))="L","LLP",IF(UPPER(MID(W159,4,1))="T","Trust",IF(UPPER(MID(W159,4,1))="A","AOP","")))))))),IF($B159="Challan","",IF(W159&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z159" s="28"/>
       <c r="AA159" s="29">
@@ -15190,10 +15190,10 @@
       <c r="V160" s="28"/>
       <c r="W160" s="28"/>
       <c r="X160" s="23">
-        <f>IF($B160&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W160)))=10,CODE(MID(TRIM(UPPER(W160)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W160)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W160)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W160)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B160="Entry",IF(AND(LEN(TRIM(UPPER(W160)))=10,CODE(MID(TRIM(UPPER(W160)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W160)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W160)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W160)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W160)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W160)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W160)),9,1))&lt;=57),"N","Y"),IF($B160="Challan","",IF(W160&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y160" s="23">
-        <f>IF($B160&lt;&gt;"Entry","",IF(LEN(W160)&lt;4,"",IF(UPPER(MID(W160,4,1))="P","Individual",IF(UPPER(MID(W160,4,1))="H","HUF",IF(UPPER(MID(W160,4,1))="C","Company",IF(UPPER(MID(W160,4,1))="F","Firm",IF(UPPER(MID(W160,4,1))="L","LLP",IF(UPPER(MID(W160,4,1))="T","Trust",IF(UPPER(MID(W160,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B160="Entry",IF(LEN(W160)&lt;4,"",IF(UPPER(MID(W160,4,1))="P","Individual",IF(UPPER(MID(W160,4,1))="H","HUF",IF(UPPER(MID(W160,4,1))="C","Company",IF(UPPER(MID(W160,4,1))="F","Firm",IF(UPPER(MID(W160,4,1))="L","LLP",IF(UPPER(MID(W160,4,1))="T","Trust",IF(UPPER(MID(W160,4,1))="A","AOP","")))))))),IF($B160="Challan","",IF(W160&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z160" s="28"/>
       <c r="AA160" s="29">
@@ -15268,10 +15268,10 @@
       <c r="V161" s="28"/>
       <c r="W161" s="28"/>
       <c r="X161" s="23">
-        <f>IF($B161&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W161)))=10,CODE(MID(TRIM(UPPER(W161)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W161)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W161)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W161)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B161="Entry",IF(AND(LEN(TRIM(UPPER(W161)))=10,CODE(MID(TRIM(UPPER(W161)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W161)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W161)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W161)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W161)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W161)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W161)),9,1))&lt;=57),"N","Y"),IF($B161="Challan","",IF(W161&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y161" s="23">
-        <f>IF($B161&lt;&gt;"Entry","",IF(LEN(W161)&lt;4,"",IF(UPPER(MID(W161,4,1))="P","Individual",IF(UPPER(MID(W161,4,1))="H","HUF",IF(UPPER(MID(W161,4,1))="C","Company",IF(UPPER(MID(W161,4,1))="F","Firm",IF(UPPER(MID(W161,4,1))="L","LLP",IF(UPPER(MID(W161,4,1))="T","Trust",IF(UPPER(MID(W161,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B161="Entry",IF(LEN(W161)&lt;4,"",IF(UPPER(MID(W161,4,1))="P","Individual",IF(UPPER(MID(W161,4,1))="H","HUF",IF(UPPER(MID(W161,4,1))="C","Company",IF(UPPER(MID(W161,4,1))="F","Firm",IF(UPPER(MID(W161,4,1))="L","LLP",IF(UPPER(MID(W161,4,1))="T","Trust",IF(UPPER(MID(W161,4,1))="A","AOP","")))))))),IF($B161="Challan","",IF(W161&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z161" s="28"/>
       <c r="AA161" s="29">
@@ -15346,10 +15346,10 @@
       <c r="V162" s="28"/>
       <c r="W162" s="28"/>
       <c r="X162" s="23">
-        <f>IF($B162&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W162)))=10,CODE(MID(TRIM(UPPER(W162)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W162)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W162)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W162)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B162="Entry",IF(AND(LEN(TRIM(UPPER(W162)))=10,CODE(MID(TRIM(UPPER(W162)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W162)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W162)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W162)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W162)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W162)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W162)),9,1))&lt;=57),"N","Y"),IF($B162="Challan","",IF(W162&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y162" s="23">
-        <f>IF($B162&lt;&gt;"Entry","",IF(LEN(W162)&lt;4,"",IF(UPPER(MID(W162,4,1))="P","Individual",IF(UPPER(MID(W162,4,1))="H","HUF",IF(UPPER(MID(W162,4,1))="C","Company",IF(UPPER(MID(W162,4,1))="F","Firm",IF(UPPER(MID(W162,4,1))="L","LLP",IF(UPPER(MID(W162,4,1))="T","Trust",IF(UPPER(MID(W162,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B162="Entry",IF(LEN(W162)&lt;4,"",IF(UPPER(MID(W162,4,1))="P","Individual",IF(UPPER(MID(W162,4,1))="H","HUF",IF(UPPER(MID(W162,4,1))="C","Company",IF(UPPER(MID(W162,4,1))="F","Firm",IF(UPPER(MID(W162,4,1))="L","LLP",IF(UPPER(MID(W162,4,1))="T","Trust",IF(UPPER(MID(W162,4,1))="A","AOP","")))))))),IF($B162="Challan","",IF(W162&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z162" s="28"/>
       <c r="AA162" s="29">
@@ -15424,10 +15424,10 @@
       <c r="V163" s="28"/>
       <c r="W163" s="28"/>
       <c r="X163" s="23">
-        <f>IF($B163&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W163)))=10,CODE(MID(TRIM(UPPER(W163)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W163)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W163)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W163)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B163="Entry",IF(AND(LEN(TRIM(UPPER(W163)))=10,CODE(MID(TRIM(UPPER(W163)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W163)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W163)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W163)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W163)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W163)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W163)),9,1))&lt;=57),"N","Y"),IF($B163="Challan","",IF(W163&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y163" s="23">
-        <f>IF($B163&lt;&gt;"Entry","",IF(LEN(W163)&lt;4,"",IF(UPPER(MID(W163,4,1))="P","Individual",IF(UPPER(MID(W163,4,1))="H","HUF",IF(UPPER(MID(W163,4,1))="C","Company",IF(UPPER(MID(W163,4,1))="F","Firm",IF(UPPER(MID(W163,4,1))="L","LLP",IF(UPPER(MID(W163,4,1))="T","Trust",IF(UPPER(MID(W163,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B163="Entry",IF(LEN(W163)&lt;4,"",IF(UPPER(MID(W163,4,1))="P","Individual",IF(UPPER(MID(W163,4,1))="H","HUF",IF(UPPER(MID(W163,4,1))="C","Company",IF(UPPER(MID(W163,4,1))="F","Firm",IF(UPPER(MID(W163,4,1))="L","LLP",IF(UPPER(MID(W163,4,1))="T","Trust",IF(UPPER(MID(W163,4,1))="A","AOP","")))))))),IF($B163="Challan","",IF(W163&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z163" s="28"/>
       <c r="AA163" s="29">
@@ -15502,10 +15502,10 @@
       <c r="V164" s="28"/>
       <c r="W164" s="28"/>
       <c r="X164" s="23">
-        <f>IF($B164&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W164)))=10,CODE(MID(TRIM(UPPER(W164)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W164)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W164)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W164)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B164="Entry",IF(AND(LEN(TRIM(UPPER(W164)))=10,CODE(MID(TRIM(UPPER(W164)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W164)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W164)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W164)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W164)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W164)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W164)),9,1))&lt;=57),"N","Y"),IF($B164="Challan","",IF(W164&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y164" s="23">
-        <f>IF($B164&lt;&gt;"Entry","",IF(LEN(W164)&lt;4,"",IF(UPPER(MID(W164,4,1))="P","Individual",IF(UPPER(MID(W164,4,1))="H","HUF",IF(UPPER(MID(W164,4,1))="C","Company",IF(UPPER(MID(W164,4,1))="F","Firm",IF(UPPER(MID(W164,4,1))="L","LLP",IF(UPPER(MID(W164,4,1))="T","Trust",IF(UPPER(MID(W164,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B164="Entry",IF(LEN(W164)&lt;4,"",IF(UPPER(MID(W164,4,1))="P","Individual",IF(UPPER(MID(W164,4,1))="H","HUF",IF(UPPER(MID(W164,4,1))="C","Company",IF(UPPER(MID(W164,4,1))="F","Firm",IF(UPPER(MID(W164,4,1))="L","LLP",IF(UPPER(MID(W164,4,1))="T","Trust",IF(UPPER(MID(W164,4,1))="A","AOP","")))))))),IF($B164="Challan","",IF(W164&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z164" s="28"/>
       <c r="AA164" s="29">
@@ -15580,10 +15580,10 @@
       <c r="V165" s="28"/>
       <c r="W165" s="28"/>
       <c r="X165" s="23">
-        <f>IF($B165&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W165)))=10,CODE(MID(TRIM(UPPER(W165)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W165)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W165)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W165)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B165="Entry",IF(AND(LEN(TRIM(UPPER(W165)))=10,CODE(MID(TRIM(UPPER(W165)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W165)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W165)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W165)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W165)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W165)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W165)),9,1))&lt;=57),"N","Y"),IF($B165="Challan","",IF(W165&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y165" s="23">
-        <f>IF($B165&lt;&gt;"Entry","",IF(LEN(W165)&lt;4,"",IF(UPPER(MID(W165,4,1))="P","Individual",IF(UPPER(MID(W165,4,1))="H","HUF",IF(UPPER(MID(W165,4,1))="C","Company",IF(UPPER(MID(W165,4,1))="F","Firm",IF(UPPER(MID(W165,4,1))="L","LLP",IF(UPPER(MID(W165,4,1))="T","Trust",IF(UPPER(MID(W165,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B165="Entry",IF(LEN(W165)&lt;4,"",IF(UPPER(MID(W165,4,1))="P","Individual",IF(UPPER(MID(W165,4,1))="H","HUF",IF(UPPER(MID(W165,4,1))="C","Company",IF(UPPER(MID(W165,4,1))="F","Firm",IF(UPPER(MID(W165,4,1))="L","LLP",IF(UPPER(MID(W165,4,1))="T","Trust",IF(UPPER(MID(W165,4,1))="A","AOP","")))))))),IF($B165="Challan","",IF(W165&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z165" s="28"/>
       <c r="AA165" s="29">
@@ -15658,10 +15658,10 @@
       <c r="V166" s="28"/>
       <c r="W166" s="28"/>
       <c r="X166" s="23">
-        <f>IF($B166&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W166)))=10,CODE(MID(TRIM(UPPER(W166)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W166)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W166)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W166)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B166="Entry",IF(AND(LEN(TRIM(UPPER(W166)))=10,CODE(MID(TRIM(UPPER(W166)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W166)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W166)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W166)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W166)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W166)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W166)),9,1))&lt;=57),"N","Y"),IF($B166="Challan","",IF(W166&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y166" s="23">
-        <f>IF($B166&lt;&gt;"Entry","",IF(LEN(W166)&lt;4,"",IF(UPPER(MID(W166,4,1))="P","Individual",IF(UPPER(MID(W166,4,1))="H","HUF",IF(UPPER(MID(W166,4,1))="C","Company",IF(UPPER(MID(W166,4,1))="F","Firm",IF(UPPER(MID(W166,4,1))="L","LLP",IF(UPPER(MID(W166,4,1))="T","Trust",IF(UPPER(MID(W166,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B166="Entry",IF(LEN(W166)&lt;4,"",IF(UPPER(MID(W166,4,1))="P","Individual",IF(UPPER(MID(W166,4,1))="H","HUF",IF(UPPER(MID(W166,4,1))="C","Company",IF(UPPER(MID(W166,4,1))="F","Firm",IF(UPPER(MID(W166,4,1))="L","LLP",IF(UPPER(MID(W166,4,1))="T","Trust",IF(UPPER(MID(W166,4,1))="A","AOP","")))))))),IF($B166="Challan","",IF(W166&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z166" s="28"/>
       <c r="AA166" s="29">
@@ -15736,10 +15736,10 @@
       <c r="V167" s="28"/>
       <c r="W167" s="28"/>
       <c r="X167" s="23">
-        <f>IF($B167&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W167)))=10,CODE(MID(TRIM(UPPER(W167)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W167)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W167)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W167)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B167="Entry",IF(AND(LEN(TRIM(UPPER(W167)))=10,CODE(MID(TRIM(UPPER(W167)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W167)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W167)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W167)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W167)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W167)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W167)),9,1))&lt;=57),"N","Y"),IF($B167="Challan","",IF(W167&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y167" s="23">
-        <f>IF($B167&lt;&gt;"Entry","",IF(LEN(W167)&lt;4,"",IF(UPPER(MID(W167,4,1))="P","Individual",IF(UPPER(MID(W167,4,1))="H","HUF",IF(UPPER(MID(W167,4,1))="C","Company",IF(UPPER(MID(W167,4,1))="F","Firm",IF(UPPER(MID(W167,4,1))="L","LLP",IF(UPPER(MID(W167,4,1))="T","Trust",IF(UPPER(MID(W167,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B167="Entry",IF(LEN(W167)&lt;4,"",IF(UPPER(MID(W167,4,1))="P","Individual",IF(UPPER(MID(W167,4,1))="H","HUF",IF(UPPER(MID(W167,4,1))="C","Company",IF(UPPER(MID(W167,4,1))="F","Firm",IF(UPPER(MID(W167,4,1))="L","LLP",IF(UPPER(MID(W167,4,1))="T","Trust",IF(UPPER(MID(W167,4,1))="A","AOP","")))))))),IF($B167="Challan","",IF(W167&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z167" s="28"/>
       <c r="AA167" s="29">
@@ -15814,10 +15814,10 @@
       <c r="V168" s="28"/>
       <c r="W168" s="28"/>
       <c r="X168" s="23">
-        <f>IF($B168&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W168)))=10,CODE(MID(TRIM(UPPER(W168)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W168)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W168)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W168)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B168="Entry",IF(AND(LEN(TRIM(UPPER(W168)))=10,CODE(MID(TRIM(UPPER(W168)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W168)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W168)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W168)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W168)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W168)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W168)),9,1))&lt;=57),"N","Y"),IF($B168="Challan","",IF(W168&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y168" s="23">
-        <f>IF($B168&lt;&gt;"Entry","",IF(LEN(W168)&lt;4,"",IF(UPPER(MID(W168,4,1))="P","Individual",IF(UPPER(MID(W168,4,1))="H","HUF",IF(UPPER(MID(W168,4,1))="C","Company",IF(UPPER(MID(W168,4,1))="F","Firm",IF(UPPER(MID(W168,4,1))="L","LLP",IF(UPPER(MID(W168,4,1))="T","Trust",IF(UPPER(MID(W168,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B168="Entry",IF(LEN(W168)&lt;4,"",IF(UPPER(MID(W168,4,1))="P","Individual",IF(UPPER(MID(W168,4,1))="H","HUF",IF(UPPER(MID(W168,4,1))="C","Company",IF(UPPER(MID(W168,4,1))="F","Firm",IF(UPPER(MID(W168,4,1))="L","LLP",IF(UPPER(MID(W168,4,1))="T","Trust",IF(UPPER(MID(W168,4,1))="A","AOP","")))))))),IF($B168="Challan","",IF(W168&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z168" s="28"/>
       <c r="AA168" s="29">
@@ -15892,10 +15892,10 @@
       <c r="V169" s="28"/>
       <c r="W169" s="28"/>
       <c r="X169" s="23">
-        <f>IF($B169&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W169)))=10,CODE(MID(TRIM(UPPER(W169)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W169)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W169)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W169)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B169="Entry",IF(AND(LEN(TRIM(UPPER(W169)))=10,CODE(MID(TRIM(UPPER(W169)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W169)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W169)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W169)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W169)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W169)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W169)),9,1))&lt;=57),"N","Y"),IF($B169="Challan","",IF(W169&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y169" s="23">
-        <f>IF($B169&lt;&gt;"Entry","",IF(LEN(W169)&lt;4,"",IF(UPPER(MID(W169,4,1))="P","Individual",IF(UPPER(MID(W169,4,1))="H","HUF",IF(UPPER(MID(W169,4,1))="C","Company",IF(UPPER(MID(W169,4,1))="F","Firm",IF(UPPER(MID(W169,4,1))="L","LLP",IF(UPPER(MID(W169,4,1))="T","Trust",IF(UPPER(MID(W169,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B169="Entry",IF(LEN(W169)&lt;4,"",IF(UPPER(MID(W169,4,1))="P","Individual",IF(UPPER(MID(W169,4,1))="H","HUF",IF(UPPER(MID(W169,4,1))="C","Company",IF(UPPER(MID(W169,4,1))="F","Firm",IF(UPPER(MID(W169,4,1))="L","LLP",IF(UPPER(MID(W169,4,1))="T","Trust",IF(UPPER(MID(W169,4,1))="A","AOP","")))))))),IF($B169="Challan","",IF(W169&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z169" s="28"/>
       <c r="AA169" s="29">
@@ -15970,10 +15970,10 @@
       <c r="V170" s="28"/>
       <c r="W170" s="28"/>
       <c r="X170" s="23">
-        <f>IF($B170&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W170)))=10,CODE(MID(TRIM(UPPER(W170)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W170)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W170)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W170)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B170="Entry",IF(AND(LEN(TRIM(UPPER(W170)))=10,CODE(MID(TRIM(UPPER(W170)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W170)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W170)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W170)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W170)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W170)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W170)),9,1))&lt;=57),"N","Y"),IF($B170="Challan","",IF(W170&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y170" s="23">
-        <f>IF($B170&lt;&gt;"Entry","",IF(LEN(W170)&lt;4,"",IF(UPPER(MID(W170,4,1))="P","Individual",IF(UPPER(MID(W170,4,1))="H","HUF",IF(UPPER(MID(W170,4,1))="C","Company",IF(UPPER(MID(W170,4,1))="F","Firm",IF(UPPER(MID(W170,4,1))="L","LLP",IF(UPPER(MID(W170,4,1))="T","Trust",IF(UPPER(MID(W170,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B170="Entry",IF(LEN(W170)&lt;4,"",IF(UPPER(MID(W170,4,1))="P","Individual",IF(UPPER(MID(W170,4,1))="H","HUF",IF(UPPER(MID(W170,4,1))="C","Company",IF(UPPER(MID(W170,4,1))="F","Firm",IF(UPPER(MID(W170,4,1))="L","LLP",IF(UPPER(MID(W170,4,1))="T","Trust",IF(UPPER(MID(W170,4,1))="A","AOP","")))))))),IF($B170="Challan","",IF(W170&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z170" s="28"/>
       <c r="AA170" s="29">
@@ -16048,10 +16048,10 @@
       <c r="V171" s="28"/>
       <c r="W171" s="28"/>
       <c r="X171" s="23">
-        <f>IF($B171&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W171)))=10,CODE(MID(TRIM(UPPER(W171)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W171)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W171)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W171)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B171="Entry",IF(AND(LEN(TRIM(UPPER(W171)))=10,CODE(MID(TRIM(UPPER(W171)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W171)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W171)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W171)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W171)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W171)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W171)),9,1))&lt;=57),"N","Y"),IF($B171="Challan","",IF(W171&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y171" s="23">
-        <f>IF($B171&lt;&gt;"Entry","",IF(LEN(W171)&lt;4,"",IF(UPPER(MID(W171,4,1))="P","Individual",IF(UPPER(MID(W171,4,1))="H","HUF",IF(UPPER(MID(W171,4,1))="C","Company",IF(UPPER(MID(W171,4,1))="F","Firm",IF(UPPER(MID(W171,4,1))="L","LLP",IF(UPPER(MID(W171,4,1))="T","Trust",IF(UPPER(MID(W171,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B171="Entry",IF(LEN(W171)&lt;4,"",IF(UPPER(MID(W171,4,1))="P","Individual",IF(UPPER(MID(W171,4,1))="H","HUF",IF(UPPER(MID(W171,4,1))="C","Company",IF(UPPER(MID(W171,4,1))="F","Firm",IF(UPPER(MID(W171,4,1))="L","LLP",IF(UPPER(MID(W171,4,1))="T","Trust",IF(UPPER(MID(W171,4,1))="A","AOP","")))))))),IF($B171="Challan","",IF(W171&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z171" s="28"/>
       <c r="AA171" s="29">
@@ -16126,10 +16126,10 @@
       <c r="V172" s="28"/>
       <c r="W172" s="28"/>
       <c r="X172" s="23">
-        <f>IF($B172&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W172)))=10,CODE(MID(TRIM(UPPER(W172)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W172)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W172)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W172)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B172="Entry",IF(AND(LEN(TRIM(UPPER(W172)))=10,CODE(MID(TRIM(UPPER(W172)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W172)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W172)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W172)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W172)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W172)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W172)),9,1))&lt;=57),"N","Y"),IF($B172="Challan","",IF(W172&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y172" s="23">
-        <f>IF($B172&lt;&gt;"Entry","",IF(LEN(W172)&lt;4,"",IF(UPPER(MID(W172,4,1))="P","Individual",IF(UPPER(MID(W172,4,1))="H","HUF",IF(UPPER(MID(W172,4,1))="C","Company",IF(UPPER(MID(W172,4,1))="F","Firm",IF(UPPER(MID(W172,4,1))="L","LLP",IF(UPPER(MID(W172,4,1))="T","Trust",IF(UPPER(MID(W172,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B172="Entry",IF(LEN(W172)&lt;4,"",IF(UPPER(MID(W172,4,1))="P","Individual",IF(UPPER(MID(W172,4,1))="H","HUF",IF(UPPER(MID(W172,4,1))="C","Company",IF(UPPER(MID(W172,4,1))="F","Firm",IF(UPPER(MID(W172,4,1))="L","LLP",IF(UPPER(MID(W172,4,1))="T","Trust",IF(UPPER(MID(W172,4,1))="A","AOP","")))))))),IF($B172="Challan","",IF(W172&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z172" s="28"/>
       <c r="AA172" s="29">
@@ -16204,10 +16204,10 @@
       <c r="V173" s="28"/>
       <c r="W173" s="28"/>
       <c r="X173" s="23">
-        <f>IF($B173&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W173)))=10,CODE(MID(TRIM(UPPER(W173)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W173)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W173)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W173)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B173="Entry",IF(AND(LEN(TRIM(UPPER(W173)))=10,CODE(MID(TRIM(UPPER(W173)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W173)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W173)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W173)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W173)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W173)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W173)),9,1))&lt;=57),"N","Y"),IF($B173="Challan","",IF(W173&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y173" s="23">
-        <f>IF($B173&lt;&gt;"Entry","",IF(LEN(W173)&lt;4,"",IF(UPPER(MID(W173,4,1))="P","Individual",IF(UPPER(MID(W173,4,1))="H","HUF",IF(UPPER(MID(W173,4,1))="C","Company",IF(UPPER(MID(W173,4,1))="F","Firm",IF(UPPER(MID(W173,4,1))="L","LLP",IF(UPPER(MID(W173,4,1))="T","Trust",IF(UPPER(MID(W173,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B173="Entry",IF(LEN(W173)&lt;4,"",IF(UPPER(MID(W173,4,1))="P","Individual",IF(UPPER(MID(W173,4,1))="H","HUF",IF(UPPER(MID(W173,4,1))="C","Company",IF(UPPER(MID(W173,4,1))="F","Firm",IF(UPPER(MID(W173,4,1))="L","LLP",IF(UPPER(MID(W173,4,1))="T","Trust",IF(UPPER(MID(W173,4,1))="A","AOP","")))))))),IF($B173="Challan","",IF(W173&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z173" s="28"/>
       <c r="AA173" s="29">
@@ -16282,10 +16282,10 @@
       <c r="V174" s="28"/>
       <c r="W174" s="28"/>
       <c r="X174" s="23">
-        <f>IF($B174&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W174)))=10,CODE(MID(TRIM(UPPER(W174)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W174)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W174)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W174)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B174="Entry",IF(AND(LEN(TRIM(UPPER(W174)))=10,CODE(MID(TRIM(UPPER(W174)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W174)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W174)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W174)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W174)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W174)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W174)),9,1))&lt;=57),"N","Y"),IF($B174="Challan","",IF(W174&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y174" s="23">
-        <f>IF($B174&lt;&gt;"Entry","",IF(LEN(W174)&lt;4,"",IF(UPPER(MID(W174,4,1))="P","Individual",IF(UPPER(MID(W174,4,1))="H","HUF",IF(UPPER(MID(W174,4,1))="C","Company",IF(UPPER(MID(W174,4,1))="F","Firm",IF(UPPER(MID(W174,4,1))="L","LLP",IF(UPPER(MID(W174,4,1))="T","Trust",IF(UPPER(MID(W174,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B174="Entry",IF(LEN(W174)&lt;4,"",IF(UPPER(MID(W174,4,1))="P","Individual",IF(UPPER(MID(W174,4,1))="H","HUF",IF(UPPER(MID(W174,4,1))="C","Company",IF(UPPER(MID(W174,4,1))="F","Firm",IF(UPPER(MID(W174,4,1))="L","LLP",IF(UPPER(MID(W174,4,1))="T","Trust",IF(UPPER(MID(W174,4,1))="A","AOP","")))))))),IF($B174="Challan","",IF(W174&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z174" s="28"/>
       <c r="AA174" s="29">
@@ -16360,10 +16360,10 @@
       <c r="V175" s="28"/>
       <c r="W175" s="28"/>
       <c r="X175" s="23">
-        <f>IF($B175&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W175)))=10,CODE(MID(TRIM(UPPER(W175)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W175)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W175)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W175)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B175="Entry",IF(AND(LEN(TRIM(UPPER(W175)))=10,CODE(MID(TRIM(UPPER(W175)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W175)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W175)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W175)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W175)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W175)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W175)),9,1))&lt;=57),"N","Y"),IF($B175="Challan","",IF(W175&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y175" s="23">
-        <f>IF($B175&lt;&gt;"Entry","",IF(LEN(W175)&lt;4,"",IF(UPPER(MID(W175,4,1))="P","Individual",IF(UPPER(MID(W175,4,1))="H","HUF",IF(UPPER(MID(W175,4,1))="C","Company",IF(UPPER(MID(W175,4,1))="F","Firm",IF(UPPER(MID(W175,4,1))="L","LLP",IF(UPPER(MID(W175,4,1))="T","Trust",IF(UPPER(MID(W175,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B175="Entry",IF(LEN(W175)&lt;4,"",IF(UPPER(MID(W175,4,1))="P","Individual",IF(UPPER(MID(W175,4,1))="H","HUF",IF(UPPER(MID(W175,4,1))="C","Company",IF(UPPER(MID(W175,4,1))="F","Firm",IF(UPPER(MID(W175,4,1))="L","LLP",IF(UPPER(MID(W175,4,1))="T","Trust",IF(UPPER(MID(W175,4,1))="A","AOP","")))))))),IF($B175="Challan","",IF(W175&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z175" s="28"/>
       <c r="AA175" s="29">
@@ -16438,10 +16438,10 @@
       <c r="V176" s="28"/>
       <c r="W176" s="28"/>
       <c r="X176" s="23">
-        <f>IF($B176&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W176)))=10,CODE(MID(TRIM(UPPER(W176)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W176)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W176)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W176)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B176="Entry",IF(AND(LEN(TRIM(UPPER(W176)))=10,CODE(MID(TRIM(UPPER(W176)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W176)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W176)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W176)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W176)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W176)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W176)),9,1))&lt;=57),"N","Y"),IF($B176="Challan","",IF(W176&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y176" s="23">
-        <f>IF($B176&lt;&gt;"Entry","",IF(LEN(W176)&lt;4,"",IF(UPPER(MID(W176,4,1))="P","Individual",IF(UPPER(MID(W176,4,1))="H","HUF",IF(UPPER(MID(W176,4,1))="C","Company",IF(UPPER(MID(W176,4,1))="F","Firm",IF(UPPER(MID(W176,4,1))="L","LLP",IF(UPPER(MID(W176,4,1))="T","Trust",IF(UPPER(MID(W176,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B176="Entry",IF(LEN(W176)&lt;4,"",IF(UPPER(MID(W176,4,1))="P","Individual",IF(UPPER(MID(W176,4,1))="H","HUF",IF(UPPER(MID(W176,4,1))="C","Company",IF(UPPER(MID(W176,4,1))="F","Firm",IF(UPPER(MID(W176,4,1))="L","LLP",IF(UPPER(MID(W176,4,1))="T","Trust",IF(UPPER(MID(W176,4,1))="A","AOP","")))))))),IF($B176="Challan","",IF(W176&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z176" s="28"/>
       <c r="AA176" s="29">
@@ -16516,10 +16516,10 @@
       <c r="V177" s="28"/>
       <c r="W177" s="28"/>
       <c r="X177" s="23">
-        <f>IF($B177&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W177)))=10,CODE(MID(TRIM(UPPER(W177)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W177)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W177)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W177)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B177="Entry",IF(AND(LEN(TRIM(UPPER(W177)))=10,CODE(MID(TRIM(UPPER(W177)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W177)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W177)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W177)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W177)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W177)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W177)),9,1))&lt;=57),"N","Y"),IF($B177="Challan","",IF(W177&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y177" s="23">
-        <f>IF($B177&lt;&gt;"Entry","",IF(LEN(W177)&lt;4,"",IF(UPPER(MID(W177,4,1))="P","Individual",IF(UPPER(MID(W177,4,1))="H","HUF",IF(UPPER(MID(W177,4,1))="C","Company",IF(UPPER(MID(W177,4,1))="F","Firm",IF(UPPER(MID(W177,4,1))="L","LLP",IF(UPPER(MID(W177,4,1))="T","Trust",IF(UPPER(MID(W177,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B177="Entry",IF(LEN(W177)&lt;4,"",IF(UPPER(MID(W177,4,1))="P","Individual",IF(UPPER(MID(W177,4,1))="H","HUF",IF(UPPER(MID(W177,4,1))="C","Company",IF(UPPER(MID(W177,4,1))="F","Firm",IF(UPPER(MID(W177,4,1))="L","LLP",IF(UPPER(MID(W177,4,1))="T","Trust",IF(UPPER(MID(W177,4,1))="A","AOP","")))))))),IF($B177="Challan","",IF(W177&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z177" s="28"/>
       <c r="AA177" s="29">
@@ -16594,10 +16594,10 @@
       <c r="V178" s="28"/>
       <c r="W178" s="28"/>
       <c r="X178" s="23">
-        <f>IF($B178&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W178)))=10,CODE(MID(TRIM(UPPER(W178)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W178)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W178)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W178)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B178="Entry",IF(AND(LEN(TRIM(UPPER(W178)))=10,CODE(MID(TRIM(UPPER(W178)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W178)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W178)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W178)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W178)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W178)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W178)),9,1))&lt;=57),"N","Y"),IF($B178="Challan","",IF(W178&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y178" s="23">
-        <f>IF($B178&lt;&gt;"Entry","",IF(LEN(W178)&lt;4,"",IF(UPPER(MID(W178,4,1))="P","Individual",IF(UPPER(MID(W178,4,1))="H","HUF",IF(UPPER(MID(W178,4,1))="C","Company",IF(UPPER(MID(W178,4,1))="F","Firm",IF(UPPER(MID(W178,4,1))="L","LLP",IF(UPPER(MID(W178,4,1))="T","Trust",IF(UPPER(MID(W178,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B178="Entry",IF(LEN(W178)&lt;4,"",IF(UPPER(MID(W178,4,1))="P","Individual",IF(UPPER(MID(W178,4,1))="H","HUF",IF(UPPER(MID(W178,4,1))="C","Company",IF(UPPER(MID(W178,4,1))="F","Firm",IF(UPPER(MID(W178,4,1))="L","LLP",IF(UPPER(MID(W178,4,1))="T","Trust",IF(UPPER(MID(W178,4,1))="A","AOP","")))))))),IF($B178="Challan","",IF(W178&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z178" s="28"/>
       <c r="AA178" s="29">
@@ -16672,10 +16672,10 @@
       <c r="V179" s="28"/>
       <c r="W179" s="28"/>
       <c r="X179" s="23">
-        <f>IF($B179&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W179)))=10,CODE(MID(TRIM(UPPER(W179)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W179)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W179)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W179)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B179="Entry",IF(AND(LEN(TRIM(UPPER(W179)))=10,CODE(MID(TRIM(UPPER(W179)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W179)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W179)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W179)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W179)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W179)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W179)),9,1))&lt;=57),"N","Y"),IF($B179="Challan","",IF(W179&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y179" s="23">
-        <f>IF($B179&lt;&gt;"Entry","",IF(LEN(W179)&lt;4,"",IF(UPPER(MID(W179,4,1))="P","Individual",IF(UPPER(MID(W179,4,1))="H","HUF",IF(UPPER(MID(W179,4,1))="C","Company",IF(UPPER(MID(W179,4,1))="F","Firm",IF(UPPER(MID(W179,4,1))="L","LLP",IF(UPPER(MID(W179,4,1))="T","Trust",IF(UPPER(MID(W179,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B179="Entry",IF(LEN(W179)&lt;4,"",IF(UPPER(MID(W179,4,1))="P","Individual",IF(UPPER(MID(W179,4,1))="H","HUF",IF(UPPER(MID(W179,4,1))="C","Company",IF(UPPER(MID(W179,4,1))="F","Firm",IF(UPPER(MID(W179,4,1))="L","LLP",IF(UPPER(MID(W179,4,1))="T","Trust",IF(UPPER(MID(W179,4,1))="A","AOP","")))))))),IF($B179="Challan","",IF(W179&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z179" s="28"/>
       <c r="AA179" s="29">
@@ -16750,10 +16750,10 @@
       <c r="V180" s="28"/>
       <c r="W180" s="28"/>
       <c r="X180" s="23">
-        <f>IF($B180&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W180)))=10,CODE(MID(TRIM(UPPER(W180)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W180)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W180)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W180)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B180="Entry",IF(AND(LEN(TRIM(UPPER(W180)))=10,CODE(MID(TRIM(UPPER(W180)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W180)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W180)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W180)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W180)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W180)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W180)),9,1))&lt;=57),"N","Y"),IF($B180="Challan","",IF(W180&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y180" s="23">
-        <f>IF($B180&lt;&gt;"Entry","",IF(LEN(W180)&lt;4,"",IF(UPPER(MID(W180,4,1))="P","Individual",IF(UPPER(MID(W180,4,1))="H","HUF",IF(UPPER(MID(W180,4,1))="C","Company",IF(UPPER(MID(W180,4,1))="F","Firm",IF(UPPER(MID(W180,4,1))="L","LLP",IF(UPPER(MID(W180,4,1))="T","Trust",IF(UPPER(MID(W180,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B180="Entry",IF(LEN(W180)&lt;4,"",IF(UPPER(MID(W180,4,1))="P","Individual",IF(UPPER(MID(W180,4,1))="H","HUF",IF(UPPER(MID(W180,4,1))="C","Company",IF(UPPER(MID(W180,4,1))="F","Firm",IF(UPPER(MID(W180,4,1))="L","LLP",IF(UPPER(MID(W180,4,1))="T","Trust",IF(UPPER(MID(W180,4,1))="A","AOP","")))))))),IF($B180="Challan","",IF(W180&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z180" s="28"/>
       <c r="AA180" s="29">
@@ -16828,10 +16828,10 @@
       <c r="V181" s="28"/>
       <c r="W181" s="28"/>
       <c r="X181" s="23">
-        <f>IF($B181&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W181)))=10,CODE(MID(TRIM(UPPER(W181)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W181)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W181)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W181)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B181="Entry",IF(AND(LEN(TRIM(UPPER(W181)))=10,CODE(MID(TRIM(UPPER(W181)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W181)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W181)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W181)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W181)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W181)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W181)),9,1))&lt;=57),"N","Y"),IF($B181="Challan","",IF(W181&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y181" s="23">
-        <f>IF($B181&lt;&gt;"Entry","",IF(LEN(W181)&lt;4,"",IF(UPPER(MID(W181,4,1))="P","Individual",IF(UPPER(MID(W181,4,1))="H","HUF",IF(UPPER(MID(W181,4,1))="C","Company",IF(UPPER(MID(W181,4,1))="F","Firm",IF(UPPER(MID(W181,4,1))="L","LLP",IF(UPPER(MID(W181,4,1))="T","Trust",IF(UPPER(MID(W181,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B181="Entry",IF(LEN(W181)&lt;4,"",IF(UPPER(MID(W181,4,1))="P","Individual",IF(UPPER(MID(W181,4,1))="H","HUF",IF(UPPER(MID(W181,4,1))="C","Company",IF(UPPER(MID(W181,4,1))="F","Firm",IF(UPPER(MID(W181,4,1))="L","LLP",IF(UPPER(MID(W181,4,1))="T","Trust",IF(UPPER(MID(W181,4,1))="A","AOP","")))))))),IF($B181="Challan","",IF(W181&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z181" s="28"/>
       <c r="AA181" s="29">
@@ -16906,10 +16906,10 @@
       <c r="V182" s="28"/>
       <c r="W182" s="28"/>
       <c r="X182" s="23">
-        <f>IF($B182&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W182)))=10,CODE(MID(TRIM(UPPER(W182)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W182)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W182)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W182)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B182="Entry",IF(AND(LEN(TRIM(UPPER(W182)))=10,CODE(MID(TRIM(UPPER(W182)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W182)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W182)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W182)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W182)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W182)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W182)),9,1))&lt;=57),"N","Y"),IF($B182="Challan","",IF(W182&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y182" s="23">
-        <f>IF($B182&lt;&gt;"Entry","",IF(LEN(W182)&lt;4,"",IF(UPPER(MID(W182,4,1))="P","Individual",IF(UPPER(MID(W182,4,1))="H","HUF",IF(UPPER(MID(W182,4,1))="C","Company",IF(UPPER(MID(W182,4,1))="F","Firm",IF(UPPER(MID(W182,4,1))="L","LLP",IF(UPPER(MID(W182,4,1))="T","Trust",IF(UPPER(MID(W182,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B182="Entry",IF(LEN(W182)&lt;4,"",IF(UPPER(MID(W182,4,1))="P","Individual",IF(UPPER(MID(W182,4,1))="H","HUF",IF(UPPER(MID(W182,4,1))="C","Company",IF(UPPER(MID(W182,4,1))="F","Firm",IF(UPPER(MID(W182,4,1))="L","LLP",IF(UPPER(MID(W182,4,1))="T","Trust",IF(UPPER(MID(W182,4,1))="A","AOP","")))))))),IF($B182="Challan","",IF(W182&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z182" s="28"/>
       <c r="AA182" s="29">
@@ -16984,10 +16984,10 @@
       <c r="V183" s="28"/>
       <c r="W183" s="28"/>
       <c r="X183" s="23">
-        <f>IF($B183&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W183)))=10,CODE(MID(TRIM(UPPER(W183)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W183)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W183)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W183)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B183="Entry",IF(AND(LEN(TRIM(UPPER(W183)))=10,CODE(MID(TRIM(UPPER(W183)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W183)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W183)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W183)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W183)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W183)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W183)),9,1))&lt;=57),"N","Y"),IF($B183="Challan","",IF(W183&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y183" s="23">
-        <f>IF($B183&lt;&gt;"Entry","",IF(LEN(W183)&lt;4,"",IF(UPPER(MID(W183,4,1))="P","Individual",IF(UPPER(MID(W183,4,1))="H","HUF",IF(UPPER(MID(W183,4,1))="C","Company",IF(UPPER(MID(W183,4,1))="F","Firm",IF(UPPER(MID(W183,4,1))="L","LLP",IF(UPPER(MID(W183,4,1))="T","Trust",IF(UPPER(MID(W183,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B183="Entry",IF(LEN(W183)&lt;4,"",IF(UPPER(MID(W183,4,1))="P","Individual",IF(UPPER(MID(W183,4,1))="H","HUF",IF(UPPER(MID(W183,4,1))="C","Company",IF(UPPER(MID(W183,4,1))="F","Firm",IF(UPPER(MID(W183,4,1))="L","LLP",IF(UPPER(MID(W183,4,1))="T","Trust",IF(UPPER(MID(W183,4,1))="A","AOP","")))))))),IF($B183="Challan","",IF(W183&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z183" s="28"/>
       <c r="AA183" s="29">
@@ -17062,10 +17062,10 @@
       <c r="V184" s="28"/>
       <c r="W184" s="28"/>
       <c r="X184" s="23">
-        <f>IF($B184&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W184)))=10,CODE(MID(TRIM(UPPER(W184)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W184)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W184)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W184)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B184="Entry",IF(AND(LEN(TRIM(UPPER(W184)))=10,CODE(MID(TRIM(UPPER(W184)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W184)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W184)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W184)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W184)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W184)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W184)),9,1))&lt;=57),"N","Y"),IF($B184="Challan","",IF(W184&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y184" s="23">
-        <f>IF($B184&lt;&gt;"Entry","",IF(LEN(W184)&lt;4,"",IF(UPPER(MID(W184,4,1))="P","Individual",IF(UPPER(MID(W184,4,1))="H","HUF",IF(UPPER(MID(W184,4,1))="C","Company",IF(UPPER(MID(W184,4,1))="F","Firm",IF(UPPER(MID(W184,4,1))="L","LLP",IF(UPPER(MID(W184,4,1))="T","Trust",IF(UPPER(MID(W184,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B184="Entry",IF(LEN(W184)&lt;4,"",IF(UPPER(MID(W184,4,1))="P","Individual",IF(UPPER(MID(W184,4,1))="H","HUF",IF(UPPER(MID(W184,4,1))="C","Company",IF(UPPER(MID(W184,4,1))="F","Firm",IF(UPPER(MID(W184,4,1))="L","LLP",IF(UPPER(MID(W184,4,1))="T","Trust",IF(UPPER(MID(W184,4,1))="A","AOP","")))))))),IF($B184="Challan","",IF(W184&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z184" s="28"/>
       <c r="AA184" s="29">
@@ -17140,10 +17140,10 @@
       <c r="V185" s="28"/>
       <c r="W185" s="28"/>
       <c r="X185" s="23">
-        <f>IF($B185&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W185)))=10,CODE(MID(TRIM(UPPER(W185)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W185)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W185)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W185)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B185="Entry",IF(AND(LEN(TRIM(UPPER(W185)))=10,CODE(MID(TRIM(UPPER(W185)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W185)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W185)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W185)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W185)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W185)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W185)),9,1))&lt;=57),"N","Y"),IF($B185="Challan","",IF(W185&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y185" s="23">
-        <f>IF($B185&lt;&gt;"Entry","",IF(LEN(W185)&lt;4,"",IF(UPPER(MID(W185,4,1))="P","Individual",IF(UPPER(MID(W185,4,1))="H","HUF",IF(UPPER(MID(W185,4,1))="C","Company",IF(UPPER(MID(W185,4,1))="F","Firm",IF(UPPER(MID(W185,4,1))="L","LLP",IF(UPPER(MID(W185,4,1))="T","Trust",IF(UPPER(MID(W185,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B185="Entry",IF(LEN(W185)&lt;4,"",IF(UPPER(MID(W185,4,1))="P","Individual",IF(UPPER(MID(W185,4,1))="H","HUF",IF(UPPER(MID(W185,4,1))="C","Company",IF(UPPER(MID(W185,4,1))="F","Firm",IF(UPPER(MID(W185,4,1))="L","LLP",IF(UPPER(MID(W185,4,1))="T","Trust",IF(UPPER(MID(W185,4,1))="A","AOP","")))))))),IF($B185="Challan","",IF(W185&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z185" s="28"/>
       <c r="AA185" s="29">
@@ -17218,10 +17218,10 @@
       <c r="V186" s="28"/>
       <c r="W186" s="28"/>
       <c r="X186" s="23">
-        <f>IF($B186&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W186)))=10,CODE(MID(TRIM(UPPER(W186)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W186)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W186)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W186)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B186="Entry",IF(AND(LEN(TRIM(UPPER(W186)))=10,CODE(MID(TRIM(UPPER(W186)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W186)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W186)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W186)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W186)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W186)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W186)),9,1))&lt;=57),"N","Y"),IF($B186="Challan","",IF(W186&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y186" s="23">
-        <f>IF($B186&lt;&gt;"Entry","",IF(LEN(W186)&lt;4,"",IF(UPPER(MID(W186,4,1))="P","Individual",IF(UPPER(MID(W186,4,1))="H","HUF",IF(UPPER(MID(W186,4,1))="C","Company",IF(UPPER(MID(W186,4,1))="F","Firm",IF(UPPER(MID(W186,4,1))="L","LLP",IF(UPPER(MID(W186,4,1))="T","Trust",IF(UPPER(MID(W186,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B186="Entry",IF(LEN(W186)&lt;4,"",IF(UPPER(MID(W186,4,1))="P","Individual",IF(UPPER(MID(W186,4,1))="H","HUF",IF(UPPER(MID(W186,4,1))="C","Company",IF(UPPER(MID(W186,4,1))="F","Firm",IF(UPPER(MID(W186,4,1))="L","LLP",IF(UPPER(MID(W186,4,1))="T","Trust",IF(UPPER(MID(W186,4,1))="A","AOP","")))))))),IF($B186="Challan","",IF(W186&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z186" s="28"/>
       <c r="AA186" s="29">
@@ -17296,10 +17296,10 @@
       <c r="V187" s="28"/>
       <c r="W187" s="28"/>
       <c r="X187" s="23">
-        <f>IF($B187&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W187)))=10,CODE(MID(TRIM(UPPER(W187)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W187)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W187)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W187)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B187="Entry",IF(AND(LEN(TRIM(UPPER(W187)))=10,CODE(MID(TRIM(UPPER(W187)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W187)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W187)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W187)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W187)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W187)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W187)),9,1))&lt;=57),"N","Y"),IF($B187="Challan","",IF(W187&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y187" s="23">
-        <f>IF($B187&lt;&gt;"Entry","",IF(LEN(W187)&lt;4,"",IF(UPPER(MID(W187,4,1))="P","Individual",IF(UPPER(MID(W187,4,1))="H","HUF",IF(UPPER(MID(W187,4,1))="C","Company",IF(UPPER(MID(W187,4,1))="F","Firm",IF(UPPER(MID(W187,4,1))="L","LLP",IF(UPPER(MID(W187,4,1))="T","Trust",IF(UPPER(MID(W187,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B187="Entry",IF(LEN(W187)&lt;4,"",IF(UPPER(MID(W187,4,1))="P","Individual",IF(UPPER(MID(W187,4,1))="H","HUF",IF(UPPER(MID(W187,4,1))="C","Company",IF(UPPER(MID(W187,4,1))="F","Firm",IF(UPPER(MID(W187,4,1))="L","LLP",IF(UPPER(MID(W187,4,1))="T","Trust",IF(UPPER(MID(W187,4,1))="A","AOP","")))))))),IF($B187="Challan","",IF(W187&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z187" s="28"/>
       <c r="AA187" s="29">
@@ -17374,10 +17374,10 @@
       <c r="V188" s="28"/>
       <c r="W188" s="28"/>
       <c r="X188" s="23">
-        <f>IF($B188&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W188)))=10,CODE(MID(TRIM(UPPER(W188)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W188)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W188)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W188)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B188="Entry",IF(AND(LEN(TRIM(UPPER(W188)))=10,CODE(MID(TRIM(UPPER(W188)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W188)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W188)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W188)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W188)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W188)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W188)),9,1))&lt;=57),"N","Y"),IF($B188="Challan","",IF(W188&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y188" s="23">
-        <f>IF($B188&lt;&gt;"Entry","",IF(LEN(W188)&lt;4,"",IF(UPPER(MID(W188,4,1))="P","Individual",IF(UPPER(MID(W188,4,1))="H","HUF",IF(UPPER(MID(W188,4,1))="C","Company",IF(UPPER(MID(W188,4,1))="F","Firm",IF(UPPER(MID(W188,4,1))="L","LLP",IF(UPPER(MID(W188,4,1))="T","Trust",IF(UPPER(MID(W188,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B188="Entry",IF(LEN(W188)&lt;4,"",IF(UPPER(MID(W188,4,1))="P","Individual",IF(UPPER(MID(W188,4,1))="H","HUF",IF(UPPER(MID(W188,4,1))="C","Company",IF(UPPER(MID(W188,4,1))="F","Firm",IF(UPPER(MID(W188,4,1))="L","LLP",IF(UPPER(MID(W188,4,1))="T","Trust",IF(UPPER(MID(W188,4,1))="A","AOP","")))))))),IF($B188="Challan","",IF(W188&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z188" s="28"/>
       <c r="AA188" s="29">
@@ -17452,10 +17452,10 @@
       <c r="V189" s="28"/>
       <c r="W189" s="28"/>
       <c r="X189" s="23">
-        <f>IF($B189&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W189)))=10,CODE(MID(TRIM(UPPER(W189)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W189)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W189)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W189)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B189="Entry",IF(AND(LEN(TRIM(UPPER(W189)))=10,CODE(MID(TRIM(UPPER(W189)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W189)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W189)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W189)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W189)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W189)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W189)),9,1))&lt;=57),"N","Y"),IF($B189="Challan","",IF(W189&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y189" s="23">
-        <f>IF($B189&lt;&gt;"Entry","",IF(LEN(W189)&lt;4,"",IF(UPPER(MID(W189,4,1))="P","Individual",IF(UPPER(MID(W189,4,1))="H","HUF",IF(UPPER(MID(W189,4,1))="C","Company",IF(UPPER(MID(W189,4,1))="F","Firm",IF(UPPER(MID(W189,4,1))="L","LLP",IF(UPPER(MID(W189,4,1))="T","Trust",IF(UPPER(MID(W189,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B189="Entry",IF(LEN(W189)&lt;4,"",IF(UPPER(MID(W189,4,1))="P","Individual",IF(UPPER(MID(W189,4,1))="H","HUF",IF(UPPER(MID(W189,4,1))="C","Company",IF(UPPER(MID(W189,4,1))="F","Firm",IF(UPPER(MID(W189,4,1))="L","LLP",IF(UPPER(MID(W189,4,1))="T","Trust",IF(UPPER(MID(W189,4,1))="A","AOP","")))))))),IF($B189="Challan","",IF(W189&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z189" s="28"/>
       <c r="AA189" s="29">
@@ -17530,10 +17530,10 @@
       <c r="V190" s="28"/>
       <c r="W190" s="28"/>
       <c r="X190" s="23">
-        <f>IF($B190&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W190)))=10,CODE(MID(TRIM(UPPER(W190)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W190)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W190)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W190)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B190="Entry",IF(AND(LEN(TRIM(UPPER(W190)))=10,CODE(MID(TRIM(UPPER(W190)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W190)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W190)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W190)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W190)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W190)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W190)),9,1))&lt;=57),"N","Y"),IF($B190="Challan","",IF(W190&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y190" s="23">
-        <f>IF($B190&lt;&gt;"Entry","",IF(LEN(W190)&lt;4,"",IF(UPPER(MID(W190,4,1))="P","Individual",IF(UPPER(MID(W190,4,1))="H","HUF",IF(UPPER(MID(W190,4,1))="C","Company",IF(UPPER(MID(W190,4,1))="F","Firm",IF(UPPER(MID(W190,4,1))="L","LLP",IF(UPPER(MID(W190,4,1))="T","Trust",IF(UPPER(MID(W190,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B190="Entry",IF(LEN(W190)&lt;4,"",IF(UPPER(MID(W190,4,1))="P","Individual",IF(UPPER(MID(W190,4,1))="H","HUF",IF(UPPER(MID(W190,4,1))="C","Company",IF(UPPER(MID(W190,4,1))="F","Firm",IF(UPPER(MID(W190,4,1))="L","LLP",IF(UPPER(MID(W190,4,1))="T","Trust",IF(UPPER(MID(W190,4,1))="A","AOP","")))))))),IF($B190="Challan","",IF(W190&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z190" s="28"/>
       <c r="AA190" s="29">
@@ -17608,10 +17608,10 @@
       <c r="V191" s="28"/>
       <c r="W191" s="28"/>
       <c r="X191" s="23">
-        <f>IF($B191&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W191)))=10,CODE(MID(TRIM(UPPER(W191)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W191)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W191)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W191)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B191="Entry",IF(AND(LEN(TRIM(UPPER(W191)))=10,CODE(MID(TRIM(UPPER(W191)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W191)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W191)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W191)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W191)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W191)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W191)),9,1))&lt;=57),"N","Y"),IF($B191="Challan","",IF(W191&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y191" s="23">
-        <f>IF($B191&lt;&gt;"Entry","",IF(LEN(W191)&lt;4,"",IF(UPPER(MID(W191,4,1))="P","Individual",IF(UPPER(MID(W191,4,1))="H","HUF",IF(UPPER(MID(W191,4,1))="C","Company",IF(UPPER(MID(W191,4,1))="F","Firm",IF(UPPER(MID(W191,4,1))="L","LLP",IF(UPPER(MID(W191,4,1))="T","Trust",IF(UPPER(MID(W191,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B191="Entry",IF(LEN(W191)&lt;4,"",IF(UPPER(MID(W191,4,1))="P","Individual",IF(UPPER(MID(W191,4,1))="H","HUF",IF(UPPER(MID(W191,4,1))="C","Company",IF(UPPER(MID(W191,4,1))="F","Firm",IF(UPPER(MID(W191,4,1))="L","LLP",IF(UPPER(MID(W191,4,1))="T","Trust",IF(UPPER(MID(W191,4,1))="A","AOP","")))))))),IF($B191="Challan","",IF(W191&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z191" s="28"/>
       <c r="AA191" s="29">
@@ -17686,10 +17686,10 @@
       <c r="V192" s="28"/>
       <c r="W192" s="28"/>
       <c r="X192" s="23">
-        <f>IF($B192&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W192)))=10,CODE(MID(TRIM(UPPER(W192)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W192)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W192)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W192)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B192="Entry",IF(AND(LEN(TRIM(UPPER(W192)))=10,CODE(MID(TRIM(UPPER(W192)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W192)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W192)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W192)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W192)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W192)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W192)),9,1))&lt;=57),"N","Y"),IF($B192="Challan","",IF(W192&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y192" s="23">
-        <f>IF($B192&lt;&gt;"Entry","",IF(LEN(W192)&lt;4,"",IF(UPPER(MID(W192,4,1))="P","Individual",IF(UPPER(MID(W192,4,1))="H","HUF",IF(UPPER(MID(W192,4,1))="C","Company",IF(UPPER(MID(W192,4,1))="F","Firm",IF(UPPER(MID(W192,4,1))="L","LLP",IF(UPPER(MID(W192,4,1))="T","Trust",IF(UPPER(MID(W192,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B192="Entry",IF(LEN(W192)&lt;4,"",IF(UPPER(MID(W192,4,1))="P","Individual",IF(UPPER(MID(W192,4,1))="H","HUF",IF(UPPER(MID(W192,4,1))="C","Company",IF(UPPER(MID(W192,4,1))="F","Firm",IF(UPPER(MID(W192,4,1))="L","LLP",IF(UPPER(MID(W192,4,1))="T","Trust",IF(UPPER(MID(W192,4,1))="A","AOP","")))))))),IF($B192="Challan","",IF(W192&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z192" s="28"/>
       <c r="AA192" s="29">
@@ -17764,10 +17764,10 @@
       <c r="V193" s="28"/>
       <c r="W193" s="28"/>
       <c r="X193" s="23">
-        <f>IF($B193&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W193)))=10,CODE(MID(TRIM(UPPER(W193)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W193)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W193)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W193)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B193="Entry",IF(AND(LEN(TRIM(UPPER(W193)))=10,CODE(MID(TRIM(UPPER(W193)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W193)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W193)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W193)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W193)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W193)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W193)),9,1))&lt;=57),"N","Y"),IF($B193="Challan","",IF(W193&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y193" s="23">
-        <f>IF($B193&lt;&gt;"Entry","",IF(LEN(W193)&lt;4,"",IF(UPPER(MID(W193,4,1))="P","Individual",IF(UPPER(MID(W193,4,1))="H","HUF",IF(UPPER(MID(W193,4,1))="C","Company",IF(UPPER(MID(W193,4,1))="F","Firm",IF(UPPER(MID(W193,4,1))="L","LLP",IF(UPPER(MID(W193,4,1))="T","Trust",IF(UPPER(MID(W193,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B193="Entry",IF(LEN(W193)&lt;4,"",IF(UPPER(MID(W193,4,1))="P","Individual",IF(UPPER(MID(W193,4,1))="H","HUF",IF(UPPER(MID(W193,4,1))="C","Company",IF(UPPER(MID(W193,4,1))="F","Firm",IF(UPPER(MID(W193,4,1))="L","LLP",IF(UPPER(MID(W193,4,1))="T","Trust",IF(UPPER(MID(W193,4,1))="A","AOP","")))))))),IF($B193="Challan","",IF(W193&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z193" s="28"/>
       <c r="AA193" s="29">
@@ -17842,10 +17842,10 @@
       <c r="V194" s="28"/>
       <c r="W194" s="28"/>
       <c r="X194" s="23">
-        <f>IF($B194&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W194)))=10,CODE(MID(TRIM(UPPER(W194)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W194)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W194)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W194)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B194="Entry",IF(AND(LEN(TRIM(UPPER(W194)))=10,CODE(MID(TRIM(UPPER(W194)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W194)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W194)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W194)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W194)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W194)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W194)),9,1))&lt;=57),"N","Y"),IF($B194="Challan","",IF(W194&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y194" s="23">
-        <f>IF($B194&lt;&gt;"Entry","",IF(LEN(W194)&lt;4,"",IF(UPPER(MID(W194,4,1))="P","Individual",IF(UPPER(MID(W194,4,1))="H","HUF",IF(UPPER(MID(W194,4,1))="C","Company",IF(UPPER(MID(W194,4,1))="F","Firm",IF(UPPER(MID(W194,4,1))="L","LLP",IF(UPPER(MID(W194,4,1))="T","Trust",IF(UPPER(MID(W194,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B194="Entry",IF(LEN(W194)&lt;4,"",IF(UPPER(MID(W194,4,1))="P","Individual",IF(UPPER(MID(W194,4,1))="H","HUF",IF(UPPER(MID(W194,4,1))="C","Company",IF(UPPER(MID(W194,4,1))="F","Firm",IF(UPPER(MID(W194,4,1))="L","LLP",IF(UPPER(MID(W194,4,1))="T","Trust",IF(UPPER(MID(W194,4,1))="A","AOP","")))))))),IF($B194="Challan","",IF(W194&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z194" s="28"/>
       <c r="AA194" s="29">
@@ -17920,10 +17920,10 @@
       <c r="V195" s="28"/>
       <c r="W195" s="28"/>
       <c r="X195" s="23">
-        <f>IF($B195&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W195)))=10,CODE(MID(TRIM(UPPER(W195)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W195)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W195)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W195)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B195="Entry",IF(AND(LEN(TRIM(UPPER(W195)))=10,CODE(MID(TRIM(UPPER(W195)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W195)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W195)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W195)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W195)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W195)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W195)),9,1))&lt;=57),"N","Y"),IF($B195="Challan","",IF(W195&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y195" s="23">
-        <f>IF($B195&lt;&gt;"Entry","",IF(LEN(W195)&lt;4,"",IF(UPPER(MID(W195,4,1))="P","Individual",IF(UPPER(MID(W195,4,1))="H","HUF",IF(UPPER(MID(W195,4,1))="C","Company",IF(UPPER(MID(W195,4,1))="F","Firm",IF(UPPER(MID(W195,4,1))="L","LLP",IF(UPPER(MID(W195,4,1))="T","Trust",IF(UPPER(MID(W195,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B195="Entry",IF(LEN(W195)&lt;4,"",IF(UPPER(MID(W195,4,1))="P","Individual",IF(UPPER(MID(W195,4,1))="H","HUF",IF(UPPER(MID(W195,4,1))="C","Company",IF(UPPER(MID(W195,4,1))="F","Firm",IF(UPPER(MID(W195,4,1))="L","LLP",IF(UPPER(MID(W195,4,1))="T","Trust",IF(UPPER(MID(W195,4,1))="A","AOP","")))))))),IF($B195="Challan","",IF(W195&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z195" s="28"/>
       <c r="AA195" s="29">
@@ -17998,10 +17998,10 @@
       <c r="V196" s="28"/>
       <c r="W196" s="28"/>
       <c r="X196" s="23">
-        <f>IF($B196&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W196)))=10,CODE(MID(TRIM(UPPER(W196)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W196)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W196)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W196)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B196="Entry",IF(AND(LEN(TRIM(UPPER(W196)))=10,CODE(MID(TRIM(UPPER(W196)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W196)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W196)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W196)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W196)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W196)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W196)),9,1))&lt;=57),"N","Y"),IF($B196="Challan","",IF(W196&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y196" s="23">
-        <f>IF($B196&lt;&gt;"Entry","",IF(LEN(W196)&lt;4,"",IF(UPPER(MID(W196,4,1))="P","Individual",IF(UPPER(MID(W196,4,1))="H","HUF",IF(UPPER(MID(W196,4,1))="C","Company",IF(UPPER(MID(W196,4,1))="F","Firm",IF(UPPER(MID(W196,4,1))="L","LLP",IF(UPPER(MID(W196,4,1))="T","Trust",IF(UPPER(MID(W196,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B196="Entry",IF(LEN(W196)&lt;4,"",IF(UPPER(MID(W196,4,1))="P","Individual",IF(UPPER(MID(W196,4,1))="H","HUF",IF(UPPER(MID(W196,4,1))="C","Company",IF(UPPER(MID(W196,4,1))="F","Firm",IF(UPPER(MID(W196,4,1))="L","LLP",IF(UPPER(MID(W196,4,1))="T","Trust",IF(UPPER(MID(W196,4,1))="A","AOP","")))))))),IF($B196="Challan","",IF(W196&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z196" s="28"/>
       <c r="AA196" s="29">
@@ -18076,10 +18076,10 @@
       <c r="V197" s="28"/>
       <c r="W197" s="28"/>
       <c r="X197" s="23">
-        <f>IF($B197&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W197)))=10,CODE(MID(TRIM(UPPER(W197)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W197)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W197)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W197)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B197="Entry",IF(AND(LEN(TRIM(UPPER(W197)))=10,CODE(MID(TRIM(UPPER(W197)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W197)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W197)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W197)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W197)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W197)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W197)),9,1))&lt;=57),"N","Y"),IF($B197="Challan","",IF(W197&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y197" s="23">
-        <f>IF($B197&lt;&gt;"Entry","",IF(LEN(W197)&lt;4,"",IF(UPPER(MID(W197,4,1))="P","Individual",IF(UPPER(MID(W197,4,1))="H","HUF",IF(UPPER(MID(W197,4,1))="C","Company",IF(UPPER(MID(W197,4,1))="F","Firm",IF(UPPER(MID(W197,4,1))="L","LLP",IF(UPPER(MID(W197,4,1))="T","Trust",IF(UPPER(MID(W197,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B197="Entry",IF(LEN(W197)&lt;4,"",IF(UPPER(MID(W197,4,1))="P","Individual",IF(UPPER(MID(W197,4,1))="H","HUF",IF(UPPER(MID(W197,4,1))="C","Company",IF(UPPER(MID(W197,4,1))="F","Firm",IF(UPPER(MID(W197,4,1))="L","LLP",IF(UPPER(MID(W197,4,1))="T","Trust",IF(UPPER(MID(W197,4,1))="A","AOP","")))))))),IF($B197="Challan","",IF(W197&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z197" s="28"/>
       <c r="AA197" s="29">
@@ -18154,10 +18154,10 @@
       <c r="V198" s="28"/>
       <c r="W198" s="28"/>
       <c r="X198" s="23">
-        <f>IF($B198&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W198)))=10,CODE(MID(TRIM(UPPER(W198)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W198)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W198)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W198)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B198="Entry",IF(AND(LEN(TRIM(UPPER(W198)))=10,CODE(MID(TRIM(UPPER(W198)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W198)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W198)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W198)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W198)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W198)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W198)),9,1))&lt;=57),"N","Y"),IF($B198="Challan","",IF(W198&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y198" s="23">
-        <f>IF($B198&lt;&gt;"Entry","",IF(LEN(W198)&lt;4,"",IF(UPPER(MID(W198,4,1))="P","Individual",IF(UPPER(MID(W198,4,1))="H","HUF",IF(UPPER(MID(W198,4,1))="C","Company",IF(UPPER(MID(W198,4,1))="F","Firm",IF(UPPER(MID(W198,4,1))="L","LLP",IF(UPPER(MID(W198,4,1))="T","Trust",IF(UPPER(MID(W198,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B198="Entry",IF(LEN(W198)&lt;4,"",IF(UPPER(MID(W198,4,1))="P","Individual",IF(UPPER(MID(W198,4,1))="H","HUF",IF(UPPER(MID(W198,4,1))="C","Company",IF(UPPER(MID(W198,4,1))="F","Firm",IF(UPPER(MID(W198,4,1))="L","LLP",IF(UPPER(MID(W198,4,1))="T","Trust",IF(UPPER(MID(W198,4,1))="A","AOP","")))))))),IF($B198="Challan","",IF(W198&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z198" s="28"/>
       <c r="AA198" s="29">
@@ -18232,10 +18232,10 @@
       <c r="V199" s="28"/>
       <c r="W199" s="28"/>
       <c r="X199" s="23">
-        <f>IF($B199&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W199)))=10,CODE(MID(TRIM(UPPER(W199)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W199)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W199)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W199)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B199="Entry",IF(AND(LEN(TRIM(UPPER(W199)))=10,CODE(MID(TRIM(UPPER(W199)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W199)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W199)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W199)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W199)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W199)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W199)),9,1))&lt;=57),"N","Y"),IF($B199="Challan","",IF(W199&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y199" s="23">
-        <f>IF($B199&lt;&gt;"Entry","",IF(LEN(W199)&lt;4,"",IF(UPPER(MID(W199,4,1))="P","Individual",IF(UPPER(MID(W199,4,1))="H","HUF",IF(UPPER(MID(W199,4,1))="C","Company",IF(UPPER(MID(W199,4,1))="F","Firm",IF(UPPER(MID(W199,4,1))="L","LLP",IF(UPPER(MID(W199,4,1))="T","Trust",IF(UPPER(MID(W199,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B199="Entry",IF(LEN(W199)&lt;4,"",IF(UPPER(MID(W199,4,1))="P","Individual",IF(UPPER(MID(W199,4,1))="H","HUF",IF(UPPER(MID(W199,4,1))="C","Company",IF(UPPER(MID(W199,4,1))="F","Firm",IF(UPPER(MID(W199,4,1))="L","LLP",IF(UPPER(MID(W199,4,1))="T","Trust",IF(UPPER(MID(W199,4,1))="A","AOP","")))))))),IF($B199="Challan","",IF(W199&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z199" s="28"/>
       <c r="AA199" s="29">
@@ -18310,10 +18310,10 @@
       <c r="V200" s="28"/>
       <c r="W200" s="28"/>
       <c r="X200" s="23">
-        <f>IF($B200&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W200)))=10,CODE(MID(TRIM(UPPER(W200)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W200)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W200)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W200)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B200="Entry",IF(AND(LEN(TRIM(UPPER(W200)))=10,CODE(MID(TRIM(UPPER(W200)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W200)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W200)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W200)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W200)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W200)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W200)),9,1))&lt;=57),"N","Y"),IF($B200="Challan","",IF(W200&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y200" s="23">
-        <f>IF($B200&lt;&gt;"Entry","",IF(LEN(W200)&lt;4,"",IF(UPPER(MID(W200,4,1))="P","Individual",IF(UPPER(MID(W200,4,1))="H","HUF",IF(UPPER(MID(W200,4,1))="C","Company",IF(UPPER(MID(W200,4,1))="F","Firm",IF(UPPER(MID(W200,4,1))="L","LLP",IF(UPPER(MID(W200,4,1))="T","Trust",IF(UPPER(MID(W200,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B200="Entry",IF(LEN(W200)&lt;4,"",IF(UPPER(MID(W200,4,1))="P","Individual",IF(UPPER(MID(W200,4,1))="H","HUF",IF(UPPER(MID(W200,4,1))="C","Company",IF(UPPER(MID(W200,4,1))="F","Firm",IF(UPPER(MID(W200,4,1))="L","LLP",IF(UPPER(MID(W200,4,1))="T","Trust",IF(UPPER(MID(W200,4,1))="A","AOP","")))))))),IF($B200="Challan","",IF(W200&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z200" s="28"/>
       <c r="AA200" s="29">
@@ -18388,10 +18388,10 @@
       <c r="V201" s="28"/>
       <c r="W201" s="28"/>
       <c r="X201" s="23">
-        <f>IF($B201&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W201)))=10,CODE(MID(TRIM(UPPER(W201)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W201)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W201)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W201)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B201="Entry",IF(AND(LEN(TRIM(UPPER(W201)))=10,CODE(MID(TRIM(UPPER(W201)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W201)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W201)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W201)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W201)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W201)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W201)),9,1))&lt;=57),"N","Y"),IF($B201="Challan","",IF(W201&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y201" s="23">
-        <f>IF($B201&lt;&gt;"Entry","",IF(LEN(W201)&lt;4,"",IF(UPPER(MID(W201,4,1))="P","Individual",IF(UPPER(MID(W201,4,1))="H","HUF",IF(UPPER(MID(W201,4,1))="C","Company",IF(UPPER(MID(W201,4,1))="F","Firm",IF(UPPER(MID(W201,4,1))="L","LLP",IF(UPPER(MID(W201,4,1))="T","Trust",IF(UPPER(MID(W201,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B201="Entry",IF(LEN(W201)&lt;4,"",IF(UPPER(MID(W201,4,1))="P","Individual",IF(UPPER(MID(W201,4,1))="H","HUF",IF(UPPER(MID(W201,4,1))="C","Company",IF(UPPER(MID(W201,4,1))="F","Firm",IF(UPPER(MID(W201,4,1))="L","LLP",IF(UPPER(MID(W201,4,1))="T","Trust",IF(UPPER(MID(W201,4,1))="A","AOP","")))))))),IF($B201="Challan","",IF(W201&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z201" s="28"/>
       <c r="AA201" s="29">
@@ -18466,10 +18466,10 @@
       <c r="V202" s="28"/>
       <c r="W202" s="28"/>
       <c r="X202" s="23">
-        <f>IF($B202&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W202)))=10,CODE(MID(TRIM(UPPER(W202)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W202)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W202)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W202)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B202="Entry",IF(AND(LEN(TRIM(UPPER(W202)))=10,CODE(MID(TRIM(UPPER(W202)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W202)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W202)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W202)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W202)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W202)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W202)),9,1))&lt;=57),"N","Y"),IF($B202="Challan","",IF(W202&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y202" s="23">
-        <f>IF($B202&lt;&gt;"Entry","",IF(LEN(W202)&lt;4,"",IF(UPPER(MID(W202,4,1))="P","Individual",IF(UPPER(MID(W202,4,1))="H","HUF",IF(UPPER(MID(W202,4,1))="C","Company",IF(UPPER(MID(W202,4,1))="F","Firm",IF(UPPER(MID(W202,4,1))="L","LLP",IF(UPPER(MID(W202,4,1))="T","Trust",IF(UPPER(MID(W202,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B202="Entry",IF(LEN(W202)&lt;4,"",IF(UPPER(MID(W202,4,1))="P","Individual",IF(UPPER(MID(W202,4,1))="H","HUF",IF(UPPER(MID(W202,4,1))="C","Company",IF(UPPER(MID(W202,4,1))="F","Firm",IF(UPPER(MID(W202,4,1))="L","LLP",IF(UPPER(MID(W202,4,1))="T","Trust",IF(UPPER(MID(W202,4,1))="A","AOP","")))))))),IF($B202="Challan","",IF(W202&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z202" s="28"/>
       <c r="AA202" s="29">
@@ -18544,10 +18544,10 @@
       <c r="V203" s="28"/>
       <c r="W203" s="28"/>
       <c r="X203" s="23">
-        <f>IF($B203&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W203)))=10,CODE(MID(TRIM(UPPER(W203)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W203)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W203)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W203)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B203="Entry",IF(AND(LEN(TRIM(UPPER(W203)))=10,CODE(MID(TRIM(UPPER(W203)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W203)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W203)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W203)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W203)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W203)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W203)),9,1))&lt;=57),"N","Y"),IF($B203="Challan","",IF(W203&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y203" s="23">
-        <f>IF($B203&lt;&gt;"Entry","",IF(LEN(W203)&lt;4,"",IF(UPPER(MID(W203,4,1))="P","Individual",IF(UPPER(MID(W203,4,1))="H","HUF",IF(UPPER(MID(W203,4,1))="C","Company",IF(UPPER(MID(W203,4,1))="F","Firm",IF(UPPER(MID(W203,4,1))="L","LLP",IF(UPPER(MID(W203,4,1))="T","Trust",IF(UPPER(MID(W203,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B203="Entry",IF(LEN(W203)&lt;4,"",IF(UPPER(MID(W203,4,1))="P","Individual",IF(UPPER(MID(W203,4,1))="H","HUF",IF(UPPER(MID(W203,4,1))="C","Company",IF(UPPER(MID(W203,4,1))="F","Firm",IF(UPPER(MID(W203,4,1))="L","LLP",IF(UPPER(MID(W203,4,1))="T","Trust",IF(UPPER(MID(W203,4,1))="A","AOP","")))))))),IF($B203="Challan","",IF(W203&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z203" s="28"/>
       <c r="AA203" s="29">
@@ -18622,10 +18622,10 @@
       <c r="V204" s="28"/>
       <c r="W204" s="28"/>
       <c r="X204" s="23">
-        <f>IF($B204&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W204)))=10,CODE(MID(TRIM(UPPER(W204)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W204)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W204)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W204)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B204="Entry",IF(AND(LEN(TRIM(UPPER(W204)))=10,CODE(MID(TRIM(UPPER(W204)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W204)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W204)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W204)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W204)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W204)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W204)),9,1))&lt;=57),"N","Y"),IF($B204="Challan","",IF(W204&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y204" s="23">
-        <f>IF($B204&lt;&gt;"Entry","",IF(LEN(W204)&lt;4,"",IF(UPPER(MID(W204,4,1))="P","Individual",IF(UPPER(MID(W204,4,1))="H","HUF",IF(UPPER(MID(W204,4,1))="C","Company",IF(UPPER(MID(W204,4,1))="F","Firm",IF(UPPER(MID(W204,4,1))="L","LLP",IF(UPPER(MID(W204,4,1))="T","Trust",IF(UPPER(MID(W204,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B204="Entry",IF(LEN(W204)&lt;4,"",IF(UPPER(MID(W204,4,1))="P","Individual",IF(UPPER(MID(W204,4,1))="H","HUF",IF(UPPER(MID(W204,4,1))="C","Company",IF(UPPER(MID(W204,4,1))="F","Firm",IF(UPPER(MID(W204,4,1))="L","LLP",IF(UPPER(MID(W204,4,1))="T","Trust",IF(UPPER(MID(W204,4,1))="A","AOP","")))))))),IF($B204="Challan","",IF(W204&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z204" s="28"/>
       <c r="AA204" s="29">
@@ -18700,10 +18700,10 @@
       <c r="V205" s="28"/>
       <c r="W205" s="28"/>
       <c r="X205" s="23">
-        <f>IF($B205&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W205)))=10,CODE(MID(TRIM(UPPER(W205)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W205)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W205)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W205)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B205="Entry",IF(AND(LEN(TRIM(UPPER(W205)))=10,CODE(MID(TRIM(UPPER(W205)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W205)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W205)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W205)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W205)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W205)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W205)),9,1))&lt;=57),"N","Y"),IF($B205="Challan","",IF(W205&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y205" s="23">
-        <f>IF($B205&lt;&gt;"Entry","",IF(LEN(W205)&lt;4,"",IF(UPPER(MID(W205,4,1))="P","Individual",IF(UPPER(MID(W205,4,1))="H","HUF",IF(UPPER(MID(W205,4,1))="C","Company",IF(UPPER(MID(W205,4,1))="F","Firm",IF(UPPER(MID(W205,4,1))="L","LLP",IF(UPPER(MID(W205,4,1))="T","Trust",IF(UPPER(MID(W205,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B205="Entry",IF(LEN(W205)&lt;4,"",IF(UPPER(MID(W205,4,1))="P","Individual",IF(UPPER(MID(W205,4,1))="H","HUF",IF(UPPER(MID(W205,4,1))="C","Company",IF(UPPER(MID(W205,4,1))="F","Firm",IF(UPPER(MID(W205,4,1))="L","LLP",IF(UPPER(MID(W205,4,1))="T","Trust",IF(UPPER(MID(W205,4,1))="A","AOP","")))))))),IF($B205="Challan","",IF(W205&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z205" s="28"/>
       <c r="AA205" s="29">
@@ -18778,10 +18778,10 @@
       <c r="V206" s="28"/>
       <c r="W206" s="28"/>
       <c r="X206" s="23">
-        <f>IF($B206&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W206)))=10,CODE(MID(TRIM(UPPER(W206)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W206)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W206)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W206)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B206="Entry",IF(AND(LEN(TRIM(UPPER(W206)))=10,CODE(MID(TRIM(UPPER(W206)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W206)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W206)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W206)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W206)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W206)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W206)),9,1))&lt;=57),"N","Y"),IF($B206="Challan","",IF(W206&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y206" s="23">
-        <f>IF($B206&lt;&gt;"Entry","",IF(LEN(W206)&lt;4,"",IF(UPPER(MID(W206,4,1))="P","Individual",IF(UPPER(MID(W206,4,1))="H","HUF",IF(UPPER(MID(W206,4,1))="C","Company",IF(UPPER(MID(W206,4,1))="F","Firm",IF(UPPER(MID(W206,4,1))="L","LLP",IF(UPPER(MID(W206,4,1))="T","Trust",IF(UPPER(MID(W206,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B206="Entry",IF(LEN(W206)&lt;4,"",IF(UPPER(MID(W206,4,1))="P","Individual",IF(UPPER(MID(W206,4,1))="H","HUF",IF(UPPER(MID(W206,4,1))="C","Company",IF(UPPER(MID(W206,4,1))="F","Firm",IF(UPPER(MID(W206,4,1))="L","LLP",IF(UPPER(MID(W206,4,1))="T","Trust",IF(UPPER(MID(W206,4,1))="A","AOP","")))))))),IF($B206="Challan","",IF(W206&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z206" s="28"/>
       <c r="AA206" s="29">
@@ -18856,10 +18856,10 @@
       <c r="V207" s="28"/>
       <c r="W207" s="28"/>
       <c r="X207" s="23">
-        <f>IF($B207&lt;&gt;"Entry","",IF(AND(LEN(TRIM(UPPER(W207)))=10,CODE(MID(TRIM(UPPER(W207)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W207)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W207)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W207)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),9,1))&lt;=57),"N","Y"))</f>
+        <f>IF($B207="Entry",IF(AND(LEN(TRIM(UPPER(W207)))=10,CODE(MID(TRIM(UPPER(W207)),1,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),1,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),2,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),2,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),3,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),3,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),4,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),4,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),5,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),5,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),10,1))&gt;=65,CODE(MID(TRIM(UPPER(W207)),10,1))&lt;=90,CODE(MID(TRIM(UPPER(W207)),6,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),6,1))&lt;=57,CODE(MID(TRIM(UPPER(W207)),7,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),7,1))&lt;=57,CODE(MID(TRIM(UPPER(W207)),8,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),8,1))&lt;=57,CODE(MID(TRIM(UPPER(W207)),9,1))&gt;=48,CODE(MID(TRIM(UPPER(W207)),9,1))&lt;=57),"N","Y"),IF($B207="Challan","",IF(W207&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Y207" s="23">
-        <f>IF($B207&lt;&gt;"Entry","",IF(LEN(W207)&lt;4,"",IF(UPPER(MID(W207,4,1))="P","Individual",IF(UPPER(MID(W207,4,1))="H","HUF",IF(UPPER(MID(W207,4,1))="C","Company",IF(UPPER(MID(W207,4,1))="F","Firm",IF(UPPER(MID(W207,4,1))="L","LLP",IF(UPPER(MID(W207,4,1))="T","Trust",IF(UPPER(MID(W207,4,1))="A","AOP",""))))))))</f>
+        <f>IF($B207="Entry",IF(LEN(W207)&lt;4,"",IF(UPPER(MID(W207,4,1))="P","Individual",IF(UPPER(MID(W207,4,1))="H","HUF",IF(UPPER(MID(W207,4,1))="C","Company",IF(UPPER(MID(W207,4,1))="F","Firm",IF(UPPER(MID(W207,4,1))="L","LLP",IF(UPPER(MID(W207,4,1))="T","Trust",IF(UPPER(MID(W207,4,1))="A","AOP","")))))))),IF($B207="Challan","",IF(W207&lt;&gt;"","◄ Set Row Type","")))</f>
       </c>
       <c r="Z207" s="28"/>
       <c r="AA207" s="29">

</xml_diff>